<commit_message>
tracker: note feature/swiggy-prompt-injection deleted, superseded by merged fix branch
P6-S14 was never independently PR-ed to dev -- fix/swiggy-sse-market-intel
branched off its tip and shipped it as part of PR #87 instead. Deleted the
now-fully-superseded feature/swiggy-prompt-injection branch (remote + local)
and recorded the merge on the P6-S35 row.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -346,7 +346,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -488,11 +488,44 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00C9C9C9"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9C9C9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9C9C9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9C9C9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9C9C9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9C9C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -812,6 +845,8 @@
     <xf numFmtId="0" fontId="25" fillId="32" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13785,7 +13820,7 @@
           <t>P6-S02</t>
         </is>
       </c>
-      <c r="B9" s="101" t="n"/>
+      <c r="B9" s="113" t="n"/>
       <c r="C9" s="102" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -14028,7 +14063,7 @@
           <t>P6-S03c</t>
         </is>
       </c>
-      <c r="B14" s="92" t="n"/>
+      <c r="B14" s="113" t="n"/>
       <c r="C14" s="93" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -14271,7 +14306,7 @@
           <t>P6-S06</t>
         </is>
       </c>
-      <c r="B19" s="101" t="n"/>
+      <c r="B19" s="113" t="n"/>
       <c r="C19" s="102" t="inlineStr">
         <is>
           <t>Integrations</t>
@@ -14426,7 +14461,7 @@
           <t>P6-S08</t>
         </is>
       </c>
-      <c r="B22" s="92" t="n"/>
+      <c r="B22" s="114" t="n"/>
       <c r="C22" s="93" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14491,7 +14526,7 @@
           <t>P6-S09</t>
         </is>
       </c>
-      <c r="B23" s="101" t="n"/>
+      <c r="B23" s="113" t="n"/>
       <c r="C23" s="102" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14644,7 +14679,7 @@
           <t>P6-S11</t>
         </is>
       </c>
-      <c r="B26" s="92" t="n"/>
+      <c r="B26" s="114" t="n"/>
       <c r="C26" s="93" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14711,7 +14746,7 @@
           <t>P6-S12</t>
         </is>
       </c>
-      <c r="B27" s="101" t="n"/>
+      <c r="B27" s="114" t="n"/>
       <c r="C27" s="102" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14778,7 +14813,7 @@
           <t>P6-S13</t>
         </is>
       </c>
-      <c r="B28" s="92" t="n"/>
+      <c r="B28" s="113" t="n"/>
       <c r="C28" s="93" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15021,7 +15056,7 @@
           <t>P6-F15</t>
         </is>
       </c>
-      <c r="B33" s="101" t="n"/>
+      <c r="B33" s="114" t="n"/>
       <c r="C33" s="102" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15088,7 +15123,7 @@
           <t>P6-F16</t>
         </is>
       </c>
-      <c r="B34" s="92" t="n"/>
+      <c r="B34" s="114" t="n"/>
       <c r="C34" s="93" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -15137,7 +15172,7 @@
           <t>P6-F16b</t>
         </is>
       </c>
-      <c r="B35" s="101" t="n"/>
+      <c r="B35" s="114" t="n"/>
       <c r="C35" s="102" t="inlineStr">
         <is>
           <t>Docs</t>
@@ -15186,7 +15221,7 @@
           <t>P6-F17</t>
         </is>
       </c>
-      <c r="B36" s="92" t="n"/>
+      <c r="B36" s="113" t="n"/>
       <c r="C36" s="93" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15272,7 +15307,7 @@
       </c>
       <c r="B38" s="92" t="inlineStr">
         <is>
-          <t>feature/swiggy-prompt-injection</t>
+          <t>feature/swiggy-prompt-injection (deleted post-merge)</t>
         </is>
       </c>
       <c r="C38" s="93" t="inlineStr">
@@ -15287,7 +15322,7 @@
       </c>
       <c r="E38" s="94" t="inlineStr">
         <is>
-          <t>Swiggy enricher prompt_text injected into 3 LLM prompts: (1) menu_intelligence gets ## Market Context (competitor prices, alerts); (2) inventory gets ## Live Procurement Options (Instamart prices per shortage item); (3) reservation gets ## Occupancy Signal (area HIGH/MEDIUM/LOW). LLM now references Swiggy data in reasoning — e.g. "Order tomatoes via Instamart at Rs.24/kg". Frontend: AgentCard swiggySignal prop shows orange Swiggy badge in card header with one-line market signal (area tonight: HIGH, 5 Instamart prices live, 2 pricing alerts).</t>
+          <t>Swiggy enricher prompt_text injected into 3 LLM prompts: (1) menu_intelligence gets ## Market Context (competitor prices, alerts); (2) inventory gets ## Live Procurement Options (Instamart prices per shortage item); (3) reservation gets ## Occupancy Signal (area HIGH/MEDIUM/LOW). LLM now references Swiggy data in reasoning — e.g. "Order tomatoes via Instamart at Rs.24/kg". Frontend: AgentCard swiggySignal prop shows orange Swiggy badge in card header with one-line market signal (area tonight: HIGH, 5 Instamart prices live, 2 pricing alerts). Never independently PR-ed to dev -- fix/swiggy-sse-market-intel branched off its tip and shipped it as part of that PR instead; feature/swiggy-prompt-injection deleted 2026-07-03 (remote + local), fully superseded.</t>
         </is>
       </c>
       <c r="F38" s="94" t="inlineStr">
@@ -15357,7 +15392,7 @@
       </c>
       <c r="E40" s="94" t="inlineStr">
         <is>
-          <t>Fixed Instamart procurement card rendering nothing despite live shortage data: frontend read item.name/item.in_stock but backend ProcurementEnricher sends item.ingredient/item.inStock (confirmed against the enricher's own test contract). Found and fixed a cost/token-attribution race: reservation and inventory nodes share the 'fast' LLM tier and run in true parallel; _inject() draining the shared provider usage buffer at node start/end let one node's drain steal the other's usage records. Fixed via per-node contextvar tagging (bind_llm_usage_node/drain_usage(node=...)) in llm/base.py + graph.py. Converted ~11 files across the Swiggy integration layer + cache/vector-memory infra from stdlib logging to structlog -- the app never calls logging.basicConfig(), so every .info()/.debug() call on those modules was being silently dropped, and .warning() lines printed unstructured with no run correlation.</t>
+          <t>Fixed Instamart procurement card rendering nothing despite live shortage data: frontend read item.name/item.in_stock but backend ProcurementEnricher sends item.ingredient/item.inStock (confirmed against the enricher's own test contract). Found and fixed a cost/token-attribution race: reservation and inventory nodes share the 'fast' LLM tier and run in true parallel; _inject() draining the shared provider usage buffer at node start/end let one node's drain steal the other's usage records. Fixed via per-node contextvar tagging (bind_llm_usage_node/drain_usage(node=...)) in llm/base.py + graph.py. Converted ~11 files across the Swiggy integration layer + cache/vector-memory infra from stdlib logging to structlog -- the app never calls logging.basicConfig(), so every .info()/.debug() call on those modules was being silently dropped, and .warning() lines printed unstructured with no run correlation. Merged to dev via PR #87, 2026-07-03.</t>
         </is>
       </c>
       <c r="F40" s="94" t="inlineStr">
@@ -15411,7 +15446,7 @@
           <t>P6-S36</t>
         </is>
       </c>
-      <c r="B41" s="101" t="n"/>
+      <c r="B41" s="114" t="n"/>
       <c r="C41" s="102" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15478,7 +15513,7 @@
           <t>P6-S37</t>
         </is>
       </c>
-      <c r="B42" s="92" t="n"/>
+      <c r="B42" s="114" t="n"/>
       <c r="C42" s="93" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -15545,7 +15580,7 @@
           <t>P6-S38</t>
         </is>
       </c>
-      <c r="B43" s="101" t="n"/>
+      <c r="B43" s="114" t="n"/>
       <c r="C43" s="102" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15612,7 +15647,7 @@
           <t>P6-S39</t>
         </is>
       </c>
-      <c r="B44" s="92" t="n"/>
+      <c r="B44" s="114" t="n"/>
       <c r="C44" s="93" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15679,7 +15714,7 @@
           <t>P6-S40</t>
         </is>
       </c>
-      <c r="B45" s="101" t="n"/>
+      <c r="B45" s="114" t="n"/>
       <c r="C45" s="102" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15746,7 +15781,7 @@
           <t>P6-S41</t>
         </is>
       </c>
-      <c r="B46" s="92" t="n"/>
+      <c r="B46" s="114" t="n"/>
       <c r="C46" s="93" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15813,7 +15848,7 @@
           <t>P6-S42</t>
         </is>
       </c>
-      <c r="B47" s="101" t="n"/>
+      <c r="B47" s="114" t="n"/>
       <c r="C47" s="102" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15880,7 +15915,7 @@
           <t>P6-S47</t>
         </is>
       </c>
-      <c r="B48" s="92" t="n"/>
+      <c r="B48" s="114" t="n"/>
       <c r="C48" s="93" t="inlineStr">
         <is>
           <t>Security</t>
@@ -15939,7 +15974,7 @@
           <t>P6-S48</t>
         </is>
       </c>
-      <c r="B49" s="101" t="n"/>
+      <c r="B49" s="113" t="n"/>
       <c r="C49" s="102" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16023,20 +16058,20 @@
           <t>DO FIRST — no staging creds needed  |  each task: own branch → PR → merge dev → merge main → docs + screenshots + tracker updated</t>
         </is>
       </c>
-      <c r="B51" s="109" t="n"/>
-      <c r="C51" s="109" t="n"/>
-      <c r="D51" s="109" t="n"/>
-      <c r="E51" s="109" t="n"/>
-      <c r="F51" s="109" t="n"/>
-      <c r="G51" s="109" t="n"/>
-      <c r="H51" s="109" t="n"/>
-      <c r="I51" s="109" t="n"/>
-      <c r="J51" s="109" t="n"/>
-      <c r="K51" s="109" t="n"/>
-      <c r="L51" s="109" t="n"/>
-      <c r="M51" s="109" t="n"/>
-      <c r="N51" s="109" t="n"/>
-      <c r="O51" s="109" t="n"/>
+      <c r="B51" s="61" t="n"/>
+      <c r="C51" s="61" t="n"/>
+      <c r="D51" s="61" t="n"/>
+      <c r="E51" s="61" t="n"/>
+      <c r="F51" s="61" t="n"/>
+      <c r="G51" s="61" t="n"/>
+      <c r="H51" s="61" t="n"/>
+      <c r="I51" s="61" t="n"/>
+      <c r="J51" s="61" t="n"/>
+      <c r="K51" s="61" t="n"/>
+      <c r="L51" s="61" t="n"/>
+      <c r="M51" s="61" t="n"/>
+      <c r="N51" s="61" t="n"/>
+      <c r="O51" s="61" t="n"/>
     </row>
     <row r="52" ht="8" customHeight="1" s="65">
       <c r="A52" s="99" t="n"/>
@@ -16114,7 +16149,7 @@
           <t>P6-MI02</t>
         </is>
       </c>
-      <c r="B54" s="92" t="n"/>
+      <c r="B54" s="114" t="n"/>
       <c r="C54" s="93" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16163,7 +16198,7 @@
           <t>P6-MI03</t>
         </is>
       </c>
-      <c r="B55" s="101" t="n"/>
+      <c r="B55" s="113" t="n"/>
       <c r="C55" s="102" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -17543,20 +17578,20 @@
           <t>→ DEMO 1  |  all above on main, docs updated, screenshots done — record full Swiggy read + AI + voice + live monitor demo ←</t>
         </is>
       </c>
-      <c r="B89" s="109" t="n"/>
-      <c r="C89" s="109" t="n"/>
-      <c r="D89" s="109" t="n"/>
-      <c r="E89" s="109" t="n"/>
-      <c r="F89" s="109" t="n"/>
-      <c r="G89" s="109" t="n"/>
-      <c r="H89" s="109" t="n"/>
-      <c r="I89" s="109" t="n"/>
-      <c r="J89" s="109" t="n"/>
-      <c r="K89" s="109" t="n"/>
-      <c r="L89" s="109" t="n"/>
-      <c r="M89" s="109" t="n"/>
-      <c r="N89" s="109" t="n"/>
-      <c r="O89" s="109" t="n"/>
+      <c r="B89" s="61" t="n"/>
+      <c r="C89" s="61" t="n"/>
+      <c r="D89" s="61" t="n"/>
+      <c r="E89" s="61" t="n"/>
+      <c r="F89" s="61" t="n"/>
+      <c r="G89" s="61" t="n"/>
+      <c r="H89" s="61" t="n"/>
+      <c r="I89" s="61" t="n"/>
+      <c r="J89" s="61" t="n"/>
+      <c r="K89" s="61" t="n"/>
+      <c r="L89" s="61" t="n"/>
+      <c r="M89" s="61" t="n"/>
+      <c r="N89" s="61" t="n"/>
+      <c r="O89" s="61" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
tracker: fix P6-S42 ID collision, restore sequential S-numbering across both sheets
Adding P6-S42 for the CI dependency-conflict fix (previous commit) collided
with an already-existing P6-S42 (ProcurementExecutor) on the Staging Creds +
Phase 7 sheet -- missed because that task lives on a different sheet than
where the new row was added. Renumbered the entire S31..S46 tail (spanning
both Phase 6 and Staging Creds + Phase 7 sheets) up by one so the CI-fix task
takes S31 (the correct next slot after S30) and every task after it shifts
to S32..S47, with all Depends On cross-references updated to match. Verified
no duplicate Task IDs remain anywhere in the workbook.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -20,10 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -458,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -640,6 +639,7 @@
     <xf numFmtId="0" fontId="24" fillId="28" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="19" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -651,11 +651,13 @@
     <xf numFmtId="0" fontId="15" fillId="25" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -673,20 +675,11 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -981,7 +974,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" s="72">
-      <c r="A1" s="83" t="inlineStr">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>CortexKitchen — Project Dashboard</t>
         </is>
@@ -1019,7 +1012,7 @@
     <row r="3" ht="14.4" customHeight="1" s="72">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Current milestone: Phase 6 -- P6-S21-S30 (this branch's hardening fixes) complete; inventory now cites live Swiggy Instamart prices end-to-end, replan loop + critic converge to approved on first pass. Next: P6-MI01-04 (market intel expansion) or P6-S38-S41 (follow-ups).</t>
+          <t>Current milestone: Phase 6 -- P6-S21-S30 (this branch's hardening fixes) complete; inventory now cites live Swiggy Instamart prices end-to-end, replan loop + critic converge to approved on first pass. Next: P6-MI01-04 (market intel expansion) or P6-S39-S41 (follow-ups).</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1132,7 +1125,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Pending from Swiggy. Needed ONLY for checkout + book_table (P6-S42, P6-S43). Everything else works with production OAuth token.</t>
+          <t>Pending from Swiggy. Needed ONLY for checkout + book_table (P6-S43, P6-S44). Everything else works with production OAuth token.</t>
         </is>
       </c>
       <c r="C6" s="1" t="n"/>
@@ -8023,34 +8016,34 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" s="72">
-      <c r="A1" s="84" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>CortexKitchen — Phase Tracker (P0 through P6-S11 complete)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16.05" customHeight="1" s="72">
-      <c r="A2" s="78" t="inlineStr">
+      <c r="A2" s="79" t="inlineStr">
         <is>
           <t>Phase 6 planned tasks (P6-01 onwards) live in the Phase 6 sheet  ·  This sheet = historical record only</t>
         </is>
       </c>
-      <c r="B2" s="74" t="n"/>
-      <c r="C2" s="74" t="n"/>
-      <c r="D2" s="74" t="n"/>
-      <c r="E2" s="74" t="n"/>
-      <c r="F2" s="74" t="n"/>
-      <c r="G2" s="74" t="n"/>
-      <c r="H2" s="74" t="n"/>
-      <c r="I2" s="74" t="n"/>
-      <c r="J2" s="74" t="n"/>
-      <c r="K2" s="74" t="n"/>
-      <c r="L2" s="74" t="n"/>
-      <c r="M2" s="74" t="n"/>
-      <c r="N2" s="74" t="n"/>
-      <c r="O2" s="74" t="n"/>
-      <c r="P2" s="74" t="n"/>
-      <c r="Q2" s="75" t="n"/>
+      <c r="B2" s="75" t="n"/>
+      <c r="C2" s="75" t="n"/>
+      <c r="D2" s="75" t="n"/>
+      <c r="E2" s="75" t="n"/>
+      <c r="F2" s="75" t="n"/>
+      <c r="G2" s="75" t="n"/>
+      <c r="H2" s="75" t="n"/>
+      <c r="I2" s="75" t="n"/>
+      <c r="J2" s="75" t="n"/>
+      <c r="K2" s="75" t="n"/>
+      <c r="L2" s="75" t="n"/>
+      <c r="M2" s="75" t="n"/>
+      <c r="N2" s="75" t="n"/>
+      <c r="O2" s="75" t="n"/>
+      <c r="P2" s="75" t="n"/>
+      <c r="Q2" s="76" t="n"/>
     </row>
     <row r="3" ht="19.95" customHeight="1" s="72">
       <c r="A3" s="5" t="inlineStr">
@@ -8140,27 +8133,27 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" s="72">
-      <c r="A4" s="77" t="inlineStr">
+      <c r="A4" s="78" t="inlineStr">
         <is>
           <t>Phase 0</t>
         </is>
       </c>
-      <c r="B4" s="74" t="n"/>
-      <c r="C4" s="74" t="n"/>
-      <c r="D4" s="74" t="n"/>
-      <c r="E4" s="74" t="n"/>
-      <c r="F4" s="74" t="n"/>
-      <c r="G4" s="74" t="n"/>
-      <c r="H4" s="74" t="n"/>
-      <c r="I4" s="74" t="n"/>
-      <c r="J4" s="74" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="74" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="74" t="n"/>
-      <c r="O4" s="74" t="n"/>
-      <c r="P4" s="74" t="n"/>
-      <c r="Q4" s="75" t="n"/>
+      <c r="B4" s="75" t="n"/>
+      <c r="C4" s="75" t="n"/>
+      <c r="D4" s="75" t="n"/>
+      <c r="E4" s="75" t="n"/>
+      <c r="F4" s="75" t="n"/>
+      <c r="G4" s="75" t="n"/>
+      <c r="H4" s="75" t="n"/>
+      <c r="I4" s="75" t="n"/>
+      <c r="J4" s="75" t="n"/>
+      <c r="K4" s="75" t="n"/>
+      <c r="L4" s="75" t="n"/>
+      <c r="M4" s="75" t="n"/>
+      <c r="N4" s="75" t="n"/>
+      <c r="O4" s="75" t="n"/>
+      <c r="P4" s="75" t="n"/>
+      <c r="Q4" s="76" t="n"/>
     </row>
     <row r="5" ht="48" customHeight="1" s="72">
       <c r="A5" s="19" t="inlineStr">
@@ -8548,27 +8541,27 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" s="72">
-      <c r="A10" s="77" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
         <is>
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="B10" s="74" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="74" t="n"/>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="74" t="n"/>
-      <c r="H10" s="74" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="74" t="n"/>
-      <c r="M10" s="74" t="n"/>
-      <c r="N10" s="74" t="n"/>
-      <c r="O10" s="74" t="n"/>
-      <c r="P10" s="74" t="n"/>
-      <c r="Q10" s="75" t="n"/>
+      <c r="B10" s="75" t="n"/>
+      <c r="C10" s="75" t="n"/>
+      <c r="D10" s="75" t="n"/>
+      <c r="E10" s="75" t="n"/>
+      <c r="F10" s="75" t="n"/>
+      <c r="G10" s="75" t="n"/>
+      <c r="H10" s="75" t="n"/>
+      <c r="I10" s="75" t="n"/>
+      <c r="J10" s="75" t="n"/>
+      <c r="K10" s="75" t="n"/>
+      <c r="L10" s="75" t="n"/>
+      <c r="M10" s="75" t="n"/>
+      <c r="N10" s="75" t="n"/>
+      <c r="O10" s="75" t="n"/>
+      <c r="P10" s="75" t="n"/>
+      <c r="Q10" s="76" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1" s="72">
       <c r="A11" s="24" t="inlineStr">
@@ -9501,27 +9494,27 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="72">
-      <c r="A23" s="76" t="inlineStr">
+      <c r="A23" s="77" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="B23" s="74" t="n"/>
-      <c r="C23" s="74" t="n"/>
-      <c r="D23" s="74" t="n"/>
-      <c r="E23" s="74" t="n"/>
-      <c r="F23" s="74" t="n"/>
-      <c r="G23" s="74" t="n"/>
-      <c r="H23" s="74" t="n"/>
-      <c r="I23" s="74" t="n"/>
-      <c r="J23" s="74" t="n"/>
-      <c r="K23" s="74" t="n"/>
-      <c r="L23" s="74" t="n"/>
-      <c r="M23" s="74" t="n"/>
-      <c r="N23" s="74" t="n"/>
-      <c r="O23" s="74" t="n"/>
-      <c r="P23" s="74" t="n"/>
-      <c r="Q23" s="75" t="n"/>
+      <c r="B23" s="75" t="n"/>
+      <c r="C23" s="75" t="n"/>
+      <c r="D23" s="75" t="n"/>
+      <c r="E23" s="75" t="n"/>
+      <c r="F23" s="75" t="n"/>
+      <c r="G23" s="75" t="n"/>
+      <c r="H23" s="75" t="n"/>
+      <c r="I23" s="75" t="n"/>
+      <c r="J23" s="75" t="n"/>
+      <c r="K23" s="75" t="n"/>
+      <c r="L23" s="75" t="n"/>
+      <c r="M23" s="75" t="n"/>
+      <c r="N23" s="75" t="n"/>
+      <c r="O23" s="75" t="n"/>
+      <c r="P23" s="75" t="n"/>
+      <c r="Q23" s="76" t="n"/>
     </row>
     <row r="24" ht="48" customHeight="1" s="72">
       <c r="A24" s="24" t="inlineStr">
@@ -9986,27 +9979,27 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="72">
-      <c r="A30" s="76" t="inlineStr">
+      <c r="A30" s="77" t="inlineStr">
         <is>
           <t>Phase 3</t>
         </is>
       </c>
-      <c r="B30" s="74" t="n"/>
-      <c r="C30" s="74" t="n"/>
-      <c r="D30" s="74" t="n"/>
-      <c r="E30" s="74" t="n"/>
-      <c r="F30" s="74" t="n"/>
-      <c r="G30" s="74" t="n"/>
-      <c r="H30" s="74" t="n"/>
-      <c r="I30" s="74" t="n"/>
-      <c r="J30" s="74" t="n"/>
-      <c r="K30" s="74" t="n"/>
-      <c r="L30" s="74" t="n"/>
-      <c r="M30" s="74" t="n"/>
-      <c r="N30" s="74" t="n"/>
-      <c r="O30" s="74" t="n"/>
-      <c r="P30" s="74" t="n"/>
-      <c r="Q30" s="75" t="n"/>
+      <c r="B30" s="75" t="n"/>
+      <c r="C30" s="75" t="n"/>
+      <c r="D30" s="75" t="n"/>
+      <c r="E30" s="75" t="n"/>
+      <c r="F30" s="75" t="n"/>
+      <c r="G30" s="75" t="n"/>
+      <c r="H30" s="75" t="n"/>
+      <c r="I30" s="75" t="n"/>
+      <c r="J30" s="75" t="n"/>
+      <c r="K30" s="75" t="n"/>
+      <c r="L30" s="75" t="n"/>
+      <c r="M30" s="75" t="n"/>
+      <c r="N30" s="75" t="n"/>
+      <c r="O30" s="75" t="n"/>
+      <c r="P30" s="75" t="n"/>
+      <c r="Q30" s="76" t="n"/>
     </row>
     <row r="31" ht="48" customHeight="1" s="72">
       <c r="A31" s="24" t="inlineStr">
@@ -10394,27 +10387,27 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" s="72">
-      <c r="A36" s="81" t="inlineStr">
+      <c r="A36" s="82" t="inlineStr">
         <is>
           <t>Demo prep</t>
         </is>
       </c>
-      <c r="B36" s="74" t="n"/>
-      <c r="C36" s="74" t="n"/>
-      <c r="D36" s="74" t="n"/>
-      <c r="E36" s="74" t="n"/>
-      <c r="F36" s="74" t="n"/>
-      <c r="G36" s="74" t="n"/>
-      <c r="H36" s="74" t="n"/>
-      <c r="I36" s="74" t="n"/>
-      <c r="J36" s="74" t="n"/>
-      <c r="K36" s="74" t="n"/>
-      <c r="L36" s="74" t="n"/>
-      <c r="M36" s="74" t="n"/>
-      <c r="N36" s="74" t="n"/>
-      <c r="O36" s="74" t="n"/>
-      <c r="P36" s="74" t="n"/>
-      <c r="Q36" s="75" t="n"/>
+      <c r="B36" s="75" t="n"/>
+      <c r="C36" s="75" t="n"/>
+      <c r="D36" s="75" t="n"/>
+      <c r="E36" s="75" t="n"/>
+      <c r="F36" s="75" t="n"/>
+      <c r="G36" s="75" t="n"/>
+      <c r="H36" s="75" t="n"/>
+      <c r="I36" s="75" t="n"/>
+      <c r="J36" s="75" t="n"/>
+      <c r="K36" s="75" t="n"/>
+      <c r="L36" s="75" t="n"/>
+      <c r="M36" s="75" t="n"/>
+      <c r="N36" s="75" t="n"/>
+      <c r="O36" s="75" t="n"/>
+      <c r="P36" s="75" t="n"/>
+      <c r="Q36" s="76" t="n"/>
     </row>
     <row r="37" ht="48" customHeight="1" s="72">
       <c r="A37" s="32" t="inlineStr">
@@ -10648,27 +10641,27 @@
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="72">
-      <c r="A40" s="73" t="inlineStr">
+      <c r="A40" s="74" t="inlineStr">
         <is>
           <t>Phase 4</t>
         </is>
       </c>
-      <c r="B40" s="74" t="n"/>
-      <c r="C40" s="74" t="n"/>
-      <c r="D40" s="74" t="n"/>
-      <c r="E40" s="74" t="n"/>
-      <c r="F40" s="74" t="n"/>
-      <c r="G40" s="74" t="n"/>
-      <c r="H40" s="74" t="n"/>
-      <c r="I40" s="74" t="n"/>
-      <c r="J40" s="74" t="n"/>
-      <c r="K40" s="74" t="n"/>
-      <c r="L40" s="74" t="n"/>
-      <c r="M40" s="74" t="n"/>
-      <c r="N40" s="74" t="n"/>
-      <c r="O40" s="74" t="n"/>
-      <c r="P40" s="74" t="n"/>
-      <c r="Q40" s="75" t="n"/>
+      <c r="B40" s="75" t="n"/>
+      <c r="C40" s="75" t="n"/>
+      <c r="D40" s="75" t="n"/>
+      <c r="E40" s="75" t="n"/>
+      <c r="F40" s="75" t="n"/>
+      <c r="G40" s="75" t="n"/>
+      <c r="H40" s="75" t="n"/>
+      <c r="I40" s="75" t="n"/>
+      <c r="J40" s="75" t="n"/>
+      <c r="K40" s="75" t="n"/>
+      <c r="L40" s="75" t="n"/>
+      <c r="M40" s="75" t="n"/>
+      <c r="N40" s="75" t="n"/>
+      <c r="O40" s="75" t="n"/>
+      <c r="P40" s="75" t="n"/>
+      <c r="Q40" s="76" t="n"/>
     </row>
     <row r="41" ht="48" customHeight="1" s="72">
       <c r="A41" s="24" t="inlineStr">
@@ -11672,27 +11665,27 @@
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" s="72">
-      <c r="A54" s="73" t="inlineStr">
+      <c r="A54" s="74" t="inlineStr">
         <is>
           <t>Phase 5</t>
         </is>
       </c>
-      <c r="B54" s="74" t="n"/>
-      <c r="C54" s="74" t="n"/>
-      <c r="D54" s="74" t="n"/>
-      <c r="E54" s="74" t="n"/>
-      <c r="F54" s="74" t="n"/>
-      <c r="G54" s="74" t="n"/>
-      <c r="H54" s="74" t="n"/>
-      <c r="I54" s="74" t="n"/>
-      <c r="J54" s="74" t="n"/>
-      <c r="K54" s="74" t="n"/>
-      <c r="L54" s="74" t="n"/>
-      <c r="M54" s="74" t="n"/>
-      <c r="N54" s="74" t="n"/>
-      <c r="O54" s="74" t="n"/>
-      <c r="P54" s="74" t="n"/>
-      <c r="Q54" s="75" t="n"/>
+      <c r="B54" s="75" t="n"/>
+      <c r="C54" s="75" t="n"/>
+      <c r="D54" s="75" t="n"/>
+      <c r="E54" s="75" t="n"/>
+      <c r="F54" s="75" t="n"/>
+      <c r="G54" s="75" t="n"/>
+      <c r="H54" s="75" t="n"/>
+      <c r="I54" s="75" t="n"/>
+      <c r="J54" s="75" t="n"/>
+      <c r="K54" s="75" t="n"/>
+      <c r="L54" s="75" t="n"/>
+      <c r="M54" s="75" t="n"/>
+      <c r="N54" s="75" t="n"/>
+      <c r="O54" s="75" t="n"/>
+      <c r="P54" s="75" t="n"/>
+      <c r="Q54" s="76" t="n"/>
     </row>
     <row r="55" ht="48" customHeight="1" s="72">
       <c r="A55" s="19" t="inlineStr">
@@ -12618,27 +12611,27 @@
       </c>
     </row>
     <row r="68" ht="18" customHeight="1" s="72">
-      <c r="A68" s="79" t="inlineStr">
+      <c r="A68" s="80" t="inlineStr">
         <is>
           <t>Phase 6</t>
         </is>
       </c>
-      <c r="B68" s="74" t="n"/>
-      <c r="C68" s="74" t="n"/>
-      <c r="D68" s="74" t="n"/>
-      <c r="E68" s="74" t="n"/>
-      <c r="F68" s="74" t="n"/>
-      <c r="G68" s="74" t="n"/>
-      <c r="H68" s="74" t="n"/>
-      <c r="I68" s="74" t="n"/>
-      <c r="J68" s="74" t="n"/>
-      <c r="K68" s="74" t="n"/>
-      <c r="L68" s="74" t="n"/>
-      <c r="M68" s="74" t="n"/>
-      <c r="N68" s="74" t="n"/>
-      <c r="O68" s="74" t="n"/>
-      <c r="P68" s="74" t="n"/>
-      <c r="Q68" s="75" t="n"/>
+      <c r="B68" s="75" t="n"/>
+      <c r="C68" s="75" t="n"/>
+      <c r="D68" s="75" t="n"/>
+      <c r="E68" s="75" t="n"/>
+      <c r="F68" s="75" t="n"/>
+      <c r="G68" s="75" t="n"/>
+      <c r="H68" s="75" t="n"/>
+      <c r="I68" s="75" t="n"/>
+      <c r="J68" s="75" t="n"/>
+      <c r="K68" s="75" t="n"/>
+      <c r="L68" s="75" t="n"/>
+      <c r="M68" s="75" t="n"/>
+      <c r="N68" s="75" t="n"/>
+      <c r="O68" s="75" t="n"/>
+      <c r="P68" s="75" t="n"/>
+      <c r="Q68" s="76" t="n"/>
     </row>
     <row r="69" ht="48" customHeight="1" s="72">
       <c r="A69" s="24" t="inlineStr">
@@ -13229,22 +13222,23 @@
   <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col width="12" customWidth="1" style="40" min="1" max="1"/>
-    <col width="27" customWidth="1" style="40" min="2" max="2"/>
-    <col width="15" customWidth="1" style="40" min="3" max="3"/>
-    <col width="32" customWidth="1" style="40" min="4" max="4"/>
-    <col width="58" customWidth="1" style="40" min="5" max="5"/>
-    <col width="40" customWidth="1" style="40" min="6" max="6"/>
-    <col width="30" customWidth="1" style="40" min="7" max="7"/>
-    <col width="13" customWidth="1" style="40" min="8" max="8"/>
-    <col width="11" customWidth="1" style="40" min="9" max="9"/>
+    <col width="12" customWidth="1" style="71" min="1" max="1"/>
+    <col width="27" customWidth="1" style="71" min="2" max="2"/>
+    <col width="15" customWidth="1" style="71" min="3" max="3"/>
+    <col width="32" customWidth="1" style="71" min="4" max="4"/>
+    <col width="58" customWidth="1" style="71" min="5" max="5"/>
+    <col width="40" customWidth="1" style="71" min="6" max="6"/>
+    <col width="30" customWidth="1" style="71" min="7" max="7"/>
+    <col width="13" customWidth="1" style="71" min="8" max="8"/>
+    <col width="11" customWidth="1" style="71" min="9" max="9"/>
     <col width="10" customWidth="1" style="72" min="10" max="10"/>
-    <col width="12" customWidth="1" style="40" min="11" max="11"/>
+    <col width="12" customWidth="1" style="71" min="11" max="11"/>
     <col width="12" customWidth="1" style="72" min="12" max="12"/>
     <col width="9" customWidth="1" style="72" min="13" max="13"/>
     <col width="16" customWidth="1" style="72" min="14" max="14"/>
     <col width="46" customWidth="1" style="72" min="15" max="15"/>
-    <col width="12" customWidth="1" style="40" min="16" max="16384"/>
+    <col width="12" customWidth="1" style="71" min="16" max="16"/>
+    <col width="12" customWidth="1" style="71" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.95" customHeight="1" s="72">
@@ -13330,7 +13324,7 @@
           <t>P6-S01</t>
         </is>
       </c>
-      <c r="B2" s="65" t="inlineStr">
+      <c r="B2" s="66" t="inlineStr">
         <is>
           <t>feature/per-node-model-routing</t>
         </is>
@@ -13418,7 +13412,7 @@
           <t>P6-S02</t>
         </is>
       </c>
-      <c r="B4" s="65" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
         <is>
           <t>feature/assumption-diffing</t>
         </is>
@@ -13506,7 +13500,7 @@
           <t>P6-S03</t>
         </is>
       </c>
-      <c r="B6" s="65" t="inlineStr">
+      <c r="B6" s="66" t="inlineStr">
         <is>
           <t>feature/drop-diff1-reseed-data</t>
         </is>
@@ -13594,7 +13588,7 @@
           <t>P6-S04</t>
         </is>
       </c>
-      <c r="B8" s="65" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
         <is>
           <t>feature/swiggy-base-connector</t>
         </is>
@@ -13665,7 +13659,7 @@
           <t>P6-S05</t>
         </is>
       </c>
-      <c r="B9" s="67" t="n"/>
+      <c r="B9" s="68" t="n"/>
       <c r="C9" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -13749,7 +13743,7 @@
           <t>P6-S06</t>
         </is>
       </c>
-      <c r="B11" s="68" t="inlineStr">
+      <c r="B11" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-sync-orders</t>
         </is>
@@ -13837,7 +13831,7 @@
           <t>P6-S07</t>
         </is>
       </c>
-      <c r="B13" s="68" t="inlineStr">
+      <c r="B13" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-base-connector</t>
         </is>
@@ -13908,7 +13902,7 @@
           <t>P6-S08</t>
         </is>
       </c>
-      <c r="B14" s="67" t="n"/>
+      <c r="B14" s="68" t="n"/>
       <c r="C14" s="46" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -13992,7 +13986,7 @@
           <t>P6-S09</t>
         </is>
       </c>
-      <c r="B16" s="65" t="inlineStr">
+      <c r="B16" s="66" t="inlineStr">
         <is>
           <t>feature/agent-intelligence</t>
         </is>
@@ -14080,7 +14074,7 @@
           <t>P6-S10</t>
         </is>
       </c>
-      <c r="B18" s="65" t="inlineStr">
+      <c r="B18" s="66" t="inlineStr">
         <is>
           <t>feature/swiggy-sync-feedback-reservations</t>
         </is>
@@ -14102,7 +14096,7 @@
       </c>
       <c r="F18" s="47" t="inlineStr">
         <is>
-          <t>feat: reservation sync skeleton — get_booking_status → reservations table, register_booking_order_id for DineoutExecutor (P6-S43)</t>
+          <t>feat: reservation sync skeleton — get_booking_status → reservations table, register_booking_order_id for DineoutExecutor (P6-S44)</t>
         </is>
       </c>
       <c r="G18" s="47" t="inlineStr">
@@ -14151,7 +14145,7 @@
           <t>P6-S11</t>
         </is>
       </c>
-      <c r="B19" s="67" t="n"/>
+      <c r="B19" s="68" t="n"/>
       <c r="C19" s="55" t="inlineStr">
         <is>
           <t>Integrations</t>
@@ -14235,7 +14229,7 @@
           <t>P6-S12</t>
         </is>
       </c>
-      <c r="B21" s="68" t="inlineStr">
+      <c r="B21" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-market-intel-enrichers</t>
         </is>
@@ -14306,7 +14300,7 @@
           <t>P6-S13</t>
         </is>
       </c>
-      <c r="B22" s="66" t="n"/>
+      <c r="B22" s="67" t="n"/>
       <c r="C22" s="46" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14371,7 +14365,7 @@
           <t>P6-S14</t>
         </is>
       </c>
-      <c r="B23" s="67" t="n"/>
+      <c r="B23" s="68" t="n"/>
       <c r="C23" s="55" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14384,7 +14378,7 @@
       </c>
       <c r="E23" s="56" t="inlineStr">
         <is>
-          <t>Create enrichers/procurement.py. search_products (per shortage item, max 5 calls/run) + your_go_to_items (frequent reorders). Output: [{ingredient, spinId, price, unit, inStock}]. spinId MUST persist in OrchestratorState — required for Instamart checkout in P6-S42. Redis cache 30 min. Returns None on any failure; inventory node falls back to its own analysis.</t>
+          <t>Create enrichers/procurement.py. search_products (per shortage item, max 5 calls/run) + your_go_to_items (frequent reorders). Output: [{ingredient, spinId, price, unit, inStock}]. spinId MUST persist in OrchestratorState — required for Instamart checkout in P6-S43. Redis cache 30 min. Returns None on any failure; inventory node falls back to its own analysis.</t>
         </is>
       </c>
       <c r="F23" s="56" t="inlineStr">
@@ -14453,7 +14447,7 @@
           <t>P6-S15</t>
         </is>
       </c>
-      <c r="B25" s="68" t="inlineStr">
+      <c r="B25" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-market-intel-node</t>
         </is>
@@ -14524,7 +14518,7 @@
           <t>P6-S16</t>
         </is>
       </c>
-      <c r="B26" s="66" t="n"/>
+      <c r="B26" s="67" t="n"/>
       <c r="C26" s="46" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14591,7 +14585,7 @@
           <t>P6-S17</t>
         </is>
       </c>
-      <c r="B27" s="66" t="n"/>
+      <c r="B27" s="67" t="n"/>
       <c r="C27" s="55" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14658,7 +14652,7 @@
           <t>P6-S18</t>
         </is>
       </c>
-      <c r="B28" s="67" t="n"/>
+      <c r="B28" s="68" t="n"/>
       <c r="C28" s="46" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -14742,7 +14736,7 @@
           <t>P6-S19</t>
         </is>
       </c>
-      <c r="B30" s="65" t="inlineStr">
+      <c r="B30" s="66" t="inlineStr">
         <is>
           <t>feature/swiggy-chatbot-tools</t>
         </is>
@@ -14830,7 +14824,7 @@
           <t>P6-F01</t>
         </is>
       </c>
-      <c r="B32" s="65" t="inlineStr">
+      <c r="B32" s="66" t="inlineStr">
         <is>
           <t>feature/swiggy-connectors-ui</t>
         </is>
@@ -14901,7 +14895,7 @@
           <t>P6-F02</t>
         </is>
       </c>
-      <c r="B33" s="66" t="n"/>
+      <c r="B33" s="67" t="n"/>
       <c r="C33" s="55" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -14968,7 +14962,7 @@
           <t>P6-F03</t>
         </is>
       </c>
-      <c r="B34" s="66" t="n"/>
+      <c r="B34" s="67" t="n"/>
       <c r="C34" s="46" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -15017,7 +15011,7 @@
           <t>P6-F04</t>
         </is>
       </c>
-      <c r="B35" s="66" t="n"/>
+      <c r="B35" s="67" t="n"/>
       <c r="C35" s="55" t="inlineStr">
         <is>
           <t>Docs</t>
@@ -15066,7 +15060,7 @@
           <t>P6-F05</t>
         </is>
       </c>
-      <c r="B36" s="67" t="n"/>
+      <c r="B36" s="68" t="n"/>
       <c r="C36" s="46" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15150,7 +15144,7 @@
           <t>P6-S20</t>
         </is>
       </c>
-      <c r="B38" s="65" t="inlineStr">
+      <c r="B38" s="66" t="inlineStr">
         <is>
           <t>feature/swiggy-prompt-injection (deleted post-merge)</t>
         </is>
@@ -15220,7 +15214,7 @@
           <t>P6-S21</t>
         </is>
       </c>
-      <c r="B40" s="65" t="inlineStr">
+      <c r="B40" s="66" t="inlineStr">
         <is>
           <t>fix/swiggy-sse-market-intel</t>
         </is>
@@ -15291,7 +15285,7 @@
           <t>P6-S22</t>
         </is>
       </c>
-      <c r="B41" s="66" t="n"/>
+      <c r="B41" s="67" t="n"/>
       <c r="C41" s="55" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15358,7 +15352,7 @@
           <t>P6-S23</t>
         </is>
       </c>
-      <c r="B42" s="66" t="n"/>
+      <c r="B42" s="67" t="n"/>
       <c r="C42" s="46" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -15425,7 +15419,7 @@
           <t>P6-S24</t>
         </is>
       </c>
-      <c r="B43" s="66" t="n"/>
+      <c r="B43" s="67" t="n"/>
       <c r="C43" s="55" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -15492,7 +15486,7 @@
           <t>P6-S25</t>
         </is>
       </c>
-      <c r="B44" s="66" t="n"/>
+      <c r="B44" s="67" t="n"/>
       <c r="C44" s="46" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15559,7 +15553,7 @@
           <t>P6-S26</t>
         </is>
       </c>
-      <c r="B45" s="66" t="n"/>
+      <c r="B45" s="67" t="n"/>
       <c r="C45" s="55" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15626,7 +15620,7 @@
           <t>P6-S27</t>
         </is>
       </c>
-      <c r="B46" s="66" t="n"/>
+      <c r="B46" s="67" t="n"/>
       <c r="C46" s="46" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15693,7 +15687,7 @@
           <t>P6-S28</t>
         </is>
       </c>
-      <c r="B47" s="66" t="n"/>
+      <c r="B47" s="67" t="n"/>
       <c r="C47" s="55" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -15760,7 +15754,7 @@
           <t>P6-S29</t>
         </is>
       </c>
-      <c r="B48" s="66" t="n"/>
+      <c r="B48" s="67" t="n"/>
       <c r="C48" s="46" t="inlineStr">
         <is>
           <t>Security</t>
@@ -15819,7 +15813,7 @@
           <t>P6-S30</t>
         </is>
       </c>
-      <c r="B49" s="67" t="n"/>
+      <c r="B49" s="68" t="n"/>
       <c r="C49" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -15880,13 +15874,13 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="7.95" customHeight="1" s="72">
+    <row r="50" ht="108" customHeight="1" s="72">
       <c r="A50" s="44" t="inlineStr">
         <is>
-          <t>P6-S42</t>
-        </is>
-      </c>
-      <c r="B50" s="67" t="inlineStr">
+          <t>P6-S31</t>
+        </is>
+      </c>
+      <c r="B50" s="68" t="inlineStr">
         <is>
           <t>fix/ci-fastapi-starlette-conflict</t>
         </is>
@@ -15974,7 +15968,7 @@
           <t>P6-MI01</t>
         </is>
       </c>
-      <c r="B52" s="68" t="inlineStr">
+      <c r="B52" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-market-intel-expansion</t>
         </is>
@@ -16027,7 +16021,7 @@
           <t>P6-MI02</t>
         </is>
       </c>
-      <c r="B53" s="66" t="n"/>
+      <c r="B53" s="67" t="n"/>
       <c r="C53" s="46" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16076,7 +16070,7 @@
           <t>P6-MI03</t>
         </is>
       </c>
-      <c r="B54" s="67" t="n"/>
+      <c r="B54" s="68" t="n"/>
       <c r="C54" s="55" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -16142,7 +16136,7 @@
           <t>P6-MI04</t>
         </is>
       </c>
-      <c r="B56" s="68" t="inlineStr">
+      <c r="B56" s="69" t="inlineStr">
         <is>
           <t>feature/swiggy-chatbot-expansion</t>
         </is>
@@ -16209,10 +16203,10 @@
     <row r="58" ht="73.05" customHeight="1" s="72">
       <c r="A58" s="62" t="inlineStr">
         <is>
-          <t>P6-S31</t>
-        </is>
-      </c>
-      <c r="B58" s="68" t="inlineStr">
+          <t>P6-S32</t>
+        </is>
+      </c>
+      <c r="B58" s="69" t="inlineStr">
         <is>
           <t>feature/action-queue</t>
         </is>
@@ -16297,10 +16291,10 @@
     <row r="60" ht="73.05" customHeight="1" s="72">
       <c r="A60" s="62" t="inlineStr">
         <is>
-          <t>P6-S32</t>
-        </is>
-      </c>
-      <c r="B60" s="68" t="n"/>
+          <t>P6-S33</t>
+        </is>
+      </c>
+      <c r="B60" s="69" t="n"/>
       <c r="C60" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16381,10 +16375,10 @@
     <row r="62" ht="73.05" customHeight="1" s="72">
       <c r="A62" s="62" t="inlineStr">
         <is>
-          <t>P6-S33</t>
-        </is>
-      </c>
-      <c r="B62" s="68" t="n"/>
+          <t>P6-S34</t>
+        </is>
+      </c>
+      <c r="B62" s="69" t="n"/>
       <c r="C62" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16436,7 +16430,7 @@
       </c>
       <c r="N62" s="55" t="inlineStr">
         <is>
-          <t>P6-S32</t>
+          <t>P6-S33</t>
         </is>
       </c>
       <c r="O62" s="56" t="inlineStr">
@@ -16465,10 +16459,10 @@
     <row r="64" ht="85.95" customHeight="1" s="72">
       <c r="A64" s="62" t="inlineStr">
         <is>
-          <t>P6-S34</t>
-        </is>
-      </c>
-      <c r="B64" s="68" t="inlineStr">
+          <t>P6-S35</t>
+        </is>
+      </c>
+      <c r="B64" s="69" t="inlineStr">
         <is>
           <t>feature/workflow-system</t>
         </is>
@@ -16553,10 +16547,10 @@
     <row r="66" ht="99" customHeight="1" s="72">
       <c r="A66" s="62" t="inlineStr">
         <is>
-          <t>P6-S35</t>
-        </is>
-      </c>
-      <c r="B66" s="68" t="n"/>
+          <t>P6-S36</t>
+        </is>
+      </c>
+      <c r="B66" s="69" t="n"/>
       <c r="C66" s="55" t="inlineStr">
         <is>
           <t>Product</t>
@@ -16608,7 +16602,7 @@
       </c>
       <c r="N66" s="55" t="inlineStr">
         <is>
-          <t>P6-S22-UNRESOLVED, P6-S42</t>
+          <t>P6-S22-UNRESOLVED, P6-S43</t>
         </is>
       </c>
       <c r="O66" s="56" t="inlineStr">
@@ -16637,10 +16631,10 @@
     <row r="68" ht="73.05" customHeight="1" s="72">
       <c r="A68" s="62" t="inlineStr">
         <is>
-          <t>P6-S36</t>
-        </is>
-      </c>
-      <c r="B68" s="68" t="n"/>
+          <t>P6-S37</t>
+        </is>
+      </c>
+      <c r="B68" s="69" t="n"/>
       <c r="C68" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -16692,7 +16686,7 @@
       </c>
       <c r="N68" s="55" t="inlineStr">
         <is>
-          <t>P6-S31</t>
+          <t>P6-S32</t>
         </is>
       </c>
       <c r="O68" s="56" t="inlineStr">
@@ -16721,10 +16715,10 @@
     <row r="70" ht="85.95" customHeight="1" s="72">
       <c r="A70" s="62" t="inlineStr">
         <is>
-          <t>P6-S37</t>
-        </is>
-      </c>
-      <c r="B70" s="68" t="inlineStr">
+          <t>P6-S38</t>
+        </is>
+      </c>
+      <c r="B70" s="69" t="inlineStr">
         <is>
           <t>feature/debate-critic</t>
         </is>
@@ -16780,7 +16774,7 @@
       </c>
       <c r="N70" s="55" t="inlineStr">
         <is>
-          <t>P6-S34</t>
+          <t>P6-S35</t>
         </is>
       </c>
       <c r="O70" s="56" t="inlineStr">
@@ -16812,7 +16806,7 @@
           <t>P6-R01</t>
         </is>
       </c>
-      <c r="B72" s="68" t="inlineStr">
+      <c r="B72" s="69" t="inlineStr">
         <is>
           <t>feature/voice-interface</t>
         </is>
@@ -16868,7 +16862,7 @@
       </c>
       <c r="N72" s="55" t="inlineStr">
         <is>
-          <t>P6-S43</t>
+          <t>P6-S44</t>
         </is>
       </c>
       <c r="O72" s="56" t="inlineStr">
@@ -16900,7 +16894,7 @@
           <t>P6-F06</t>
         </is>
       </c>
-      <c r="B74" s="68" t="inlineStr">
+      <c r="B74" s="69" t="inlineStr">
         <is>
           <t>feature/action-queue-ui</t>
         </is>
@@ -16961,7 +16955,7 @@
       </c>
       <c r="O74" s="56" t="inlineStr">
         <is>
-          <t>Depends on P6-S31 (action_queue in plan API response)</t>
+          <t>Depends on P6-S32 (action_queue in plan API response)</t>
         </is>
       </c>
     </row>
@@ -16988,7 +16982,7 @@
           <t>P6-F07</t>
         </is>
       </c>
-      <c r="B76" s="68" t="n"/>
+      <c r="B76" s="69" t="n"/>
       <c r="C76" s="55" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -17040,7 +17034,7 @@
       </c>
       <c r="N76" s="55" t="inlineStr">
         <is>
-          <t>P6-S43</t>
+          <t>P6-S44</t>
         </is>
       </c>
       <c r="O76" s="56" t="inlineStr">
@@ -17072,7 +17066,7 @@
           <t>P6-F08</t>
         </is>
       </c>
-      <c r="B78" s="68" t="n"/>
+      <c r="B78" s="69" t="n"/>
       <c r="C78" s="55" t="inlineStr">
         <is>
           <t>Frontend</t>
@@ -17085,7 +17079,7 @@
       </c>
       <c r="E78" s="56" t="inlineStr">
         <is>
-          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S35). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
+          <t>New route /live. Kitchen display-grade SSE feed from LiveMonitorService (P6-S36). Shows active Swiggy delivery orders with ETA countdown, Instamart procurement status with delivery ETA, alert banner on delivery spike or ingredient arrival. Swiggy logo + 'Live via Swiggy MCP' badge. Page shows inactive state outside service hours (12-14h, 19-22h IST).</t>
         </is>
       </c>
       <c r="F78" s="56" t="inlineStr">
@@ -17124,7 +17118,7 @@
       </c>
       <c r="N78" s="55" t="inlineStr">
         <is>
-          <t>P6-S35</t>
+          <t>P6-S36</t>
         </is>
       </c>
       <c r="O78" s="56" t="inlineStr">
@@ -17153,10 +17147,10 @@
     <row r="80" ht="124.95" customHeight="1" s="72">
       <c r="A80" s="62" t="inlineStr">
         <is>
-          <t>P6-S38</t>
-        </is>
-      </c>
-      <c r="B80" s="68" t="n"/>
+          <t>P6-S39</t>
+        </is>
+      </c>
+      <c r="B80" s="69" t="n"/>
       <c r="C80" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -17229,10 +17223,10 @@
     <row r="82" ht="112.05" customHeight="1" s="72">
       <c r="A82" s="62" t="inlineStr">
         <is>
-          <t>P6-S39</t>
-        </is>
-      </c>
-      <c r="B82" s="68" t="n"/>
+          <t>P6-S40</t>
+        </is>
+      </c>
+      <c r="B82" s="69" t="n"/>
       <c r="C82" s="55" t="inlineStr">
         <is>
           <t>Product</t>
@@ -17305,10 +17299,10 @@
     <row r="84" ht="99" customHeight="1" s="72">
       <c r="A84" s="62" t="inlineStr">
         <is>
-          <t>P6-S40</t>
-        </is>
-      </c>
-      <c r="B84" s="68" t="n"/>
+          <t>P6-S41</t>
+        </is>
+      </c>
+      <c r="B84" s="69" t="n"/>
       <c r="C84" s="55" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -17381,10 +17375,10 @@
     <row r="86" ht="151.05" customHeight="1" s="72">
       <c r="A86" s="62" t="inlineStr">
         <is>
-          <t>P6-S41</t>
-        </is>
-      </c>
-      <c r="B86" s="68" t="n"/>
+          <t>P6-S42</t>
+        </is>
+      </c>
+      <c r="B86" s="69" t="n"/>
       <c r="C86" s="55" t="inlineStr">
         <is>
           <t>Product</t>
@@ -17451,7 +17445,7 @@
       <c r="O87" s="52" t="n"/>
     </row>
     <row r="88" ht="28.05" customHeight="1" s="72">
-      <c r="A88" s="69" t="inlineStr">
+      <c r="A88" s="70" t="inlineStr">
         <is>
           <t>→ DEMO 1  |  all above on main, docs updated, screenshots done — record full Swiggy read + AI + voice + live monitor demo ←</t>
         </is>
@@ -17570,16 +17564,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="85" t="inlineStr">
+      <c r="A2" s="83" t="inlineStr">
         <is>
           <t>BLOCKED — needs Swiggy staging creds (write tools: checkout, book_table)</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="41" t="inlineStr">
         <is>
-          <t>P6-S42</t>
+          <t>P6-S43</t>
         </is>
       </c>
       <c r="B4" s="41" t="inlineStr">
@@ -17609,7 +17604,7 @@
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>docs/SWIGGY_INTEGRATION.md (P6-S42 executor section)</t>
+          <t>docs/SWIGGY_INTEGRATION.md (P6-S43 executor section)</t>
         </is>
       </c>
       <c r="H4" s="41" t="inlineStr">
@@ -17627,7 +17622,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K4" s="70" t="n"/>
+      <c r="K4" s="42" t="n"/>
       <c r="L4" s="41" t="inlineStr">
         <is>
           <t>W5</t>
@@ -17638,7 +17633,7 @@
       </c>
       <c r="N4" s="41" t="inlineStr">
         <is>
-          <t>P6-S31, P6-S14</t>
+          <t>P6-S32, P6-S14</t>
         </is>
       </c>
       <c r="O4" s="41" t="inlineStr">
@@ -17647,10 +17642,11 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t>P6-S43</t>
+          <t>P6-S44</t>
         </is>
       </c>
       <c r="B6" s="41" t="inlineStr">
@@ -17698,7 +17694,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K6" s="70" t="n"/>
+      <c r="K6" s="42" t="n"/>
       <c r="L6" s="41" t="inlineStr">
         <is>
           <t>W5</t>
@@ -17709,7 +17705,7 @@
       </c>
       <c r="N6" s="41" t="inlineStr">
         <is>
-          <t>P6-S31</t>
+          <t>P6-S32</t>
         </is>
       </c>
       <c r="O6" s="41" t="inlineStr">
@@ -17718,10 +17714,11 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>P6-S44</t>
+          <t>P6-S45</t>
         </is>
       </c>
       <c r="B8" s="41" t="inlineStr">
@@ -17769,7 +17766,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K8" s="70" t="n"/>
+      <c r="K8" s="42" t="n"/>
       <c r="L8" s="41" t="inlineStr">
         <is>
           <t>W9</t>
@@ -17780,7 +17777,7 @@
       </c>
       <c r="N8" s="41" t="inlineStr">
         <is>
-          <t>P6-S37</t>
+          <t>P6-S38</t>
         </is>
       </c>
       <c r="O8" s="41" t="inlineStr">
@@ -17789,20 +17786,22 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="85" t="inlineStr">
+      <c r="A10" s="83" t="inlineStr">
         <is>
           <t>WHEN RECEIVED — Sarvam AI access + AWS credits</t>
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>P6-S45</t>
-        </is>
-      </c>
-      <c r="B12" s="70" t="n"/>
+          <t>P6-S46</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="n"/>
       <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -17843,8 +17842,8 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K12" s="70" t="n"/>
-      <c r="L12" s="70" t="n"/>
+      <c r="K12" s="42" t="n"/>
+      <c r="L12" s="42" t="n"/>
       <c r="M12" s="41" t="n">
         <v>0</v>
       </c>
@@ -17859,13 +17858,14 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>P6-S46</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="n"/>
+          <t>P6-S47</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="n"/>
       <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -17906,8 +17906,8 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K14" s="70" t="n"/>
-      <c r="L14" s="70" t="n"/>
+      <c r="K14" s="42" t="n"/>
+      <c r="L14" s="42" t="n"/>
       <c r="M14" s="41" t="n">
         <v>0</v>
       </c>
@@ -17922,27 +17922,30 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" s="85" t="inlineStr">
+      <c r="A16" s="83" t="inlineStr">
         <is>
           <t>→ DEMO 2 / POTENTIAL DEMO  |  all above on main, staging write tools + Sarvam voice + AWS hosted — record full product demo ←</t>
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
-      <c r="A18" s="85" t="inlineStr">
+      <c r="A18" s="83" t="inlineStr">
         <is>
           <t>DOCS + PHASE 6 MILESTONE MERGE</t>
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
           <t>P6-D01</t>
         </is>
       </c>
-      <c r="B20" s="70" t="n"/>
+      <c r="B20" s="42" t="n"/>
       <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Docs</t>
@@ -17983,7 +17986,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K20" s="70" t="n"/>
+      <c r="K20" s="42" t="n"/>
       <c r="L20" s="41" t="inlineStr">
         <is>
           <t>W8</t>
@@ -18003,13 +18006,14 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="41" t="inlineStr">
         <is>
           <t>P6-D02</t>
         </is>
       </c>
-      <c r="B22" s="70" t="n"/>
+      <c r="B22" s="42" t="n"/>
       <c r="C22" s="41" t="inlineStr">
         <is>
           <t>Docs</t>
@@ -18050,7 +18054,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K22" s="70" t="n"/>
+      <c r="K22" s="42" t="n"/>
       <c r="L22" s="41" t="inlineStr">
         <is>
           <t>W8</t>
@@ -18070,13 +18074,14 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="41" t="inlineStr">
         <is>
           <t>P6-D03</t>
         </is>
       </c>
-      <c r="B24" s="70" t="n"/>
+      <c r="B24" s="42" t="n"/>
       <c r="C24" s="41" t="inlineStr">
         <is>
           <t>Release</t>
@@ -18117,7 +18122,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K24" s="70" t="n"/>
+      <c r="K24" s="42" t="n"/>
       <c r="L24" s="41" t="inlineStr">
         <is>
           <t>W8</t>
@@ -18137,13 +18142,15 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
-      <c r="A26" s="85" t="inlineStr">
+      <c r="A26" s="83" t="inlineStr">
         <is>
           <t>PHASE 7 — Production, CI/CD, Public Release</t>
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="41" t="inlineStr">
         <is>
@@ -18195,7 +18202,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K28" s="70" t="n"/>
+      <c r="K28" s="42" t="n"/>
       <c r="L28" s="41" t="inlineStr">
         <is>
           <t>P7</t>
@@ -18215,6 +18222,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
@@ -18266,7 +18274,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K30" s="70" t="n"/>
+      <c r="K30" s="42" t="n"/>
       <c r="L30" s="41" t="inlineStr">
         <is>
           <t>P7</t>
@@ -18286,6 +18294,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="41" t="inlineStr">
         <is>
@@ -18337,7 +18346,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K32" s="70" t="n"/>
+      <c r="K32" s="42" t="n"/>
       <c r="L32" s="41" t="inlineStr">
         <is>
           <t>P7</t>
@@ -18357,6 +18366,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="41" t="inlineStr">
         <is>
@@ -18408,7 +18418,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K34" s="70" t="n"/>
+      <c r="K34" s="42" t="n"/>
       <c r="L34" s="41" t="inlineStr">
         <is>
           <t>P7</t>
@@ -18428,6 +18438,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="41" t="inlineStr">
         <is>
@@ -18479,7 +18490,7 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K36" s="70" t="n"/>
+      <c r="K36" s="42" t="n"/>
       <c r="L36" s="41" t="inlineStr">
         <is>
           <t>P7</t>
@@ -18527,7 +18538,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.95" customHeight="1" s="72">
-      <c r="A1" s="84" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>CortexKitchen v2 — Documentation Strategy (Phase 6)</t>
         </is>
@@ -18656,7 +18667,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>P6-S43 — NEW</t>
+          <t>P6-S44 — NEW</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -18678,7 +18689,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>P6-S04, P6-S15, P6-S18, P6-S43</t>
+          <t>P6-S04, P6-S15, P6-S18, P6-S44</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -18744,7 +18755,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>P6-S05, P6-S18, P6-S43</t>
+          <t>P6-S05, P6-S18, P6-S44</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -18766,7 +18777,7 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>P6-S04, P6-S06, P6-S18, P6-S43</t>
+          <t>P6-S04, P6-S06, P6-S18, P6-S44</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -18910,7 +18921,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.95" customHeight="1" s="72">
-      <c r="A1" s="84" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>CortexKitchen — Git Branching Rules</t>
         </is>

</xml_diff>

<commit_message>
tracker: record hard constraint on P6-F09..F12 -- redesign must not strip existing depth
User reviewed a direction-only prototype (single summary screen, color/type/theme only)
and pushed back that the actual redesign must never remove agent detail drill-downs,
critic reasoning/revision history, or /runs comparisons -- the new visual direction gets
applied to all existing depth, not used as an excuse to simplify it away.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -17211,7 +17211,7 @@
       </c>
       <c r="E80" s="56" t="inlineStr">
         <is>
-          <t>Add a parallel light-mode palette alongside the existing ink/ember dark tokens in globals.css (Tailwind v4 @theme), wire a theme toggle (persisted via localStorage, defaults to system prefers-color-scheme) accessible from every page's header/nav, and audit + replace ad-hoc opacity-based dark-only utility classes (text-white/65, bg-white/[0.02], etc.) across all ~35 dashboard/runs/chat components with theme-aware tokens so both modes render correctly. Target users skew middle-aged restaurant owners/managers who may find a dark-only dev-tool aesthetic hard to read or off-putting -- a toggle makes the product usable for both preferences, not just engineers.</t>
+          <t>Add a parallel light-mode palette alongside the existing ink/ember dark tokens in globals.css (Tailwind v4 @theme), wire a theme toggle (persisted via localStorage, defaults to system prefers-color-scheme) accessible from every page's header/nav, and audit + replace ad-hoc opacity-based dark-only utility classes (text-white/65, bg-white/[0.02], etc.) across all ~35 dashboard/runs/chat components with theme-aware tokens so both modes render correctly. Target users skew middle-aged restaurant owners/managers who may find a dark-only dev-tool aesthetic hard to read or off-putting -- a toggle makes the product usable for both preferences, not just engineers. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
         </is>
       </c>
       <c r="F80" s="56" t="inlineStr">
@@ -17271,7 +17271,7 @@
       </c>
       <c r="E82" s="56" t="inlineStr">
         <is>
-          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language.</t>
+          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
         </is>
       </c>
       <c r="F82" s="56" t="inlineStr">
@@ -17335,7 +17335,7 @@
       </c>
       <c r="E84" s="56" t="inlineStr">
         <is>
-          <t>The single /dashboard page currently tries to show demand forecast + reservations + complaints + inventory + market intel + menu + critic + connector status all at once -- reads as a diagnostics dump a manager could get lost in. Restructure into: a lightweight /dashboard 'Today' view (KPIs, alerts, pending actions only -- what a manager checks first each morning), a dedicated /operations page for the 5 planning-agent outputs in plain-language framing (not raw JSON-shaped cards), and Swiggy Market Intelligence promoted to its own dedicated /market page (competitor pricing, occupancy, Instamart procurement) so it has a clear, demo-able home separate from internal ops data -- matching the product's own internal-vs-Swiggy-data distinction already documented in CLAUDE.md.</t>
+          <t>The single /dashboard page currently tries to show demand forecast + reservations + complaints + inventory + market intel + menu + critic + connector status all at once -- reads as a diagnostics dump a manager could get lost in. Restructure into: a lightweight /dashboard 'Today' view (KPIs, alerts, pending actions only -- what a manager checks first each morning), a dedicated /operations page for the 5 planning-agent outputs in plain-language framing (not raw JSON-shaped cards), and Swiggy Market Intelligence promoted to its own dedicated /market page (competitor pricing, occupancy, Instamart procurement) so it has a clear, demo-able home separate from internal ops data -- matching the product's own internal-vs-Swiggy-data distinction already documented in CLAUDE.md. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
         </is>
       </c>
       <c r="F84" s="56" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="E86" s="56" t="inlineStr">
         <is>
-          <t>Apply the new design system to /runs. Restyle from a dense monospace debug trace (raw dimension-score grids, 10+ revision-reason text blocks) into something a manager can skim in under a minute. Fix the currently-unstyled raw Next.js 404 on /runs/{id} deep links -- give each run its own real page.</t>
+          <t>Apply the new design system to /runs. Restyle from a dense monospace debug trace (raw dimension-score grids, 10+ revision-reason text blocks) into something a manager can skim in under a minute. Fix the currently-unstyled raw Next.js 404 on /runs/{id} deep links -- give each run its own real page. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
         </is>
       </c>
       <c r="F86" s="56" t="inlineStr">

</xml_diff>

<commit_message>
tracker: mark P6-F09 Completed, note F10 partial overlap
Light/dark theme system fully built, applied across all pages, and
verified with a real authenticated browser session -- not just the
direction-prototype pages. Noted on P6-F10 that its ember-accent-contrast
fix already landed as part of F09 (was blocking basic light-mode
readability), so remaining F10 scope is just the monospace-as-accent
typography rebalance.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -501,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -727,6 +728,12 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -17211,7 +17218,7 @@
       </c>
       <c r="E80" s="56" t="inlineStr">
         <is>
-          <t>Add a parallel light-mode palette alongside the existing ink/ember dark tokens in globals.css (Tailwind v4 @theme), wire a theme toggle (persisted via localStorage, defaults to system prefers-color-scheme) accessible from every page's header/nav, and audit + replace ad-hoc opacity-based dark-only utility classes (text-white/65, bg-white/[0.02], etc.) across all ~35 dashboard/runs/chat components with theme-aware tokens so both modes render correctly. Target users skew middle-aged restaurant owners/managers who may find a dark-only dev-tool aesthetic hard to read or off-putting -- a toggle makes the product usable for both preferences, not just engineers. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
+          <t>Add a parallel light-mode palette alongside the existing ink/ember dark tokens in globals.css (Tailwind v4 @theme), wire a theme toggle (persisted via localStorage, defaults to system prefers-color-scheme) accessible from every page's header/nav, and audit + replace ad-hoc opacity-based dark-only utility classes (text-white/65, bg-white/[0.02], etc.) across all ~35 dashboard/runs/chat components with theme-aware tokens so both modes render correctly. Target users skew middle-aged restaurant owners/managers who may find a dark-only dev-tool aesthetic hard to read or off-putting -- a toggle makes the product usable for both preferences, not just engineers. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts. DONE 2026-07-04: light-mode token layer + toggle built and applied across all ~30 pages/components (not just the 5 touched in the direction prototype), via a boundary-safe scripted class rename so the same old class always maps to the same new token. 3 real bugs found only by driving the app in a browser (not catchable by a class-rename script alone): ember accent text washed out on light badges (fixed via --color-accent token), DatePicker select/date-input had inline style={{background:...}} overriding the className entirely, and no explicit color-scheme meant native &lt;select&gt;/&lt;option&gt; rendered with OS dark chrome regardless of page theme. Verified end-to-end with a real registered test account across dashboard/runs/connectors/chat in both themes -- zero console errors, zero hydration warnings, tsc + eslint clean.</t>
         </is>
       </c>
       <c r="F80" s="56" t="inlineStr">
@@ -17226,7 +17233,7 @@
       </c>
       <c r="H80" s="63" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I80" s="49" t="inlineStr">
@@ -17239,10 +17246,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K80" s="55" t="n"/>
-      <c r="L80" s="59" t="n"/>
+      <c r="K80" s="84" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L80" s="85" t="n">
+        <v>46207</v>
+      </c>
       <c r="M80" s="58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N80" s="55" t="n"/>
       <c r="O80" s="56" t="inlineStr">
@@ -17271,7 +17282,7 @@
       </c>
       <c r="E82" s="56" t="inlineStr">
         <is>
-          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
+          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts. NOTE: the ember-accent-text contrast fix (text-ember-300/400 -&gt; --color-accent token) was already done as part of P6-F09 verification, since it was blocking basic light-mode readability, not a nice-to-have. Remaining F10 scope: pull font-mono back from being the default label voice everywhere to a true accent.</t>
         </is>
       </c>
       <c r="F82" s="56" t="inlineStr">

</xml_diff>

<commit_message>
tracker: mark P6-F10 Completed
Typography rebalance done in two passes -- mechanical (uppercase-tracked
labels) then per-instance judgment (remaining bare font-mono usages,
since this codebase used monospace for real data, category labels, and
prose all mixed together). Also fixed a second legacy hardcoded-color
blind spot (bg-navy-*/text-gold-*) found while auditing context.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -17282,7 +17282,7 @@
       </c>
       <c r="E82" s="56" t="inlineStr">
         <is>
-          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts. NOTE: the ember-accent-text contrast fix (text-ember-300/400 -&gt; --color-accent token) was already done as part of P6-F09 verification, since it was blocking basic light-mode readability, not a nice-to-have. Remaining F10 scope: pull font-mono back from being the default label voice everywhere to a true accent.</t>
+          <t>Dashboard/runs pages currently lean on Space Mono uppercase micro-labels (font-mono text-[9px] uppercase tracking-wider) as the primary label voice for nearly everything -- this is what reads as an engineering console rather than a product, not the color palette. Rebalance: reserve monospace for true accents only (IDs, exact prices/timestamps, code-like values); extend the existing Instrument Serif display font + warm ink/ember palette (already used well on the landing page) into section headers and key numbers elsewhere for warmth and hierarchy, matching the landing page's already-elite feel instead of inventing a new typographic language. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts. NOTE: the ember-accent-text contrast fix (text-ember-300/400 -&gt; --color-accent token) was already done as part of P6-F09 verification, since it was blocking basic light-mode readability, not a nice-to-have. Remaining F10 scope: pull font-mono back from being the default label voice everywhere to a true accent. DONE 2026-07-4: two-pass conversion -- (1) mechanical pass on the specific font-mono+uppercase+tracking- combination (171 label class-strings, always a decorative label in this codebase, never data), (2) per-instance judgment pass on the remaining ~89 bare font-mono usages, since this codebase used monospace for three genuinely different things (real data, category/status labels, and even prose/error messages) that no single mechanical rule could tell apart. Demoted buttons/links/status words/category badges/prose; kept genuine data (prices, IDs, timestamps, scores, deltas, code blocks). Also caught 2 more instances of hardcoded legacy bg-navy-*/text-gold-* colors (a different legacy palette than bg-ink-*, missed by the original P6-F09 conversion script) while auditing context file-by-file. Verified in browser (dashboard, runs) both themes -- zero console errors, tsc clean.</t>
         </is>
       </c>
       <c r="F82" s="56" t="inlineStr">
@@ -17297,7 +17297,7 @@
       </c>
       <c r="H82" s="63" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I82" s="49" t="inlineStr">
@@ -17310,10 +17310,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K82" s="55" t="n"/>
-      <c r="L82" s="59" t="n"/>
+      <c r="K82" s="84" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L82" s="85" t="n">
+        <v>46207</v>
+      </c>
       <c r="M82" s="58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N82" s="55" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tracker: mark P6-F11 Completed, add P6-F18/F19 for market analytics + Today redesign
P6-F11 (dashboard split into /dashboard, /operations, /market) shipped in
PR #89 -- was still marked Planned. Added P6-F18 (live market intelligence +
business analytics endpoints) and P6-F19 (Today dashboard redesign: modal
planning flow, warm theme, NavBar cleanup, date-relative seed data) to cover
the rest of that merge, both Completed.

Note: eaef859's commit message and an earlier CLAUDE.md pass informally
tagged the analytics work "P6-F16", which collides with an already-used tag
from the 2026-07-01 PR (F14/F15/F17) that never got tracker rows. P6-F18 is
the correct sequential tracker ID; git history is left as-is.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Tracker ( 1 - 5 )" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staging Creds + Phase 7" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Strategy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git Practices" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Phase Tracker ( 1 - 5 )" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Phase 6" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Staging Creds + Phase 7" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Doc Strategy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Git Practices" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -502,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -735,6 +735,8 @@
     <xf numFmtId="166" fontId="21" fillId="23" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13270,7 +13272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O96"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="12" customWidth="1" style="71" min="1" max="1"/>
@@ -17350,12 +17352,12 @@
       </c>
       <c r="E84" s="56" t="inlineStr">
         <is>
-          <t>The single /dashboard page currently tries to show demand forecast + reservations + complaints + inventory + market intel + menu + critic + connector status all at once -- reads as a diagnostics dump a manager could get lost in. Restructure into: a lightweight /dashboard 'Today' view (KPIs, alerts, pending actions only -- what a manager checks first each morning), a dedicated /operations page for the 5 planning-agent outputs in plain-language framing (not raw JSON-shaped cards), and Swiggy Market Intelligence promoted to its own dedicated /market page (competitor pricing, occupancy, Instamart procurement) so it has a clear, demo-able home separate from internal ops data -- matching the product's own internal-vs-Swiggy-data distinction already documented in CLAUDE.md. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts.</t>
+          <t>The single /dashboard page currently tries to show demand forecast + reservations + complaints + inventory + market intel + menu + critic + connector status all at once -- reads as a diagnostics dump a manager could get lost in. Restructure into: a lightweight /dashboard 'Today' view (KPIs, alerts, pending actions only -- what a manager checks first each morning), a dedicated /operations page for the 5 planning-agent outputs in plain-language framing (not raw JSON-shaped cards), and Swiggy Market Intelligence promoted to its own dedicated /market page (competitor pricing, occupancy, Instamart procurement) so it has a clear, demo-able home separate from internal ops data -- matching the product's own internal-vs-Swiggy-data distinction already documented in CLAUDE.md. HARD CONSTRAINT (user, 2026-07-04): this redesign must never strip existing detail views, cards, or pages for a cleaner look -- agent detail drill-downs, full critic dimension breakdown + reasoning + revision history, /runs comparisons, all of it stays. Apply the new visual direction (light/dark theme, Instrument Serif + Plus Jakarta Sans, monospace as accent not primary label voice, semantic severity color kept separate from agent-category color) TO that existing depth -- never as a reason to cut it. A direction prototype (single summary screen only, not the full app) was reviewed and approved for tone/color/type before this task starts. DONE 2026-07-04: split shipped -- /dashboard is now the lightweight 'Today' view (TodayIdleState: business KPIs, market intel teaser, actionable ops snapshot), /operations holds the 5 agent-card detail + CriticBanner + ForecastChart + ManagerActionPanel (via useSelectedRun, reads ?run={id} or falls back to most recent), /market is the dedicated Swiggy market intelligence page. Verified end-to-end via Playwright: fresh register -&gt; idle state renders clean in both themes -&gt; trigger a plan via the new PlanShiftModal -&gt; auto-redirects to /operations?run={id} with the CriticBanner visible on landing, zero console errors.</t>
         </is>
       </c>
       <c r="F84" s="56" t="inlineStr">
         <is>
-          <t>feat: split dashboard into /dashboard (Today), /operations, /market</t>
+          <t>feat(P6-F11/F12): redesign Today dashboard -- modal planning flow, market-aware layout, warm theme</t>
         </is>
       </c>
       <c r="G84" s="56" t="inlineStr">
@@ -17365,7 +17367,7 @@
       </c>
       <c r="H84" s="63" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I84" s="49" t="inlineStr">
@@ -17378,10 +17380,14 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K84" s="55" t="n"/>
-      <c r="L84" s="59" t="n"/>
+      <c r="K84" s="84" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L84" s="85" t="n">
+        <v>46207</v>
+      </c>
       <c r="M84" s="58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N84" s="55" t="inlineStr">
         <is>
@@ -17760,7 +17766,183 @@
       <c r="O95" s="52" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="70" t="inlineStr">
+      <c r="A96" s="62" t="inlineStr">
+        <is>
+          <t>P6-F18</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>feature/design-system-theming</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Live market intelligence + business analytics endpoints, independent of planning runs</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>GET /api/v1/market/pulse calls CompetitorEnricher/OccupancyEnricher/ProcurementEnricher directly (no planning run required) and structures diff_pct/direction comparisons server-side, since the raw enrichers return loosely-typed dicts, not a UI-ready shape. GET /api/v1/business/performance computes real revenue/profit via a new MenuItem.cost_price column, daily trend, yesterday/today snapshots, top/bottom dishes, dine-in vs delivery channel split, complaints grouped by keyword-matched category, and peak-hours demand (orders only, so future-dated reservation seed rows don't skew 'when are we actually busy'). DONE 2026-07-04: verified against seeded data -- revenue, margin, and complaint-category counts all match expected values. NOTE: this commit's message (eaef859) and an earlier CLAUDE.md pass informally used the tag 'P6-F16', which collides with an already-used tag from the P6-F14/F15/F17 PR (2026-07-01) that was never given tracker rows -- P6-F18 is the correct sequential tracker ID; the git history is left as-is rather than rewritten.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>feat(P6-F16 in commit msg / P6-F18 in tracker): live market intelligence + business analytics, independent of planning runs</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>CLAUDE.md (API routes section, Swiggy token/circuit-breaker gotcha)</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K96" s="87" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L96" s="87" t="n">
+        <v>46207</v>
+      </c>
+      <c r="M96" t="n">
+        <v>1</v>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>P6-S15</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Hit /market/pulse and /business/performance directly against seeded data; confirm revenue/margin/complaint-category numbers match the seed script, and market pulse returns swiggy_connected + live comparisons when the token is valid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="86" t="n"/>
+      <c r="B97" s="86" t="n"/>
+      <c r="C97" s="86" t="n"/>
+      <c r="D97" s="86" t="n"/>
+      <c r="E97" s="86" t="n"/>
+      <c r="F97" s="86" t="n"/>
+      <c r="G97" s="86" t="n"/>
+      <c r="H97" s="86" t="n"/>
+      <c r="I97" s="86" t="n"/>
+      <c r="J97" s="86" t="n"/>
+      <c r="K97" s="86" t="n"/>
+      <c r="L97" s="86" t="n"/>
+      <c r="M97" s="86" t="n"/>
+      <c r="N97" s="86" t="n"/>
+      <c r="O97" s="86" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="62" t="inlineStr">
+        <is>
+          <t>P6-F19</t>
+        </is>
+      </c>
+      <c r="B98" s="69" t="inlineStr">
+        <is>
+          <t>feature/design-system-theming</t>
+        </is>
+      </c>
+      <c r="C98" s="55" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D98" s="56" t="inlineStr">
+        <is>
+          <t>Today dashboard redesign: modal planning flow, warm theme, NavBar cleanup, date-relative seed data</t>
+        </is>
+      </c>
+      <c r="E98" s="56" t="inlineStr">
+        <is>
+          <t>TodayIdleState fully rewritten around a manager's actual priorities: overall performance chart, actionable 'tonight at a glance' reservations/inventory snapshot, yesterday's business KPIs with channel split, menu performance (top/bottom sellers), peak hours paired with a merged guest-sentiment + complaint-theme card, and a consolidated market intelligence card teasing into /market. 'Plan your next shift' now opens PlanShiftModal instead of running inline. NavBar: removed the scenario dropdown (the modal owns scenario selection now) and the stale 'Friday Rush -- not planned yet' status chip; warmer brand mark and active-tab styling. globals.css light-mode tokens rebuilt around a warm stone/parchment palette instead of cool blue-gray. Also fixed a glitch where the critic-approved banner flashed on /dashboard for one frame and vanished on redirect to /operations -- /operations now shows CriticBanner directly instead of burying the verdict in the Manager Brief modal. seed_demo_data.py no longer hardcodes 2026 calendar dates -- SEED_AS_OF anchors to run-time so 'Today' always reflects live state, and inventory was rebalanced from a permanent 11/18 shortage state to 3/18 genuinely low items. DONE 2026-07-04: verified end-to-end via Playwright (fresh register, both themes, full plan-run -&gt; redirect -&gt; critic banner flow), zero console errors.</t>
+        </is>
+      </c>
+      <c r="F98" s="56" t="inlineStr">
+        <is>
+          <t>feat(P6-F11/F12): redesign Today dashboard -- modal planning flow, market-aware layout, warm theme</t>
+        </is>
+      </c>
+      <c r="G98" s="56" t="inlineStr">
+        <is>
+          <t>CLAUDE.md (page map, theming section)</t>
+        </is>
+      </c>
+      <c r="H98" s="63" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I98" s="49" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J98" s="55" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K98" s="84" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L98" s="85" t="n">
+        <v>46207</v>
+      </c>
+      <c r="M98" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="N98" s="55" t="inlineStr">
+        <is>
+          <t>P6-F11; P6-F18</t>
+        </is>
+      </c>
+      <c r="O98" s="56" t="inlineStr">
+        <is>
+          <t>Playwright: register -&gt; idle state renders clean (light+dark, no console errors) -&gt; open PlanShiftModal -&gt; Generate Plan -&gt; auto-redirect to /operations?run={id} with CriticBanner visible, no flash/glitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="86" t="n"/>
+      <c r="B99" s="86" t="n"/>
+      <c r="C99" s="86" t="n"/>
+      <c r="D99" s="86" t="n"/>
+      <c r="E99" s="86" t="n"/>
+      <c r="F99" s="86" t="n"/>
+      <c r="G99" s="86" t="n"/>
+      <c r="H99" s="86" t="n"/>
+      <c r="I99" s="86" t="n"/>
+      <c r="J99" s="86" t="n"/>
+      <c r="K99" s="86" t="n"/>
+      <c r="L99" s="86" t="n"/>
+      <c r="M99" s="86" t="n"/>
+      <c r="N99" s="86" t="n"/>
+      <c r="O99" s="86" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="70" t="inlineStr">
         <is>
           <t>→ DEMO 1  |  all above on main, docs updated, screenshots done — record full Swiggy read + AI + voice + live monitor demo ←</t>
         </is>
@@ -17769,7 +17951,6 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="B40:B49"/>
-    <mergeCell ref="A96:O96"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="B52:B54"/>
@@ -17777,6 +17958,7 @@
     <mergeCell ref="B32:B36"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B25:B28"/>
+    <mergeCell ref="A100:O100"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tracker: fix P6-MI05-MI14 completion dates -- 2026-07-06 (actual merge date), not 2026-07-05
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -16386,7 +16386,7 @@
       </c>
       <c r="E53" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: search_menu(query=dish_name) confirmed to return ZERO results for every query tested against this Swiggy sandbox -- real API calls, real zero value, not a bug. Removed _search_dish_prices entirely rather than ship a permanently-empty feature. The per-dish competitor table this task specified was superseded by a structurally different fix instead (see P6-MI12): exact dish-name matching between our menu and competitor menus turned out to never reliably align ("Butter Chicken" vs "Butter Chicken Masala" vs "Murgh Makhani"), so dish_prices was replaced by keyword-in-name category classification. dish_prices/DishPriceEntry models removed from market.py and lib/api.ts.</t>
+          <t>DONE 2026-07-06: search_menu(query=dish_name) confirmed to return ZERO results for every query tested against this Swiggy sandbox -- real API calls, real zero value, not a bug. Removed _search_dish_prices entirely rather than ship a permanently-empty feature. The per-dish competitor table this task specified was superseded by a structurally different fix instead (see P6-MI12): exact dish-name matching between our menu and competitor menus turned out to never reliably align ("Butter Chicken" vs "Butter Chicken Masala" vs "Murgh Makhani"), so dish_prices was replaced by keyword-in-name category classification. dish_prices/DishPriceEntry models removed from market.py and lib/api.ts.</t>
         </is>
       </c>
       <c r="F53" s="44" t="inlineStr">
@@ -16415,10 +16415,10 @@
         </is>
       </c>
       <c r="K53" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L53" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M53" s="47" t="n">
         <v>1</v>
@@ -16457,7 +16457,7 @@
       </c>
       <c r="E54" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: fetch_food_coupons(restaurantId, addressId) called per open competitor (max 3), filtered to COD-compatible (requiresOnlinePayment=False), building competitor_deals: [{restaurant, title, discount, code}]. Injected into menu_intel prompt and shown as its own "Competitor Swiggy Deals" card on /market with full discount/code detail per restaurant (not capped to the first result).</t>
+          <t>DONE 2026-07-06: fetch_food_coupons(restaurantId, addressId) called per open competitor (max 3), filtered to COD-compatible (requiresOnlinePayment=False), building competitor_deals: [{restaurant, title, discount, code}]. Injected into menu_intel prompt and shown as its own "Competitor Swiggy Deals" card on /market with full discount/code detail per restaurant (not capped to the first result).</t>
         </is>
       </c>
       <c r="F54" s="44" t="inlineStr">
@@ -16486,10 +16486,10 @@
         </is>
       </c>
       <c r="K54" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L54" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M54" s="47" t="n">
         <v>1</v>
@@ -16528,7 +16528,7 @@
       </c>
       <c r="E55" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: get_restaurant_details(restaurantId, lat, lng) called for top 3 open Dineout competitors, parsing deals[]/amenities/highlights/avgRating -&gt; competitor_dineout_deals (ALL deals per restaurant shown, not just the first). get_available_slots deals[] parsed with zero extra calls -&gt; slot_deals_found, aggregated by time-of-day (_aggregate_slot_availability_by_time) and rendered as OccupancyBySlotChart (status-colored HIGH/MEDIUM/LOW). Injected into reservation node prompt via OccupancyEnricher.</t>
+          <t>DONE 2026-07-06: get_restaurant_details(restaurantId, lat, lng) called for top 3 open Dineout competitors, parsing deals[]/amenities/highlights/avgRating -&gt; competitor_dineout_deals (ALL deals per restaurant shown, not just the first). get_available_slots deals[] parsed with zero extra calls -&gt; slot_deals_found, aggregated by time-of-day (_aggregate_slot_availability_by_time) and rendered as OccupancyBySlotChart (status-colored HIGH/MEDIUM/LOW). Injected into reservation node prompt via OccupancyEnricher.</t>
         </is>
       </c>
       <c r="F55" s="44" t="inlineStr">
@@ -16557,10 +16557,10 @@
         </is>
       </c>
       <c r="K55" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L55" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M55" s="47" t="n">
         <v>1</v>
@@ -16599,7 +16599,7 @@
       </c>
       <c r="E56" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: Diff 7 added to EvaluationSanityChecker -- fires when market_intel_a.tonight_busy is True AND dineout_deals_count &gt;= 2, flagging that predicted walk-in demand may be absorbed by competitor promotions. Total active assumption diffs: 7.</t>
+          <t>DONE 2026-07-06: Diff 7 added to EvaluationSanityChecker -- fires when market_intel_a.tonight_busy is True AND dineout_deals_count &gt;= 2, flagging that predicted walk-in demand may be absorbed by competitor promotions. Total active assumption diffs: 7.</t>
         </is>
       </c>
       <c r="F56" s="44" t="inlineStr">
@@ -16628,10 +16628,10 @@
         </is>
       </c>
       <c r="K56" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L56" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M56" s="47" t="n">
         <v>1</v>
@@ -16670,7 +16670,7 @@
       </c>
       <c r="E57" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: Pricing impact model added (elasticity model: gap_pct * -0.8 = volume_change_pct; weekly_revenue_impact_inr computed per flagged item, top 5 by absolute impact returned). Rendered as a diverging PricingImpactChart (rose = at-risk, emerald = upside) on /market, honestly scoped to exact dish-name matches only -- a smaller "Exact Menu Matches" card, since exact matching across restaurants is unreliable (see P6-MI12).</t>
+          <t>DONE 2026-07-06: Pricing impact model added (elasticity model: gap_pct * -0.8 = volume_change_pct; weekly_revenue_impact_inr computed per flagged item, top 5 by absolute impact returned). Rendered as a diverging PricingImpactChart (rose = at-risk, emerald = upside) on /market, honestly scoped to exact dish-name matches only -- a smaller "Exact Menu Matches" card, since exact matching across restaurants is unreliable (see P6-MI12).</t>
         </is>
       </c>
       <c r="F57" s="44" t="inlineStr">
@@ -16699,10 +16699,10 @@
         </is>
       </c>
       <c r="K57" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L57" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M57" s="47" t="n">
         <v>1</v>
@@ -16741,7 +16741,7 @@
       </c>
       <c r="E58" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: ScenarioRecommender (domain/services/scenario_recommender.py) built -- LLM-based recommendation with a deterministic rule-based fallback, factoring in recent run history, live market_intel signals, calendar context (INDIAN_HOLIDAYS_2026 added to core/constants.py, 20 holidays), and inventory shortage count. GET /planning/recommend?target_date=YYYY-MM-DD added to api/routes/planning.py.</t>
+          <t>DONE 2026-07-06: ScenarioRecommender (domain/services/scenario_recommender.py) built -- LLM-based recommendation with a deterministic rule-based fallback, factoring in recent run history, live market_intel signals, calendar context (INDIAN_HOLIDAYS_2026 added to core/constants.py, 20 holidays), and inventory shortage count. GET /planning/recommend?target_date=YYYY-MM-DD added to api/routes/planning.py.</t>
         </is>
       </c>
       <c r="F58" s="44" t="inlineStr">
@@ -16770,10 +16770,10 @@
         </is>
       </c>
       <c r="K58" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L58" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M58" s="47" t="n">
         <v>1</v>
@@ -16812,7 +16812,7 @@
       </c>
       <c r="E59" s="44" t="inlineStr">
         <is>
-          <t>DONE 2026-07-05: GET /market/trends?days=N added -- reads market_intel from stored PlanningRun.final_response across past runs (zero new Swiggy calls), returns per-dish area_avg price history + occupancy signal history. MarketTrendChart.tsx renders both as recharts line charts on /market, dish-selectable, empty state when fewer than 3 data points.</t>
+          <t>DONE 2026-07-06: GET /market/trends?days=N added -- reads market_intel from stored PlanningRun.final_response across past runs (zero new Swiggy calls), returns per-dish area_avg price history + occupancy signal history. MarketTrendChart.tsx renders both as recharts line charts on /market, dish-selectable, empty state when fewer than 3 data points.</t>
         </is>
       </c>
       <c r="F59" s="44" t="inlineStr">
@@ -16841,10 +16841,10 @@
         </is>
       </c>
       <c r="K59" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L59" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M59" s="47" t="n">
         <v>1</v>
@@ -16912,10 +16912,10 @@
         </is>
       </c>
       <c r="K60" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L60" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M60" s="47" t="n">
         <v>1</v>
@@ -16983,10 +16983,10 @@
         </is>
       </c>
       <c r="K61" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L61" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M61" s="47" t="n">
         <v>1</v>
@@ -17050,10 +17050,10 @@
         </is>
       </c>
       <c r="K62" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="L62" s="46" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="M62" s="47" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
tracker: fix branch attribution -- MI01/02/03 marked Superseded (delivered via MI07/MI11/MI12), MI09/10/11 corrected from placeholder branch names to feature/swiggy-market-intel-extended
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -16152,161 +16152,169 @@
       <c r="O48" s="87" t="n"/>
     </row>
     <row r="49" ht="52.05" customHeight="1" s="77">
-      <c r="A49" s="52" t="inlineStr">
+      <c r="A49" s="72" t="inlineStr">
         <is>
           <t>P6-MI01</t>
         </is>
       </c>
-      <c r="B49" s="53" t="inlineStr">
-        <is>
-          <t>feature/swiggy-market-intel-expansion</t>
-        </is>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
+      <c r="B49" s="73" t="inlineStr">
+        <is>
+          <t>feature/swiggy-market-intel-extended</t>
+        </is>
+      </c>
+      <c r="C49" s="73" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D49" s="53" t="inlineStr">
+      <c r="D49" s="73" t="inlineStr">
         <is>
           <t>Competitor deal &amp; offer intelligence</t>
         </is>
       </c>
-      <c r="E49" s="53" t="inlineStr">
-        <is>
-          <t>Surface deal and amenity data from get_restaurant_details (already called in OccupancyEnricher but data discarded). Extract: deals[], isFree, title, amenities[], highlights[], avgRating per competitor. Add to market_intel_output as competitor_deals list. Show in Market Intelligence panel: Competitor X running 20% off deal. Has live music + valet. No new API calls — uses data already fetched.</t>
-        </is>
-      </c>
-      <c r="F49" s="53" t="inlineStr">
+      <c r="E49" s="73" t="inlineStr">
+        <is>
+          <t>Surface deal and amenity data from get_restaurant_details (already called in OccupancyEnricher but data discarded). Extract: deals[], isFree, title, amenities[], highlights[], avgRating per competitor. Add to market_intel_output as competitor_deals list. Show in Market Intelligence panel: Competitor X running 20% off deal. Has live music + valet. No new API calls — uses data already fetched. SUPERSEDED 2026-07-06 -- delivered as part of P6-MI07 (get_restaurant_details + slot deals[]) on feature/swiggy-market-intel-extended; never built as its own separate task.</t>
+        </is>
+      </c>
+      <c r="F49" s="73" t="inlineStr">
         <is>
           <t>feat: surface competitor deal and amenity intelligence from Dineout MCP</t>
         </is>
       </c>
-      <c r="G49" s="53" t="inlineStr">
+      <c r="G49" s="73" t="inlineStr">
         <is>
           <t>docs/AGENTS.md (OccupancyEnricher output extended)</t>
         </is>
       </c>
-      <c r="H49" s="54" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I49" s="52" t="inlineStr">
+      <c r="H49" s="74" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="I49" s="72" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J49" s="52" t="n"/>
-      <c r="K49" s="52" t="n"/>
-      <c r="L49" s="52" t="n"/>
-      <c r="M49" s="55" t="n">
+      <c r="J49" s="72" t="n"/>
+      <c r="K49" s="72" t="n"/>
+      <c r="L49" s="72" t="n"/>
+      <c r="M49" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="N49" s="53" t="n"/>
-      <c r="O49" s="53" t="n"/>
+      <c r="N49" s="73" t="n"/>
+      <c r="O49" s="73" t="n"/>
     </row>
     <row r="50" ht="52.05" customHeight="1" s="77">
-      <c r="A50" s="56" t="inlineStr">
+      <c r="A50" s="72" t="inlineStr">
         <is>
           <t>P6-MI02</t>
         </is>
       </c>
-      <c r="B50" s="57" t="n"/>
-      <c r="C50" s="57" t="inlineStr">
+      <c r="B50" s="73" t="inlineStr">
+        <is>
+          <t>feature/swiggy-market-intel-extended</t>
+        </is>
+      </c>
+      <c r="C50" s="73" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
-      <c r="D50" s="57" t="inlineStr">
+      <c r="D50" s="73" t="inlineStr">
         <is>
           <t>Competitor price trend tracking</t>
         </is>
       </c>
-      <c r="E50" s="57" t="inlineStr">
-        <is>
-          <t>New table: market_snapshots (org_id, snapshot_type, data jsonb, captured_at). After each planning run, persist competitor_pricing dict from CompetitorEnricher. MarketIntelService computes week-over-week delta per dish. market_intel_output gains price_trends field: [{dish, current_avg, prev_avg, delta_pct, direction}]. Panel shows: Biryani area avg up 18pct vs last week. Zero new Swiggy API calls - just persisting what we already fetch.</t>
-        </is>
-      </c>
-      <c r="F50" s="57" t="inlineStr">
+      <c r="E50" s="73" t="inlineStr">
+        <is>
+          <t>New table: market_snapshots (org_id, snapshot_type, data jsonb, captured_at). After each planning run, persist competitor_pricing dict from CompetitorEnricher. MarketIntelService computes week-over-week delta per dish. market_intel_output gains price_trends field: [{dish, current_avg, prev_avg, delta_pct, direction}]. Panel shows: Biryani area avg up 18pct vs last week. Zero new Swiggy API calls - just persisting what we already fetch. SUPERSEDED 2026-07-06 -- P6-MI11 achieved the same trend-view outcome by reading directly from stored PlanningRun.final_response on feature/swiggy-market-intel-extended; the dedicated market_snapshots table this task specified was never built.</t>
+        </is>
+      </c>
+      <c r="F50" s="73" t="inlineStr">
         <is>
           <t>feat: competitor price trend tracking — persist snapshots, week-over-week delta</t>
         </is>
       </c>
-      <c r="G50" s="57" t="inlineStr">
+      <c r="G50" s="73" t="inlineStr">
         <is>
           <t>docs/DATA_MODEL.md (market_snapshots table), docs/AGENTS.md</t>
         </is>
       </c>
-      <c r="H50" s="54" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I50" s="56" t="inlineStr">
+      <c r="H50" s="74" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="I50" s="72" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J50" s="56" t="n"/>
-      <c r="K50" s="56" t="n"/>
-      <c r="L50" s="56" t="n"/>
-      <c r="M50" s="58" t="n">
+      <c r="J50" s="72" t="n"/>
+      <c r="K50" s="72" t="n"/>
+      <c r="L50" s="72" t="n"/>
+      <c r="M50" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="N50" s="57" t="n"/>
-      <c r="O50" s="57" t="n"/>
+      <c r="N50" s="73" t="n"/>
+      <c r="O50" s="73" t="n"/>
     </row>
     <row r="51" ht="52.05" customHeight="1" s="77">
-      <c r="A51" s="52" t="inlineStr">
+      <c r="A51" s="72" t="inlineStr">
         <is>
           <t>P6-MI03</t>
         </is>
       </c>
-      <c r="B51" s="53" t="n"/>
-      <c r="C51" s="53" t="inlineStr">
+      <c r="B51" s="73" t="inlineStr">
+        <is>
+          <t>feature/swiggy-market-intel-extended</t>
+        </is>
+      </c>
+      <c r="C51" s="73" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D51" s="53" t="inlineStr">
+      <c r="D51" s="73" t="inlineStr">
         <is>
           <t>Category-level pricing analysis</t>
         </is>
       </c>
-      <c r="E51" s="53" t="inlineStr">
-        <is>
-          <t>CompetitorEnricher currently returns flat dish-&gt;price dict. Extend to group by inferred category (biryani/starters/mains/drinks). Compute area avg per category. Compare against restaurant menu categories. Output: [{category, your_avg, area_avg, diff_pct, verdict}]. menu_intelligence prompt gains: Your North Indian mains avg Rs.320 vs area Rs.275 (+16pct). Your starters Rs.180 vs area Rs.210 (-14pct underpriced). No new API calls - aggregation on existing CompetitorEnricher output.</t>
-        </is>
-      </c>
-      <c r="F51" s="53" t="inlineStr">
+      <c r="E51" s="73" t="inlineStr">
+        <is>
+          <t>CompetitorEnricher currently returns flat dish-&gt;price dict. Extend to group by inferred category (biryani/starters/mains/drinks). Compute area avg per category. Compare against restaurant menu categories. Output: [{category, your_avg, area_avg, diff_pct, verdict}]. menu_intelligence prompt gains: Your North Indian mains avg Rs.320 vs area Rs.275 (+16pct). Your starters Rs.180 vs area Rs.210 (-14pct underpriced). No new API calls - aggregation on existing CompetitorEnricher output. SUPERSEDED 2026-07-06 -- delivered (and extended with named cheapest/priciest dishes) as part of P6-MI12 on feature/swiggy-market-intel-extended; never built as its own separate task.</t>
+        </is>
+      </c>
+      <c r="F51" s="73" t="inlineStr">
         <is>
           <t>feat: category-level pricing — group competitor prices by category vs your menu</t>
         </is>
       </c>
-      <c r="G51" s="53" t="inlineStr">
+      <c r="G51" s="73" t="inlineStr">
         <is>
           <t>docs/AGENTS.md (CompetitorEnricher output extended)</t>
         </is>
       </c>
-      <c r="H51" s="54" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I51" s="52" t="inlineStr">
+      <c r="H51" s="74" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="I51" s="72" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J51" s="52" t="n"/>
-      <c r="K51" s="52" t="n"/>
-      <c r="L51" s="52" t="n"/>
-      <c r="M51" s="55" t="n">
+      <c r="J51" s="72" t="n"/>
+      <c r="K51" s="72" t="n"/>
+      <c r="L51" s="72" t="n"/>
+      <c r="M51" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="N51" s="53" t="n"/>
-      <c r="O51" s="53" t="n"/>
+      <c r="N51" s="73" t="n"/>
+      <c r="O51" s="73" t="n"/>
     </row>
     <row r="52" ht="52.05" customHeight="1" s="77">
       <c r="A52" s="56" t="inlineStr">
@@ -16655,7 +16663,7 @@
       </c>
       <c r="B57" s="44" t="inlineStr">
         <is>
-          <t>feature/pricing-impact-model</t>
+          <t>feature/swiggy-market-intel-extended</t>
         </is>
       </c>
       <c r="C57" s="44" t="inlineStr">
@@ -16726,7 +16734,7 @@
       </c>
       <c r="B58" s="44" t="inlineStr">
         <is>
-          <t>feature/scenario-recommendation</t>
+          <t>feature/swiggy-market-intel-extended</t>
         </is>
       </c>
       <c r="C58" s="44" t="inlineStr">
@@ -16797,7 +16805,7 @@
       </c>
       <c r="B59" s="44" t="inlineStr">
         <is>
-          <t>feature/trend-analytics</t>
+          <t>feature/swiggy-market-intel-extended</t>
         </is>
       </c>
       <c r="C59" s="44" t="inlineStr">

</xml_diff>

<commit_message>
tracker: renumber P6-A1-A36 to match actual build sequence after the procurement/Action Queue deferral
Task IDs now read strictly top-to-bottom matching the real order we'll
build in, not just physical position with old labels. All Depends On
references remapped in both the Phase 6 sheet and the Staging Creds +
Phase 7 sheet (including inline prose mentions).
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -17338,7 +17338,7 @@
     <row r="69" ht="52.05" customHeight="1" s="82">
       <c r="A69" s="42" t="inlineStr">
         <is>
-          <t>P6-A8</t>
+          <t>P6-A5</t>
         </is>
       </c>
       <c r="B69" s="92" t="inlineStr">
@@ -17401,7 +17401,7 @@
     <row r="70" ht="7.95" customHeight="1" s="82">
       <c r="A70" s="42" t="inlineStr">
         <is>
-          <t>P6-A14</t>
+          <t>P6-A6</t>
         </is>
       </c>
       <c r="B70" s="92" t="inlineStr">
@@ -17464,7 +17464,7 @@
     <row r="71" ht="18" customHeight="1" s="82">
       <c r="A71" s="42" t="inlineStr">
         <is>
-          <t>P6-A15</t>
+          <t>P6-A7</t>
         </is>
       </c>
       <c r="B71" s="72" t="n"/>
@@ -17515,7 +17515,7 @@
       </c>
       <c r="N71" s="70" t="inlineStr">
         <is>
-          <t>P6-A14</t>
+          <t>P6-A6</t>
         </is>
       </c>
       <c r="O71" s="70" t="inlineStr">
@@ -17527,7 +17527,7 @@
     <row r="72" ht="52.05" customHeight="1" s="82">
       <c r="A72" s="42" t="inlineStr">
         <is>
-          <t>P6-A18</t>
+          <t>P6-A8</t>
         </is>
       </c>
       <c r="B72" s="92" t="inlineStr">
@@ -17590,7 +17590,7 @@
     <row r="73" ht="52.05" customHeight="1" s="82">
       <c r="A73" s="42" t="inlineStr">
         <is>
-          <t>P6-A19</t>
+          <t>P6-A9</t>
         </is>
       </c>
       <c r="B73" s="72" t="n"/>
@@ -17649,7 +17649,7 @@
     <row r="74" ht="18" customHeight="1" s="82">
       <c r="A74" s="42" t="inlineStr">
         <is>
-          <t>P6-A20</t>
+          <t>P6-A10</t>
         </is>
       </c>
       <c r="B74" s="92" t="inlineStr">
@@ -17669,7 +17669,7 @@
       </c>
       <c r="E74" s="70" t="inlineStr">
         <is>
-          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A16) exists or once real customers have multiple outlets.</t>
+          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A31) exists or once real customers have multiple outlets.</t>
         </is>
       </c>
       <c r="F74" s="70" t="inlineStr">
@@ -17712,7 +17712,7 @@
     <row r="75" ht="52.05" customHeight="1" s="82">
       <c r="A75" s="42" t="inlineStr">
         <is>
-          <t>P6-A21</t>
+          <t>P6-A11</t>
         </is>
       </c>
       <c r="B75" s="72" t="n"/>
@@ -17763,7 +17763,7 @@
       </c>
       <c r="N75" s="70" t="inlineStr">
         <is>
-          <t>P6-A20</t>
+          <t>P6-A10</t>
         </is>
       </c>
       <c r="O75" s="70" t="inlineStr">
@@ -17775,7 +17775,7 @@
     <row r="76" ht="52.05" customHeight="1" s="82">
       <c r="A76" s="42" t="inlineStr">
         <is>
-          <t>P6-A24</t>
+          <t>P6-A12</t>
         </is>
       </c>
       <c r="B76" s="92" t="inlineStr">
@@ -17838,7 +17838,7 @@
     <row r="77" ht="52.05" customHeight="1" s="82">
       <c r="A77" s="42" t="inlineStr">
         <is>
-          <t>P6-A25</t>
+          <t>P6-A13</t>
         </is>
       </c>
       <c r="B77" s="72" t="n"/>
@@ -17889,7 +17889,7 @@
       </c>
       <c r="N77" s="70" t="inlineStr">
         <is>
-          <t>P6-A24</t>
+          <t>P6-A12</t>
         </is>
       </c>
       <c r="O77" s="70" t="inlineStr">
@@ -17901,7 +17901,7 @@
     <row r="78" ht="52.05" customHeight="1" s="82">
       <c r="A78" s="42" t="inlineStr">
         <is>
-          <t>P6-A26</t>
+          <t>P6-A14</t>
         </is>
       </c>
       <c r="B78" s="92" t="inlineStr">
@@ -17964,7 +17964,7 @@
     <row r="79" ht="18" customHeight="1" s="82">
       <c r="A79" s="42" t="inlineStr">
         <is>
-          <t>P6-A27</t>
+          <t>P6-A15</t>
         </is>
       </c>
       <c r="B79" s="72" t="n"/>
@@ -18023,7 +18023,7 @@
     <row r="80" ht="52.05" customHeight="1" s="82">
       <c r="A80" s="42" t="inlineStr">
         <is>
-          <t>P6-A28</t>
+          <t>P6-A16</t>
         </is>
       </c>
       <c r="B80" s="92" t="inlineStr">
@@ -18086,7 +18086,7 @@
     <row r="81" ht="7.95" customHeight="1" s="82">
       <c r="A81" s="42" t="inlineStr">
         <is>
-          <t>P6-A29</t>
+          <t>P6-A17</t>
         </is>
       </c>
       <c r="B81" s="71" t="n"/>
@@ -18145,7 +18145,7 @@
     <row r="82" ht="52.05" customHeight="1" s="82">
       <c r="A82" s="42" t="inlineStr">
         <is>
-          <t>P6-A30</t>
+          <t>P6-A18</t>
         </is>
       </c>
       <c r="B82" s="72" t="n"/>
@@ -18204,7 +18204,7 @@
     <row r="83" ht="52.05" customHeight="1" s="82">
       <c r="A83" s="42" t="inlineStr">
         <is>
-          <t>P6-A31</t>
+          <t>P6-A19</t>
         </is>
       </c>
       <c r="B83" s="92" t="inlineStr">
@@ -18267,7 +18267,7 @@
     <row r="84" ht="7.95" customHeight="1" s="82">
       <c r="A84" s="42" t="inlineStr">
         <is>
-          <t>P6-A33</t>
+          <t>P6-A20</t>
         </is>
       </c>
       <c r="B84" s="92" t="inlineStr">
@@ -18330,7 +18330,7 @@
     <row r="85" ht="18" customHeight="1" s="82">
       <c r="A85" s="42" t="inlineStr">
         <is>
-          <t>P6-A34</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="B85" s="92" t="inlineStr">
@@ -18393,7 +18393,7 @@
     <row r="86" ht="52.05" customHeight="1" s="82">
       <c r="A86" s="42" t="inlineStr">
         <is>
-          <t>P6-A35</t>
+          <t>P6-A22</t>
         </is>
       </c>
       <c r="B86" s="92" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="N86" s="70" t="inlineStr">
         <is>
-          <t>P6-A8</t>
+          <t>P6-A5</t>
         </is>
       </c>
       <c r="O86" s="70" t="inlineStr">
@@ -18484,7 +18484,7 @@
     <row r="89" ht="39.6" customHeight="1" s="82">
       <c r="A89" s="42" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="B89" s="92" t="inlineStr">
@@ -18547,7 +18547,7 @@
     <row r="90" ht="39.6" customHeight="1" s="82">
       <c r="A90" s="42" t="inlineStr">
         <is>
-          <t>P6-A6</t>
+          <t>P6-A24</t>
         </is>
       </c>
       <c r="B90" s="72" t="n"/>
@@ -18598,7 +18598,7 @@
       </c>
       <c r="N90" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O90" s="70" t="inlineStr">
@@ -18610,7 +18610,7 @@
     <row r="91" ht="39.6" customHeight="1" s="82">
       <c r="A91" s="42" t="inlineStr">
         <is>
-          <t>P6-A7</t>
+          <t>P6-A25</t>
         </is>
       </c>
       <c r="B91" s="92" t="inlineStr">
@@ -18665,7 +18665,7 @@
       </c>
       <c r="N91" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O91" s="70" t="inlineStr">
@@ -18677,7 +18677,7 @@
     <row r="92" ht="39.6" customHeight="1" s="82">
       <c r="A92" s="42" t="inlineStr">
         <is>
-          <t>P6-A9</t>
+          <t>P6-A26</t>
         </is>
       </c>
       <c r="B92" s="72" t="n"/>
@@ -18728,7 +18728,7 @@
       </c>
       <c r="N92" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O92" s="70" t="inlineStr">
@@ -18740,7 +18740,7 @@
     <row r="93" ht="39.6" customHeight="1" s="82">
       <c r="A93" s="42" t="inlineStr">
         <is>
-          <t>P6-A10</t>
+          <t>P6-A27</t>
         </is>
       </c>
       <c r="B93" s="92" t="inlineStr">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="N93" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O93" s="70" t="inlineStr">
@@ -18807,7 +18807,7 @@
     <row r="94" ht="39.6" customHeight="1" s="82">
       <c r="A94" s="42" t="inlineStr">
         <is>
-          <t>P6-A11</t>
+          <t>P6-A28</t>
         </is>
       </c>
       <c r="B94" s="72" t="n"/>
@@ -18858,7 +18858,7 @@
       </c>
       <c r="N94" s="70" t="inlineStr">
         <is>
-          <t>P6-A5, P6-A10</t>
+          <t>P6-A23, P6-A27</t>
         </is>
       </c>
       <c r="O94" s="70" t="inlineStr">
@@ -18870,7 +18870,7 @@
     <row r="95" ht="52.8" customHeight="1" s="82">
       <c r="A95" s="42" t="inlineStr">
         <is>
-          <t>P6-A12</t>
+          <t>P6-A29</t>
         </is>
       </c>
       <c r="B95" s="92" t="inlineStr">
@@ -18890,7 +18890,7 @@
       </c>
       <c r="E95" s="70" t="inlineStr">
         <is>
-          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A17.</t>
+          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A32.</t>
         </is>
       </c>
       <c r="F95" s="70" t="inlineStr">
@@ -18925,7 +18925,7 @@
       </c>
       <c r="N95" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O95" s="70" t="inlineStr">
@@ -18937,7 +18937,7 @@
     <row r="96" ht="171.6" customHeight="1" s="82">
       <c r="A96" s="42" t="inlineStr">
         <is>
-          <t>P6-A13</t>
+          <t>P6-A30</t>
         </is>
       </c>
       <c r="B96" s="72" t="n"/>
@@ -18953,7 +18953,7 @@
       </c>
       <c r="E96" s="70" t="inlineStr">
         <is>
-          <t>Same pattern as P6-A7 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
+          <t>Same pattern as P6-A25 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
         </is>
       </c>
       <c r="F96" s="70" t="inlineStr">
@@ -18988,7 +18988,7 @@
       </c>
       <c r="N96" s="70" t="inlineStr">
         <is>
-          <t>P6-A5, P6-A12</t>
+          <t>P6-A23, P6-A29</t>
         </is>
       </c>
       <c r="O96" s="70" t="inlineStr">
@@ -19000,7 +19000,7 @@
     <row r="97" ht="39.6" customHeight="1" s="82">
       <c r="A97" s="42" t="inlineStr">
         <is>
-          <t>P6-A16</t>
+          <t>P6-A31</t>
         </is>
       </c>
       <c r="B97" s="92" t="inlineStr">
@@ -19063,7 +19063,7 @@
     <row r="98" ht="39.6" customHeight="1" s="82">
       <c r="A98" s="42" t="inlineStr">
         <is>
-          <t>P6-A17</t>
+          <t>P6-A32</t>
         </is>
       </c>
       <c r="B98" s="72" t="n"/>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="N98" s="70" t="inlineStr">
         <is>
-          <t>P6-A16</t>
+          <t>P6-A31</t>
         </is>
       </c>
       <c r="O98" s="70" t="inlineStr">
@@ -19126,7 +19126,7 @@
     <row r="99" ht="52.8" customHeight="1" s="82">
       <c r="A99" s="42" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A33</t>
         </is>
       </c>
       <c r="B99" s="92" t="inlineStr">
@@ -19181,7 +19181,7 @@
       </c>
       <c r="N99" s="70" t="inlineStr">
         <is>
-          <t>P6-A5</t>
+          <t>P6-A23</t>
         </is>
       </c>
       <c r="O99" s="70" t="inlineStr">
@@ -19193,7 +19193,7 @@
     <row r="100" ht="171.6" customHeight="1" s="82">
       <c r="A100" s="42" t="inlineStr">
         <is>
-          <t>P6-A23</t>
+          <t>P6-A34</t>
         </is>
       </c>
       <c r="B100" s="72" t="n"/>
@@ -19209,7 +19209,7 @@
       </c>
       <c r="E100" s="70" t="inlineStr">
         <is>
-          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A17 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
+          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A32 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
         </is>
       </c>
       <c r="F100" s="70" t="inlineStr">
@@ -19244,7 +19244,7 @@
       </c>
       <c r="N100" s="70" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A33</t>
         </is>
       </c>
       <c r="O100" s="70" t="inlineStr">
@@ -19256,7 +19256,7 @@
     <row r="101">
       <c r="A101" s="42" t="inlineStr">
         <is>
-          <t>P6-A32</t>
+          <t>P6-A35</t>
         </is>
       </c>
       <c r="B101" s="92" t="inlineStr">
@@ -19311,7 +19311,7 @@
       </c>
       <c r="N101" s="70" t="inlineStr">
         <is>
-          <t>P6-A6</t>
+          <t>P6-A24</t>
         </is>
       </c>
       <c r="O101" s="70" t="inlineStr">
@@ -19560,7 +19560,7 @@
       </c>
       <c r="E4" s="68" t="inlineStr">
         <is>
-          <t>Phase A (P6-A12) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
+          <t>Phase A (P6-A29) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
         </is>
       </c>
       <c r="F4" s="68" t="inlineStr">
@@ -19595,7 +19595,7 @@
       </c>
       <c r="N4" s="68" t="inlineStr">
         <is>
-          <t>P6-A12, P6-S14</t>
+          <t>P6-A29, P6-S14</t>
         </is>
       </c>
       <c r="O4" s="68" t="inlineStr">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="E6" s="68" t="inlineStr">
         <is>
-          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A13) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
+          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A30) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
         </is>
       </c>
       <c r="F6" s="68" t="inlineStr">
@@ -19679,7 +19679,7 @@
       </c>
       <c r="N6" s="68" t="inlineStr">
         <is>
-          <t>P6-A13</t>
+          <t>P6-A30</t>
         </is>
       </c>
       <c r="O6" s="68" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="E8" s="68" t="inlineStr">
         <is>
-          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A9) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
+          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A26) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
         </is>
       </c>
       <c r="F8" s="68" t="inlineStr">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="N8" s="68" t="inlineStr">
         <is>
-          <t>P6-A9, P7-1, P7-2</t>
+          <t>P6-A26, P7-1, P7-2</t>
         </is>
       </c>
       <c r="O8" s="68" t="inlineStr">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="N14" s="68" t="inlineStr">
         <is>
-          <t>P6-A34</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O14" s="68" t="inlineStr">
@@ -20684,6 +20684,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="68" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tracker: delete P6-A5 (anomaly investigation agent) -- can't be genuinely demonstrated on seeded data, cascade-renumber A6-A36 to A5-A35
Its real value only shows up once real sales history exists to detect a
genuine deviation from; on seeded data any anomaly would have to be staged,
which proves less than it looks like. Cleared the stale dependency on the
now-deleted task from what's now P6-A21 (/live page reframed) rather than
remap it to something unrelated.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -189,6 +189,7 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font/>
   </fonts>
   <fills count="22">
     <fill>
@@ -302,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -465,11 +466,12 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -755,6 +757,7 @@
     <xf numFmtId="0" fontId="14" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17145,7 +17148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:O41"/>
+  <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.109375" customWidth="1" style="72" min="1" max="1"/>
@@ -17261,7 +17264,7 @@
       </c>
       <c r="E3" s="90" t="inlineStr">
         <is>
-          <t>CompetitorEnricher already computes menu_breadth, cuisine_crowding, veg_mix, and competitor_landscape, and OccupancyEnricher computes slot_availability_by_time -- all of it reaches /market/pulse and the /market page, but NONE of it is passed into _build_prompt(), so menu_intelligence, the critic, and the actual generated plan never see it. Wire these into CompetitorEnricher._build_prompt() (and OccupancyEnricher's equivalent) so the LLM reasoning actually reflects everything already being computed, not just category pricing/positioning/deals/pricing impact. Also absorbed in this same branch (originally planned as a separate task, P6-A5, before it turned out to ship in the same PR): floating chat widget (bottom-right bubble, expandable to the full /chat page) backed by real conversation persistence -- new ChatSession/ChatMessage tables (chat history previously lived only in frontend React state per page load, nothing was queryable server-side), GET /chat/sessions (list past threads) + GET /chat/sessions/{id} (full thread), and a shared ChatSessionContext so the floating widget and the full /chat page never lose context switching between them. LIVE-VERIFIED 2026-07-06 against the real running backend (not just unit tests): cleared the stale Redis cache from before this change, confirmed CompetitorEnricher._build_prompt() now genuinely includes Menu breadth/Cuisine crowding/veg-non-veg mix/Competitor landscape sections against the real Swiggy account.</t>
+          <t>CompetitorEnricher already computes menu_breadth, cuisine_crowding, veg_mix, and competitor_landscape, and OccupancyEnricher computes slot_availability_by_time -- all of it reaches /market/pulse and the /market page, but NONE of it is passed into _build_prompt(), so menu_intelligence, the critic, and the actual generated plan never see it. Wire these into CompetitorEnricher._build_prompt() (and OccupancyEnricher's equivalent) so the LLM reasoning actually reflects everything already being computed, not just category pricing/positioning/deals/pricing impact. Also absorbed in this same branch (originally planned as a separate task, before it turned out to ship in the same PR): floating chat widget (bottom-right bubble, expandable to the full /chat page) backed by real conversation persistence -- new ChatSession/ChatMessage tables (chat history previously lived only in frontend React state per page load, nothing was queryable server-side), GET /chat/sessions (list past threads) + GET /chat/sessions/{id} (full thread), and a shared ChatSessionContext so the floating widget and the full /chat page never lose context switching between them. LIVE-VERIFIED 2026-07-06 against the real running backend (not just unit tests): cleared the stale Redis cache from before this change, confirmed CompetitorEnricher._build_prompt() now genuinely includes Menu breadth/Cuisine crowding/veg-non-veg mix/Competitor landscape sections against the real Swiggy account.</t>
         </is>
       </c>
       <c r="F3" s="90" t="inlineStr">
@@ -17515,2086 +17518,2004 @@
       </c>
     </row>
     <row r="7" ht="52.05" customFormat="1" customHeight="1" s="97">
-      <c r="A7" s="92" t="n"/>
-      <c r="B7" s="93" t="n"/>
-      <c r="C7" s="94" t="n"/>
-      <c r="D7" s="94" t="n"/>
-      <c r="E7" s="94" t="n"/>
-      <c r="F7" s="94" t="n"/>
-      <c r="G7" s="94" t="n"/>
-      <c r="H7" s="95" t="n"/>
-      <c r="I7" s="92" t="n"/>
-      <c r="J7" s="92" t="n"/>
-      <c r="K7" s="92" t="n"/>
-      <c r="L7" s="92" t="n"/>
-      <c r="M7" s="96" t="n"/>
-      <c r="N7" s="94" t="n"/>
-      <c r="O7" s="94" t="n"/>
+      <c r="A7" s="65" t="inlineStr">
+        <is>
+          <t>P6-A5</t>
+        </is>
+      </c>
+      <c r="B7" s="98" t="inlineStr">
+        <is>
+          <t>feature/multi-platform-connectors</t>
+        </is>
+      </c>
+      <c r="C7" s="90" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D7" s="90" t="inlineStr">
+        <is>
+          <t>Zomato stub connector</t>
+        </is>
+      </c>
+      <c r="E7" s="90" t="inlineStr">
+        <is>
+          <t>ZomatoConnector class following the exact BaseConnector shape (sync()/enrich()) as SwiggyConnector, registered in provider_registry.py's CAPABILITY_PROVIDERS as an actually-real (if non-functional) connector rather than a placeholder string. Proves the multi-provider architecture is real, not Swiggy-only. No live Zomato API call required -- returns a clear 'not yet connected' state.</t>
+        </is>
+      </c>
+      <c r="F7" s="90" t="inlineStr">
+        <is>
+          <t>feat: ZomatoConnector stub -- proves multi-provider architecture, no live API required</t>
+        </is>
+      </c>
+      <c r="G7" s="90" t="inlineStr">
+        <is>
+          <t>CLAUDE.md, docs/CONNECTORS.md</t>
+        </is>
+      </c>
+      <c r="H7" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I7" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J7" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K7" s="89" t="n"/>
+      <c r="L7" s="89" t="n"/>
+      <c r="M7" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="90" t="n"/>
+      <c r="O7" s="90" t="inlineStr">
+        <is>
+          <t>connector registers correctly in provider_registry; enrich() returns a clean not-connected state, never raises</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52.05" customHeight="1" s="72">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="65" t="inlineStr">
+        <is>
+          <t>P6-A6</t>
+        </is>
+      </c>
+      <c r="B8" s="69" t="n"/>
+      <c r="C8" s="90" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D8" s="90" t="inlineStr">
+        <is>
+          <t>Public review aggregation connectors (Google/Zomato reviews)</t>
+        </is>
+      </c>
+      <c r="E8" s="90" t="inlineStr">
+        <is>
+          <t>GoogleReviewsConnector / ZomatoReviewsConnector following the same BaseConnector pattern, pulling public review data (not internal complaints) into complaint_intelligence as an additional source type. Extends the Feedback model's source concept rather than inventing a parallel system.</t>
+        </is>
+      </c>
+      <c r="F8" s="90" t="inlineStr">
+        <is>
+          <t>feat: public review aggregation -- Google/Zomato reviews via BaseConnector pattern</t>
+        </is>
+      </c>
+      <c r="G8" s="90" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/CONNECTORS.md</t>
+        </is>
+      </c>
+      <c r="H8" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I8" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J8" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K8" s="89" t="n"/>
+      <c r="L8" s="89" t="n"/>
+      <c r="M8" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="90" t="inlineStr">
         <is>
           <t>P6-A5</t>
         </is>
       </c>
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>feature/anomaly-agent</t>
-        </is>
-      </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="O8" s="90" t="inlineStr">
+        <is>
+          <t>reviews ingested with correct source tag; complaint_intelligence node correctly surfaces public-review-sourced themes alongside internal ones</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="7.95" customHeight="1" s="72">
+      <c r="A9" s="65" t="inlineStr">
+        <is>
+          <t>P6-A7</t>
+        </is>
+      </c>
+      <c r="B9" s="98" t="inlineStr">
+        <is>
+          <t>feature/financial-compliance</t>
+        </is>
+      </c>
+      <c r="C9" s="90" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D9" s="90" t="inlineStr">
+        <is>
+          <t>Financial scorecard -- Expense ledger + real P&amp;L</t>
+        </is>
+      </c>
+      <c r="E9" s="90" t="inlineStr">
+        <is>
+          <t>New Expense model (category: rent/utilities/marketing/labor-later/other, amount, recurrence). Extends business.py's existing revenue/margin computation into a real daily/weekly P&amp;L and one composite health score. Designed so labor slots in later as just another Expense category, not a rewrite.</t>
+        </is>
+      </c>
+      <c r="F9" s="90" t="inlineStr">
+        <is>
+          <t>feat: financial scorecard -- Expense ledger, real P&amp;L, composite health score</t>
+        </is>
+      </c>
+      <c r="G9" s="90" t="inlineStr">
+        <is>
+          <t>docs/APIS.md</t>
+        </is>
+      </c>
+      <c r="H9" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I9" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J9" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K9" s="89" t="n"/>
+      <c r="L9" s="89" t="n"/>
+      <c r="M9" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="90" t="n"/>
+      <c r="O9" s="90" t="inlineStr">
+        <is>
+          <t>P&amp;L numbers match seeded expense + revenue data; health score computes deterministically from known inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="72">
+      <c r="A10" s="65" t="inlineStr">
+        <is>
+          <t>P6-A8</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="n"/>
+      <c r="C10" s="90" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D10" s="90" t="inlineStr">
+        <is>
+          <t>Compliance / Obligations calendar</t>
+        </is>
+      </c>
+      <c r="E10" s="90" t="inlineStr">
+        <is>
+          <t>Generalized Obligation model (type: license-renewal/GST-filing/inspection/other, due_date, status) with reminders delivered through the existing Phase-5 email digest mechanism rather than a new one-off sender. Not a GST computation/invoicing layer -- just a dated-obligation tracker with reminders.</t>
+        </is>
+      </c>
+      <c r="F10" s="90" t="inlineStr">
+        <is>
+          <t>feat: compliance/obligations calendar -- reminder engine reusing the existing email digest</t>
+        </is>
+      </c>
+      <c r="G10" s="90" t="inlineStr">
+        <is>
+          <t>docs/APIS.md</t>
+        </is>
+      </c>
+      <c r="H10" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I10" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J10" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K10" s="89" t="n"/>
+      <c r="L10" s="89" t="n"/>
+      <c r="M10" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="90" t="n"/>
+      <c r="O10" s="90" t="inlineStr">
+        <is>
+          <t>reminder fires at the correct lead-time before due_date; reuses existing digest delivery path</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52.05" customHeight="1" s="72">
+      <c r="A11" s="65" t="inlineStr">
+        <is>
+          <t>P6-A9</t>
+        </is>
+      </c>
+      <c r="B11" s="98" t="inlineStr">
+        <is>
+          <t>feature/location-architecture</t>
+        </is>
+      </c>
+      <c r="C11" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D11" s="90" t="inlineStr">
+        <is>
+          <t>Location-aware enrichers (hedge for multi-location)</t>
+        </is>
+      </c>
+      <c r="E11" s="90" t="inlineStr">
+        <is>
+          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A30) exists or once real customers have multiple outlets.</t>
+        </is>
+      </c>
+      <c r="F11" s="90" t="inlineStr">
+        <is>
+          <t>feat: location-aware enrichers -- pass address/location context through instead of one hardcoded address</t>
+        </is>
+      </c>
+      <c r="G11" s="90" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H11" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I11" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J11" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K11" s="89" t="n"/>
+      <c r="L11" s="89" t="n"/>
+      <c r="M11" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="90" t="n"/>
+      <c r="O11" s="90" t="inlineStr">
+        <is>
+          <t>enrichers accept and correctly use a passed-in address_id, defaulting to the existing single-address behavior when none given</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52.05" customHeight="1" s="72">
+      <c r="A12" s="65" t="inlineStr">
+        <is>
+          <t>P6-A10</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="n"/>
+      <c r="C12" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D12" s="90" t="inlineStr">
+        <is>
+          <t>Multi-location / Restaurant entity -- STRATEGIC, needs explicit go/no-go</t>
+        </is>
+      </c>
+      <c r="E12" s="90" t="inlineStr">
+        <is>
+          <t>Introduce Restaurant as a first-class entity between Organization and everything else (menu, inventory, planning runs, Swiggy connector -- each physical location has its own Swiggy restaurant ID). Add restaurant_id to MenuItem/InventoryItem/PlanningRun/connectors. Cheaper to do now while the schema is small than to retrofit later. NOT started until the user confirms real near-term demand justifies it over other Phase A work.</t>
+        </is>
+      </c>
+      <c r="F12" s="90" t="inlineStr">
+        <is>
+          <t>feat: Restaurant entity -- first-class multi-location support</t>
+        </is>
+      </c>
+      <c r="G12" s="90" t="inlineStr">
+        <is>
+          <t>docs/DATA_MODEL.md, docs/DECISIONS.md</t>
+        </is>
+      </c>
+      <c r="H12" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I12" s="89" t="inlineStr">
+        <is>
+          <t>Low (pending go/no-go)</t>
+        </is>
+      </c>
+      <c r="J12" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K12" s="89" t="n"/>
+      <c r="L12" s="89" t="n"/>
+      <c r="M12" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="90" t="inlineStr">
+        <is>
+          <t>P6-A9</t>
+        </is>
+      </c>
+      <c r="O12" s="90" t="inlineStr">
+        <is>
+          <t>existing single-location orgs continue to work unchanged (default restaurant backfilled); cross-location query test once 2+ restaurants exist</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="72">
+      <c r="A13" s="65" t="inlineStr">
+        <is>
+          <t>P6-A11</t>
+        </is>
+      </c>
+      <c r="B13" s="98" t="inlineStr">
+        <is>
+          <t>feature/chatbot-dineout-tools</t>
+        </is>
+      </c>
+      <c r="C13" s="90" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D13" s="90" t="inlineStr">
+        <is>
+          <t>Chatbot -- Dineout competitive query tools</t>
+        </is>
+      </c>
+      <c r="E13" s="90" t="inlineStr">
+        <is>
+          <t>3 Groq function-calling tools for the existing chatbot: get_competitor_deals, get_area_occupancy, get_trending_dishes -- all using Swiggy's existing read-only Dineout MCP (search_restaurants_dineout, get_restaurant_details, get_available_slots), already-proven tools. (Formerly P6-MI04; renumbered as part of the Phase 6 replan.)</t>
+        </is>
+      </c>
+      <c r="F13" s="90" t="inlineStr">
+        <is>
+          <t>feat: chatbot Dineout tools -- competitor deals, area occupancy, trending dishes</t>
+        </is>
+      </c>
+      <c r="G13" s="90" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="H13" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I13" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J13" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K13" s="89" t="n"/>
+      <c r="L13" s="89" t="n"/>
+      <c r="M13" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="90" t="n"/>
+      <c r="O13" s="90" t="inlineStr">
+        <is>
+          <t>all 3 tools callable from /chat; correct Swiggy data returned; graceful None on failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52.05" customHeight="1" s="72">
+      <c r="A14" s="65" t="inlineStr">
+        <is>
+          <t>P6-A12</t>
+        </is>
+      </c>
+      <c r="B14" s="69" t="n"/>
+      <c r="C14" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D14" s="90" t="inlineStr">
+        <is>
+          <t>Structured outputs -- tool_choice=required across chatbot tools</t>
+        </is>
+      </c>
+      <c r="E14" s="90" t="inlineStr">
+        <is>
+          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema across all chatbot tools (Swiggy and internal). Chatbot function calls never hallucinate JSON.</t>
+        </is>
+      </c>
+      <c r="F14" s="90" t="inlineStr">
+        <is>
+          <t>feat: structured outputs -- tool_choice=required across all chatbot tools</t>
+        </is>
+      </c>
+      <c r="G14" s="90" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="H14" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I14" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J14" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K14" s="89" t="n"/>
+      <c r="L14" s="89" t="n"/>
+      <c r="M14" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="90" t="inlineStr">
+        <is>
+          <t>P6-A11</t>
+        </is>
+      </c>
+      <c r="O14" s="90" t="inlineStr">
+        <is>
+          <t>schema validation test; chatbot returns valid JSON on repeated calls</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52.05" customHeight="1" s="72">
+      <c r="A15" s="65" t="inlineStr">
+        <is>
+          <t>P6-A13</t>
+        </is>
+      </c>
+      <c r="B15" s="98" t="inlineStr">
+        <is>
+          <t>feature/llm-cost-quality</t>
+        </is>
+      </c>
+      <c r="C15" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D15" s="90" t="inlineStr">
+        <is>
+          <t>Prompt caching -- critic + aggregator</t>
+        </is>
+      </c>
+      <c r="E15" s="90" t="inlineStr">
+        <is>
+          <t>Add prompt-caching headers to critic and aggregator LLM calls (both have long, repeated system prompts). Cuts LLM cost per planning run; invisible to a demo but real cost hygiene.</t>
+        </is>
+      </c>
+      <c r="F15" s="90" t="inlineStr">
+        <is>
+          <t>feat: prompt caching -- cut LLM costs on critic and aggregator nodes</t>
+        </is>
+      </c>
+      <c r="G15" s="90" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H15" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I15" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J15" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K15" s="89" t="n"/>
+      <c r="L15" s="89" t="n"/>
+      <c r="M15" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="90" t="n"/>
+      <c r="O15" s="90" t="inlineStr">
+        <is>
+          <t>cost log shows cache_hit=true on second run of the same scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52.05" customHeight="1" s="72">
+      <c r="A16" s="65" t="inlineStr">
+        <is>
+          <t>P6-A14</t>
+        </is>
+      </c>
+      <c r="B16" s="69" t="n"/>
+      <c r="C16" s="90" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
-        <is>
-          <t>Anomaly-triggered investigation agent</t>
-        </is>
-      </c>
-      <c r="E8" s="43" t="inlineStr">
-        <is>
-          <t>A reactive service that, given a detected anomaly (e.g. a dish's sales dropped sharply vs the same weekday last period), chains the existing enrichers/services (CompetitorEnricher, complaint_intelligence, inventory) to synthesize one diagnosis instead of a human cross-referencing multiple dashboard cards. Ships with anomaly detection for the single clearest case first (dish-level sales drop) rather than a general anomaly framework. This is the clearest expression of 'separate synthesis layer' -- no single platform (Swiggy, a POS) could produce this alone.</t>
-        </is>
-      </c>
-      <c r="F8" s="43" t="inlineStr">
-        <is>
-          <t>feat: anomaly-triggered investigation agent -- reactive cross-signal diagnosis</t>
-        </is>
-      </c>
-      <c r="G8" s="43" t="inlineStr">
+      <c r="D16" s="90" t="inlineStr">
+        <is>
+          <t>Multi-agent debate critic</t>
+        </is>
+      </c>
+      <c r="E16" s="90" t="inlineStr">
+        <is>
+          <t>Two LLM critic instances (optimistic vs conservative), structured debate, moderator resolves disagreement. Marginal demo-visible upside over the existing single critic given the added cost/latency -- kept low priority.</t>
+        </is>
+      </c>
+      <c r="F16" s="90" t="inlineStr">
+        <is>
+          <t>feat: multi-agent debate critic -- consensus scoring</t>
+        </is>
+      </c>
+      <c r="G16" s="90" t="inlineStr">
         <is>
           <t>docs/AGENTS.md</t>
         </is>
       </c>
-      <c r="H8" s="41" t="inlineStr">
+      <c r="H16" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I8" s="42" t="inlineStr">
+      <c r="I16" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J16" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K16" s="89" t="n"/>
+      <c r="L16" s="89" t="n"/>
+      <c r="M16" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="90" t="n"/>
+      <c r="O16" s="90" t="inlineStr">
+        <is>
+          <t>debate resolves on test plans; disagreement cases escalate correctly</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52.05" customHeight="1" s="72">
+      <c r="A17" s="65" t="inlineStr">
+        <is>
+          <t>P6-A15</t>
+        </is>
+      </c>
+      <c r="B17" s="98" t="inlineStr">
+        <is>
+          <t>feature/ci-eval-hygiene</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D17" s="90" t="inlineStr">
+        <is>
+          <t>Fix SQLite/JSONB CI test-infra gap</t>
+        </is>
+      </c>
+      <c r="E17" s="90" t="inlineStr">
+        <is>
+          <t>test_swiggy_reservation_sync.py and test_connector_repository.py are excluded from CI because SQLite can't render Postgres JSONB columns. Either a SQLite-compatible fallback type or a Postgres CI service container.</t>
+        </is>
+      </c>
+      <c r="F17" s="90" t="inlineStr">
+        <is>
+          <t>fix: SQLite-compatible JSONB handling (or Postgres CI service) for excluded test files</t>
+        </is>
+      </c>
+      <c r="G17" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H17" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I17" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J17" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K17" s="89" t="n"/>
+      <c r="L17" s="89" t="n"/>
+      <c r="M17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="90" t="n"/>
+      <c r="O17" s="90" t="inlineStr">
+        <is>
+          <t>previously-excluded test files run in CI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="72">
+      <c r="A18" s="65" t="inlineStr">
+        <is>
+          <t>P6-A16</t>
+        </is>
+      </c>
+      <c r="B18" s="70" t="n"/>
+      <c r="C18" s="90" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D18" s="90" t="inlineStr">
+        <is>
+          <t>Promote reviewed RAGAS/DeepEval candidates</t>
+        </is>
+      </c>
+      <c r="E18" s="90" t="inlineStr">
+        <is>
+          <t>Recurring habit of running the existing candidate-generation scripts and hand-promoting reviewed candidates into the curated eval datasets.</t>
+        </is>
+      </c>
+      <c r="F18" s="90" t="inlineStr">
+        <is>
+          <t>chore: promote reviewed eval candidates into curated datasets</t>
+        </is>
+      </c>
+      <c r="G18" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H18" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I18" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J18" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K18" s="89" t="n"/>
+      <c r="L18" s="89" t="n"/>
+      <c r="M18" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="90" t="n"/>
+      <c r="O18" s="90" t="inlineStr">
+        <is>
+          <t>N/A -- ongoing process, not a one-time build</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52.05" customHeight="1" s="72">
+      <c r="A19" s="65" t="inlineStr">
+        <is>
+          <t>P6-A17</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="n"/>
+      <c r="C19" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D19" s="90" t="inlineStr">
+        <is>
+          <t>Regenerate golden_runs.json against real data</t>
+        </is>
+      </c>
+      <c r="E19" s="90" t="inlineStr">
+        <is>
+          <t>The key-path bug in build_golden_dataset.py is already fixed; the checked-in fixture still reflects the old broken extraction. Regenerate once real run history exists.</t>
+        </is>
+      </c>
+      <c r="F19" s="90" t="inlineStr">
+        <is>
+          <t>chore: regenerate golden_runs.json with corrected extraction logic</t>
+        </is>
+      </c>
+      <c r="G19" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H19" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I19" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J19" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K19" s="89" t="n"/>
+      <c r="L19" s="89" t="n"/>
+      <c r="M19" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="90" t="n"/>
+      <c r="O19" s="90" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="7.95" customHeight="1" s="72">
+      <c r="A20" s="65" t="inlineStr">
+        <is>
+          <t>P6-A18</t>
+        </is>
+      </c>
+      <c r="B20" s="98" t="inlineStr">
+        <is>
+          <t>feature/menu-engineering-matrix</t>
+        </is>
+      </c>
+      <c r="C20" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D20" s="90" t="inlineStr">
+        <is>
+          <t>Menu engineering matrix UI</t>
+        </is>
+      </c>
+      <c r="E20" s="90" t="inlineStr">
+        <is>
+          <t>Stars/plow-horses/dogs/puzzles quadrant chart using margin_pct x quantity, both already computed in business.py -- just needs quadrant classification + a chart.</t>
+        </is>
+      </c>
+      <c r="F20" s="90" t="inlineStr">
+        <is>
+          <t>feat: menu engineering matrix -- margin x popularity quadrant chart</t>
+        </is>
+      </c>
+      <c r="G20" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H20" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I20" s="89" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J8" s="42" t="inlineStr">
+      <c r="J20" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K8" s="42" t="n"/>
-      <c r="L8" s="42" t="n"/>
-      <c r="M8" s="44" t="n">
+      <c r="K20" s="89" t="n"/>
+      <c r="L20" s="89" t="n"/>
+      <c r="M20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="43" t="n"/>
-      <c r="O8" s="43" t="inlineStr">
-        <is>
-          <t>given a synthetic sales-drop + competitor-deal fixture, agent correctly attributes cause</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="7.95" customHeight="1" s="72">
-      <c r="A9" s="42" t="inlineStr">
-        <is>
-          <t>P6-A6</t>
-        </is>
-      </c>
-      <c r="B9" s="68" t="inlineStr">
-        <is>
-          <t>feature/multi-platform-connectors</t>
-        </is>
-      </c>
-      <c r="C9" s="43" t="inlineStr">
-        <is>
-          <t>Integrations</t>
-        </is>
-      </c>
-      <c r="D9" s="43" t="inlineStr">
-        <is>
-          <t>Zomato stub connector</t>
-        </is>
-      </c>
-      <c r="E9" s="43" t="inlineStr">
-        <is>
-          <t>ZomatoConnector class following the exact BaseConnector shape (sync()/enrich()) as SwiggyConnector, registered in provider_registry.py's CAPABILITY_PROVIDERS as an actually-real (if non-functional) connector rather than a placeholder string. Proves the multi-provider architecture is real, not Swiggy-only. No live Zomato API call required -- returns a clear 'not yet connected' state.</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
-        <is>
-          <t>feat: ZomatoConnector stub -- proves multi-provider architecture, no live API required</t>
-        </is>
-      </c>
-      <c r="G9" s="43" t="inlineStr">
-        <is>
-          <t>CLAUDE.md, docs/CONNECTORS.md</t>
-        </is>
-      </c>
-      <c r="H9" s="41" t="inlineStr">
+      <c r="N20" s="90" t="n"/>
+      <c r="O20" s="90" t="inlineStr">
+        <is>
+          <t>quadrant classification unit test; chart renders correctly</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52.05" customHeight="1" s="72">
+      <c r="A21" s="65" t="inlineStr">
+        <is>
+          <t>P6-A19</t>
+        </is>
+      </c>
+      <c r="B21" s="98" t="inlineStr">
+        <is>
+          <t>feature/pages-redesign</t>
+        </is>
+      </c>
+      <c r="C21" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D21" s="90" t="inlineStr">
+        <is>
+          <t>all page redesign via claude design</t>
+        </is>
+      </c>
+      <c r="E21" s="90" t="inlineStr">
+        <is>
+          <t>Apply the existing design system to /runs -- currently the weakest-looking screen (dense monospace debug trace). Fix the unstyled raw 404 on /runs/{id} deep links.</t>
+        </is>
+      </c>
+      <c r="F21" s="90" t="inlineStr">
+        <is>
+          <t>feat: redesign /runs history page + fix /runs/{id} deep-link 404</t>
+        </is>
+      </c>
+      <c r="G21" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H21" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I9" s="42" t="inlineStr">
+      <c r="I21" s="89" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J9" s="42" t="inlineStr">
+      <c r="J21" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K9" s="42" t="n"/>
-      <c r="L9" s="42" t="n"/>
-      <c r="M9" s="44" t="n">
+      <c r="K21" s="89" t="n"/>
+      <c r="L21" s="89" t="n"/>
+      <c r="M21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="43" t="n"/>
-      <c r="O9" s="43" t="inlineStr">
-        <is>
-          <t>connector registers correctly in provider_registry; enrich() returns a clean not-connected state, never raises</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="72">
-      <c r="A10" s="42" t="inlineStr">
-        <is>
-          <t>P6-A7</t>
-        </is>
-      </c>
-      <c r="B10" s="69" t="n"/>
-      <c r="C10" s="43" t="inlineStr">
-        <is>
-          <t>Integrations</t>
-        </is>
-      </c>
-      <c r="D10" s="43" t="inlineStr">
-        <is>
-          <t>Public review aggregation connectors (Google/Zomato reviews)</t>
-        </is>
-      </c>
-      <c r="E10" s="43" t="inlineStr">
-        <is>
-          <t>GoogleReviewsConnector / ZomatoReviewsConnector following the same BaseConnector pattern, pulling public review data (not internal complaints) into complaint_intelligence as an additional source type. Extends the Feedback model's source concept rather than inventing a parallel system.</t>
-        </is>
-      </c>
-      <c r="F10" s="43" t="inlineStr">
-        <is>
-          <t>feat: public review aggregation -- Google/Zomato reviews via BaseConnector pattern</t>
-        </is>
-      </c>
-      <c r="G10" s="43" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md, docs/CONNECTORS.md</t>
-        </is>
-      </c>
-      <c r="H10" s="41" t="inlineStr">
+      <c r="N21" s="90" t="n"/>
+      <c r="O21" s="90" t="inlineStr">
+        <is>
+          <t>direct navigation to /runs/{id} renders the run, not a 404</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52.05" customHeight="1" s="72">
+      <c r="A22" s="65" t="inlineStr">
+        <is>
+          <t>P6-A20</t>
+        </is>
+      </c>
+      <c r="B22" s="98" t="inlineStr">
+        <is>
+          <t>feature/voice-interface</t>
+        </is>
+      </c>
+      <c r="C22" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D22" s="90" t="inlineStr">
+        <is>
+          <t>Voice interface</t>
+        </is>
+      </c>
+      <c r="E22" s="90" t="inlineStr">
+        <is>
+          <t>Whisper transcription on browser-recorded question, existing RAG chatbot answers, TTS reads back.</t>
+        </is>
+      </c>
+      <c r="F22" s="90" t="inlineStr">
+        <is>
+          <t>feat: voice interface -- Whisper transcription + RAG answer + TTS readback</t>
+        </is>
+      </c>
+      <c r="G22" s="90" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md</t>
+        </is>
+      </c>
+      <c r="H22" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I10" s="42" t="inlineStr">
+      <c r="I22" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J22" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K22" s="89" t="n"/>
+      <c r="L22" s="89" t="n"/>
+      <c r="M22" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="90" t="n"/>
+      <c r="O22" s="90" t="inlineStr">
+        <is>
+          <t>transcription accuracy smoke test; end-to-end voice -&gt; RAG answer -&gt; TTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="7.95" customHeight="1" s="72">
+      <c r="A23" s="65" t="inlineStr">
+        <is>
+          <t>P6-A21</t>
+        </is>
+      </c>
+      <c r="B23" s="98" t="inlineStr">
+        <is>
+          <t>feature/live-page-redesign</t>
+        </is>
+      </c>
+      <c r="C23" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D23" s="90" t="inlineStr">
+        <is>
+          <t>/live page -- reframed as alerts/synthesis overlay</t>
+        </is>
+      </c>
+      <c r="E23" s="90" t="inlineStr">
+        <is>
+          <t>NOT a live order board (that's POS/aggregator territory and touches personal Swiggy consumer data). Instead: an alerts-and-synthesis overlay surfacing cross-referenced signals (e.g. 'order running late -- here's why, per our own data') during service hours.</t>
+        </is>
+      </c>
+      <c r="F23" s="90" t="inlineStr">
+        <is>
+          <t>feat: /live page -- alerts and synthesis overlay, not a live order feed</t>
+        </is>
+      </c>
+      <c r="G23" s="90" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md</t>
+        </is>
+      </c>
+      <c r="H23" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I23" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J23" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K23" s="89" t="n"/>
+      <c r="L23" s="89" t="n"/>
+      <c r="M23" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="90" t="n"/>
+      <c r="O23" s="90" t="inlineStr">
+        <is>
+          <t>manual verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="72">
+      <c r="A24" s="111" t="n"/>
+      <c r="B24" s="111" t="n"/>
+      <c r="C24" s="111" t="n"/>
+      <c r="D24" s="111" t="n"/>
+      <c r="E24" s="111" t="n"/>
+      <c r="F24" s="111" t="n"/>
+      <c r="G24" s="111" t="n"/>
+      <c r="H24" s="111" t="n"/>
+      <c r="I24" s="111" t="n"/>
+      <c r="J24" s="111" t="n"/>
+      <c r="K24" s="111" t="n"/>
+      <c r="L24" s="111" t="n"/>
+      <c r="M24" s="111" t="n"/>
+      <c r="N24" s="111" t="n"/>
+      <c r="O24" s="111" t="n"/>
+    </row>
+    <row r="25" ht="52.05" customHeight="1" s="72">
+      <c r="A25" s="109" t="inlineStr">
+        <is>
+          <t>DEFERRED TO END OF PHASE A -- pending direct restaurant-owner research into real procurement/approval workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52.8" customHeight="1" s="72">
+      <c r="A26" s="65" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="B26" s="98" t="inlineStr">
+        <is>
+          <t>feature/action-queue</t>
+        </is>
+      </c>
+      <c r="C26" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D26" s="90" t="inlineStr">
+        <is>
+          <t>ActionQueueService + action_queue table</t>
+        </is>
+      </c>
+      <c r="E26" s="90" t="inlineStr">
+        <is>
+          <t>New table (org_id, action_type [AUTO/APPROVE_REQUIRED/RECOMMENDATION], payload jsonb, status [PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED], approved_by, executed_at, error). ActionQueueService CRUD + status transitions. Plan output gains an action_queue section in the API response. Foundational -- every other agentic task below (workflow triggers, dynamic pricing, executors, trust-ladder) writes into this same table rather than inventing its own approval mechanism. DEFERRED to end of Phase A -- its main real-world value (approving reorder suggestions) is exactly the workflow that needs real restaurant-owner input first; building the approval UX before that research risks designing around the wrong assumptions.</t>
+        </is>
+      </c>
+      <c r="F26" s="90" t="inlineStr">
+        <is>
+          <t>feat: ActionQueueService + action_queue table -- 3-tier action model with approval lifecycle</t>
+        </is>
+      </c>
+      <c r="G26" s="90" t="inlineStr">
+        <is>
+          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md, docs/DECISIONS.md</t>
+        </is>
+      </c>
+      <c r="H26" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I26" s="89" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J26" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K26" s="89" t="n"/>
+      <c r="L26" s="89" t="n"/>
+      <c r="M26" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="90" t="n"/>
+      <c r="O26" s="90" t="inlineStr">
+        <is>
+          <t>CRUD + status-transition unit tests; plan output includes action_queue section</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="39.6" customHeight="1" s="72">
+      <c r="A27" s="65" t="inlineStr">
+        <is>
+          <t>P6-A23</t>
+        </is>
+      </c>
+      <c r="B27" s="69" t="n"/>
+      <c r="C27" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D27" s="90" t="inlineStr">
+        <is>
+          <t>Action Queue UI</t>
+        </is>
+      </c>
+      <c r="E27" s="90" t="inlineStr">
+        <is>
+          <t>Approve/reject list with type badges, Instamart cart-preview modal before approving checkout, procurement tracker (placed orders, status, ETA) in the inventory panel.</t>
+        </is>
+      </c>
+      <c r="F27" s="90" t="inlineStr">
+        <is>
+          <t>feat: Action Queue UI -- approve/reject with cart preview, procurement tracker</t>
+        </is>
+      </c>
+      <c r="G27" s="90" t="inlineStr">
+        <is>
+          <t>None (frontend only)</t>
+        </is>
+      </c>
+      <c r="H27" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I27" s="89" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J27" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K27" s="89" t="n"/>
+      <c r="L27" s="89" t="n"/>
+      <c r="M27" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O27" s="90" t="inlineStr">
+        <is>
+          <t>typecheck clean; manual verification against live action_queue data</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="39.6" customHeight="1" s="72">
+      <c r="A28" s="65" t="inlineStr">
+        <is>
+          <t>P6-A24</t>
+        </is>
+      </c>
+      <c r="B28" s="98" t="inlineStr">
+        <is>
+          <t>feature/agentic-automation</t>
+        </is>
+      </c>
+      <c r="C28" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D28" s="90" t="inlineStr">
+        <is>
+          <t>Workflow trigger engine (scoped: 2-3 built-in triggers, not a user-defined builder)</t>
+        </is>
+      </c>
+      <c r="E28" s="90" t="inlineStr">
+        <is>
+          <t>A small WorkflowEngine evaluating built-in conditions after each planning run and auto-creating action_queue rows. Ships with 2-3 real triggers to start: (1) 2+ critical shortages found -&gt; queue an urgent restock action, (2) tonight_busy + 2+ competitor Dineout deals live -&gt; queue a pricing/promo review action. Deliberately NOT the full owner-defined trigger/condition/action builder from the original workflow-system idea -- that's a much bigger UI/DB investment for marginal demo value beyond just having the triggers exist.</t>
+        </is>
+      </c>
+      <c r="F28" s="90" t="inlineStr">
+        <is>
+          <t>feat: workflow trigger engine -- built-in triggers auto-queue actions post-planning-run</t>
+        </is>
+      </c>
+      <c r="G28" s="90" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H28" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I28" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J28" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K28" s="89" t="n"/>
+      <c r="L28" s="89" t="n"/>
+      <c r="M28" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O28" s="90" t="inlineStr">
+        <is>
+          <t>each trigger condition fires correctly and produces the right queued action</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="39.6" customHeight="1" s="72">
+      <c r="A29" s="65" t="inlineStr">
+        <is>
+          <t>P6-A25</t>
+        </is>
+      </c>
+      <c r="B29" s="69" t="n"/>
+      <c r="C29" s="90" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D29" s="90" t="inlineStr">
+        <is>
+          <t>Trust-ladder mechanic on the Action Queue</t>
+        </is>
+      </c>
+      <c r="E29" s="90" t="inlineStr">
+        <is>
+          <t>Track consecutive unedited approvals per action_type. After N consecutive approvals (default 3) of the same type, offer 'always do this automatically' -- promotes future instances of that action_type straight to AUTO tier for that org. Makes 'autonomous' a visible, explainable mechanic rather than a claim.</t>
+        </is>
+      </c>
+      <c r="F29" s="90" t="inlineStr">
+        <is>
+          <t>feat: trust-ladder -- auto-promote repeatedly-approved action types to AUTO tier</t>
+        </is>
+      </c>
+      <c r="G29" s="90" t="inlineStr">
+        <is>
+          <t>docs/ACTION_QUEUE.md</t>
+        </is>
+      </c>
+      <c r="H29" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I29" s="89" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J10" s="42" t="inlineStr">
+      <c r="J29" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K10" s="42" t="n"/>
-      <c r="L10" s="42" t="n"/>
-      <c r="M10" s="44" t="n">
+      <c r="K29" s="89" t="n"/>
+      <c r="L29" s="89" t="n"/>
+      <c r="M29" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="43" t="inlineStr">
-        <is>
-          <t>P6-A6</t>
-        </is>
-      </c>
-      <c r="O10" s="43" t="inlineStr">
-        <is>
-          <t>reviews ingested with correct source tag; complaint_intelligence node correctly surfaces public-review-sourced themes alongside internal ones</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="52.05" customHeight="1" s="72">
-      <c r="A11" s="42" t="inlineStr">
-        <is>
-          <t>P6-A8</t>
-        </is>
-      </c>
-      <c r="B11" s="68" t="inlineStr">
-        <is>
-          <t>feature/financial-compliance</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="D11" s="43" t="inlineStr">
-        <is>
-          <t>Financial scorecard -- Expense ledger + real P&amp;L</t>
-        </is>
-      </c>
-      <c r="E11" s="43" t="inlineStr">
-        <is>
-          <t>New Expense model (category: rent/utilities/marketing/labor-later/other, amount, recurrence). Extends business.py's existing revenue/margin computation into a real daily/weekly P&amp;L and one composite health score. Designed so labor slots in later as just another Expense category, not a rewrite.</t>
-        </is>
-      </c>
-      <c r="F11" s="43" t="inlineStr">
-        <is>
-          <t>feat: financial scorecard -- Expense ledger, real P&amp;L, composite health score</t>
-        </is>
-      </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="N29" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O29" s="90" t="inlineStr">
+        <is>
+          <t>N consecutive approvals triggers promotion prompt; promoted type skips approval next time</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="39.6" customHeight="1" s="72">
+      <c r="A30" s="65" t="inlineStr">
+        <is>
+          <t>P6-A26</t>
+        </is>
+      </c>
+      <c r="B30" s="98" t="inlineStr">
+        <is>
+          <t>feature/dynamic-pricing</t>
+        </is>
+      </c>
+      <c r="C30" s="90" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D30" s="90" t="inlineStr">
+        <is>
+          <t>Dynamic pricing engine -- PriceChangeProposal (internal menu only)</t>
+        </is>
+      </c>
+      <c r="E30" s="90" t="inlineStr">
+        <is>
+          <t>New PriceChangeProposal model (item, current_price, suggested_price, reason, source, created_at). Computed from existing category_pricing/positioning data already in CompetitorEnricher. Surfaces as a new action_type in the Action Queue -- approving it updates your own MenuItem.price. Explicitly scoped to internal-only; does NOT attempt to sync price changes out to live Swiggy/Zomato listings (that needs Partner API access we don't have).</t>
+        </is>
+      </c>
+      <c r="F30" s="90" t="inlineStr">
+        <is>
+          <t>feat: dynamic pricing engine -- competitor-data-driven price suggestions via the Action Queue</t>
+        </is>
+      </c>
+      <c r="G30" s="90" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H30" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I30" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J30" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K30" s="89" t="n"/>
+      <c r="L30" s="89" t="n"/>
+      <c r="M30" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O30" s="90" t="inlineStr">
+        <is>
+          <t>suggestion computed correctly from category_pricing gap; approving updates MenuItem.price; PriceChangeProposal row persists as an audit trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="39.6" customHeight="1" s="72">
+      <c r="A31" s="65" t="inlineStr">
+        <is>
+          <t>P6-A27</t>
+        </is>
+      </c>
+      <c r="B31" s="69" t="n"/>
+      <c r="C31" s="90" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D31" s="90" t="inlineStr">
+        <is>
+          <t>Outcome / recommendation-learning memory</t>
+        </is>
+      </c>
+      <c r="E31" s="90" t="inlineStr">
+        <is>
+          <t>Extend the existing Qdrant-backed cross-session memory pattern (P6-S09) to track whether past actions/recommendations actually worked (e.g. did an approved price change move margin next week? did an approved restock prevent a stockout?). Feed this back into future confidence scoring on similar suggestions.</t>
+        </is>
+      </c>
+      <c r="F31" s="90" t="inlineStr">
+        <is>
+          <t>feat: outcome-learning memory -- track whether past AI actions worked, feed back into future confidence</t>
+        </is>
+      </c>
+      <c r="G31" s="90" t="inlineStr">
+        <is>
+          <t>docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H31" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I31" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J31" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K31" s="89" t="n"/>
+      <c r="L31" s="89" t="n"/>
+      <c r="M31" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22, P6-A26</t>
+        </is>
+      </c>
+      <c r="O31" s="90" t="inlineStr">
+        <is>
+          <t>outcome recorded correctly against the originating action; confidence score shifts on repeat suggestion of the same type after a bad outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="39.6" customHeight="1" s="72">
+      <c r="A32" s="65" t="inlineStr">
+        <is>
+          <t>P6-A28</t>
+        </is>
+      </c>
+      <c r="B32" s="98" t="inlineStr">
+        <is>
+          <t>feature/procurement-dineout-executors</t>
+        </is>
+      </c>
+      <c r="C32" s="90" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D32" s="90" t="inlineStr">
+        <is>
+          <t>ProcurementExecutor -- full flow, mocked final checkout call</t>
+        </is>
+      </c>
+      <c r="E32" s="90" t="inlineStr">
+        <is>
+          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A31.</t>
+        </is>
+      </c>
+      <c r="F32" s="90" t="inlineStr">
+        <is>
+          <t>feat: ProcurementExecutor -- full approval-gated Instamart flow, checkout call mocked pending staging creds</t>
+        </is>
+      </c>
+      <c r="G32" s="90" t="inlineStr">
+        <is>
+          <t>docs/ACTION_QUEUE.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H32" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I32" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J32" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K32" s="89" t="n"/>
+      <c r="L32" s="89" t="n"/>
+      <c r="M32" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O32" s="90" t="inlineStr">
+        <is>
+          <t>full flow test with mocked checkout; interrupt() pauses correctly; procurement_orders row created with a clear 'simulated' flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="39.6" customHeight="1" s="72">
+      <c r="A33" s="65" t="inlineStr">
+        <is>
+          <t>P6-A29</t>
+        </is>
+      </c>
+      <c r="B33" s="69" t="n"/>
+      <c r="C33" s="90" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D33" s="90" t="inlineStr">
+        <is>
+          <t>DineoutExecutor -- full flow, mocked final book_table call</t>
+        </is>
+      </c>
+      <c r="E33" s="90" t="inlineStr">
+        <is>
+          <t>Same pattern as P6-A24 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
+        </is>
+      </c>
+      <c r="F33" s="90" t="inlineStr">
+        <is>
+          <t>feat: DineoutExecutor -- full approval-gated Dineout booking flow, book_table call mocked pending staging creds</t>
+        </is>
+      </c>
+      <c r="G33" s="90" t="inlineStr">
+        <is>
+          <t>docs/ACTION_QUEUE.md</t>
+        </is>
+      </c>
+      <c r="H33" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I33" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J33" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K33" s="89" t="n"/>
+      <c r="L33" s="89" t="n"/>
+      <c r="M33" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22, P6-A28</t>
+        </is>
+      </c>
+      <c r="O33" s="90" t="inlineStr">
+        <is>
+          <t>full flow test with mocked book_table; reservations row created with a clear 'simulated' flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="52.8" customHeight="1" s="72">
+      <c r="A34" s="65" t="inlineStr">
+        <is>
+          <t>P6-A30</t>
+        </is>
+      </c>
+      <c r="B34" s="98" t="inlineStr">
+        <is>
+          <t>feature/recipe-vendor-foundations</t>
+        </is>
+      </c>
+      <c r="C34" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D34" s="90" t="inlineStr">
+        <is>
+          <t>Recipe + RecipeIngredient model</t>
+        </is>
+      </c>
+      <c r="E34" s="90" t="inlineStr">
+        <is>
+          <t>New Recipe (menu_item_id) + RecipeIngredient (recipe_id, ingredient, quantity, unit) tables. Bridges MenuItem and inventory -- unlocks live-computed cost_price (from real ingredient prices) instead of manual entry, and real per-dish inventory depletion instead of aggregate-only shortage tracking. DEFERRED to end of Phase A alongside the rest of the procurement/Action Queue cluster, pending direct restaurant-owner research into how real procurement actually works.</t>
+        </is>
+      </c>
+      <c r="F34" s="90" t="inlineStr">
+        <is>
+          <t>feat: Recipe + RecipeIngredient models -- dish-to-ingredient yield mapping</t>
+        </is>
+      </c>
+      <c r="G34" s="90" t="inlineStr">
+        <is>
+          <t>docs/DATA_MODEL.md</t>
+        </is>
+      </c>
+      <c r="H34" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I34" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J34" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K34" s="89" t="n"/>
+      <c r="L34" s="89" t="n"/>
+      <c r="M34" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="90" t="n"/>
+      <c r="O34" s="90" t="inlineStr">
+        <is>
+          <t>recipe costing test (sum of ingredient costs matches computed cost_price); depletion test (a sale reduces linked ingredient stock by the right amount)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="171.6" customHeight="1" s="72">
+      <c r="A35" s="65" t="inlineStr">
+        <is>
+          <t>P6-A31</t>
+        </is>
+      </c>
+      <c r="B35" s="69" t="n"/>
+      <c r="C35" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D35" s="90" t="inlineStr">
+        <is>
+          <t>Vendor/Supplier model</t>
+        </is>
+      </c>
+      <c r="E35" s="90" t="inlineStr">
+        <is>
+          <t>New Vendor model (name, category, is_online, contact) + VendorPriceQuote (vendor_id, ingredient, price, quoted_at). Instamart becomes one Vendor among several (an 'online' vendor with live API pricing); local mandi/wholesale vendors become trackable entities with manually-entered or periodically-surveyed prices. Scoped as tracking/comparison only, not a marketplace. DEFERRED to end of Phase A -- exact procurement medium (Instamart API vs a WhatsApp-dispatch message to a local vendor vs other) intentionally left open pending direct conversation with a real restaurant owner/manager about their actual ordering process, before committing to a design.</t>
+        </is>
+      </c>
+      <c r="F35" s="90" t="inlineStr">
+        <is>
+          <t>feat: Vendor/Supplier model -- Instamart becomes one vendor among many, not the only source</t>
+        </is>
+      </c>
+      <c r="G35" s="90" t="inlineStr">
+        <is>
+          <t>docs/DATA_MODEL.md</t>
+        </is>
+      </c>
+      <c r="H35" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I35" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J35" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K35" s="89" t="n"/>
+      <c r="L35" s="89" t="n"/>
+      <c r="M35" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="90" t="inlineStr">
+        <is>
+          <t>P6-A30</t>
+        </is>
+      </c>
+      <c r="O35" s="90" t="inlineStr">
+        <is>
+          <t>vendor price comparison query returns correct cheapest-vendor-per-ingredient</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="39.6" customHeight="1" s="72">
+      <c r="A36" s="65" t="inlineStr">
+        <is>
+          <t>P6-A32</t>
+        </is>
+      </c>
+      <c r="B36" s="98" t="inlineStr">
+        <is>
+          <t>feature/mcp-expansion</t>
+        </is>
+      </c>
+      <c r="C36" s="90" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D36" s="90" t="inlineStr">
+        <is>
+          <t>Internal MCP server -- get_market_brief / get_action_queue / approve_action</t>
+        </is>
+      </c>
+      <c r="E36" s="90" t="inlineStr">
+        <is>
+          <t>3 new tools on CortexKitchen's own MCP server (mcp_server.py), JWT-authenticated, calling MarketIntelService and ActionQueueService live. Lets an owner ask Claude Desktop directly about their restaurant and approve actions from there.</t>
+        </is>
+      </c>
+      <c r="F36" s="90" t="inlineStr">
+        <is>
+          <t>feat: 3 new MCP tools -- get_market_brief, get_action_queue, approve_action</t>
+        </is>
+      </c>
+      <c r="G36" s="90" t="inlineStr">
+        <is>
+          <t>docs/APIS.md, docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H36" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I36" s="89" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J36" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K36" s="89" t="n"/>
+      <c r="L36" s="89" t="n"/>
+      <c r="M36" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="90" t="inlineStr">
+        <is>
+          <t>P6-A22</t>
+        </is>
+      </c>
+      <c r="O36" s="90" t="inlineStr">
+        <is>
+          <t>all 3 tools smoke-tested in Claude Desktop; approve_action triggers the same approval path as the web UI; JWT enforced</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="39.6" customHeight="1" s="72">
+      <c r="A37" s="65" t="inlineStr">
+        <is>
+          <t>P6-A33</t>
+        </is>
+      </c>
+      <c r="B37" s="69" t="n"/>
+      <c r="C37" s="90" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D37" s="90" t="inlineStr">
+        <is>
+          <t>Internal MCP server -- expand further (menu insights, forecast, what-if)</t>
+        </is>
+      </c>
+      <c r="E37" s="90" t="inlineStr">
+        <is>
+          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A31 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
+        </is>
+      </c>
+      <c r="F37" s="90" t="inlineStr">
+        <is>
+          <t>feat: expand internal MCP server -- menu insights, forecast, what-if simulator as tools</t>
+        </is>
+      </c>
+      <c r="G37" s="90" t="inlineStr">
         <is>
           <t>docs/APIS.md</t>
         </is>
       </c>
-      <c r="H11" s="41" t="inlineStr">
+      <c r="H37" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I11" s="42" t="inlineStr">
+      <c r="I37" s="89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J37" s="89" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K37" s="89" t="n"/>
+      <c r="L37" s="89" t="n"/>
+      <c r="M37" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="90" t="inlineStr">
+        <is>
+          <t>P6-A32</t>
+        </is>
+      </c>
+      <c r="O37" s="90" t="inlineStr">
+        <is>
+          <t>each new tool smoke-tested in Claude Desktop; correct data returned matching the equivalent API endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="52.8" customHeight="1" s="72">
+      <c r="A38" s="65" t="inlineStr">
+        <is>
+          <t>P6-A34</t>
+        </is>
+      </c>
+      <c r="B38" s="98" t="inlineStr">
+        <is>
+          <t>feature/brief-page</t>
+        </is>
+      </c>
+      <c r="C38" s="90" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D38" s="90" t="inlineStr">
+        <is>
+          <t>/brief page</t>
+        </is>
+      </c>
+      <c r="E38" s="90" t="inlineStr">
+        <is>
+          <t>Daily morning briefing -- overnight performance, today's forecast vs yesterday, top 3 action priorities, market snapshot. Single-screen showcase of the whole system's intelligence.</t>
+        </is>
+      </c>
+      <c r="F38" s="90" t="inlineStr">
+        <is>
+          <t>feat: /brief page -- daily morning operational briefing</t>
+        </is>
+      </c>
+      <c r="G38" s="90" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H38" s="108" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I38" s="89" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J11" s="42" t="inlineStr">
+      <c r="J38" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K11" s="42" t="n"/>
-      <c r="L11" s="42" t="n"/>
-      <c r="M11" s="44" t="n">
+      <c r="K38" s="89" t="n"/>
+      <c r="L38" s="89" t="n"/>
+      <c r="M38" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="43" t="n"/>
-      <c r="O11" s="43" t="inlineStr">
-        <is>
-          <t>P&amp;L numbers match seeded expense + revenue data; health score computes deterministically from known inputs</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="52.05" customHeight="1" s="72">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>P6-A9</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n"/>
-      <c r="C12" s="43" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="D12" s="43" t="inlineStr">
-        <is>
-          <t>Compliance / Obligations calendar</t>
-        </is>
-      </c>
-      <c r="E12" s="43" t="inlineStr">
-        <is>
-          <t>Generalized Obligation model (type: license-renewal/GST-filing/inspection/other, due_date, status) with reminders delivered through the existing Phase-5 email digest mechanism rather than a new one-off sender. Not a GST computation/invoicing layer -- just a dated-obligation tracker with reminders.</t>
-        </is>
-      </c>
-      <c r="F12" s="43" t="inlineStr">
-        <is>
-          <t>feat: compliance/obligations calendar -- reminder engine reusing the existing email digest</t>
-        </is>
-      </c>
-      <c r="G12" s="43" t="inlineStr">
-        <is>
-          <t>docs/APIS.md</t>
-        </is>
-      </c>
-      <c r="H12" s="41" t="inlineStr">
+      <c r="N38" s="90" t="inlineStr">
+        <is>
+          <t>P6-A23</t>
+        </is>
+      </c>
+      <c r="O38" s="90" t="inlineStr">
+        <is>
+          <t>manual verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="171.6" customHeight="1" s="72">
+      <c r="A39" s="65" t="inlineStr">
+        <is>
+          <t>P6-A35</t>
+        </is>
+      </c>
+      <c r="B39" s="98" t="n"/>
+      <c r="C39" s="90" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D39" s="90" t="inlineStr">
+        <is>
+          <t>Post-Phase-A documentation, test, CI, observability, and eval refresh</t>
+        </is>
+      </c>
+      <c r="E39" s="90" t="inlineStr">
+        <is>
+          <t>Once Phase A ships, a lot of new surface area will have landed at once -- Action Queue, workflow triggers, the anomaly agent, both executors, new connectors (Zomato stub, reviews), new data models (Recipe, Vendor, Expense, Obligation), MCP expansion. Do a full pass rather than letting docs drift: update every docs/*.md file, CLAUDE.md, README, and any screenshots referenced in docs to reflect what actually shipped. Audit test coverage for every new service/model added in Phase A -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (anomaly diagnoses, dynamic pricing suggestions), since the existing eval sets predate all of this and won't catch regressions in it.</t>
+        </is>
+      </c>
+      <c r="F39" s="90" t="inlineStr">
+        <is>
+          <t>docs: full documentation, test-coverage, CI, and eval refresh after the Phase A agentic core ships</t>
+        </is>
+      </c>
+      <c r="G39" s="90" t="inlineStr">
+        <is>
+          <t>All docs/*.md, CLAUDE.md, README.md</t>
+        </is>
+      </c>
+      <c r="H39" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I12" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J12" s="42" t="inlineStr">
+      <c r="I39" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J39" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K12" s="42" t="n"/>
-      <c r="L12" s="42" t="n"/>
-      <c r="M12" s="44" t="n">
+      <c r="K39" s="89" t="n"/>
+      <c r="L39" s="89" t="n"/>
+      <c r="M39" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="43" t="n"/>
-      <c r="O12" s="43" t="inlineStr">
-        <is>
-          <t>reminder fires at the correct lead-time before due_date; reuses existing digest delivery path</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="72">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>P6-A10</t>
-        </is>
-      </c>
-      <c r="B13" s="68" t="inlineStr">
-        <is>
-          <t>feature/location-architecture</t>
-        </is>
-      </c>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D13" s="43" t="inlineStr">
-        <is>
-          <t>Location-aware enrichers (hedge for multi-location)</t>
-        </is>
-      </c>
-      <c r="E13" s="43" t="inlineStr">
-        <is>
-          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A31) exists or once real customers have multiple outlets.</t>
-        </is>
-      </c>
-      <c r="F13" s="43" t="inlineStr">
-        <is>
-          <t>feat: location-aware enrichers -- pass address/location context through instead of one hardcoded address</t>
-        </is>
-      </c>
-      <c r="G13" s="43" t="inlineStr">
-        <is>
-          <t>CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="H13" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I13" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J13" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K13" s="42" t="n"/>
-      <c r="L13" s="42" t="n"/>
-      <c r="M13" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="43" t="n"/>
-      <c r="O13" s="43" t="inlineStr">
-        <is>
-          <t>enrichers accept and correctly use a passed-in address_id, defaulting to the existing single-address behavior when none given</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="52.05" customHeight="1" s="72">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>P6-A11</t>
-        </is>
-      </c>
-      <c r="B14" s="69" t="n"/>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D14" s="43" t="inlineStr">
-        <is>
-          <t>Multi-location / Restaurant entity -- STRATEGIC, needs explicit go/no-go</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="inlineStr">
-        <is>
-          <t>Introduce Restaurant as a first-class entity between Organization and everything else (menu, inventory, planning runs, Swiggy connector -- each physical location has its own Swiggy restaurant ID). Add restaurant_id to MenuItem/InventoryItem/PlanningRun/connectors. Cheaper to do now while the schema is small than to retrofit later. NOT started until the user confirms real near-term demand justifies it over other Phase A work.</t>
-        </is>
-      </c>
-      <c r="F14" s="43" t="inlineStr">
-        <is>
-          <t>feat: Restaurant entity -- first-class multi-location support</t>
-        </is>
-      </c>
-      <c r="G14" s="43" t="inlineStr">
-        <is>
-          <t>docs/DATA_MODEL.md, docs/DECISIONS.md</t>
-        </is>
-      </c>
-      <c r="H14" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I14" s="42" t="inlineStr">
-        <is>
-          <t>Low (pending go/no-go)</t>
-        </is>
-      </c>
-      <c r="J14" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K14" s="42" t="n"/>
-      <c r="L14" s="42" t="n"/>
-      <c r="M14" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="43" t="inlineStr">
-        <is>
-          <t>P6-A10</t>
-        </is>
-      </c>
-      <c r="O14" s="43" t="inlineStr">
-        <is>
-          <t>existing single-location orgs continue to work unchanged (default restaurant backfilled); cross-location query test once 2+ restaurants exist</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="52.05" customHeight="1" s="72">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>P6-A12</t>
-        </is>
-      </c>
-      <c r="B15" s="68" t="inlineStr">
-        <is>
-          <t>feature/chatbot-dineout-tools</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D15" s="43" t="inlineStr">
-        <is>
-          <t>Chatbot -- Dineout competitive query tools</t>
-        </is>
-      </c>
-      <c r="E15" s="43" t="inlineStr">
-        <is>
-          <t>3 Groq function-calling tools for the existing chatbot: get_competitor_deals, get_area_occupancy, get_trending_dishes -- all using Swiggy's existing read-only Dineout MCP (search_restaurants_dineout, get_restaurant_details, get_available_slots), already-proven tools. (Formerly P6-MI04; renumbered as part of the Phase 6 replan.)</t>
-        </is>
-      </c>
-      <c r="F15" s="43" t="inlineStr">
-        <is>
-          <t>feat: chatbot Dineout tools -- competitor deals, area occupancy, trending dishes</t>
-        </is>
-      </c>
-      <c r="G15" s="43" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md</t>
-        </is>
-      </c>
-      <c r="H15" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I15" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J15" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K15" s="42" t="n"/>
-      <c r="L15" s="42" t="n"/>
-      <c r="M15" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="43" t="n"/>
-      <c r="O15" s="43" t="inlineStr">
-        <is>
-          <t>all 3 tools callable from /chat; correct Swiggy data returned; graceful None on failure</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="52.05" customHeight="1" s="72">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>P6-A13</t>
-        </is>
-      </c>
-      <c r="B16" s="69" t="n"/>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D16" s="43" t="inlineStr">
-        <is>
-          <t>Structured outputs -- tool_choice=required across chatbot tools</t>
-        </is>
-      </c>
-      <c r="E16" s="43" t="inlineStr">
-        <is>
-          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema across all chatbot tools (Swiggy and internal). Chatbot function calls never hallucinate JSON.</t>
-        </is>
-      </c>
-      <c r="F16" s="43" t="inlineStr">
-        <is>
-          <t>feat: structured outputs -- tool_choice=required across all chatbot tools</t>
-        </is>
-      </c>
-      <c r="G16" s="43" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md</t>
-        </is>
-      </c>
-      <c r="H16" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I16" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J16" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K16" s="42" t="n"/>
-      <c r="L16" s="42" t="n"/>
-      <c r="M16" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="43" t="inlineStr">
-        <is>
-          <t>P6-A12</t>
-        </is>
-      </c>
-      <c r="O16" s="43" t="inlineStr">
-        <is>
-          <t>schema validation test; chatbot returns valid JSON on repeated calls</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="52.05" customHeight="1" s="72">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>P6-A14</t>
-        </is>
-      </c>
-      <c r="B17" s="68" t="inlineStr">
-        <is>
-          <t>feature/llm-cost-quality</t>
-        </is>
-      </c>
-      <c r="C17" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D17" s="43" t="inlineStr">
-        <is>
-          <t>Prompt caching -- critic + aggregator</t>
-        </is>
-      </c>
-      <c r="E17" s="43" t="inlineStr">
-        <is>
-          <t>Add prompt-caching headers to critic and aggregator LLM calls (both have long, repeated system prompts). Cuts LLM cost per planning run; invisible to a demo but real cost hygiene.</t>
-        </is>
-      </c>
-      <c r="F17" s="43" t="inlineStr">
-        <is>
-          <t>feat: prompt caching -- cut LLM costs on critic and aggregator nodes</t>
-        </is>
-      </c>
-      <c r="G17" s="43" t="inlineStr">
-        <is>
-          <t>docs/ARCHITECTURE.md</t>
-        </is>
-      </c>
-      <c r="H17" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I17" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J17" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K17" s="42" t="n"/>
-      <c r="L17" s="42" t="n"/>
-      <c r="M17" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="43" t="n"/>
-      <c r="O17" s="43" t="inlineStr">
-        <is>
-          <t>cost log shows cache_hit=true on second run of the same scenario</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="72">
-      <c r="A18" s="42" t="inlineStr">
-        <is>
-          <t>P6-A15</t>
-        </is>
-      </c>
-      <c r="B18" s="69" t="n"/>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>Agents</t>
-        </is>
-      </c>
-      <c r="D18" s="43" t="inlineStr">
-        <is>
-          <t>Multi-agent debate critic</t>
-        </is>
-      </c>
-      <c r="E18" s="43" t="inlineStr">
-        <is>
-          <t>Two LLM critic instances (optimistic vs conservative), structured debate, moderator resolves disagreement. Marginal demo-visible upside over the existing single critic given the added cost/latency -- kept low priority.</t>
-        </is>
-      </c>
-      <c r="F18" s="43" t="inlineStr">
-        <is>
-          <t>feat: multi-agent debate critic -- consensus scoring</t>
-        </is>
-      </c>
-      <c r="G18" s="43" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md</t>
-        </is>
-      </c>
-      <c r="H18" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I18" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J18" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K18" s="42" t="n"/>
-      <c r="L18" s="42" t="n"/>
-      <c r="M18" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="43" t="n"/>
-      <c r="O18" s="43" t="inlineStr">
-        <is>
-          <t>debate resolves on test plans; disagreement cases escalate correctly</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="52.05" customHeight="1" s="72">
-      <c r="A19" s="42" t="inlineStr">
-        <is>
-          <t>P6-A16</t>
-        </is>
-      </c>
-      <c r="B19" s="68" t="inlineStr">
-        <is>
-          <t>feature/ci-eval-hygiene</t>
-        </is>
-      </c>
-      <c r="C19" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t>Fix SQLite/JSONB CI test-infra gap</t>
-        </is>
-      </c>
-      <c r="E19" s="43" t="inlineStr">
-        <is>
-          <t>test_swiggy_reservation_sync.py and test_connector_repository.py are excluded from CI because SQLite can't render Postgres JSONB columns. Either a SQLite-compatible fallback type or a Postgres CI service container.</t>
-        </is>
-      </c>
-      <c r="F19" s="43" t="inlineStr">
-        <is>
-          <t>fix: SQLite-compatible JSONB handling (or Postgres CI service) for excluded test files</t>
-        </is>
-      </c>
-      <c r="G19" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H19" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I19" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J19" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K19" s="42" t="n"/>
-      <c r="L19" s="42" t="n"/>
-      <c r="M19" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="43" t="n"/>
-      <c r="O19" s="43" t="inlineStr">
-        <is>
-          <t>previously-excluded test files run in CI</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="7.95" customHeight="1" s="72">
-      <c r="A20" s="42" t="inlineStr">
-        <is>
-          <t>P6-A17</t>
-        </is>
-      </c>
-      <c r="B20" s="70" t="n"/>
-      <c r="C20" s="43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D20" s="43" t="inlineStr">
-        <is>
-          <t>Promote reviewed RAGAS/DeepEval candidates</t>
-        </is>
-      </c>
-      <c r="E20" s="43" t="inlineStr">
-        <is>
-          <t>Recurring habit of running the existing candidate-generation scripts and hand-promoting reviewed candidates into the curated eval datasets.</t>
-        </is>
-      </c>
-      <c r="F20" s="43" t="inlineStr">
-        <is>
-          <t>chore: promote reviewed eval candidates into curated datasets</t>
-        </is>
-      </c>
-      <c r="G20" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H20" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I20" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J20" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K20" s="42" t="n"/>
-      <c r="L20" s="42" t="n"/>
-      <c r="M20" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="43" t="n"/>
-      <c r="O20" s="43" t="inlineStr">
-        <is>
-          <t>N/A -- ongoing process, not a one-time build</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="52.05" customHeight="1" s="72">
-      <c r="A21" s="42" t="inlineStr">
-        <is>
-          <t>P6-A18</t>
-        </is>
-      </c>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D21" s="43" t="inlineStr">
-        <is>
-          <t>Regenerate golden_runs.json against real data</t>
-        </is>
-      </c>
-      <c r="E21" s="43" t="inlineStr">
-        <is>
-          <t>The key-path bug in build_golden_dataset.py is already fixed; the checked-in fixture still reflects the old broken extraction. Regenerate once real run history exists.</t>
-        </is>
-      </c>
-      <c r="F21" s="43" t="inlineStr">
-        <is>
-          <t>chore: regenerate golden_runs.json with corrected extraction logic</t>
-        </is>
-      </c>
-      <c r="G21" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H21" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I21" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J21" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K21" s="42" t="n"/>
-      <c r="L21" s="42" t="n"/>
-      <c r="M21" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="43" t="n"/>
-      <c r="O21" s="43" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="52.05" customHeight="1" s="72">
-      <c r="A22" s="42" t="inlineStr">
-        <is>
-          <t>P6-A19</t>
-        </is>
-      </c>
-      <c r="B22" s="68" t="inlineStr">
-        <is>
-          <t>feature/menu-engineering-matrix</t>
-        </is>
-      </c>
-      <c r="C22" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D22" s="43" t="inlineStr">
-        <is>
-          <t>Menu engineering matrix UI</t>
-        </is>
-      </c>
-      <c r="E22" s="43" t="inlineStr">
-        <is>
-          <t>Stars/plow-horses/dogs/puzzles quadrant chart using margin_pct x quantity, both already computed in business.py -- just needs quadrant classification + a chart.</t>
-        </is>
-      </c>
-      <c r="F22" s="43" t="inlineStr">
-        <is>
-          <t>feat: menu engineering matrix -- margin x popularity quadrant chart</t>
-        </is>
-      </c>
-      <c r="G22" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H22" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I22" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J22" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K22" s="42" t="n"/>
-      <c r="L22" s="42" t="n"/>
-      <c r="M22" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="43" t="n"/>
-      <c r="O22" s="43" t="inlineStr">
-        <is>
-          <t>quadrant classification unit test; chart renders correctly</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="7.95" customHeight="1" s="72">
-      <c r="A23" s="42" t="inlineStr">
-        <is>
-          <t>P6-A20</t>
-        </is>
-      </c>
-      <c r="B23" s="68" t="inlineStr">
-        <is>
-          <t>feature/pages-redesign</t>
-        </is>
-      </c>
-      <c r="C23" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D23" s="43" t="inlineStr">
-        <is>
-          <t>all page redesign via claude design</t>
-        </is>
-      </c>
-      <c r="E23" s="43" t="inlineStr">
-        <is>
-          <t>Apply the existing design system to /runs -- currently the weakest-looking screen (dense monospace debug trace). Fix the unstyled raw 404 on /runs/{id} deep links.</t>
-        </is>
-      </c>
-      <c r="F23" s="43" t="inlineStr">
-        <is>
-          <t>feat: redesign /runs history page + fix /runs/{id} deep-link 404</t>
-        </is>
-      </c>
-      <c r="G23" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H23" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I23" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J23" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K23" s="42" t="n"/>
-      <c r="L23" s="42" t="n"/>
-      <c r="M23" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="43" t="n"/>
-      <c r="O23" s="43" t="inlineStr">
-        <is>
-          <t>direct navigation to /runs/{id} renders the run, not a 404</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1" s="72">
-      <c r="A24" s="42" t="inlineStr">
-        <is>
-          <t>P6-A21</t>
-        </is>
-      </c>
-      <c r="B24" s="68" t="inlineStr">
-        <is>
-          <t>feature/voice-interface</t>
-        </is>
-      </c>
-      <c r="C24" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D24" s="43" t="inlineStr">
-        <is>
-          <t>Voice interface</t>
-        </is>
-      </c>
-      <c r="E24" s="43" t="inlineStr">
-        <is>
-          <t>Whisper transcription on browser-recorded question, existing RAG chatbot answers, TTS reads back.</t>
-        </is>
-      </c>
-      <c r="F24" s="43" t="inlineStr">
-        <is>
-          <t>feat: voice interface -- Whisper transcription + RAG answer + TTS readback</t>
-        </is>
-      </c>
-      <c r="G24" s="43" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md</t>
-        </is>
-      </c>
-      <c r="H24" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I24" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J24" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K24" s="42" t="n"/>
-      <c r="L24" s="42" t="n"/>
-      <c r="M24" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="43" t="n"/>
-      <c r="O24" s="43" t="inlineStr">
-        <is>
-          <t>transcription accuracy smoke test; end-to-end voice -&gt; RAG answer -&gt; TTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="52.05" customHeight="1" s="72">
-      <c r="A25" s="42" t="inlineStr">
-        <is>
-          <t>P6-A22</t>
-        </is>
-      </c>
-      <c r="B25" s="68" t="inlineStr">
-        <is>
-          <t>feature/live-page-redesign</t>
-        </is>
-      </c>
-      <c r="C25" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D25" s="43" t="inlineStr">
-        <is>
-          <t>/live page -- reframed as alerts/synthesis overlay</t>
-        </is>
-      </c>
-      <c r="E25" s="43" t="inlineStr">
-        <is>
-          <t>NOT a live order board (that's POS/aggregator territory and touches personal Swiggy consumer data). Instead: an alerts-and-synthesis overlay surfacing cross-referenced signals (e.g. 'order running late -- here's why, per our own data') during service hours.</t>
-        </is>
-      </c>
-      <c r="F25" s="43" t="inlineStr">
-        <is>
-          <t>feat: /live page -- alerts and synthesis overlay, not a live order feed</t>
-        </is>
-      </c>
-      <c r="G25" s="43" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md</t>
-        </is>
-      </c>
-      <c r="H25" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I25" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J25" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K25" s="42" t="n"/>
-      <c r="L25" s="42" t="n"/>
-      <c r="M25" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="43" t="inlineStr">
-        <is>
-          <t>P6-A5</t>
-        </is>
-      </c>
-      <c r="O25" s="43" t="inlineStr">
-        <is>
-          <t>manual verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="52.8" customHeight="1" s="72">
-      <c r="A26" s="67" t="n"/>
-      <c r="B26" s="67" t="n"/>
-      <c r="C26" s="67" t="n"/>
-      <c r="D26" s="67" t="n"/>
-      <c r="E26" s="67" t="n"/>
-      <c r="F26" s="67" t="n"/>
-      <c r="G26" s="67" t="n"/>
-      <c r="H26" s="67" t="n"/>
-      <c r="I26" s="67" t="n"/>
-      <c r="J26" s="67" t="n"/>
-      <c r="K26" s="67" t="n"/>
-      <c r="L26" s="67" t="n"/>
-      <c r="M26" s="67" t="n"/>
-      <c r="N26" s="67" t="n"/>
-      <c r="O26" s="67" t="n"/>
-    </row>
-    <row r="27" ht="39.6" customHeight="1" s="72">
-      <c r="A27" s="109" t="inlineStr">
-        <is>
-          <t>DEFERRED TO END OF PHASE A -- pending direct restaurant-owner research into real procurement/approval workflow</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="39.6" customHeight="1" s="72">
-      <c r="A28" s="42" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="B28" s="68" t="inlineStr">
-        <is>
-          <t>feature/action-queue</t>
-        </is>
-      </c>
-      <c r="C28" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D28" s="43" t="inlineStr">
-        <is>
-          <t>ActionQueueService + action_queue table</t>
-        </is>
-      </c>
-      <c r="E28" s="43" t="inlineStr">
-        <is>
-          <t>New table (org_id, action_type [AUTO/APPROVE_REQUIRED/RECOMMENDATION], payload jsonb, status [PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED], approved_by, executed_at, error). ActionQueueService CRUD + status transitions. Plan output gains an action_queue section in the API response. Foundational -- every other agentic task below (workflow triggers, dynamic pricing, executors, trust-ladder) writes into this same table rather than inventing its own approval mechanism. DEFERRED to end of Phase A -- its main real-world value (approving reorder suggestions) is exactly the workflow that needs real restaurant-owner input first; building the approval UX before that research risks designing around the wrong assumptions.</t>
-        </is>
-      </c>
-      <c r="F28" s="43" t="inlineStr">
-        <is>
-          <t>feat: ActionQueueService + action_queue table -- 3-tier action model with approval lifecycle</t>
-        </is>
-      </c>
-      <c r="G28" s="43" t="inlineStr">
-        <is>
-          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md, docs/DECISIONS.md</t>
-        </is>
-      </c>
-      <c r="H28" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I28" s="42" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="J28" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K28" s="42" t="n"/>
-      <c r="L28" s="42" t="n"/>
-      <c r="M28" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="43" t="n"/>
-      <c r="O28" s="43" t="inlineStr">
-        <is>
-          <t>CRUD + status-transition unit tests; plan output includes action_queue section</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="39.6" customHeight="1" s="72">
-      <c r="A29" s="42" t="inlineStr">
-        <is>
-          <t>P6-A24</t>
-        </is>
-      </c>
-      <c r="B29" s="69" t="n"/>
-      <c r="C29" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D29" s="43" t="inlineStr">
-        <is>
-          <t>Action Queue UI</t>
-        </is>
-      </c>
-      <c r="E29" s="43" t="inlineStr">
-        <is>
-          <t>Approve/reject list with type badges, Instamart cart-preview modal before approving checkout, procurement tracker (placed orders, status, ETA) in the inventory panel.</t>
-        </is>
-      </c>
-      <c r="F29" s="43" t="inlineStr">
-        <is>
-          <t>feat: Action Queue UI -- approve/reject with cart preview, procurement tracker</t>
-        </is>
-      </c>
-      <c r="G29" s="43" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H29" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I29" s="42" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="J29" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K29" s="42" t="n"/>
-      <c r="L29" s="42" t="n"/>
-      <c r="M29" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O29" s="43" t="inlineStr">
-        <is>
-          <t>typecheck clean; manual verification against live action_queue data</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="39.6" customHeight="1" s="72">
-      <c r="A30" s="42" t="inlineStr">
-        <is>
-          <t>P6-A25</t>
-        </is>
-      </c>
-      <c r="B30" s="68" t="inlineStr">
-        <is>
-          <t>feature/agentic-automation</t>
-        </is>
-      </c>
-      <c r="C30" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D30" s="43" t="inlineStr">
-        <is>
-          <t>Workflow trigger engine (scoped: 2-3 built-in triggers, not a user-defined builder)</t>
-        </is>
-      </c>
-      <c r="E30" s="43" t="inlineStr">
-        <is>
-          <t>A small WorkflowEngine evaluating built-in conditions after each planning run and auto-creating action_queue rows. Ships with 2-3 real triggers to start: (1) 2+ critical shortages found -&gt; queue an urgent restock action, (2) tonight_busy + 2+ competitor Dineout deals live -&gt; queue a pricing/promo review action. Deliberately NOT the full owner-defined trigger/condition/action builder from the original workflow-system idea -- that's a much bigger UI/DB investment for marginal demo value beyond just having the triggers exist.</t>
-        </is>
-      </c>
-      <c r="F30" s="43" t="inlineStr">
-        <is>
-          <t>feat: workflow trigger engine -- built-in triggers auto-queue actions post-planning-run</t>
-        </is>
-      </c>
-      <c r="G30" s="43" t="inlineStr">
-        <is>
-          <t>docs/ARCHITECTURE.md</t>
-        </is>
-      </c>
-      <c r="H30" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I30" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J30" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K30" s="42" t="n"/>
-      <c r="L30" s="42" t="n"/>
-      <c r="M30" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O30" s="43" t="inlineStr">
-        <is>
-          <t>each trigger condition fires correctly and produces the right queued action</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="39.6" customHeight="1" s="72">
-      <c r="A31" s="42" t="inlineStr">
-        <is>
-          <t>P6-A26</t>
-        </is>
-      </c>
-      <c r="B31" s="69" t="n"/>
-      <c r="C31" s="43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D31" s="43" t="inlineStr">
-        <is>
-          <t>Trust-ladder mechanic on the Action Queue</t>
-        </is>
-      </c>
-      <c r="E31" s="43" t="inlineStr">
-        <is>
-          <t>Track consecutive unedited approvals per action_type. After N consecutive approvals (default 3) of the same type, offer 'always do this automatically' -- promotes future instances of that action_type straight to AUTO tier for that org. Makes 'autonomous' a visible, explainable mechanic rather than a claim.</t>
-        </is>
-      </c>
-      <c r="F31" s="43" t="inlineStr">
-        <is>
-          <t>feat: trust-ladder -- auto-promote repeatedly-approved action types to AUTO tier</t>
-        </is>
-      </c>
-      <c r="G31" s="43" t="inlineStr">
-        <is>
-          <t>docs/ACTION_QUEUE.md</t>
-        </is>
-      </c>
-      <c r="H31" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I31" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J31" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K31" s="42" t="n"/>
-      <c r="L31" s="42" t="n"/>
-      <c r="M31" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O31" s="43" t="inlineStr">
-        <is>
-          <t>N consecutive approvals triggers promotion prompt; promoted type skips approval next time</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="39.6" customHeight="1" s="72">
-      <c r="A32" s="42" t="inlineStr">
-        <is>
-          <t>P6-A27</t>
-        </is>
-      </c>
-      <c r="B32" s="68" t="inlineStr">
-        <is>
-          <t>feature/dynamic-pricing</t>
-        </is>
-      </c>
-      <c r="C32" s="43" t="inlineStr">
-        <is>
-          <t>Agents</t>
-        </is>
-      </c>
-      <c r="D32" s="43" t="inlineStr">
-        <is>
-          <t>Dynamic pricing engine -- PriceChangeProposal (internal menu only)</t>
-        </is>
-      </c>
-      <c r="E32" s="43" t="inlineStr">
-        <is>
-          <t>New PriceChangeProposal model (item, current_price, suggested_price, reason, source, created_at). Computed from existing category_pricing/positioning data already in CompetitorEnricher. Surfaces as a new action_type in the Action Queue -- approving it updates your own MenuItem.price. Explicitly scoped to internal-only; does NOT attempt to sync price changes out to live Swiggy/Zomato listings (that needs Partner API access we don't have).</t>
-        </is>
-      </c>
-      <c r="F32" s="43" t="inlineStr">
-        <is>
-          <t>feat: dynamic pricing engine -- competitor-data-driven price suggestions via the Action Queue</t>
-        </is>
-      </c>
-      <c r="G32" s="43" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md, CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="H32" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I32" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J32" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K32" s="42" t="n"/>
-      <c r="L32" s="42" t="n"/>
-      <c r="M32" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O32" s="43" t="inlineStr">
-        <is>
-          <t>suggestion computed correctly from category_pricing gap; approving updates MenuItem.price; PriceChangeProposal row persists as an audit trail</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="39.6" customHeight="1" s="72">
-      <c r="A33" s="42" t="inlineStr">
-        <is>
-          <t>P6-A28</t>
-        </is>
-      </c>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="43" t="inlineStr">
-        <is>
-          <t>Agents</t>
-        </is>
-      </c>
-      <c r="D33" s="43" t="inlineStr">
-        <is>
-          <t>Outcome / recommendation-learning memory</t>
-        </is>
-      </c>
-      <c r="E33" s="43" t="inlineStr">
-        <is>
-          <t>Extend the existing Qdrant-backed cross-session memory pattern (P6-S09) to track whether past actions/recommendations actually worked (e.g. did an approved price change move margin next week? did an approved restock prevent a stockout?). Feed this back into future confidence scoring on similar suggestions.</t>
-        </is>
-      </c>
-      <c r="F33" s="43" t="inlineStr">
-        <is>
-          <t>feat: outcome-learning memory -- track whether past AI actions worked, feed back into future confidence</t>
-        </is>
-      </c>
-      <c r="G33" s="43" t="inlineStr">
-        <is>
-          <t>docs/ARCHITECTURE.md</t>
-        </is>
-      </c>
-      <c r="H33" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I33" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J33" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K33" s="42" t="n"/>
-      <c r="L33" s="42" t="n"/>
-      <c r="M33" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23, P6-A27</t>
-        </is>
-      </c>
-      <c r="O33" s="43" t="inlineStr">
-        <is>
-          <t>outcome recorded correctly against the originating action; confidence score shifts on repeat suggestion of the same type after a bad outcome</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="52.8" customHeight="1" s="72">
-      <c r="A34" s="42" t="inlineStr">
-        <is>
-          <t>P6-A29</t>
-        </is>
-      </c>
-      <c r="B34" s="68" t="inlineStr">
-        <is>
-          <t>feature/procurement-dineout-executors</t>
-        </is>
-      </c>
-      <c r="C34" s="43" t="inlineStr">
-        <is>
-          <t>Agents</t>
-        </is>
-      </c>
-      <c r="D34" s="43" t="inlineStr">
-        <is>
-          <t>ProcurementExecutor -- full flow, mocked final checkout call</t>
-        </is>
-      </c>
-      <c r="E34" s="43" t="inlineStr">
-        <is>
-          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A32.</t>
-        </is>
-      </c>
-      <c r="F34" s="43" t="inlineStr">
-        <is>
-          <t>feat: ProcurementExecutor -- full approval-gated Instamart flow, checkout call mocked pending staging creds</t>
-        </is>
-      </c>
-      <c r="G34" s="43" t="inlineStr">
-        <is>
-          <t>docs/ACTION_QUEUE.md, CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="H34" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I34" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J34" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K34" s="42" t="n"/>
-      <c r="L34" s="42" t="n"/>
-      <c r="M34" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O34" s="43" t="inlineStr">
-        <is>
-          <t>full flow test with mocked checkout; interrupt() pauses correctly; procurement_orders row created with a clear 'simulated' flag</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="171.6" customHeight="1" s="72">
-      <c r="A35" s="42" t="inlineStr">
-        <is>
-          <t>P6-A30</t>
-        </is>
-      </c>
-      <c r="B35" s="69" t="n"/>
-      <c r="C35" s="43" t="inlineStr">
-        <is>
-          <t>Agents</t>
-        </is>
-      </c>
-      <c r="D35" s="43" t="inlineStr">
-        <is>
-          <t>DineoutExecutor -- full flow, mocked final book_table call</t>
-        </is>
-      </c>
-      <c r="E35" s="43" t="inlineStr">
-        <is>
-          <t>Same pattern as P6-A25 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
-        </is>
-      </c>
-      <c r="F35" s="43" t="inlineStr">
-        <is>
-          <t>feat: DineoutExecutor -- full approval-gated Dineout booking flow, book_table call mocked pending staging creds</t>
-        </is>
-      </c>
-      <c r="G35" s="43" t="inlineStr">
-        <is>
-          <t>docs/ACTION_QUEUE.md</t>
-        </is>
-      </c>
-      <c r="H35" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I35" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J35" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K35" s="42" t="n"/>
-      <c r="L35" s="42" t="n"/>
-      <c r="M35" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23, P6-A29</t>
-        </is>
-      </c>
-      <c r="O35" s="43" t="inlineStr">
-        <is>
-          <t>full flow test with mocked book_table; reservations row created with a clear 'simulated' flag</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="39.6" customHeight="1" s="72">
-      <c r="A36" s="42" t="inlineStr">
-        <is>
-          <t>P6-A31</t>
-        </is>
-      </c>
-      <c r="B36" s="68" t="inlineStr">
-        <is>
-          <t>feature/recipe-vendor-foundations</t>
-        </is>
-      </c>
-      <c r="C36" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D36" s="43" t="inlineStr">
-        <is>
-          <t>Recipe + RecipeIngredient model</t>
-        </is>
-      </c>
-      <c r="E36" s="43" t="inlineStr">
-        <is>
-          <t>New Recipe (menu_item_id) + RecipeIngredient (recipe_id, ingredient, quantity, unit) tables. Bridges MenuItem and inventory -- unlocks live-computed cost_price (from real ingredient prices) instead of manual entry, and real per-dish inventory depletion instead of aggregate-only shortage tracking. DEFERRED to end of Phase A alongside the rest of the procurement/Action Queue cluster, pending direct restaurant-owner research into how real procurement actually works.</t>
-        </is>
-      </c>
-      <c r="F36" s="43" t="inlineStr">
-        <is>
-          <t>feat: Recipe + RecipeIngredient models -- dish-to-ingredient yield mapping</t>
-        </is>
-      </c>
-      <c r="G36" s="43" t="inlineStr">
-        <is>
-          <t>docs/DATA_MODEL.md</t>
-        </is>
-      </c>
-      <c r="H36" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I36" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J36" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K36" s="42" t="n"/>
-      <c r="L36" s="42" t="n"/>
-      <c r="M36" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="43" t="n"/>
-      <c r="O36" s="43" t="inlineStr">
-        <is>
-          <t>recipe costing test (sum of ingredient costs matches computed cost_price); depletion test (a sale reduces linked ingredient stock by the right amount)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="39.6" customHeight="1" s="72">
-      <c r="A37" s="42" t="inlineStr">
-        <is>
-          <t>P6-A32</t>
-        </is>
-      </c>
-      <c r="B37" s="69" t="n"/>
-      <c r="C37" s="43" t="inlineStr">
-        <is>
-          <t>Infra</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="inlineStr">
-        <is>
-          <t>Vendor/Supplier model</t>
-        </is>
-      </c>
-      <c r="E37" s="43" t="inlineStr">
-        <is>
-          <t>New Vendor model (name, category, is_online, contact) + VendorPriceQuote (vendor_id, ingredient, price, quoted_at). Instamart becomes one Vendor among several (an 'online' vendor with live API pricing); local mandi/wholesale vendors become trackable entities with manually-entered or periodically-surveyed prices. Scoped as tracking/comparison only, not a marketplace. DEFERRED to end of Phase A -- exact procurement medium (Instamart API vs a WhatsApp-dispatch message to a local vendor vs other) intentionally left open pending direct conversation with a real restaurant owner/manager about their actual ordering process, before committing to a design.</t>
-        </is>
-      </c>
-      <c r="F37" s="43" t="inlineStr">
-        <is>
-          <t>feat: Vendor/Supplier model -- Instamart becomes one vendor among many, not the only source</t>
-        </is>
-      </c>
-      <c r="G37" s="43" t="inlineStr">
-        <is>
-          <t>docs/DATA_MODEL.md</t>
-        </is>
-      </c>
-      <c r="H37" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I37" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J37" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K37" s="42" t="n"/>
-      <c r="L37" s="42" t="n"/>
-      <c r="M37" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="43" t="inlineStr">
-        <is>
-          <t>P6-A31</t>
-        </is>
-      </c>
-      <c r="O37" s="43" t="inlineStr">
-        <is>
-          <t>vendor price comparison query returns correct cheapest-vendor-per-ingredient</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="52.8" customHeight="1" s="72">
-      <c r="A38" s="42" t="inlineStr">
-        <is>
-          <t>P6-A33</t>
-        </is>
-      </c>
-      <c r="B38" s="68" t="inlineStr">
-        <is>
-          <t>feature/mcp-expansion</t>
-        </is>
-      </c>
-      <c r="C38" s="43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D38" s="43" t="inlineStr">
-        <is>
-          <t>Internal MCP server -- get_market_brief / get_action_queue / approve_action</t>
-        </is>
-      </c>
-      <c r="E38" s="43" t="inlineStr">
-        <is>
-          <t>3 new tools on CortexKitchen's own MCP server (mcp_server.py), JWT-authenticated, calling MarketIntelService and ActionQueueService live. Lets an owner ask Claude Desktop directly about their restaurant and approve actions from there.</t>
-        </is>
-      </c>
-      <c r="F38" s="43" t="inlineStr">
-        <is>
-          <t>feat: 3 new MCP tools -- get_market_brief, get_action_queue, approve_action</t>
-        </is>
-      </c>
-      <c r="G38" s="43" t="inlineStr">
-        <is>
-          <t>docs/APIS.md, docs/ARCHITECTURE.md</t>
-        </is>
-      </c>
-      <c r="H38" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I38" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J38" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K38" s="42" t="n"/>
-      <c r="L38" s="42" t="n"/>
-      <c r="M38" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="43" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="O38" s="43" t="inlineStr">
-        <is>
-          <t>all 3 tools smoke-tested in Claude Desktop; approve_action triggers the same approval path as the web UI; JWT enforced</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="171.6" customHeight="1" s="72">
-      <c r="A39" s="42" t="inlineStr">
-        <is>
-          <t>P6-A34</t>
-        </is>
-      </c>
-      <c r="B39" s="69" t="n"/>
-      <c r="C39" s="43" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D39" s="43" t="inlineStr">
-        <is>
-          <t>Internal MCP server -- expand further (menu insights, forecast, what-if)</t>
-        </is>
-      </c>
-      <c r="E39" s="43" t="inlineStr">
-        <is>
-          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A32 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
-        </is>
-      </c>
-      <c r="F39" s="43" t="inlineStr">
-        <is>
-          <t>feat: expand internal MCP server -- menu insights, forecast, what-if simulator as tools</t>
-        </is>
-      </c>
-      <c r="G39" s="43" t="inlineStr">
-        <is>
-          <t>docs/APIS.md</t>
-        </is>
-      </c>
-      <c r="H39" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I39" s="42" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J39" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K39" s="42" t="n"/>
-      <c r="L39" s="42" t="n"/>
-      <c r="M39" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="43" t="inlineStr">
-        <is>
-          <t>P6-A33</t>
-        </is>
-      </c>
-      <c r="O39" s="43" t="inlineStr">
-        <is>
-          <t>each new tool smoke-tested in Claude Desktop; correct data returned matching the equivalent API endpoint</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="39.6" customHeight="1" s="72">
-      <c r="A40" s="42" t="inlineStr">
-        <is>
-          <t>P6-A35</t>
-        </is>
-      </c>
-      <c r="B40" s="68" t="inlineStr">
-        <is>
-          <t>feature/brief-page</t>
-        </is>
-      </c>
-      <c r="C40" s="43" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D40" s="43" t="inlineStr">
-        <is>
-          <t>/brief page</t>
-        </is>
-      </c>
-      <c r="E40" s="43" t="inlineStr">
-        <is>
-          <t>Daily morning briefing -- overnight performance, today's forecast vs yesterday, top 3 action priorities, market snapshot. Single-screen showcase of the whole system's intelligence.</t>
-        </is>
-      </c>
-      <c r="F40" s="43" t="inlineStr">
-        <is>
-          <t>feat: /brief page -- daily morning operational briefing</t>
-        </is>
-      </c>
-      <c r="G40" s="43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H40" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I40" s="42" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J40" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K40" s="42" t="n"/>
-      <c r="L40" s="42" t="n"/>
-      <c r="M40" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="43" t="inlineStr">
-        <is>
-          <t>P6-A24</t>
-        </is>
-      </c>
-      <c r="O40" s="43" t="inlineStr">
-        <is>
-          <t>manual verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="171.6" customHeight="1" s="72">
-      <c r="A41" s="42" t="inlineStr">
-        <is>
-          <t>P6-A36</t>
-        </is>
-      </c>
-      <c r="B41" s="68" t="n"/>
-      <c r="C41" s="43" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D41" s="43" t="inlineStr">
-        <is>
-          <t>Post-Phase-A documentation, test, CI, observability, and eval refresh</t>
-        </is>
-      </c>
-      <c r="E41" s="43" t="inlineStr">
-        <is>
-          <t>Once Phase A ships, a lot of new surface area will have landed at once -- Action Queue, workflow triggers, the anomaly agent, both executors, new connectors (Zomato stub, reviews), new data models (Recipe, Vendor, Expense, Obligation), MCP expansion. Do a full pass rather than letting docs drift: update every docs/*.md file, CLAUDE.md, README, and any screenshots referenced in docs to reflect what actually shipped. Audit test coverage for every new service/model added in Phase A -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (anomaly diagnoses, dynamic pricing suggestions), since the existing eval sets predate all of this and won't catch regressions in it.</t>
-        </is>
-      </c>
-      <c r="F41" s="43" t="inlineStr">
-        <is>
-          <t>docs: full documentation, test-coverage, CI, and eval refresh after the Phase A agentic core ships</t>
-        </is>
-      </c>
-      <c r="G41" s="43" t="inlineStr">
-        <is>
-          <t>All docs/*.md, CLAUDE.md, README.md</t>
-        </is>
-      </c>
-      <c r="H41" s="41" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I41" s="42" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J41" s="42" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K41" s="42" t="n"/>
-      <c r="L41" s="42" t="n"/>
-      <c r="M41" s="44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="43" t="inlineStr">
+      <c r="N39" s="90" t="inlineStr">
         <is>
           <t>All P6-A tasks</t>
         </is>
       </c>
-      <c r="O41" s="43" t="inlineStr">
+      <c r="O39" s="90" t="inlineStr">
         <is>
           <t>Every new service/model has test coverage; CI includes all new test files; RAGAS/DeepEval sets include at least one case per new agentic behavior; docs/screenshots match shipped behavior</t>
         </is>
       </c>
     </row>
+    <row r="40" ht="39.6" customHeight="1" s="72"/>
+    <row r="41" ht="171.6" customHeight="1" s="72"/>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="B17:B19"/>
     <mergeCell ref="B32:B33"/>
     <mergeCell ref="B36:B37"/>
     <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="A27:O27"/>
+    <mergeCell ref="B15:B16"/>
     <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B19:B21"/>
     <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B26:B27"/>
     <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B15:B16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -19744,7 +19665,7 @@
       </c>
       <c r="E4" s="62" t="inlineStr">
         <is>
-          <t>Phase A (P6-A29) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
+          <t>Phase A (P6-A28) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
         </is>
       </c>
       <c r="F4" s="62" t="inlineStr">
@@ -19779,7 +19700,7 @@
       </c>
       <c r="N4" s="62" t="inlineStr">
         <is>
-          <t>P6-A29, P6-S14</t>
+          <t>P6-A28, P6-S14</t>
         </is>
       </c>
       <c r="O4" s="62" t="inlineStr">
@@ -19828,7 +19749,7 @@
       </c>
       <c r="E6" s="62" t="inlineStr">
         <is>
-          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A30) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
+          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A29) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
         </is>
       </c>
       <c r="F6" s="62" t="inlineStr">
@@ -19863,7 +19784,7 @@
       </c>
       <c r="N6" s="62" t="inlineStr">
         <is>
-          <t>P6-A30</t>
+          <t>P6-A29</t>
         </is>
       </c>
       <c r="O6" s="62" t="inlineStr">
@@ -19908,7 +19829,7 @@
       </c>
       <c r="E8" s="62" t="inlineStr">
         <is>
-          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A26) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
+          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A25) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
         </is>
       </c>
       <c r="F8" s="62" t="inlineStr">
@@ -19943,7 +19864,7 @@
       </c>
       <c r="N8" s="62" t="inlineStr">
         <is>
-          <t>P6-A26, P7-1, P7-2</t>
+          <t>P6-A25, P7-1, P7-2</t>
         </is>
       </c>
       <c r="O8" s="62" t="inlineStr">
@@ -20131,7 +20052,7 @@
       </c>
       <c r="N14" s="62" t="inlineStr">
         <is>
-          <t>P6-A21</t>
+          <t>P6-A20</t>
         </is>
       </c>
       <c r="O14" s="62" t="inlineStr">

</xml_diff>

<commit_message>
tracker: mark P6-A5 (Zomato stub connector) Completed
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -17540,7 +17540,7 @@
       </c>
       <c r="E7" s="90" t="inlineStr">
         <is>
-          <t>ZomatoConnector class following the exact BaseConnector shape (sync()/enrich()) as SwiggyConnector, registered in provider_registry.py's CAPABILITY_PROVIDERS as an actually-real (if non-functional) connector rather than a placeholder string. Proves the multi-provider architecture is real, not Swiggy-only. No live Zomato API call required -- returns a clear 'not yet connected' state.</t>
+          <t>ZomatoConnector class following the exact BaseConnector shape (sync()/enrich()) as SwiggyConnector, registered in provider_registry.py's CAPABILITY_PROVIDERS as an actually-real (if non-functional) connector rather than a placeholder string. Proves the multi-provider architecture is real, not Swiggy-only. No live Zomato API call required -- returns a clear 'not yet connected' state. Moved BaseConnector out of the swiggy package to a shared location (app/infrastructure/base_connector.py) as part of this task, since a genuinely platform-agnostic base class living inside a Swiggy-specific package undercut its own point.</t>
         </is>
       </c>
       <c r="F7" s="90" t="inlineStr">
@@ -17555,7 +17555,7 @@
       </c>
       <c r="H7" s="108" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I7" s="89" t="inlineStr">
@@ -17568,10 +17568,18 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K7" s="89" t="n"/>
-      <c r="L7" s="89" t="n"/>
+      <c r="K7" s="89" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="L7" s="89" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
       <c r="M7" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="90" t="n"/>
       <c r="O7" s="90" t="inlineStr">

</xml_diff>

<commit_message>
tracker: defer P6-A6 (review aggregation) to Phase 7 as P7-15 -- needs a real restaurant, cascade-renumber A7-A35 to A6-A34
Unlike the Zomato stub connector (which only needed to prove the
architecture), this task's entire value is real review data -- there's no
actual Google/Zomato business listing for this restaurant yet, so even a
demoable version isn't possible until a real restaurant customer exists.
Added a new 'BLOCKED -- needs a real restaurant' section to the Staging
Creds + Phase 7 sheet distinct from the existing Swiggy-creds and
Sarvam/AWS blockers, since this is a different kind of blocker entirely.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -471,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -758,6 +758,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17594,30 +17598,34 @@
           <t>P6-A6</t>
         </is>
       </c>
-      <c r="B8" s="69" t="n"/>
+      <c r="B8" s="98" t="inlineStr">
+        <is>
+          <t>feature/financial-compliance</t>
+        </is>
+      </c>
       <c r="C8" s="90" t="inlineStr">
         <is>
-          <t>Integrations</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="D8" s="90" t="inlineStr">
         <is>
-          <t>Public review aggregation connectors (Google/Zomato reviews)</t>
+          <t>Financial scorecard -- Expense ledger + real P&amp;L</t>
         </is>
       </c>
       <c r="E8" s="90" t="inlineStr">
         <is>
-          <t>GoogleReviewsConnector / ZomatoReviewsConnector following the same BaseConnector pattern, pulling public review data (not internal complaints) into complaint_intelligence as an additional source type. Extends the Feedback model's source concept rather than inventing a parallel system.</t>
+          <t>New Expense model (category: rent/utilities/marketing/labor-later/other, amount, recurrence). Extends business.py's existing revenue/margin computation into a real daily/weekly P&amp;L and one composite health score. Designed so labor slots in later as just another Expense category, not a rewrite.</t>
         </is>
       </c>
       <c r="F8" s="90" t="inlineStr">
         <is>
-          <t>feat: public review aggregation -- Google/Zomato reviews via BaseConnector pattern</t>
+          <t>feat: financial scorecard -- Expense ledger, real P&amp;L, composite health score</t>
         </is>
       </c>
       <c r="G8" s="90" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md, docs/CONNECTORS.md</t>
+          <t>docs/APIS.md</t>
         </is>
       </c>
       <c r="H8" s="108" t="inlineStr">
@@ -17640,14 +17648,10 @@
       <c r="M8" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="90" t="inlineStr">
-        <is>
-          <t>P6-A5</t>
-        </is>
-      </c>
+      <c r="N8" s="90" t="n"/>
       <c r="O8" s="90" t="inlineStr">
         <is>
-          <t>reviews ingested with correct source tag; complaint_intelligence node correctly surfaces public-review-sourced themes alongside internal ones</t>
+          <t>P&amp;L numbers match seeded expense + revenue data; health score computes deterministically from known inputs</t>
         </is>
       </c>
     </row>
@@ -17657,11 +17661,7 @@
           <t>P6-A7</t>
         </is>
       </c>
-      <c r="B9" s="98" t="inlineStr">
-        <is>
-          <t>feature/financial-compliance</t>
-        </is>
-      </c>
+      <c r="B9" s="69" t="n"/>
       <c r="C9" s="90" t="inlineStr">
         <is>
           <t>Backend</t>
@@ -17669,17 +17669,17 @@
       </c>
       <c r="D9" s="90" t="inlineStr">
         <is>
-          <t>Financial scorecard -- Expense ledger + real P&amp;L</t>
+          <t>Compliance / Obligations calendar</t>
         </is>
       </c>
       <c r="E9" s="90" t="inlineStr">
         <is>
-          <t>New Expense model (category: rent/utilities/marketing/labor-later/other, amount, recurrence). Extends business.py's existing revenue/margin computation into a real daily/weekly P&amp;L and one composite health score. Designed so labor slots in later as just another Expense category, not a rewrite.</t>
+          <t>Generalized Obligation model (type: license-renewal/GST-filing/inspection/other, due_date, status) with reminders delivered through the existing Phase-5 email digest mechanism rather than a new one-off sender. Not a GST computation/invoicing layer -- just a dated-obligation tracker with reminders.</t>
         </is>
       </c>
       <c r="F9" s="90" t="inlineStr">
         <is>
-          <t>feat: financial scorecard -- Expense ledger, real P&amp;L, composite health score</t>
+          <t>feat: compliance/obligations calendar -- reminder engine reusing the existing email digest</t>
         </is>
       </c>
       <c r="G9" s="90" t="inlineStr">
@@ -17694,7 +17694,7 @@
       </c>
       <c r="I9" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J9" s="89" t="inlineStr">
@@ -17710,7 +17710,7 @@
       <c r="N9" s="90" t="n"/>
       <c r="O9" s="90" t="inlineStr">
         <is>
-          <t>P&amp;L numbers match seeded expense + revenue data; health score computes deterministically from known inputs</t>
+          <t>reminder fires at the correct lead-time before due_date; reuses existing digest delivery path</t>
         </is>
       </c>
     </row>
@@ -17720,30 +17720,34 @@
           <t>P6-A8</t>
         </is>
       </c>
-      <c r="B10" s="69" t="n"/>
+      <c r="B10" s="98" t="inlineStr">
+        <is>
+          <t>feature/location-architecture</t>
+        </is>
+      </c>
       <c r="C10" s="90" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D10" s="90" t="inlineStr">
         <is>
-          <t>Compliance / Obligations calendar</t>
+          <t>Location-aware enrichers (hedge for multi-location)</t>
         </is>
       </c>
       <c r="E10" s="90" t="inlineStr">
         <is>
-          <t>Generalized Obligation model (type: license-renewal/GST-filing/inspection/other, due_date, status) with reminders delivered through the existing Phase-5 email digest mechanism rather than a new one-off sender. Not a GST computation/invoicing layer -- just a dated-obligation tracker with reminders.</t>
+          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A29) exists or once real customers have multiple outlets.</t>
         </is>
       </c>
       <c r="F10" s="90" t="inlineStr">
         <is>
-          <t>feat: compliance/obligations calendar -- reminder engine reusing the existing email digest</t>
+          <t>feat: location-aware enrichers -- pass address/location context through instead of one hardcoded address</t>
         </is>
       </c>
       <c r="G10" s="90" t="inlineStr">
         <is>
-          <t>docs/APIS.md</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="H10" s="108" t="inlineStr">
@@ -17769,7 +17773,7 @@
       <c r="N10" s="90" t="n"/>
       <c r="O10" s="90" t="inlineStr">
         <is>
-          <t>reminder fires at the correct lead-time before due_date; reuses existing digest delivery path</t>
+          <t>enrichers accept and correctly use a passed-in address_id, defaulting to the existing single-address behavior when none given</t>
         </is>
       </c>
     </row>
@@ -17779,11 +17783,7 @@
           <t>P6-A9</t>
         </is>
       </c>
-      <c r="B11" s="98" t="inlineStr">
-        <is>
-          <t>feature/location-architecture</t>
-        </is>
-      </c>
+      <c r="B11" s="69" t="n"/>
       <c r="C11" s="90" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -17791,22 +17791,22 @@
       </c>
       <c r="D11" s="90" t="inlineStr">
         <is>
-          <t>Location-aware enrichers (hedge for multi-location)</t>
+          <t>Multi-location / Restaurant entity -- STRATEGIC, needs explicit go/no-go</t>
         </is>
       </c>
       <c r="E11" s="90" t="inlineStr">
         <is>
-          <t>Thread an explicit location/address context through MarketIntelService and all 3 enrichers instead of a single hardcoded SWIGGY_ADDRESS_ID -- cheap to do now, expensive to retrofit once multi-location (P6-A30) exists or once real customers have multiple outlets.</t>
+          <t>Introduce Restaurant as a first-class entity between Organization and everything else (menu, inventory, planning runs, Swiggy connector -- each physical location has its own Swiggy restaurant ID). Add restaurant_id to MenuItem/InventoryItem/PlanningRun/connectors. Cheaper to do now while the schema is small than to retrofit later. NOT started until the user confirms real near-term demand justifies it over other Phase A work.</t>
         </is>
       </c>
       <c r="F11" s="90" t="inlineStr">
         <is>
-          <t>feat: location-aware enrichers -- pass address/location context through instead of one hardcoded address</t>
+          <t>feat: Restaurant entity -- first-class multi-location support</t>
         </is>
       </c>
       <c r="G11" s="90" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>docs/DATA_MODEL.md, docs/DECISIONS.md</t>
         </is>
       </c>
       <c r="H11" s="108" t="inlineStr">
@@ -17816,7 +17816,7 @@
       </c>
       <c r="I11" s="89" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low (pending go/no-go)</t>
         </is>
       </c>
       <c r="J11" s="89" t="inlineStr">
@@ -17829,10 +17829,14 @@
       <c r="M11" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="90" t="n"/>
+      <c r="N11" s="90" t="inlineStr">
+        <is>
+          <t>P6-A8</t>
+        </is>
+      </c>
       <c r="O11" s="90" t="inlineStr">
         <is>
-          <t>enrichers accept and correctly use a passed-in address_id, defaulting to the existing single-address behavior when none given</t>
+          <t>existing single-location orgs continue to work unchanged (default restaurant backfilled); cross-location query test once 2+ restaurants exist</t>
         </is>
       </c>
     </row>
@@ -17842,30 +17846,34 @@
           <t>P6-A10</t>
         </is>
       </c>
-      <c r="B12" s="69" t="n"/>
+      <c r="B12" s="98" t="inlineStr">
+        <is>
+          <t>feature/chatbot-dineout-tools</t>
+        </is>
+      </c>
       <c r="C12" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D12" s="90" t="inlineStr">
         <is>
-          <t>Multi-location / Restaurant entity -- STRATEGIC, needs explicit go/no-go</t>
+          <t>Chatbot -- Dineout competitive query tools</t>
         </is>
       </c>
       <c r="E12" s="90" t="inlineStr">
         <is>
-          <t>Introduce Restaurant as a first-class entity between Organization and everything else (menu, inventory, planning runs, Swiggy connector -- each physical location has its own Swiggy restaurant ID). Add restaurant_id to MenuItem/InventoryItem/PlanningRun/connectors. Cheaper to do now while the schema is small than to retrofit later. NOT started until the user confirms real near-term demand justifies it over other Phase A work.</t>
+          <t>3 Groq function-calling tools for the existing chatbot: get_competitor_deals, get_area_occupancy, get_trending_dishes -- all using Swiggy's existing read-only Dineout MCP (search_restaurants_dineout, get_restaurant_details, get_available_slots), already-proven tools. (Formerly P6-MI04; renumbered as part of the Phase 6 replan.)</t>
         </is>
       </c>
       <c r="F12" s="90" t="inlineStr">
         <is>
-          <t>feat: Restaurant entity -- first-class multi-location support</t>
+          <t>feat: chatbot Dineout tools -- competitor deals, area occupancy, trending dishes</t>
         </is>
       </c>
       <c r="G12" s="90" t="inlineStr">
         <is>
-          <t>docs/DATA_MODEL.md, docs/DECISIONS.md</t>
+          <t>docs/AGENTS.md</t>
         </is>
       </c>
       <c r="H12" s="108" t="inlineStr">
@@ -17875,7 +17883,7 @@
       </c>
       <c r="I12" s="89" t="inlineStr">
         <is>
-          <t>Low (pending go/no-go)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J12" s="89" t="inlineStr">
@@ -17888,14 +17896,10 @@
       <c r="M12" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="90" t="inlineStr">
-        <is>
-          <t>P6-A9</t>
-        </is>
-      </c>
+      <c r="N12" s="90" t="n"/>
       <c r="O12" s="90" t="inlineStr">
         <is>
-          <t>existing single-location orgs continue to work unchanged (default restaurant backfilled); cross-location query test once 2+ restaurants exist</t>
+          <t>all 3 tools callable from /chat; correct Swiggy data returned; graceful None on failure</t>
         </is>
       </c>
     </row>
@@ -17905,29 +17909,25 @@
           <t>P6-A11</t>
         </is>
       </c>
-      <c r="B13" s="98" t="inlineStr">
-        <is>
-          <t>feature/chatbot-dineout-tools</t>
-        </is>
-      </c>
+      <c r="B13" s="69" t="n"/>
       <c r="C13" s="90" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D13" s="90" t="inlineStr">
         <is>
-          <t>Chatbot -- Dineout competitive query tools</t>
+          <t>Structured outputs -- tool_choice=required across chatbot tools</t>
         </is>
       </c>
       <c r="E13" s="90" t="inlineStr">
         <is>
-          <t>3 Groq function-calling tools for the existing chatbot: get_competitor_deals, get_area_occupancy, get_trending_dishes -- all using Swiggy's existing read-only Dineout MCP (search_restaurants_dineout, get_restaurant_details, get_available_slots), already-proven tools. (Formerly P6-MI04; renumbered as part of the Phase 6 replan.)</t>
+          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema across all chatbot tools (Swiggy and internal). Chatbot function calls never hallucinate JSON.</t>
         </is>
       </c>
       <c r="F13" s="90" t="inlineStr">
         <is>
-          <t>feat: chatbot Dineout tools -- competitor deals, area occupancy, trending dishes</t>
+          <t>feat: structured outputs -- tool_choice=required across all chatbot tools</t>
         </is>
       </c>
       <c r="G13" s="90" t="inlineStr">
@@ -17942,7 +17942,7 @@
       </c>
       <c r="I13" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J13" s="89" t="inlineStr">
@@ -17955,10 +17955,14 @@
       <c r="M13" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="90" t="n"/>
+      <c r="N13" s="90" t="inlineStr">
+        <is>
+          <t>P6-A10</t>
+        </is>
+      </c>
       <c r="O13" s="90" t="inlineStr">
         <is>
-          <t>all 3 tools callable from /chat; correct Swiggy data returned; graceful None on failure</t>
+          <t>schema validation test; chatbot returns valid JSON on repeated calls</t>
         </is>
       </c>
     </row>
@@ -17968,7 +17972,11 @@
           <t>P6-A12</t>
         </is>
       </c>
-      <c r="B14" s="69" t="n"/>
+      <c r="B14" s="98" t="inlineStr">
+        <is>
+          <t>feature/llm-cost-quality</t>
+        </is>
+      </c>
       <c r="C14" s="90" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -17976,22 +17984,22 @@
       </c>
       <c r="D14" s="90" t="inlineStr">
         <is>
-          <t>Structured outputs -- tool_choice=required across chatbot tools</t>
+          <t>Prompt caching -- critic + aggregator</t>
         </is>
       </c>
       <c r="E14" s="90" t="inlineStr">
         <is>
-          <t>Upgrade chatbot Groq calls to tool_choice=required + strict JSON schema across all chatbot tools (Swiggy and internal). Chatbot function calls never hallucinate JSON.</t>
+          <t>Add prompt-caching headers to critic and aggregator LLM calls (both have long, repeated system prompts). Cuts LLM cost per planning run; invisible to a demo but real cost hygiene.</t>
         </is>
       </c>
       <c r="F14" s="90" t="inlineStr">
         <is>
-          <t>feat: structured outputs -- tool_choice=required across all chatbot tools</t>
+          <t>feat: prompt caching -- cut LLM costs on critic and aggregator nodes</t>
         </is>
       </c>
       <c r="G14" s="90" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md</t>
+          <t>docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H14" s="108" t="inlineStr">
@@ -18014,14 +18022,10 @@
       <c r="M14" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="90" t="inlineStr">
-        <is>
-          <t>P6-A11</t>
-        </is>
-      </c>
+      <c r="N14" s="90" t="n"/>
       <c r="O14" s="90" t="inlineStr">
         <is>
-          <t>schema validation test; chatbot returns valid JSON on repeated calls</t>
+          <t>cost log shows cache_hit=true on second run of the same scenario</t>
         </is>
       </c>
     </row>
@@ -18031,34 +18035,30 @@
           <t>P6-A13</t>
         </is>
       </c>
-      <c r="B15" s="98" t="inlineStr">
-        <is>
-          <t>feature/llm-cost-quality</t>
-        </is>
-      </c>
+      <c r="B15" s="69" t="n"/>
       <c r="C15" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D15" s="90" t="inlineStr">
         <is>
-          <t>Prompt caching -- critic + aggregator</t>
+          <t>Multi-agent debate critic</t>
         </is>
       </c>
       <c r="E15" s="90" t="inlineStr">
         <is>
-          <t>Add prompt-caching headers to critic and aggregator LLM calls (both have long, repeated system prompts). Cuts LLM cost per planning run; invisible to a demo but real cost hygiene.</t>
+          <t>Two LLM critic instances (optimistic vs conservative), structured debate, moderator resolves disagreement. Marginal demo-visible upside over the existing single critic given the added cost/latency -- kept low priority.</t>
         </is>
       </c>
       <c r="F15" s="90" t="inlineStr">
         <is>
-          <t>feat: prompt caching -- cut LLM costs on critic and aggregator nodes</t>
+          <t>feat: multi-agent debate critic -- consensus scoring</t>
         </is>
       </c>
       <c r="G15" s="90" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md</t>
+          <t>docs/AGENTS.md</t>
         </is>
       </c>
       <c r="H15" s="108" t="inlineStr">
@@ -18084,7 +18084,7 @@
       <c r="N15" s="90" t="n"/>
       <c r="O15" s="90" t="inlineStr">
         <is>
-          <t>cost log shows cache_hit=true on second run of the same scenario</t>
+          <t>debate resolves on test plans; disagreement cases escalate correctly</t>
         </is>
       </c>
     </row>
@@ -18094,30 +18094,34 @@
           <t>P6-A14</t>
         </is>
       </c>
-      <c r="B16" s="69" t="n"/>
+      <c r="B16" s="98" t="inlineStr">
+        <is>
+          <t>feature/ci-eval-hygiene</t>
+        </is>
+      </c>
       <c r="C16" s="90" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D16" s="90" t="inlineStr">
         <is>
-          <t>Multi-agent debate critic</t>
+          <t>Fix SQLite/JSONB CI test-infra gap</t>
         </is>
       </c>
       <c r="E16" s="90" t="inlineStr">
         <is>
-          <t>Two LLM critic instances (optimistic vs conservative), structured debate, moderator resolves disagreement. Marginal demo-visible upside over the existing single critic given the added cost/latency -- kept low priority.</t>
+          <t>test_swiggy_reservation_sync.py and test_connector_repository.py are excluded from CI because SQLite can't render Postgres JSONB columns. Either a SQLite-compatible fallback type or a Postgres CI service container.</t>
         </is>
       </c>
       <c r="F16" s="90" t="inlineStr">
         <is>
-          <t>feat: multi-agent debate critic -- consensus scoring</t>
+          <t>fix: SQLite-compatible JSONB handling (or Postgres CI service) for excluded test files</t>
         </is>
       </c>
       <c r="G16" s="90" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H16" s="108" t="inlineStr">
@@ -18143,7 +18147,7 @@
       <c r="N16" s="90" t="n"/>
       <c r="O16" s="90" t="inlineStr">
         <is>
-          <t>debate resolves on test plans; disagreement cases escalate correctly</t>
+          <t>previously-excluded test files run in CI</t>
         </is>
       </c>
     </row>
@@ -18153,29 +18157,25 @@
           <t>P6-A15</t>
         </is>
       </c>
-      <c r="B17" s="98" t="inlineStr">
-        <is>
-          <t>feature/ci-eval-hygiene</t>
-        </is>
-      </c>
+      <c r="B17" s="70" t="n"/>
       <c r="C17" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D17" s="90" t="inlineStr">
         <is>
-          <t>Fix SQLite/JSONB CI test-infra gap</t>
+          <t>Promote reviewed RAGAS/DeepEval candidates</t>
         </is>
       </c>
       <c r="E17" s="90" t="inlineStr">
         <is>
-          <t>test_swiggy_reservation_sync.py and test_connector_repository.py are excluded from CI because SQLite can't render Postgres JSONB columns. Either a SQLite-compatible fallback type or a Postgres CI service container.</t>
+          <t>Recurring habit of running the existing candidate-generation scripts and hand-promoting reviewed candidates into the curated eval datasets.</t>
         </is>
       </c>
       <c r="F17" s="90" t="inlineStr">
         <is>
-          <t>fix: SQLite-compatible JSONB handling (or Postgres CI service) for excluded test files</t>
+          <t>chore: promote reviewed eval candidates into curated datasets</t>
         </is>
       </c>
       <c r="G17" s="90" t="inlineStr">
@@ -18206,7 +18206,7 @@
       <c r="N17" s="90" t="n"/>
       <c r="O17" s="90" t="inlineStr">
         <is>
-          <t>previously-excluded test files run in CI</t>
+          <t>N/A -- ongoing process, not a one-time build</t>
         </is>
       </c>
     </row>
@@ -18216,25 +18216,25 @@
           <t>P6-A16</t>
         </is>
       </c>
-      <c r="B18" s="70" t="n"/>
+      <c r="B18" s="69" t="n"/>
       <c r="C18" s="90" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D18" s="90" t="inlineStr">
         <is>
-          <t>Promote reviewed RAGAS/DeepEval candidates</t>
+          <t>Regenerate golden_runs.json against real data</t>
         </is>
       </c>
       <c r="E18" s="90" t="inlineStr">
         <is>
-          <t>Recurring habit of running the existing candidate-generation scripts and hand-promoting reviewed candidates into the curated eval datasets.</t>
+          <t>The key-path bug in build_golden_dataset.py is already fixed; the checked-in fixture still reflects the old broken extraction. Regenerate once real run history exists.</t>
         </is>
       </c>
       <c r="F18" s="90" t="inlineStr">
         <is>
-          <t>chore: promote reviewed eval candidates into curated datasets</t>
+          <t>chore: regenerate golden_runs.json with corrected extraction logic</t>
         </is>
       </c>
       <c r="G18" s="90" t="inlineStr">
@@ -18265,7 +18265,7 @@
       <c r="N18" s="90" t="n"/>
       <c r="O18" s="90" t="inlineStr">
         <is>
-          <t>N/A -- ongoing process, not a one-time build</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -18275,25 +18275,29 @@
           <t>P6-A17</t>
         </is>
       </c>
-      <c r="B19" s="69" t="n"/>
+      <c r="B19" s="98" t="inlineStr">
+        <is>
+          <t>feature/menu-engineering-matrix</t>
+        </is>
+      </c>
       <c r="C19" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D19" s="90" t="inlineStr">
         <is>
-          <t>Regenerate golden_runs.json against real data</t>
+          <t>Menu engineering matrix UI</t>
         </is>
       </c>
       <c r="E19" s="90" t="inlineStr">
         <is>
-          <t>The key-path bug in build_golden_dataset.py is already fixed; the checked-in fixture still reflects the old broken extraction. Regenerate once real run history exists.</t>
+          <t>Stars/plow-horses/dogs/puzzles quadrant chart using margin_pct x quantity, both already computed in business.py -- just needs quadrant classification + a chart.</t>
         </is>
       </c>
       <c r="F19" s="90" t="inlineStr">
         <is>
-          <t>chore: regenerate golden_runs.json with corrected extraction logic</t>
+          <t>feat: menu engineering matrix -- margin x popularity quadrant chart</t>
         </is>
       </c>
       <c r="G19" s="90" t="inlineStr">
@@ -18308,7 +18312,7 @@
       </c>
       <c r="I19" s="89" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J19" s="89" t="inlineStr">
@@ -18324,7 +18328,7 @@
       <c r="N19" s="90" t="n"/>
       <c r="O19" s="90" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>quadrant classification unit test; chart renders correctly</t>
         </is>
       </c>
     </row>
@@ -18336,7 +18340,7 @@
       </c>
       <c r="B20" s="98" t="inlineStr">
         <is>
-          <t>feature/menu-engineering-matrix</t>
+          <t>feature/pages-redesign</t>
         </is>
       </c>
       <c r="C20" s="90" t="inlineStr">
@@ -18346,17 +18350,17 @@
       </c>
       <c r="D20" s="90" t="inlineStr">
         <is>
-          <t>Menu engineering matrix UI</t>
+          <t>all page redesign via claude design</t>
         </is>
       </c>
       <c r="E20" s="90" t="inlineStr">
         <is>
-          <t>Stars/plow-horses/dogs/puzzles quadrant chart using margin_pct x quantity, both already computed in business.py -- just needs quadrant classification + a chart.</t>
+          <t>Apply the existing design system to /runs -- currently the weakest-looking screen (dense monospace debug trace). Fix the unstyled raw 404 on /runs/{id} deep links.</t>
         </is>
       </c>
       <c r="F20" s="90" t="inlineStr">
         <is>
-          <t>feat: menu engineering matrix -- margin x popularity quadrant chart</t>
+          <t>feat: redesign /runs history page + fix /runs/{id} deep-link 404</t>
         </is>
       </c>
       <c r="G20" s="90" t="inlineStr">
@@ -18371,7 +18375,7 @@
       </c>
       <c r="I20" s="89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J20" s="89" t="inlineStr">
@@ -18387,7 +18391,7 @@
       <c r="N20" s="90" t="n"/>
       <c r="O20" s="90" t="inlineStr">
         <is>
-          <t>quadrant classification unit test; chart renders correctly</t>
+          <t>direct navigation to /runs/{id} renders the run, not a 404</t>
         </is>
       </c>
     </row>
@@ -18399,7 +18403,7 @@
       </c>
       <c r="B21" s="98" t="inlineStr">
         <is>
-          <t>feature/pages-redesign</t>
+          <t>feature/voice-interface</t>
         </is>
       </c>
       <c r="C21" s="90" t="inlineStr">
@@ -18409,22 +18413,22 @@
       </c>
       <c r="D21" s="90" t="inlineStr">
         <is>
-          <t>all page redesign via claude design</t>
+          <t>Voice interface</t>
         </is>
       </c>
       <c r="E21" s="90" t="inlineStr">
         <is>
-          <t>Apply the existing design system to /runs -- currently the weakest-looking screen (dense monospace debug trace). Fix the unstyled raw 404 on /runs/{id} deep links.</t>
+          <t>Whisper transcription on browser-recorded question, existing RAG chatbot answers, TTS reads back.</t>
         </is>
       </c>
       <c r="F21" s="90" t="inlineStr">
         <is>
-          <t>feat: redesign /runs history page + fix /runs/{id} deep-link 404</t>
+          <t>feat: voice interface -- Whisper transcription + RAG answer + TTS readback</t>
         </is>
       </c>
       <c r="G21" s="90" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>docs/PRODUCT_MODES.md</t>
         </is>
       </c>
       <c r="H21" s="108" t="inlineStr">
@@ -18434,7 +18438,7 @@
       </c>
       <c r="I21" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J21" s="89" t="inlineStr">
@@ -18450,7 +18454,7 @@
       <c r="N21" s="90" t="n"/>
       <c r="O21" s="90" t="inlineStr">
         <is>
-          <t>direct navigation to /runs/{id} renders the run, not a 404</t>
+          <t>transcription accuracy smoke test; end-to-end voice -&gt; RAG answer -&gt; TTS</t>
         </is>
       </c>
     </row>
@@ -18462,7 +18466,7 @@
       </c>
       <c r="B22" s="98" t="inlineStr">
         <is>
-          <t>feature/voice-interface</t>
+          <t>feature/live-page-redesign</t>
         </is>
       </c>
       <c r="C22" s="90" t="inlineStr">
@@ -18472,17 +18476,17 @@
       </c>
       <c r="D22" s="90" t="inlineStr">
         <is>
-          <t>Voice interface</t>
+          <t>/live page -- reframed as alerts/synthesis overlay</t>
         </is>
       </c>
       <c r="E22" s="90" t="inlineStr">
         <is>
-          <t>Whisper transcription on browser-recorded question, existing RAG chatbot answers, TTS reads back.</t>
+          <t>NOT a live order board (that's POS/aggregator territory and touches personal Swiggy consumer data). Instead: an alerts-and-synthesis overlay surfacing cross-referenced signals (e.g. 'order running late -- here's why, per our own data') during service hours.</t>
         </is>
       </c>
       <c r="F22" s="90" t="inlineStr">
         <is>
-          <t>feat: voice interface -- Whisper transcription + RAG answer + TTS readback</t>
+          <t>feat: /live page -- alerts and synthesis overlay, not a live order feed</t>
         </is>
       </c>
       <c r="G22" s="90" t="inlineStr">
@@ -18513,94 +18517,94 @@
       <c r="N22" s="90" t="n"/>
       <c r="O22" s="90" t="inlineStr">
         <is>
-          <t>transcription accuracy smoke test; end-to-end voice -&gt; RAG answer -&gt; TTS</t>
+          <t>manual verification</t>
         </is>
       </c>
     </row>
     <row r="23" ht="7.95" customHeight="1" s="72">
-      <c r="A23" s="65" t="inlineStr">
+      <c r="A23" s="111" t="n"/>
+      <c r="B23" s="111" t="n"/>
+      <c r="C23" s="111" t="n"/>
+      <c r="D23" s="111" t="n"/>
+      <c r="E23" s="111" t="n"/>
+      <c r="F23" s="111" t="n"/>
+      <c r="G23" s="111" t="n"/>
+      <c r="H23" s="111" t="n"/>
+      <c r="I23" s="111" t="n"/>
+      <c r="J23" s="111" t="n"/>
+      <c r="K23" s="111" t="n"/>
+      <c r="L23" s="111" t="n"/>
+      <c r="M23" s="111" t="n"/>
+      <c r="N23" s="111" t="n"/>
+      <c r="O23" s="111" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="72">
+      <c r="A24" s="109" t="inlineStr">
+        <is>
+          <t>DEFERRED TO END OF PHASE A -- pending direct restaurant-owner research into real procurement/approval workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52.05" customHeight="1" s="72">
+      <c r="A25" s="65" t="inlineStr">
         <is>
           <t>P6-A21</t>
         </is>
       </c>
-      <c r="B23" s="98" t="inlineStr">
-        <is>
-          <t>feature/live-page-redesign</t>
-        </is>
-      </c>
-      <c r="C23" s="90" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D23" s="90" t="inlineStr">
-        <is>
-          <t>/live page -- reframed as alerts/synthesis overlay</t>
-        </is>
-      </c>
-      <c r="E23" s="90" t="inlineStr">
-        <is>
-          <t>NOT a live order board (that's POS/aggregator territory and touches personal Swiggy consumer data). Instead: an alerts-and-synthesis overlay surfacing cross-referenced signals (e.g. 'order running late -- here's why, per our own data') during service hours.</t>
-        </is>
-      </c>
-      <c r="F23" s="90" t="inlineStr">
-        <is>
-          <t>feat: /live page -- alerts and synthesis overlay, not a live order feed</t>
-        </is>
-      </c>
-      <c r="G23" s="90" t="inlineStr">
-        <is>
-          <t>docs/PRODUCT_MODES.md</t>
-        </is>
-      </c>
-      <c r="H23" s="108" t="inlineStr">
+      <c r="B25" s="98" t="inlineStr">
+        <is>
+          <t>feature/action-queue</t>
+        </is>
+      </c>
+      <c r="C25" s="90" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="D25" s="90" t="inlineStr">
+        <is>
+          <t>ActionQueueService + action_queue table</t>
+        </is>
+      </c>
+      <c r="E25" s="90" t="inlineStr">
+        <is>
+          <t>New table (org_id, action_type [AUTO/APPROVE_REQUIRED/RECOMMENDATION], payload jsonb, status [PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED], approved_by, executed_at, error). ActionQueueService CRUD + status transitions. Plan output gains an action_queue section in the API response. Foundational -- every other agentic task below (workflow triggers, dynamic pricing, executors, trust-ladder) writes into this same table rather than inventing its own approval mechanism. DEFERRED to end of Phase A -- its main real-world value (approving reorder suggestions) is exactly the workflow that needs real restaurant-owner input first; building the approval UX before that research risks designing around the wrong assumptions.</t>
+        </is>
+      </c>
+      <c r="F25" s="90" t="inlineStr">
+        <is>
+          <t>feat: ActionQueueService + action_queue table -- 3-tier action model with approval lifecycle</t>
+        </is>
+      </c>
+      <c r="G25" s="90" t="inlineStr">
+        <is>
+          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md, docs/DECISIONS.md</t>
+        </is>
+      </c>
+      <c r="H25" s="108" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I23" s="89" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J23" s="89" t="inlineStr">
+      <c r="I25" s="89" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J25" s="89" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K23" s="89" t="n"/>
-      <c r="L23" s="89" t="n"/>
-      <c r="M23" s="91" t="n">
+      <c r="K25" s="89" t="n"/>
+      <c r="L25" s="89" t="n"/>
+      <c r="M25" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="90" t="n"/>
-      <c r="O23" s="90" t="inlineStr">
-        <is>
-          <t>manual verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1" s="72">
-      <c r="A24" s="111" t="n"/>
-      <c r="B24" s="111" t="n"/>
-      <c r="C24" s="111" t="n"/>
-      <c r="D24" s="111" t="n"/>
-      <c r="E24" s="111" t="n"/>
-      <c r="F24" s="111" t="n"/>
-      <c r="G24" s="111" t="n"/>
-      <c r="H24" s="111" t="n"/>
-      <c r="I24" s="111" t="n"/>
-      <c r="J24" s="111" t="n"/>
-      <c r="K24" s="111" t="n"/>
-      <c r="L24" s="111" t="n"/>
-      <c r="M24" s="111" t="n"/>
-      <c r="N24" s="111" t="n"/>
-      <c r="O24" s="111" t="n"/>
-    </row>
-    <row r="25" ht="52.05" customHeight="1" s="72">
-      <c r="A25" s="109" t="inlineStr">
-        <is>
-          <t>DEFERRED TO END OF PHASE A -- pending direct restaurant-owner research into real procurement/approval workflow</t>
+      <c r="N25" s="90" t="n"/>
+      <c r="O25" s="90" t="inlineStr">
+        <is>
+          <t>CRUD + status-transition unit tests; plan output includes action_queue section</t>
         </is>
       </c>
     </row>
@@ -18610,34 +18614,30 @@
           <t>P6-A22</t>
         </is>
       </c>
-      <c r="B26" s="98" t="inlineStr">
-        <is>
-          <t>feature/action-queue</t>
-        </is>
-      </c>
+      <c r="B26" s="69" t="n"/>
       <c r="C26" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D26" s="90" t="inlineStr">
         <is>
-          <t>ActionQueueService + action_queue table</t>
+          <t>Action Queue UI</t>
         </is>
       </c>
       <c r="E26" s="90" t="inlineStr">
         <is>
-          <t>New table (org_id, action_type [AUTO/APPROVE_REQUIRED/RECOMMENDATION], payload jsonb, status [PENDING/APPROVED/EXECUTED/REJECTED/EXPIRED], approved_by, executed_at, error). ActionQueueService CRUD + status transitions. Plan output gains an action_queue section in the API response. Foundational -- every other agentic task below (workflow triggers, dynamic pricing, executors, trust-ladder) writes into this same table rather than inventing its own approval mechanism. DEFERRED to end of Phase A -- its main real-world value (approving reorder suggestions) is exactly the workflow that needs real restaurant-owner input first; building the approval UX before that research risks designing around the wrong assumptions.</t>
+          <t>Approve/reject list with type badges, Instamart cart-preview modal before approving checkout, procurement tracker (placed orders, status, ETA) in the inventory panel.</t>
         </is>
       </c>
       <c r="F26" s="90" t="inlineStr">
         <is>
-          <t>feat: ActionQueueService + action_queue table -- 3-tier action model with approval lifecycle</t>
+          <t>feat: Action Queue UI -- approve/reject with cart preview, procurement tracker</t>
         </is>
       </c>
       <c r="G26" s="90" t="inlineStr">
         <is>
-          <t>docs/ACTION_QUEUE.md (new), docs/APIS.md, docs/DECISIONS.md</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H26" s="108" t="inlineStr">
@@ -18660,10 +18660,14 @@
       <c r="M26" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="90" t="n"/>
+      <c r="N26" s="90" t="inlineStr">
+        <is>
+          <t>P6-A21</t>
+        </is>
+      </c>
       <c r="O26" s="90" t="inlineStr">
         <is>
-          <t>CRUD + status-transition unit tests; plan output includes action_queue section</t>
+          <t>typecheck clean; manual verification against live action_queue data</t>
         </is>
       </c>
     </row>
@@ -18673,30 +18677,34 @@
           <t>P6-A23</t>
         </is>
       </c>
-      <c r="B27" s="69" t="n"/>
+      <c r="B27" s="98" t="inlineStr">
+        <is>
+          <t>feature/agentic-automation</t>
+        </is>
+      </c>
       <c r="C27" s="90" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D27" s="90" t="inlineStr">
         <is>
-          <t>Action Queue UI</t>
+          <t>Workflow trigger engine (scoped: 2-3 built-in triggers, not a user-defined builder)</t>
         </is>
       </c>
       <c r="E27" s="90" t="inlineStr">
         <is>
-          <t>Approve/reject list with type badges, Instamart cart-preview modal before approving checkout, procurement tracker (placed orders, status, ETA) in the inventory panel.</t>
+          <t>A small WorkflowEngine evaluating built-in conditions after each planning run and auto-creating action_queue rows. Ships with 2-3 real triggers to start: (1) 2+ critical shortages found -&gt; queue an urgent restock action, (2) tonight_busy + 2+ competitor Dineout deals live -&gt; queue a pricing/promo review action. Deliberately NOT the full owner-defined trigger/condition/action builder from the original workflow-system idea -- that's a much bigger UI/DB investment for marginal demo value beyond just having the triggers exist.</t>
         </is>
       </c>
       <c r="F27" s="90" t="inlineStr">
         <is>
-          <t>feat: Action Queue UI -- approve/reject with cart preview, procurement tracker</t>
+          <t>feat: workflow trigger engine -- built-in triggers auto-queue actions post-planning-run</t>
         </is>
       </c>
       <c r="G27" s="90" t="inlineStr">
         <is>
-          <t>None (frontend only)</t>
+          <t>docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H27" s="108" t="inlineStr">
@@ -18706,7 +18714,7 @@
       </c>
       <c r="I27" s="89" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J27" s="89" t="inlineStr">
@@ -18721,12 +18729,12 @@
       </c>
       <c r="N27" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O27" s="90" t="inlineStr">
         <is>
-          <t>typecheck clean; manual verification against live action_queue data</t>
+          <t>each trigger condition fires correctly and produces the right queued action</t>
         </is>
       </c>
     </row>
@@ -18736,34 +18744,30 @@
           <t>P6-A24</t>
         </is>
       </c>
-      <c r="B28" s="98" t="inlineStr">
-        <is>
-          <t>feature/agentic-automation</t>
-        </is>
-      </c>
+      <c r="B28" s="69" t="n"/>
       <c r="C28" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D28" s="90" t="inlineStr">
         <is>
-          <t>Workflow trigger engine (scoped: 2-3 built-in triggers, not a user-defined builder)</t>
+          <t>Trust-ladder mechanic on the Action Queue</t>
         </is>
       </c>
       <c r="E28" s="90" t="inlineStr">
         <is>
-          <t>A small WorkflowEngine evaluating built-in conditions after each planning run and auto-creating action_queue rows. Ships with 2-3 real triggers to start: (1) 2+ critical shortages found -&gt; queue an urgent restock action, (2) tonight_busy + 2+ competitor Dineout deals live -&gt; queue a pricing/promo review action. Deliberately NOT the full owner-defined trigger/condition/action builder from the original workflow-system idea -- that's a much bigger UI/DB investment for marginal demo value beyond just having the triggers exist.</t>
+          <t>Track consecutive unedited approvals per action_type. After N consecutive approvals (default 3) of the same type, offer 'always do this automatically' -- promotes future instances of that action_type straight to AUTO tier for that org. Makes 'autonomous' a visible, explainable mechanic rather than a claim.</t>
         </is>
       </c>
       <c r="F28" s="90" t="inlineStr">
         <is>
-          <t>feat: workflow trigger engine -- built-in triggers auto-queue actions post-planning-run</t>
+          <t>feat: trust-ladder -- auto-promote repeatedly-approved action types to AUTO tier</t>
         </is>
       </c>
       <c r="G28" s="90" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md</t>
+          <t>docs/ACTION_QUEUE.md</t>
         </is>
       </c>
       <c r="H28" s="108" t="inlineStr">
@@ -18773,7 +18777,7 @@
       </c>
       <c r="I28" s="89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J28" s="89" t="inlineStr">
@@ -18788,12 +18792,12 @@
       </c>
       <c r="N28" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O28" s="90" t="inlineStr">
         <is>
-          <t>each trigger condition fires correctly and produces the right queued action</t>
+          <t>N consecutive approvals triggers promotion prompt; promoted type skips approval next time</t>
         </is>
       </c>
     </row>
@@ -18803,30 +18807,34 @@
           <t>P6-A25</t>
         </is>
       </c>
-      <c r="B29" s="69" t="n"/>
+      <c r="B29" s="98" t="inlineStr">
+        <is>
+          <t>feature/dynamic-pricing</t>
+        </is>
+      </c>
       <c r="C29" s="90" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D29" s="90" t="inlineStr">
         <is>
-          <t>Trust-ladder mechanic on the Action Queue</t>
+          <t>Dynamic pricing engine -- PriceChangeProposal (internal menu only)</t>
         </is>
       </c>
       <c r="E29" s="90" t="inlineStr">
         <is>
-          <t>Track consecutive unedited approvals per action_type. After N consecutive approvals (default 3) of the same type, offer 'always do this automatically' -- promotes future instances of that action_type straight to AUTO tier for that org. Makes 'autonomous' a visible, explainable mechanic rather than a claim.</t>
+          <t>New PriceChangeProposal model (item, current_price, suggested_price, reason, source, created_at). Computed from existing category_pricing/positioning data already in CompetitorEnricher. Surfaces as a new action_type in the Action Queue -- approving it updates your own MenuItem.price. Explicitly scoped to internal-only; does NOT attempt to sync price changes out to live Swiggy/Zomato listings (that needs Partner API access we don't have).</t>
         </is>
       </c>
       <c r="F29" s="90" t="inlineStr">
         <is>
-          <t>feat: trust-ladder -- auto-promote repeatedly-approved action types to AUTO tier</t>
+          <t>feat: dynamic pricing engine -- competitor-data-driven price suggestions via the Action Queue</t>
         </is>
       </c>
       <c r="G29" s="90" t="inlineStr">
         <is>
-          <t>docs/ACTION_QUEUE.md</t>
+          <t>docs/AGENTS.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H29" s="108" t="inlineStr">
@@ -18836,7 +18844,7 @@
       </c>
       <c r="I29" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J29" s="89" t="inlineStr">
@@ -18851,12 +18859,12 @@
       </c>
       <c r="N29" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O29" s="90" t="inlineStr">
         <is>
-          <t>N consecutive approvals triggers promotion prompt; promoted type skips approval next time</t>
+          <t>suggestion computed correctly from category_pricing gap; approving updates MenuItem.price; PriceChangeProposal row persists as an audit trail</t>
         </is>
       </c>
     </row>
@@ -18866,11 +18874,7 @@
           <t>P6-A26</t>
         </is>
       </c>
-      <c r="B30" s="98" t="inlineStr">
-        <is>
-          <t>feature/dynamic-pricing</t>
-        </is>
-      </c>
+      <c r="B30" s="69" t="n"/>
       <c r="C30" s="90" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -18878,22 +18882,22 @@
       </c>
       <c r="D30" s="90" t="inlineStr">
         <is>
-          <t>Dynamic pricing engine -- PriceChangeProposal (internal menu only)</t>
+          <t>Outcome / recommendation-learning memory</t>
         </is>
       </c>
       <c r="E30" s="90" t="inlineStr">
         <is>
-          <t>New PriceChangeProposal model (item, current_price, suggested_price, reason, source, created_at). Computed from existing category_pricing/positioning data already in CompetitorEnricher. Surfaces as a new action_type in the Action Queue -- approving it updates your own MenuItem.price. Explicitly scoped to internal-only; does NOT attempt to sync price changes out to live Swiggy/Zomato listings (that needs Partner API access we don't have).</t>
+          <t>Extend the existing Qdrant-backed cross-session memory pattern (P6-S09) to track whether past actions/recommendations actually worked (e.g. did an approved price change move margin next week? did an approved restock prevent a stockout?). Feed this back into future confidence scoring on similar suggestions.</t>
         </is>
       </c>
       <c r="F30" s="90" t="inlineStr">
         <is>
-          <t>feat: dynamic pricing engine -- competitor-data-driven price suggestions via the Action Queue</t>
+          <t>feat: outcome-learning memory -- track whether past AI actions worked, feed back into future confidence</t>
         </is>
       </c>
       <c r="G30" s="90" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md, CLAUDE.md</t>
+          <t>docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H30" s="108" t="inlineStr">
@@ -18903,7 +18907,7 @@
       </c>
       <c r="I30" s="89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J30" s="89" t="inlineStr">
@@ -18918,12 +18922,12 @@
       </c>
       <c r="N30" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A21, P6-A25</t>
         </is>
       </c>
       <c r="O30" s="90" t="inlineStr">
         <is>
-          <t>suggestion computed correctly from category_pricing gap; approving updates MenuItem.price; PriceChangeProposal row persists as an audit trail</t>
+          <t>outcome recorded correctly against the originating action; confidence score shifts on repeat suggestion of the same type after a bad outcome</t>
         </is>
       </c>
     </row>
@@ -18933,7 +18937,11 @@
           <t>P6-A27</t>
         </is>
       </c>
-      <c r="B31" s="69" t="n"/>
+      <c r="B31" s="98" t="inlineStr">
+        <is>
+          <t>feature/procurement-dineout-executors</t>
+        </is>
+      </c>
       <c r="C31" s="90" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -18941,22 +18949,22 @@
       </c>
       <c r="D31" s="90" t="inlineStr">
         <is>
-          <t>Outcome / recommendation-learning memory</t>
+          <t>ProcurementExecutor -- full flow, mocked final checkout call</t>
         </is>
       </c>
       <c r="E31" s="90" t="inlineStr">
         <is>
-          <t>Extend the existing Qdrant-backed cross-session memory pattern (P6-S09) to track whether past actions/recommendations actually worked (e.g. did an approved price change move margin next week? did an approved restock prevent a stockout?). Feed this back into future confidence scoring on similar suggestions.</t>
+          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A30.</t>
         </is>
       </c>
       <c r="F31" s="90" t="inlineStr">
         <is>
-          <t>feat: outcome-learning memory -- track whether past AI actions worked, feed back into future confidence</t>
+          <t>feat: ProcurementExecutor -- full approval-gated Instamart flow, checkout call mocked pending staging creds</t>
         </is>
       </c>
       <c r="G31" s="90" t="inlineStr">
         <is>
-          <t>docs/ARCHITECTURE.md</t>
+          <t>docs/ACTION_QUEUE.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H31" s="108" t="inlineStr">
@@ -18966,7 +18974,7 @@
       </c>
       <c r="I31" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J31" s="89" t="inlineStr">
@@ -18981,12 +18989,12 @@
       </c>
       <c r="N31" s="90" t="inlineStr">
         <is>
-          <t>P6-A22, P6-A26</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O31" s="90" t="inlineStr">
         <is>
-          <t>outcome recorded correctly against the originating action; confidence score shifts on repeat suggestion of the same type after a bad outcome</t>
+          <t>full flow test with mocked checkout; interrupt() pauses correctly; procurement_orders row created with a clear 'simulated' flag</t>
         </is>
       </c>
     </row>
@@ -18996,11 +19004,7 @@
           <t>P6-A28</t>
         </is>
       </c>
-      <c r="B32" s="98" t="inlineStr">
-        <is>
-          <t>feature/procurement-dineout-executors</t>
-        </is>
-      </c>
+      <c r="B32" s="69" t="n"/>
       <c r="C32" s="90" t="inlineStr">
         <is>
           <t>Agents</t>
@@ -19008,22 +19012,22 @@
       </c>
       <c r="D32" s="90" t="inlineStr">
         <is>
-          <t>ProcurementExecutor -- full flow, mocked final checkout call</t>
+          <t>DineoutExecutor -- full flow, mocked final book_table call</t>
         </is>
       </c>
       <c r="E32" s="90" t="inlineStr">
         <is>
-          <t>Full update_cart -&gt; get_cart -&gt; LangGraph interrupt() -&gt; owner approval (via Action Queue) -&gt; checkout flow, built completely end-to-end. The actual final checkout() call is stubbed/mocked, clearly labeled 'awaiting Swiggy staging creds' -- everything else (cart building, pricing, approval gate, procurement_orders row creation) is real. Swapping the mock for a real call is Phase B's entire scope for this task. DEFERRED to end of Phase A pending direct restaurant-owner research into real procurement workflow (bulk orders, WhatsApp/phone to local vendors) -- see P6-A31.</t>
+          <t>Same pattern as P6-A23 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
         </is>
       </c>
       <c r="F32" s="90" t="inlineStr">
         <is>
-          <t>feat: ProcurementExecutor -- full approval-gated Instamart flow, checkout call mocked pending staging creds</t>
+          <t>feat: DineoutExecutor -- full approval-gated Dineout booking flow, book_table call mocked pending staging creds</t>
         </is>
       </c>
       <c r="G32" s="90" t="inlineStr">
         <is>
-          <t>docs/ACTION_QUEUE.md, CLAUDE.md</t>
+          <t>docs/ACTION_QUEUE.md</t>
         </is>
       </c>
       <c r="H32" s="108" t="inlineStr">
@@ -19033,7 +19037,7 @@
       </c>
       <c r="I32" s="89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J32" s="89" t="inlineStr">
@@ -19048,12 +19052,12 @@
       </c>
       <c r="N32" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A21, P6-A27</t>
         </is>
       </c>
       <c r="O32" s="90" t="inlineStr">
         <is>
-          <t>full flow test with mocked checkout; interrupt() pauses correctly; procurement_orders row created with a clear 'simulated' flag</t>
+          <t>full flow test with mocked book_table; reservations row created with a clear 'simulated' flag</t>
         </is>
       </c>
     </row>
@@ -19063,30 +19067,34 @@
           <t>P6-A29</t>
         </is>
       </c>
-      <c r="B33" s="69" t="n"/>
+      <c r="B33" s="98" t="inlineStr">
+        <is>
+          <t>feature/recipe-vendor-foundations</t>
+        </is>
+      </c>
       <c r="C33" s="90" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D33" s="90" t="inlineStr">
         <is>
-          <t>DineoutExecutor -- full flow, mocked final book_table call</t>
+          <t>Recipe + RecipeIngredient model</t>
         </is>
       </c>
       <c r="E33" s="90" t="inlineStr">
         <is>
-          <t>Same pattern as P6-A24 for Dineout: create_cart -&gt; book_table, approval-gated via Action Queue, real logic throughout except the final book_table() call is mocked pending staging creds.</t>
+          <t>New Recipe (menu_item_id) + RecipeIngredient (recipe_id, ingredient, quantity, unit) tables. Bridges MenuItem and inventory -- unlocks live-computed cost_price (from real ingredient prices) instead of manual entry, and real per-dish inventory depletion instead of aggregate-only shortage tracking. DEFERRED to end of Phase A alongside the rest of the procurement/Action Queue cluster, pending direct restaurant-owner research into how real procurement actually works.</t>
         </is>
       </c>
       <c r="F33" s="90" t="inlineStr">
         <is>
-          <t>feat: DineoutExecutor -- full approval-gated Dineout booking flow, book_table call mocked pending staging creds</t>
+          <t>feat: Recipe + RecipeIngredient models -- dish-to-ingredient yield mapping</t>
         </is>
       </c>
       <c r="G33" s="90" t="inlineStr">
         <is>
-          <t>docs/ACTION_QUEUE.md</t>
+          <t>docs/DATA_MODEL.md</t>
         </is>
       </c>
       <c r="H33" s="108" t="inlineStr">
@@ -19096,7 +19104,7 @@
       </c>
       <c r="I33" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J33" s="89" t="inlineStr">
@@ -19109,14 +19117,10 @@
       <c r="M33" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="90" t="inlineStr">
-        <is>
-          <t>P6-A22, P6-A28</t>
-        </is>
-      </c>
+      <c r="N33" s="90" t="n"/>
       <c r="O33" s="90" t="inlineStr">
         <is>
-          <t>full flow test with mocked book_table; reservations row created with a clear 'simulated' flag</t>
+          <t>recipe costing test (sum of ingredient costs matches computed cost_price); depletion test (a sale reduces linked ingredient stock by the right amount)</t>
         </is>
       </c>
     </row>
@@ -19126,11 +19130,7 @@
           <t>P6-A30</t>
         </is>
       </c>
-      <c r="B34" s="98" t="inlineStr">
-        <is>
-          <t>feature/recipe-vendor-foundations</t>
-        </is>
-      </c>
+      <c r="B34" s="69" t="n"/>
       <c r="C34" s="90" t="inlineStr">
         <is>
           <t>Infra</t>
@@ -19138,17 +19138,17 @@
       </c>
       <c r="D34" s="90" t="inlineStr">
         <is>
-          <t>Recipe + RecipeIngredient model</t>
+          <t>Vendor/Supplier model</t>
         </is>
       </c>
       <c r="E34" s="90" t="inlineStr">
         <is>
-          <t>New Recipe (menu_item_id) + RecipeIngredient (recipe_id, ingredient, quantity, unit) tables. Bridges MenuItem and inventory -- unlocks live-computed cost_price (from real ingredient prices) instead of manual entry, and real per-dish inventory depletion instead of aggregate-only shortage tracking. DEFERRED to end of Phase A alongside the rest of the procurement/Action Queue cluster, pending direct restaurant-owner research into how real procurement actually works.</t>
+          <t>New Vendor model (name, category, is_online, contact) + VendorPriceQuote (vendor_id, ingredient, price, quoted_at). Instamart becomes one Vendor among several (an 'online' vendor with live API pricing); local mandi/wholesale vendors become trackable entities with manually-entered or periodically-surveyed prices. Scoped as tracking/comparison only, not a marketplace. DEFERRED to end of Phase A -- exact procurement medium (Instamart API vs a WhatsApp-dispatch message to a local vendor vs other) intentionally left open pending direct conversation with a real restaurant owner/manager about their actual ordering process, before committing to a design.</t>
         </is>
       </c>
       <c r="F34" s="90" t="inlineStr">
         <is>
-          <t>feat: Recipe + RecipeIngredient models -- dish-to-ingredient yield mapping</t>
+          <t>feat: Vendor/Supplier model -- Instamart becomes one vendor among many, not the only source</t>
         </is>
       </c>
       <c r="G34" s="90" t="inlineStr">
@@ -19163,7 +19163,7 @@
       </c>
       <c r="I34" s="89" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J34" s="89" t="inlineStr">
@@ -19176,10 +19176,14 @@
       <c r="M34" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="90" t="n"/>
+      <c r="N34" s="90" t="inlineStr">
+        <is>
+          <t>P6-A29</t>
+        </is>
+      </c>
       <c r="O34" s="90" t="inlineStr">
         <is>
-          <t>recipe costing test (sum of ingredient costs matches computed cost_price); depletion test (a sale reduces linked ingredient stock by the right amount)</t>
+          <t>vendor price comparison query returns correct cheapest-vendor-per-ingredient</t>
         </is>
       </c>
     </row>
@@ -19189,30 +19193,34 @@
           <t>P6-A31</t>
         </is>
       </c>
-      <c r="B35" s="69" t="n"/>
+      <c r="B35" s="98" t="inlineStr">
+        <is>
+          <t>feature/mcp-expansion</t>
+        </is>
+      </c>
       <c r="C35" s="90" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D35" s="90" t="inlineStr">
         <is>
-          <t>Vendor/Supplier model</t>
+          <t>Internal MCP server -- get_market_brief / get_action_queue / approve_action</t>
         </is>
       </c>
       <c r="E35" s="90" t="inlineStr">
         <is>
-          <t>New Vendor model (name, category, is_online, contact) + VendorPriceQuote (vendor_id, ingredient, price, quoted_at). Instamart becomes one Vendor among several (an 'online' vendor with live API pricing); local mandi/wholesale vendors become trackable entities with manually-entered or periodically-surveyed prices. Scoped as tracking/comparison only, not a marketplace. DEFERRED to end of Phase A -- exact procurement medium (Instamart API vs a WhatsApp-dispatch message to a local vendor vs other) intentionally left open pending direct conversation with a real restaurant owner/manager about their actual ordering process, before committing to a design.</t>
+          <t>3 new tools on CortexKitchen's own MCP server (mcp_server.py), JWT-authenticated, calling MarketIntelService and ActionQueueService live. Lets an owner ask Claude Desktop directly about their restaurant and approve actions from there.</t>
         </is>
       </c>
       <c r="F35" s="90" t="inlineStr">
         <is>
-          <t>feat: Vendor/Supplier model -- Instamart becomes one vendor among many, not the only source</t>
+          <t>feat: 3 new MCP tools -- get_market_brief, get_action_queue, approve_action</t>
         </is>
       </c>
       <c r="G35" s="90" t="inlineStr">
         <is>
-          <t>docs/DATA_MODEL.md</t>
+          <t>docs/APIS.md, docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H35" s="108" t="inlineStr">
@@ -19237,12 +19245,12 @@
       </c>
       <c r="N35" s="90" t="inlineStr">
         <is>
-          <t>P6-A30</t>
+          <t>P6-A21</t>
         </is>
       </c>
       <c r="O35" s="90" t="inlineStr">
         <is>
-          <t>vendor price comparison query returns correct cheapest-vendor-per-ingredient</t>
+          <t>all 3 tools smoke-tested in Claude Desktop; approve_action triggers the same approval path as the web UI; JWT enforced</t>
         </is>
       </c>
     </row>
@@ -19252,11 +19260,7 @@
           <t>P6-A32</t>
         </is>
       </c>
-      <c r="B36" s="98" t="inlineStr">
-        <is>
-          <t>feature/mcp-expansion</t>
-        </is>
-      </c>
+      <c r="B36" s="69" t="n"/>
       <c r="C36" s="90" t="inlineStr">
         <is>
           <t>Product</t>
@@ -19264,22 +19268,22 @@
       </c>
       <c r="D36" s="90" t="inlineStr">
         <is>
-          <t>Internal MCP server -- get_market_brief / get_action_queue / approve_action</t>
+          <t>Internal MCP server -- expand further (menu insights, forecast, what-if)</t>
         </is>
       </c>
       <c r="E36" s="90" t="inlineStr">
         <is>
-          <t>3 new tools on CortexKitchen's own MCP server (mcp_server.py), JWT-authenticated, calling MarketIntelService and ActionQueueService live. Lets an owner ask Claude Desktop directly about their restaurant and approve actions from there.</t>
+          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A30 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
         </is>
       </c>
       <c r="F36" s="90" t="inlineStr">
         <is>
-          <t>feat: 3 new MCP tools -- get_market_brief, get_action_queue, approve_action</t>
+          <t>feat: expand internal MCP server -- menu insights, forecast, what-if simulator as tools</t>
         </is>
       </c>
       <c r="G36" s="90" t="inlineStr">
         <is>
-          <t>docs/APIS.md, docs/ARCHITECTURE.md</t>
+          <t>docs/APIS.md</t>
         </is>
       </c>
       <c r="H36" s="108" t="inlineStr">
@@ -19289,7 +19293,7 @@
       </c>
       <c r="I36" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J36" s="89" t="inlineStr">
@@ -19304,12 +19308,12 @@
       </c>
       <c r="N36" s="90" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A31</t>
         </is>
       </c>
       <c r="O36" s="90" t="inlineStr">
         <is>
-          <t>all 3 tools smoke-tested in Claude Desktop; approve_action triggers the same approval path as the web UI; JWT enforced</t>
+          <t>each new tool smoke-tested in Claude Desktop; correct data returned matching the equivalent API endpoint</t>
         </is>
       </c>
     </row>
@@ -19319,30 +19323,34 @@
           <t>P6-A33</t>
         </is>
       </c>
-      <c r="B37" s="69" t="n"/>
+      <c r="B37" s="98" t="inlineStr">
+        <is>
+          <t>feature/brief-page</t>
+        </is>
+      </c>
       <c r="C37" s="90" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D37" s="90" t="inlineStr">
         <is>
-          <t>Internal MCP server -- expand further (menu insights, forecast, what-if)</t>
+          <t>/brief page</t>
         </is>
       </c>
       <c r="E37" s="90" t="inlineStr">
         <is>
-          <t>Wrap additional existing services as MCP tools beyond the 3 in P6-A31 -- menu insights, demand forecast, and the Phase-5 what-if simulator. Cheap since the service layer already exists; positions CortexKitchen as a general AI-accessible restaurant data layer, not just 3 utility tools.</t>
+          <t>Daily morning briefing -- overnight performance, today's forecast vs yesterday, top 3 action priorities, market snapshot. Single-screen showcase of the whole system's intelligence.</t>
         </is>
       </c>
       <c r="F37" s="90" t="inlineStr">
         <is>
-          <t>feat: expand internal MCP server -- menu insights, forecast, what-if simulator as tools</t>
+          <t>feat: /brief page -- daily morning operational briefing</t>
         </is>
       </c>
       <c r="G37" s="90" t="inlineStr">
         <is>
-          <t>docs/APIS.md</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H37" s="108" t="inlineStr">
@@ -19352,7 +19360,7 @@
       </c>
       <c r="I37" s="89" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J37" s="89" t="inlineStr">
@@ -19367,12 +19375,12 @@
       </c>
       <c r="N37" s="90" t="inlineStr">
         <is>
-          <t>P6-A32</t>
+          <t>P6-A22</t>
         </is>
       </c>
       <c r="O37" s="90" t="inlineStr">
         <is>
-          <t>each new tool smoke-tested in Claude Desktop; correct data returned matching the equivalent API endpoint</t>
+          <t>manual verification</t>
         </is>
       </c>
     </row>
@@ -19382,34 +19390,30 @@
           <t>P6-A34</t>
         </is>
       </c>
-      <c r="B38" s="98" t="inlineStr">
-        <is>
-          <t>feature/brief-page</t>
-        </is>
-      </c>
+      <c r="B38" s="98" t="n"/>
       <c r="C38" s="90" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="D38" s="90" t="inlineStr">
         <is>
-          <t>/brief page</t>
+          <t>Post-Phase-A documentation, test, CI, observability, and eval refresh</t>
         </is>
       </c>
       <c r="E38" s="90" t="inlineStr">
         <is>
-          <t>Daily morning briefing -- overnight performance, today's forecast vs yesterday, top 3 action priorities, market snapshot. Single-screen showcase of the whole system's intelligence.</t>
+          <t>Once Phase A ships, a lot of new surface area will have landed at once -- Action Queue, workflow triggers, the anomaly agent, both executors, new connectors (Zomato stub, reviews), new data models (Recipe, Vendor, Expense, Obligation), MCP expansion. Do a full pass rather than letting docs drift: update every docs/*.md file, CLAUDE.md, README, and any screenshots referenced in docs to reflect what actually shipped. Audit test coverage for every new service/model added in Phase A -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (anomaly diagnoses, dynamic pricing suggestions), since the existing eval sets predate all of this and won't catch regressions in it.</t>
         </is>
       </c>
       <c r="F38" s="90" t="inlineStr">
         <is>
-          <t>feat: /brief page -- daily morning operational briefing</t>
+          <t>docs: full documentation, test-coverage, CI, and eval refresh after the Phase A agentic core ships</t>
         </is>
       </c>
       <c r="G38" s="90" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>All docs/*.md, CLAUDE.md, README.md</t>
         </is>
       </c>
       <c r="H38" s="108" t="inlineStr">
@@ -19419,7 +19423,7 @@
       </c>
       <c r="I38" s="89" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J38" s="89" t="inlineStr">
@@ -19434,96 +19438,49 @@
       </c>
       <c r="N38" s="90" t="inlineStr">
         <is>
-          <t>P6-A23</t>
+          <t>All P6-A tasks</t>
         </is>
       </c>
       <c r="O38" s="90" t="inlineStr">
         <is>
-          <t>manual verification</t>
+          <t>Every new service/model has test coverage; CI includes all new test files; RAGAS/DeepEval sets include at least one case per new agentic behavior; docs/screenshots match shipped behavior</t>
         </is>
       </c>
     </row>
     <row r="39" ht="171.6" customHeight="1" s="72">
-      <c r="A39" s="65" t="inlineStr">
-        <is>
-          <t>P6-A35</t>
-        </is>
-      </c>
-      <c r="B39" s="98" t="n"/>
-      <c r="C39" s="90" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D39" s="90" t="inlineStr">
-        <is>
-          <t>Post-Phase-A documentation, test, CI, observability, and eval refresh</t>
-        </is>
-      </c>
-      <c r="E39" s="90" t="inlineStr">
-        <is>
-          <t>Once Phase A ships, a lot of new surface area will have landed at once -- Action Queue, workflow triggers, the anomaly agent, both executors, new connectors (Zomato stub, reviews), new data models (Recipe, Vendor, Expense, Obligation), MCP expansion. Do a full pass rather than letting docs drift: update every docs/*.md file, CLAUDE.md, README, and any screenshots referenced in docs to reflect what actually shipped. Audit test coverage for every new service/model added in Phase A -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (anomaly diagnoses, dynamic pricing suggestions), since the existing eval sets predate all of this and won't catch regressions in it.</t>
-        </is>
-      </c>
-      <c r="F39" s="90" t="inlineStr">
-        <is>
-          <t>docs: full documentation, test-coverage, CI, and eval refresh after the Phase A agentic core ships</t>
-        </is>
-      </c>
-      <c r="G39" s="90" t="inlineStr">
-        <is>
-          <t>All docs/*.md, CLAUDE.md, README.md</t>
-        </is>
-      </c>
-      <c r="H39" s="108" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I39" s="89" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J39" s="89" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K39" s="89" t="n"/>
-      <c r="L39" s="89" t="n"/>
-      <c r="M39" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="90" t="inlineStr">
-        <is>
-          <t>All P6-A tasks</t>
-        </is>
-      </c>
-      <c r="O39" s="90" t="inlineStr">
-        <is>
-          <t>Every new service/model has test coverage; CI includes all new test files; RAGAS/DeepEval sets include at least one case per new agentic behavior; docs/screenshots match shipped behavior</t>
-        </is>
-      </c>
+      <c r="A39" s="111" t="n"/>
+      <c r="B39" s="111" t="n"/>
+      <c r="C39" s="111" t="n"/>
+      <c r="D39" s="111" t="n"/>
+      <c r="E39" s="111" t="n"/>
+      <c r="F39" s="111" t="n"/>
+      <c r="G39" s="111" t="n"/>
+      <c r="H39" s="111" t="n"/>
+      <c r="I39" s="111" t="n"/>
+      <c r="J39" s="111" t="n"/>
+      <c r="K39" s="111" t="n"/>
+      <c r="L39" s="111" t="n"/>
+      <c r="M39" s="111" t="n"/>
+      <c r="N39" s="111" t="n"/>
+      <c r="O39" s="111" t="n"/>
     </row>
     <row r="40" ht="39.6" customHeight="1" s="72"/>
     <row r="41" ht="171.6" customHeight="1" s="72"/>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A25:O25"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B7:B8"/>
+  <mergeCells count="13">
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B33:B34"/>
     <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="A24:O24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -19536,7 +19493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="40.77734375" customWidth="1" style="72" min="1" max="1"/>
@@ -19673,7 +19630,7 @@
       </c>
       <c r="E4" s="62" t="inlineStr">
         <is>
-          <t>Phase A (P6-A28) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
+          <t>Phase A (P6-A27) already builds the full get_cart -&gt; update_cart -&gt; LangGraph interrupt() -&gt; owner approval -&gt; checkout flow end-to-end, with the final checkout() call mocked and labeled 'awaiting staging creds'. This task is just the swap: replace the mock with the real call. NON-IDEMPOTENT: on any 5xx from checkout, call get_orders before retrying -- never blind-retry. procurement_orders rows switch from a 'simulated' flag to real confirmed orders.</t>
         </is>
       </c>
       <c r="F4" s="62" t="inlineStr">
@@ -19708,7 +19665,7 @@
       </c>
       <c r="N4" s="62" t="inlineStr">
         <is>
-          <t>P6-A28, P6-S14</t>
+          <t>P6-A27, P6-S14</t>
         </is>
       </c>
       <c r="O4" s="62" t="inlineStr">
@@ -19757,7 +19714,7 @@
       </c>
       <c r="E6" s="62" t="inlineStr">
         <is>
-          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A29) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
+          <t>book_table in consumer MCP books a table AT another restaurant (a consumer action), not managing your own restaurant's Dineout presence -- that needs Swiggy Partner/Business API, a separate track from these creds. Phase A (P6-A28) already builds the full create_cart -&gt; book_table flow end-to-end with the final call mocked. This task swaps the mock for the real call, scoped to the consumer-booking use case only (e.g. mystery-dining a competitor for research).</t>
         </is>
       </c>
       <c r="F6" s="62" t="inlineStr">
@@ -19792,7 +19749,7 @@
       </c>
       <c r="N6" s="62" t="inlineStr">
         <is>
-          <t>P6-A29</t>
+          <t>P6-A28</t>
         </is>
       </c>
       <c r="O6" s="62" t="inlineStr">
@@ -19837,7 +19794,7 @@
       </c>
       <c r="E8" s="62" t="inlineStr">
         <is>
-          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A25) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
+          <t>Once P7-1/P7-2 prove reliable in production, extend the trust-ladder mechanic (P6-A24) to real money-touching actions -- e.g. auto-reorder a habitually-restocked ingredient without approval once trust is established.</t>
         </is>
       </c>
       <c r="F8" s="62" t="inlineStr">
@@ -19872,7 +19829,7 @@
       </c>
       <c r="N8" s="62" t="inlineStr">
         <is>
-          <t>P6-A25, P7-1, P7-2</t>
+          <t>P6-A24, P7-1, P7-2</t>
         </is>
       </c>
       <c r="O8" s="62" t="inlineStr">
@@ -20060,7 +20017,7 @@
       </c>
       <c r="N14" s="62" t="inlineStr">
         <is>
-          <t>P6-A20</t>
+          <t>P6-A19</t>
         </is>
       </c>
       <c r="O14" s="62" t="inlineStr">
@@ -20797,6 +20754,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="62" t="inlineStr">
         <is>
@@ -20864,12 +20822,83 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="110" t="inlineStr">
+        <is>
+          <t>BLOCKED -- needs a real restaurant (not seeded/synthetic data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="112" t="inlineStr">
+        <is>
+          <t>P7-15</t>
+        </is>
+      </c>
+      <c r="B42" s="112" t="inlineStr">
+        <is>
+          <t>feature/multi-platform-connectors</t>
+        </is>
+      </c>
+      <c r="C42" s="112" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="D42" s="112" t="inlineStr">
+        <is>
+          <t>Public review aggregation connectors (Google/Zomato reviews)</t>
+        </is>
+      </c>
+      <c r="E42" s="112" t="inlineStr">
+        <is>
+          <t>GoogleReviewsConnector / ZomatoReviewsConnector following the same BaseConnector pattern, pulling public review data (not internal complaints) into complaint_intelligence as an additional source type. Extends the Feedback model's source concept rather than inventing a parallel system. DEFERRED 2026-07-07 from Phase 6A -- unlike the Zomato stub connector (which only needed to prove the architecture, not pull real data), this task's entire value IS real review data. There is no real Google/Zomato business listing for this restaurant to pull reviews from yet, so even a demoable version isn't possible until a real restaurant customer exists. Revisit then.</t>
+        </is>
+      </c>
+      <c r="F42" s="112" t="inlineStr">
+        <is>
+          <t>feat: public review aggregation -- Google/Zomato reviews via BaseConnector pattern</t>
+        </is>
+      </c>
+      <c r="G42" s="112" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/CONNECTORS.md</t>
+        </is>
+      </c>
+      <c r="H42" s="112" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="I42" s="112" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J42" s="112" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K42" s="113" t="n"/>
+      <c r="L42" s="112" t="n"/>
+      <c r="M42" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="112" t="n"/>
+      <c r="O42" s="112" t="inlineStr">
+        <is>
+          <t>reviews ingested with correct source tag; complaint_intelligence node correctly surfaces public-review-sourced themes alongside internal ones</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A12:O12"/>
     <mergeCell ref="A20:O20"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A28:O28"/>
+    <mergeCell ref="A40:O40"/>
     <mergeCell ref="A18:O18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update progress tracker
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -1036,12 +1036,12 @@
     <row r="3" ht="14.4" customHeight="1" s="73">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Current: Phase 6 — 55 done (41 + P6-MI05-14). Next: P6-S32/F06 (action queue)</t>
+          <t>Current: Phase 6 -- 69 done (55 Phase 6 + 14 Phase 6A: A1-A13, A18). Next: P6-A14 (weather + holiday signals)</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>14 Swiggy tools live (search_menu confirmed non-viable, removed). Market intel: category pricing, positioning, deals, trends all shipped</t>
+          <t>Action Queue live with trust-ladder + WhatsApp vendor execution. MCP server (5 tools) + in-app chatbot both expose get_market_brief/get_action_queue/approve_action. Financial scorecard (real P&amp;L, health score) shipped.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1072,12 +1072,12 @@
     <row r="4" ht="14.4" customHeight="1" s="73">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Last done: P6-MI05-MI14 — market intel expansion + category-independent redesign + personal-data leak fix</t>
+          <t>Last done: P6-A13 -- Internal MCP server + in-app chatbot tools (get_market_brief, get_action_queue, approve_action)</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Design system, 11-node pipeline, enrichers, market/operations/connectors pages, full market intel expansion shipped</t>
+          <t>Both surfaces share ActionQueueService + action_execution_service.approve_and_execute so approval behaves identically from Claude Desktop, in-app chat, or the UI button. Live-verified against real demo org 2026-07-08.</t>
         </is>
       </c>
       <c r="C4" s="1" t="n"/>
@@ -1108,7 +1108,7 @@
     <row r="5" ht="14.4" customHeight="1" s="73">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Priority: S32/F06 (action queue) → S33/S34 → S36/F07/F08 → R01 → staging creds → P7</t>
+          <t>Priority: A14 (weather/holiday signals) -&gt; A15 (menu engineering UI) -&gt; A16 (Dineout chatbot tools) -&gt; A17 (structured outputs) -&gt; A19/A20 (eval datasets) -&gt; A21 (redesign) -&gt; A22 (voice) -&gt; A23 (docs refresh) -&gt; A24 (sync to main) -&gt; staging creds -&gt; P7</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1541,11 +1541,11 @@
         </is>
       </c>
       <c r="C16" s="18" t="n">
-        <v>0.6892</v>
+        <v>0.8734</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Swiggy-native restaurant OS: connector layer (Swiggy first, POS second), 11-node LangGraph pipeline, action queue with approval gates, 3 product modes (ops/brief/live), voice interface, 5 new frontend pages</t>
+          <t>Swiggy-native restaurant OS: connector layer, 11-node LangGraph pipeline, Action Queue with approval gates + trust ladder + WhatsApp execution, financial scorecard, MCP server + in-app chatbot tool parity, 5 new frontend pages</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: align tracker P6-A19 entry with actual work done
Original entry only described the plan. Updated to reflect what actually
shipped: the eazydiner finding (same category as zomato, removed alongside
it), the decision to keep code comments/docs as plain architectural framing
rather than legal clause citations, and verified test results (487 backend
tests, clean frontend typecheck) instead of just expected criteria.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -18425,7 +18425,7 @@
       </c>
       <c r="E19" s="70" t="inlineStr">
         <is>
-          <t>Delete the Zomato stub connector entirely -- confirmed via codebase audit this is more than a name in one file. Remove: apps/api/app/infrastructure/zomato/ (ZomatoConnector), its CAPABILITY_PROVIDERS entries in provider_registry.py (currently lists zomato alongside swiggy under 'competitor_pricing' and 'order_history' -- bad optics under clause 17 audit rights even though the connector never makes a live call), the Zomato card on the /connectors frontend page ("Import orders and customer reviews from Zomato" -- visible in any demo), and test_zomato_connector.py. Remove ConnectorType.zomato from infrastructure/db/models.py. Do NOT touch FeedbackSource.zomato (separate enum, same file) -- that's just a provenance tag for feedback that originated from a Zomato review, no live Zomato connection involved, legitimate to keep. Clause 6.1 of the signed Swiggy Integration Agreement bars partnering with any other food delivery/dining/quick-commerce platform for a similar solution -- mark P6-A5 as Removed in this tracker. The multi-provider architecture itself is NOT the compliance problem and stays intact -- BaseConnector, provider_registry.py's CAPABILITY_PROVIDERS pattern, and ConnectorType stay exactly as they are, already proven extensible by pos_square and google_reviews (neither is a food-delivery/dining/quick-commerce competitor, so both are unaffected). Only the one concrete entry naming an actual competing platform (zomato) is removed. base_connector.py's module docstring updated to state what the pattern may extend to going forward (POS systems, loyalty/rewards platforms, accounting/inventory tools, review aggregators, payment processors) and what it must not (any other food delivery/dining-out/quick-commerce platform, e.g. Zomato, EazyDiner, while clause 6.1 is in effect).</t>
+          <t>DONE on feature/compliance-fixes (commits 1cebdfa, d75dfbd). Deleted the Zomato stub connector entirely -- codebase audit found it was more than a name in one file: apps/api/app/infrastructure/zomato/ (ZomatoConnector) removed; provider_registry.py's CAPABILITY_PROVIDERS had zomato under 'competitor_pricing' and 'order_history', PLUS an eazydiner entry under 'reservation_data' found during the same audit (EazyDiner is Zomato's own dining-reservation vertical, same category, also just an unimplemented placeholder with no connector class) -- both removed, all four capability lists now read ['swiggy'] only. Removed the Zomato card from the /connectors frontend page and test_zomato_connector.py. Removed ConnectorType.zomato from infrastructure/db/models.py -- confirmed connector_type is a plain String(50) column, not a DB enum, so no Alembic migration was needed. Did NOT touch FeedbackSource.zomato (separate enum, same file) -- that's just a provenance tag for feedback that originated from a Zomato review, no live connection, legitimate to keep. The multi-provider architecture itself was never the problem and stays fully intact -- BaseConnector, provider_registry.py's pattern, and ConnectorType stay exactly as they are, already proven extensible by pos_square and google_reviews (neither is a food-delivery/dining/quick-commerce competitor). base_connector.py's docstring and provider_registry.py's comments were updated to state what the pattern extends to going forward (POS systems, loyalty/rewards platforms, accounting/inventory tools, review aggregators, payment processors) -- phrased as ordinary architectural framing ("kept single-provider for now"), not as legal/clause citations; that level of detail stays only in CLAUDE.md's dedicated compliance section, not scattered across code comments or public docs. docs/ARCHITECTURE.md, docs/DATA_MODEL.md, and docs/SWIGGY_INTEGRATION.md updated to match -- all three had stale code snippets/schema tables still listing zomato/eazydiner as live options. docs/DECISIONS.md deliberately left untouched -- it's a point-in-time ADR, not a current-state doc. scripts/seed_demo_data.py has an expense note "Swiggy/Zomato ad spend" -- left as-is, it's realistic demo financial data (a restaurant advertising on both platforms), not a technical Zomato connection; flagged to the user as a judgment call, not yet asked to change it.</t>
         </is>
       </c>
       <c r="F19" s="70" t="inlineStr">
@@ -18461,7 +18461,7 @@
       <c r="N19" s="70" t="n"/>
       <c r="O19" s="70" t="inlineStr">
         <is>
-          <t>grep -ri zomato across apps/ returns zero hits except FeedbackSource.zomato (intentionally kept); no ConnectorType.zomato in models.py; provider_registry.py competitor_pricing/order_history lists contain only swiggy; /connectors page has no Zomato card; CI passes</t>
+          <t>VERIFIED: grep -ri "zomato|eazydiner" across apps/ returns only FeedbackSource.zomato (models.py, intentionally kept) and the explanatory mentions in base_connector.py's docstring; provider_registry.py's four CAPABILITY_PROVIDERS lists contain only 'swiggy'; /connectors page has no Zomato card; test_zomato_connector.py deleted, one stray "zomato" example string in test_connector_repository.py swapped to "pos_square"; 487 backend tests pass; frontend typechecks clean (npx tsc --noEmit, zero errors).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: expand Phase 6A with live-intelligence + scenario-overhaul tasks
Replaces the narrow P6-A21 (weather + holiday signals only) with six tasks
(P6-A21-A26) on one combined branch feature/live-intelligence-signals:
weather/holidays, industry trends (RSS-only, no paid API), regulatory
alerts (FSSAI public notices), unifying all four into the existing
market_intel_node instead of a new graph node, a scenario-selection
overhaul (natural language + dynamic profiles alongside the 4 hardcoded
presets), and a conditional validation checkpoint on action-item
specificity. Renumbers P6-A22-A29 to P6-A27-A34 to keep IDs sequential;
fixes the procurement loop's dependency (now P6-A24, not P6-A21, since it
needs signals actually wired in) and every stale cross-reference to the old
numbering across the Dashboard, Phase 6B, and Staging Creds sheets.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -569,7 +569,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -944,6 +944,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1272,7 +1284,7 @@
     <row r="3" ht="14.4" customHeight="1" s="90">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Current: Phase 6A (restaurant OS). Phase 6B (guest concierge) starts after 6A syncs to main.</t>
+          <t>Current: Phase 6A (restaurant OS) -- compliance batch DONE (P6-A19, P6-A20). Live-intelligence + scenario overhaul next (P6-A21-A26). Phase 6B (guest concierge) starts after 6A syncs to main.</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1308,7 +1320,7 @@
     <row r="4" ht="14.4" customHeight="1" s="90">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Phase 6B: guest concierge — 4 tasks before staging creds, 2 blocked, then demo-ready.</t>
+          <t>Phase 6B: guest concierge -- 9 tasks (P6-B1-B9), gated on P6-B1 (Swiggy written consent, clause 2.1v) before any code.</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -1344,7 +1356,7 @@
     <row r="5" ht="14.4" customHeight="1" s="90">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Staging creds unlock: Instamart checkout (P6-A32, P6-B08) + Dineout book_table (P6-A33, P6-B07)</t>
+          <t>Staging creds unlock: Instamart checkout (within P6-A27 procurement loop; also P6-B7 Guest Concierge) + Dineout book_table (P6-B5 Guest Concierge).</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1380,7 +1392,7 @@
     <row r="6" ht="14.4" customHeight="1" s="90">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Compliance: P6-A26 (remove Zomato stub) + P6-A25 (anonymise market intel) — do these FIRST</t>
+          <t>Compliance: P6-A19 (remove Zomato stub) + P6-A20 (anonymise market intel) -- DONE, merged to dev.</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -17334,7 +17346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="90" min="1" max="1"/>
@@ -18534,636 +18546,926 @@
     </row>
     <row r="21" ht="7.95" customHeight="1" s="90"/>
     <row r="22" ht="18" customHeight="1" s="90">
-      <c r="A22" s="93" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>RESTAURANT OS — remaining planned tasks (no staging creds needed)</t>
         </is>
       </c>
-      <c r="B22" s="96" t="n"/>
-      <c r="C22" s="96" t="n"/>
-      <c r="D22" s="96" t="n"/>
-      <c r="E22" s="96" t="n"/>
-      <c r="F22" s="96" t="n"/>
-      <c r="G22" s="96" t="n"/>
-      <c r="H22" s="96" t="n"/>
-      <c r="I22" s="96" t="n"/>
-      <c r="J22" s="96" t="n"/>
-      <c r="K22" s="96" t="n"/>
-      <c r="L22" s="96" t="n"/>
-      <c r="M22" s="96" t="n"/>
-      <c r="N22" s="96" t="n"/>
-      <c r="O22" s="97" t="n"/>
     </row>
     <row r="23" ht="52.05" customHeight="1" s="90">
-      <c r="A23" s="117" t="inlineStr">
+      <c r="A23" s="136" t="inlineStr">
         <is>
           <t>P6-A21</t>
         </is>
       </c>
-      <c r="B23" s="77" t="inlineStr">
-        <is>
-          <t>feature/weather-holiday-signals</t>
-        </is>
-      </c>
-      <c r="C23" s="77" t="inlineStr">
+      <c r="B23" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C23" s="137" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D23" s="77" t="inlineStr">
-        <is>
-          <t>Weather + holiday signals in demand forecast</t>
-        </is>
-      </c>
-      <c r="E23" s="77" t="inlineStr">
-        <is>
-          <t>Integrate Open-Meteo API (free, no key needed) for weather forecast at restaurant address. Add Indian holidays list (already in constants.py). Inject both signals into demand_forecast node context: "Rain forecast tomorrow evening: +30% delivery expected, -20% dine-in." "Tomorrow is Diwali: expect 2x normal demand, start prep by 3pm." New OrchestratorState field: weather_signal (temp, condition, rain_probability). ScenarioRecommender uses both signals to suggest correct scenario. Open-Meteo endpoint: https://api.open-meteo.com/v1/forecast (latitude, longitude, hourly=precipitation_probability,temperature_2m)</t>
-        </is>
-      </c>
-      <c r="F23" s="77" t="inlineStr">
-        <is>
-          <t>feat: weather + holiday demand signals — Open-Meteo + Indian holidays in forecast node</t>
-        </is>
-      </c>
-      <c r="G23" s="77" t="inlineStr">
-        <is>
-          <t>docs/AGENTS.md (demand_forecast node updated), CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="H23" s="71" t="inlineStr">
+      <c r="D23" s="137" t="inlineStr">
+        <is>
+          <t>Live signal 1/4: Weather + holiday-awareness in demand forecast</t>
+        </is>
+      </c>
+      <c r="E23" s="137" t="inlineStr">
+        <is>
+          <t>First of four independently-failing live-intelligence services feeding the planning pipeline (P6-A24 unifies all four). New WeatherService (infrastructure/external/weather_service.py) calls Open-Meteo (free, no API key) for current + 48h forecast at the restaurant's location -- rain/heat forecasts shift the plan toward delivery-heavy staffing and prep, clear days toward walk-in/outdoor capacity. INDIAN_HOLIDAYS_2026 already exists in core/constants.py and already feeds ScenarioRecommender in the background -- this task surfaces it explicitly into demand_forecast's own prompt too ('today is Gandhi Jayanti -- public holiday, expect elevated demand'), not just the scenario suggestion. Never raises -- returns None on any failure so demand_forecast runs fine without it. New OrchestratorState field: weather_signal.</t>
+        </is>
+      </c>
+      <c r="F23" s="137" t="inlineStr">
+        <is>
+          <t>feat: weather + holiday-awareness signal -- Open-Meteo integration (live signal 1/4)</t>
+        </is>
+      </c>
+      <c r="G23" s="137" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/ARCHITECTURE.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H23" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I23" s="76" t="inlineStr">
+      <c r="I23" s="136" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J23" s="76" t="inlineStr">
+      <c r="J23" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K23" s="76" t="n"/>
-      <c r="L23" s="76" t="n"/>
-      <c r="M23" s="78" t="n">
+      <c r="K23" s="136" t="n"/>
+      <c r="L23" s="136" t="n"/>
+      <c r="M23" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="77" t="n"/>
-      <c r="O23" s="77" t="inlineStr">
-        <is>
-          <t>Weather signal in OrchestratorState; ScenarioRecommender uses it; prompt includes weather context; Open-Meteo call works for Navi Mumbai coords</t>
+      <c r="N23" s="137" t="n"/>
+      <c r="O23" s="137" t="inlineStr">
+        <is>
+          <t>Weather API call returns current+forecast conditions for a known lat/lng and gracefully degrades to None on API failure; holiday lookup correctly identifies a known date against INDIAN_HOLIDAYS_2026; both signals appear in demand_forecast's prompt on a known test date</t>
         </is>
       </c>
     </row>
     <row r="24" ht="52.05" customHeight="1" s="90">
-      <c r="A24" s="117" t="inlineStr">
+      <c r="A24" s="136" t="inlineStr">
         <is>
           <t>P6-A22</t>
         </is>
       </c>
-      <c r="B24" s="74" t="inlineStr">
+      <c r="B24" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C24" s="137" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D24" s="137" t="inlineStr">
+        <is>
+          <t>Live signal 2/4: Industry trends (RSS-only, no paid API)</t>
+        </is>
+      </c>
+      <c r="E24" s="137" t="inlineStr">
+        <is>
+          <t>Second live-intelligence service. New TrendsService -- a curated list of Indian F&amp;B/hospitality trade-press RSS feeds, fetched via feedparser (new free/open-source dependency) and summarized into a short 'what's trending' digest using the existing Groq LLM client (no new LLM integration needed). RSS-only deliberately, not Google Trends/pytrends -- pytrends scrapes Google's internal endpoint, a ToS gray area we chose to avoid given how carefully we've treated Swiggy's terms; RSS is meant for syndication, zero ToS risk. Independently fail-open: if all feeds are unreachable, returns None and does not block weather/compliance/Swiggy signals. New OrchestratorState field: trends_signal.</t>
+        </is>
+      </c>
+      <c r="F24" s="137" t="inlineStr">
+        <is>
+          <t>feat: industry trends signal -- curated RSS feeds only, no paid API (live signal 2/4)</t>
+        </is>
+      </c>
+      <c r="G24" s="137" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H24" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I24" s="136" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J24" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K24" s="136" t="n"/>
+      <c r="L24" s="136" t="n"/>
+      <c r="M24" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="137" t="n"/>
+      <c r="O24" s="137" t="inlineStr">
+        <is>
+          <t>RSS fetch+parse works against a known feed in a live test; degrades to None if all feeds are unreachable (simulated); LLM produces a coherent digest from real feed content</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52.05" customHeight="1" s="90">
+      <c r="A25" s="136" t="inlineStr">
+        <is>
+          <t>P6-A23</t>
+        </is>
+      </c>
+      <c r="B25" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C25" s="137" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D25" s="137" t="inlineStr">
+        <is>
+          <t>Live signal 3/4: Regulatory/compliance alerts (FSSAI public notices)</t>
+        </is>
+      </c>
+      <c r="E25" s="137" t="inlineStr">
+        <is>
+          <t>Third live-intelligence service. New ComplianceAlertsService scrapes FSSAI's public notifications page (fssai.gov.in/notifications.php) via beautifulsoup4 (new dependency) -- confirmed live (2026-07-11) this page has no RSS feed, is plain server-side-rendered HTML (not JS-dependent), so a lightweight parser is sufficient without a headless browser. Public government regulatory data, no ToS tension of any kind -- cleanest source of the four on that front. Explicit fail-open contract given HTML scraping is inherently more fragile than RSS (any FSSAI site redesign breaks the parser) -- must degrade to None cleanly, never raise, never block the other three signals. New OrchestratorState field: compliance_alerts_signal.</t>
+        </is>
+      </c>
+      <c r="F25" s="137" t="inlineStr">
+        <is>
+          <t>feat: regulatory/compliance alerts signal -- FSSAI public notices scrape (live signal 3/4)</t>
+        </is>
+      </c>
+      <c r="G25" s="137" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/ARCHITECTURE.md</t>
+        </is>
+      </c>
+      <c r="H25" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I25" s="136" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J25" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K25" s="136" t="n"/>
+      <c r="L25" s="136" t="n"/>
+      <c r="M25" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="137" t="n"/>
+      <c r="O25" s="137" t="inlineStr">
+        <is>
+          <t>Scrape returns real recent notices in a live test; degrades to None on parse failure (simulate an unexpected page structure); no crash on an empty result set</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52.05" customHeight="1" s="90">
+      <c r="A26" s="136" t="inlineStr">
+        <is>
+          <t>P6-A24</t>
+        </is>
+      </c>
+      <c r="B26" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C26" s="137" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D26" s="137" t="inlineStr">
+        <is>
+          <t>Live signal 4/4: Wire all live signals into the planning pipeline (unify)</t>
+        </is>
+      </c>
+      <c r="E26" s="137" t="inlineStr">
+        <is>
+          <t>Merges weather/holiday (P6-A21) + industry trends (P6-A22) + compliance alerts (P6-A23) + the existing anonymised Swiggy area signals (P6-A20) into one combined 'Area &amp; Live Signals' section. Added INSIDE the existing market_intel_node / MarketIntelService rather than a new 12th LangGraph node -- MarketIntelService already runs multiple enrichers concurrently and fails open per-enricher, so this is additive to a proven pattern, not a new one. Critically, this preserves the existing state field names (swiggy_competitor_context, swiggy_occupancy_context, market_intel_output) that 5+ files and the frontend already read by name -- confirmed via audit that renaming them would be a wide, unnecessary blast radius. No frontend SSE changes needed since the node count doesn't change. Injected into demand_forecast, menu_intelligence, and the critic's prompt via aggregator.py's _build_critic_summary. Each of the 4 sources stays independently fail-open all the way through -- one going down never blocks the others or crashes the node.</t>
+        </is>
+      </c>
+      <c r="F26" s="137" t="inlineStr">
+        <is>
+          <t>feat: wire live signals into planning pipeline -- unified Area &amp; Live Signals section</t>
+        </is>
+      </c>
+      <c r="G26" s="137" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/ARCHITECTURE.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H26" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I26" s="136" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J26" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K26" s="136" t="n"/>
+      <c r="L26" s="136" t="n"/>
+      <c r="M26" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="137" t="inlineStr">
+        <is>
+          <t>P6-A21, P6-A22, P6-A23</t>
+        </is>
+      </c>
+      <c r="O26" s="137" t="inlineStr">
+        <is>
+          <t>demand_forecast/menu_intelligence/critic prompts include all present sources; simulated failure of any one source doesn't block the others or crash the node; aggregator's critic summary includes a live-signals section; existing Swiggy state field names unchanged, all P6-A19/A20 tests still pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52.05" customHeight="1" s="90">
+      <c r="A27" s="136" t="inlineStr">
+        <is>
+          <t>P6-A25</t>
+        </is>
+      </c>
+      <c r="B27" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C27" s="137" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D27" s="137" t="inlineStr">
+        <is>
+          <t>Scenario selection overhaul -- natural language + dynamic profiles</t>
+        </is>
+      </c>
+      <c r="E27" s="137" t="inlineStr">
+        <is>
+          <t>Confirmed via audit: all 4 scenarios (friday_rush/weekday_lunch/holiday_spike/low_stock_weekend) are hardcoded end-to-end -- a Pydantic Literal type in PlanningRunRequest, ops_manager_node rejects anything else, and the frontend has the same 4-item array duplicated in dashboard/page.tsx AND TodayIdleState.tsx. demand_forecast doesn't actually branch its algorithm on scenario today -- Prophet runs identically regardless, scenario only affects labeling and target_date. This task: relax PlanningScenarioId off the hardcoded Literal to accept a custom profile payload. New service turns free-form natural language ('we're hosting an event today, expecting large turnover') into an ad-hoc scenario_profile dict (label/service_window/operational_focus, LLM-derived) -- the 4 existing presets remain as one-click shortcuts, NOT replaced (explicit product decision). ops_manager_node's SUPPORTED_SCENARIOS check updated to admit custom profiles alongside the presets. Frontend: dedupe the two duplicated SCENARIO_OPTIONS arrays into one shared source; add a natural-language text input alongside the existing tile picker in PlanShiftModal.tsx -- user's choice of either mode, not a replacement of the tiles.</t>
+        </is>
+      </c>
+      <c r="F27" s="137" t="inlineStr">
+        <is>
+          <t>feat: scenario selection overhaul -- natural-language intake + dynamic profiles alongside presets</t>
+        </is>
+      </c>
+      <c r="G27" s="137" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md, docs/ARCHITECTURE.md, docs/PRODUCT_MODES.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H27" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I27" s="136" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J27" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K27" s="136" t="n"/>
+      <c r="L27" s="136" t="n"/>
+      <c r="M27" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="137" t="n"/>
+      <c r="O27" s="137" t="inlineStr">
+        <is>
+          <t>Natural-language input produces a valid scenario_profile dict with sensible defaults for missing fields; existing 4 presets still work completely unchanged; ops_manager_node accepts a custom profile without rejecting it; frontend offers both input modes; SCENARIO_OPTIONS no longer duplicated across two files</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="52.05" customHeight="1" s="90">
+      <c r="A28" s="136" t="inlineStr">
+        <is>
+          <t>P6-A26</t>
+        </is>
+      </c>
+      <c r="B28" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C28" s="137" t="inlineStr">
+        <is>
+          <t>Eval</t>
+        </is>
+      </c>
+      <c r="D28" s="137" t="inlineStr">
+        <is>
+          <t>Validate action-item specificity after live signals land (conditional)</t>
+        </is>
+      </c>
+      <c r="E28" s="137" t="inlineStr">
+        <is>
+          <t>Not a guaranteed code task -- a validation checkpoint. Research confirmed aggregator.py/critic_service.py already favor structured, itemized output (bulleted restock actions, explicit dish names, numeric thresholds, dimension scores) over narrative paragraphs, so the 'standard, generic response' feedback is more likely an input-richness problem than a prompt-engineering problem. After P6-A24 ships, manually review 3-5 generated plans against known-rich live-signal test dates (a rain-forecast night, a real upcoming holiday, an active trend, a live FSSAI notice) to check whether output is now sufficiently specific/actionable. If yes: close this task, no further work needed. If still generic: scope a real follow-up prompt-engineering task against aggregator/critic with concrete before/after examples.</t>
+        </is>
+      </c>
+      <c r="F28" s="137" t="inlineStr">
+        <is>
+          <t>None yet -- validation checkpoint, code only if the review finds a real gap</t>
+        </is>
+      </c>
+      <c r="G28" s="137" t="inlineStr">
+        <is>
+          <t>None yet</t>
+        </is>
+      </c>
+      <c r="H28" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I28" s="136" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J28" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K28" s="136" t="n"/>
+      <c r="L28" s="136" t="n"/>
+      <c r="M28" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="137" t="inlineStr">
+        <is>
+          <t>P6-A24</t>
+        </is>
+      </c>
+      <c r="O28" s="137" t="inlineStr">
+        <is>
+          <t>N/A -- manual review checkpoint, not an automated test</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="52.05" customHeight="1" s="90">
+      <c r="A29" s="136" t="inlineStr">
+        <is>
+          <t>P6-A27</t>
+        </is>
+      </c>
+      <c r="B29" s="137" t="inlineStr">
         <is>
           <t>feature/procurement-loop-endtoend</t>
         </is>
       </c>
-      <c r="C24" s="74" t="inlineStr">
+      <c r="C29" s="137" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D24" s="74" t="inlineStr">
+      <c r="D29" s="137" t="inlineStr">
         <is>
           <t>Autonomous procurement loop — end-to-end wire</t>
         </is>
       </c>
-      <c r="E24" s="74" t="inlineStr">
+      <c r="E29" s="137" t="inlineStr">
         <is>
           <t>Connect: weather/holiday signal → demand_forecast surge → inventory shortage detection → ProcurementEnricher Instamart prices → ActionQueue APPROVE_REQUIRED action → trust ladder → checkout (staging creds) OR WhatsApp vendor fallback. This is the flagship restaurant OS demo moment. The plan output must clearly show: shortage detected → Instamart has it at Rs.24/kg → approve to order → or WhatsApp vendor if not on Instamart. Wire trust ladder: orders under Rs.500 auto-approved, over Rs.500 needs manual approval in action queue UI.</t>
         </is>
       </c>
-      <c r="F24" s="74" t="inlineStr">
+      <c r="F29" s="137" t="inlineStr">
         <is>
           <t>feat: autonomous procurement loop — weather → forecast → shortage → Instamart → action queue</t>
         </is>
       </c>
-      <c r="G24" s="74" t="inlineStr">
+      <c r="G29" s="137" t="inlineStr">
         <is>
           <t>CLAUDE.md, docs/ARCHITECTURE.md (procurement loop diagram)</t>
         </is>
       </c>
-      <c r="H24" s="71" t="inlineStr">
+      <c r="H29" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I24" s="73" t="inlineStr">
+      <c r="I29" s="136" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J24" s="73" t="inlineStr">
+      <c r="J29" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K24" s="73" t="n"/>
-      <c r="L24" s="73" t="n"/>
-      <c r="M24" s="75" t="n">
+      <c r="K29" s="136" t="n"/>
+      <c r="L29" s="136" t="n"/>
+      <c r="M29" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N24" s="74" t="inlineStr">
-        <is>
-          <t>P6-A21</t>
-        </is>
-      </c>
-      <c r="O24" s="74" t="inlineStr">
+      <c r="N29" s="137" t="inlineStr">
+        <is>
+          <t>P6-A24</t>
+        </is>
+      </c>
+      <c r="O29" s="137" t="inlineStr">
         <is>
           <t>Full loop runs end-to-end in demo; trust ladder fires correctly; action queue shows Instamart procurement with price + spinId; WhatsApp fallback triggers when product not found on Instamart</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="52.05" customHeight="1" s="90">
-      <c r="A25" s="117" t="inlineStr">
-        <is>
-          <t>P6-A23</t>
-        </is>
-      </c>
-      <c r="B25" s="77" t="inlineStr">
+    <row r="30" ht="63" customHeight="1" s="90">
+      <c r="A30" s="136" t="inlineStr">
+        <is>
+          <t>P6-A28</t>
+        </is>
+      </c>
+      <c r="B30" s="137" t="inlineStr">
         <is>
           <t>feature/instamart-event-supplies</t>
         </is>
       </c>
-      <c r="C25" s="77" t="inlineStr">
+      <c r="C30" s="137" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D25" s="77" t="inlineStr">
+      <c r="D30" s="137" t="inlineStr">
         <is>
           <t>Instamart event supplies in operator chatbot</t>
         </is>
       </c>
-      <c r="E25" s="77" t="inlineStr">
+      <c r="E30" s="137" t="inlineStr">
         <is>
           <t>Extend operator chatbot with event supplies tool: "we are hosting a birthday event tonight, need supplies." Calls search_products for non-food items: candles, paper plates, cups, napkins, soft drinks, basic decorations, cleaning supplies, batteries. Returns real Instamart prices and availability. Creates ActionQueue procurement action for approval. Key insight: Instamart is not just food ingredients — managers use it for quick supply runs that previously required leaving the restaurant. New chatbot tool: get_event_supplies(event_type, headcount)</t>
         </is>
       </c>
-      <c r="F25" s="77" t="inlineStr">
+      <c r="F30" s="137" t="inlineStr">
         <is>
           <t>feat: Instamart event supplies tool in operator chatbot</t>
         </is>
       </c>
-      <c r="G25" s="77" t="inlineStr">
+      <c r="G30" s="137" t="inlineStr">
         <is>
           <t>docs/AGENTS.md (chatbot tools updated)</t>
         </is>
       </c>
-      <c r="H25" s="71" t="inlineStr">
+      <c r="H30" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I25" s="76" t="inlineStr">
+      <c r="I30" s="136" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J25" s="76" t="inlineStr">
+      <c r="J30" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K25" s="76" t="n"/>
-      <c r="L25" s="76" t="n"/>
-      <c r="M25" s="78" t="n">
+      <c r="K30" s="136" t="n"/>
+      <c r="L30" s="136" t="n"/>
+      <c r="M30" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="77" t="n"/>
-      <c r="O25" s="77" t="inlineStr">
+      <c r="N30" s="137" t="n"/>
+      <c r="O30" s="137" t="inlineStr">
         <is>
           <t>search_products returns real results for non-food queries; ActionQueue action created; trust ladder applied; chatbot responds naturally to event supply requests</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="52.05" customHeight="1" s="90">
-      <c r="A26" s="117" t="inlineStr">
-        <is>
-          <t>P6-A24</t>
-        </is>
-      </c>
-      <c r="B26" s="74" t="inlineStr">
+    <row r="31" ht="18" customHeight="1" s="90">
+      <c r="A31" s="139" t="inlineStr">
+        <is>
+          <t>P6-A29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>feature/menu-engineering-matrix</t>
         </is>
       </c>
-      <c r="C26" s="74" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="D26" s="74" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Menu engineering matrix UI</t>
         </is>
       </c>
-      <c r="E26" s="74" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Visual matrix: dish margin (y-axis) vs order popularity (x-axis). Four quadrants: Stars (high margin + high orders — promote), Plowhorses (low margin + high orders — reprice or remove), Puzzles (high margin + low orders — market better), Dogs (low margin + low orders — remove). Data from BusinessAnalyticsService (already has margin + popularity). Interactive: click a dish to see full margin breakdown. Shown on /operations page as a new panel. Connects to planning: critic uses quadrant data to validate menu recommendations.</t>
         </is>
       </c>
-      <c r="F26" s="74" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>feat: menu engineering matrix — margin vs popularity quadrant chart</t>
         </is>
       </c>
-      <c r="G26" s="74" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>None (frontend only)</t>
         </is>
       </c>
-      <c r="H26" s="71" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I26" s="73" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J26" s="73" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K26" s="73" t="n"/>
-      <c r="L26" s="73" t="n"/>
-      <c r="M26" s="75" t="n">
+      <c r="M31" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="74" t="n"/>
-      <c r="O26" s="74" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>Matrix renders with correct quadrant assignment; click through shows dish margin detail; Stars/Plowhorses/Puzzles/Dogs correctly classified</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="52.05" customHeight="1" s="90">
-      <c r="A27" s="117" t="inlineStr">
-        <is>
-          <t>P6-A25</t>
-        </is>
-      </c>
-      <c r="B27" s="77" t="inlineStr">
+    <row r="32" ht="52.05" customHeight="1" s="90">
+      <c r="A32" s="136" t="inlineStr">
+        <is>
+          <t>P6-A30</t>
+        </is>
+      </c>
+      <c r="B32" s="137" t="inlineStr">
         <is>
           <t>feature/structured-outputs</t>
         </is>
       </c>
-      <c r="C27" s="77" t="inlineStr">
+      <c r="C32" s="137" t="inlineStr">
         <is>
           <t>Agents</t>
         </is>
       </c>
-      <c r="D27" s="77" t="inlineStr">
+      <c r="D32" s="137" t="inlineStr">
         <is>
           <t>Structured outputs — tool_choice=required across chatbot</t>
         </is>
       </c>
-      <c r="E27" s="77" t="inlineStr">
+      <c r="E32" s="137" t="inlineStr">
         <is>
           <t>Force structured JSON outputs from Groq function calling. Eliminates cases where chatbot returns freeform text instead of calling the right tool. Add response validation layer. Makes chatbot more reliable for demo — no unexpected text responses.</t>
         </is>
       </c>
-      <c r="F27" s="77" t="inlineStr">
+      <c r="F32" s="137" t="inlineStr">
         <is>
           <t>feat: structured outputs — force tool_choice=required in chatbot</t>
         </is>
       </c>
-      <c r="G27" s="77" t="inlineStr">
+      <c r="G32" s="137" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H27" s="71" t="inlineStr">
+      <c r="H32" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I27" s="76" t="inlineStr">
+      <c r="I32" s="136" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J27" s="76" t="inlineStr">
+      <c r="J32" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K27" s="76" t="n"/>
-      <c r="L27" s="76" t="n"/>
-      <c r="M27" s="78" t="n">
+      <c r="K32" s="136" t="n"/>
+      <c r="L32" s="136" t="n"/>
+      <c r="M32" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N27" s="77" t="n"/>
-      <c r="O27" s="77" t="inlineStr">
+      <c r="N32" s="137" t="n"/>
+      <c r="O32" s="137" t="inlineStr">
         <is>
           <t>Chatbot always calls a tool when one applies; no unexpected freeform responses; existing chatbot tests pass</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="52.05" customHeight="1" s="90">
-      <c r="A28" s="117" t="inlineStr">
-        <is>
-          <t>P6-A26</t>
-        </is>
-      </c>
-      <c r="B28" s="74" t="inlineStr">
+    <row r="33" ht="52.05" customHeight="1" s="90">
+      <c r="A33" s="136" t="inlineStr">
+        <is>
+          <t>P6-A31</t>
+        </is>
+      </c>
+      <c r="B33" s="137" t="inlineStr">
         <is>
           <t>feature/voice-interface</t>
         </is>
       </c>
-      <c r="C28" s="74" t="inlineStr">
+      <c r="C33" s="137" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="D28" s="74" t="inlineStr">
+      <c r="D33" s="137" t="inlineStr">
         <is>
           <t>Voice interface — Whisper transcription + TTS response</t>
         </is>
       </c>
-      <c r="E28" s="74" t="inlineStr">
+      <c r="E33" s="137" t="inlineStr">
         <is>
           <t>Restaurant operator speaks to CortexKitchen instead of typing. Browser MediaRecorder API captures audio. Whisper (via Groq) transcribes to text. Existing chatbot processes the text query. TTS reads back the response. Use case: manager walking the floor asks questions hands-free. "What does the plan say about staffing tonight?" "How many covers are we expecting?" Add mic button to existing /chat page. Works for operator side only initially.</t>
         </is>
       </c>
-      <c r="F28" s="74" t="inlineStr">
+      <c r="F33" s="137" t="inlineStr">
         <is>
           <t>feat: voice interface — Whisper transcription + TTS on /chat page</t>
         </is>
       </c>
-      <c r="G28" s="74" t="inlineStr">
+      <c r="G33" s="137" t="inlineStr">
         <is>
           <t>docs/PRODUCT_MODES.md (voice mode section)</t>
         </is>
       </c>
-      <c r="H28" s="71" t="inlineStr">
+      <c r="H33" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I28" s="73" t="inlineStr">
+      <c r="I33" s="136" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J28" s="73" t="inlineStr">
+      <c r="J33" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K28" s="73" t="n"/>
-      <c r="L28" s="73" t="n"/>
-      <c r="M28" s="75" t="n">
+      <c r="K33" s="136" t="n"/>
+      <c r="L33" s="136" t="n"/>
+      <c r="M33" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N28" s="74" t="n"/>
-      <c r="O28" s="74" t="inlineStr">
+      <c r="N33" s="137" t="n"/>
+      <c r="O33" s="137" t="inlineStr">
         <is>
           <t>Audio recorded and transcribed correctly; chatbot processes transcription; TTS plays response; mic button shows recording state</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="52.05" customHeight="1" s="90">
-      <c r="A29" s="117" t="inlineStr">
+    <row r="34" ht="7.95" customHeight="1" s="90">
+      <c r="A34" s="136" t="inlineStr">
+        <is>
+          <t>P6-A32</t>
+        </is>
+      </c>
+      <c r="B34" s="137" t="inlineStr">
+        <is>
+          <t>feature/eval-pipeline</t>
+        </is>
+      </c>
+      <c r="C34" s="137" t="inlineStr">
+        <is>
+          <t>Eval</t>
+        </is>
+      </c>
+      <c r="D34" s="137" t="inlineStr">
+        <is>
+          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
+        </is>
+      </c>
+      <c r="E34" s="137" t="inlineStr">
+        <is>
+          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
+        </is>
+      </c>
+      <c r="F34" s="137" t="inlineStr">
+        <is>
+          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
+        </is>
+      </c>
+      <c r="G34" s="137" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H34" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I34" s="136" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J34" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K34" s="136" t="n"/>
+      <c r="L34" s="136" t="n"/>
+      <c r="M34" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="137" t="inlineStr">
         <is>
           <t>P6-A27</t>
         </is>
       </c>
-      <c r="B29" s="77" t="inlineStr">
-        <is>
-          <t>feature/eval-pipeline</t>
-        </is>
-      </c>
-      <c r="C29" s="77" t="inlineStr">
-        <is>
-          <t>Eval</t>
-        </is>
-      </c>
-      <c r="D29" s="77" t="inlineStr">
-        <is>
-          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
-        </is>
-      </c>
-      <c r="E29" s="77" t="inlineStr">
-        <is>
-          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
-        </is>
-      </c>
-      <c r="F29" s="77" t="inlineStr">
-        <is>
-          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
-        </is>
-      </c>
-      <c r="G29" s="77" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H29" s="71" t="inlineStr">
+      <c r="O34" s="137" t="inlineStr">
+        <is>
+          <t>CI eval gate passes; golden_runs.json reflects current system; regressions caught in 2+ test scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DOCS + SYNC — end of Phase 6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="136" t="inlineStr">
+        <is>
+          <t>P6-A33</t>
+        </is>
+      </c>
+      <c r="B37" s="137" t="inlineStr">
+        <is>
+          <t>feature/documentation</t>
+        </is>
+      </c>
+      <c r="C37" s="137" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D37" s="137" t="inlineStr">
+        <is>
+          <t>Whole-system documentation + screenshots refresh</t>
+        </is>
+      </c>
+      <c r="E37" s="137" t="inlineStr">
+        <is>
+          <t>Update all docs to reflect: new two-sided product vision, compliance changes (Zomato removed, market intel anonymised), autonomous procurement loop, weather signals, voice interface. New product vision statement in README. Screenshots of the operator portal (dashboard, operations, market, action queue, chat) for portfolio -- Guest Concierge screenshots belong to Phase 6B docs (P6-B9), not here, since Guest Concierge does not exist yet at this point.</t>
+        </is>
+      </c>
+      <c r="F37" s="137" t="inlineStr">
+        <is>
+          <t>docs: whole-system documentation refresh — new product vision</t>
+        </is>
+      </c>
+      <c r="G37" s="137" t="inlineStr">
+        <is>
+          <t>README.md, docs/ARCHITECTURE.md, docs/AGENTS.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H37" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I29" s="76" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J29" s="76" t="inlineStr">
+      <c r="I37" s="136" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J37" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K29" s="76" t="n"/>
-      <c r="L29" s="76" t="n"/>
-      <c r="M29" s="78" t="n">
+      <c r="K37" s="136" t="n"/>
+      <c r="L37" s="136" t="n"/>
+      <c r="M37" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N29" s="77" t="inlineStr">
-        <is>
-          <t>P6-A22</t>
-        </is>
-      </c>
-      <c r="O29" s="77" t="inlineStr">
-        <is>
-          <t>CI eval gate passes; golden_runs.json reflects current system; regressions caught in 2+ test scenarios</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="63" customHeight="1" s="90"/>
-    <row r="31" ht="18" customHeight="1" s="90">
-      <c r="A31" s="118" t="inlineStr">
-        <is>
-          <t>DOCS + SYNC — end of Phase 6A</t>
-        </is>
-      </c>
-      <c r="B31" s="131" t="n"/>
-      <c r="C31" s="131" t="n"/>
-      <c r="D31" s="131" t="n"/>
-      <c r="E31" s="131" t="n"/>
-      <c r="F31" s="131" t="n"/>
-      <c r="G31" s="131" t="n"/>
-      <c r="H31" s="131" t="n"/>
-      <c r="I31" s="131" t="n"/>
-      <c r="J31" s="131" t="n"/>
-      <c r="K31" s="131" t="n"/>
-      <c r="L31" s="131" t="n"/>
-      <c r="M31" s="131" t="n"/>
-      <c r="N31" s="131" t="n"/>
-      <c r="O31" s="131" t="n"/>
-    </row>
-    <row r="32" ht="52.05" customHeight="1" s="90">
-      <c r="A32" s="120" t="inlineStr">
-        <is>
-          <t>P6-A28</t>
-        </is>
-      </c>
-      <c r="B32" s="81" t="inlineStr">
-        <is>
-          <t>feature/documentation</t>
-        </is>
-      </c>
-      <c r="C32" s="81" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D32" s="81" t="inlineStr">
-        <is>
-          <t>Whole-system documentation + screenshots refresh</t>
-        </is>
-      </c>
-      <c r="E32" s="81" t="inlineStr">
-        <is>
-          <t>Update all docs to reflect: new two-sided product vision, compliance changes (Zomato removed, market intel anonymised), autonomous procurement loop, weather signals, voice interface. New product vision statement in README. Screenshots of the operator portal (dashboard, operations, market, action queue, chat) for portfolio -- Guest Concierge screenshots belong to Phase 6B docs (P6-B9), not here, since Guest Concierge does not exist yet at this point.</t>
-        </is>
-      </c>
-      <c r="F32" s="81" t="inlineStr">
-        <is>
-          <t>docs: whole-system documentation refresh — new product vision</t>
-        </is>
-      </c>
-      <c r="G32" s="81" t="inlineStr">
-        <is>
-          <t>README.md, docs/ARCHITECTURE.md, docs/AGENTS.md, CLAUDE.md</t>
-        </is>
-      </c>
-      <c r="H32" s="71" t="inlineStr">
+      <c r="N37" s="137" t="inlineStr">
+        <is>
+          <t>P6-A32</t>
+        </is>
+      </c>
+      <c r="O37" s="137" t="inlineStr">
+        <is>
+          <t>README reflects two-sided platform; all compliance changes documented; screenshots current</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="136" t="inlineStr">
+        <is>
+          <t>P6-A34</t>
+        </is>
+      </c>
+      <c r="B38" s="137" t="inlineStr">
+        <is>
+          <t>dev -&gt; main</t>
+        </is>
+      </c>
+      <c r="C38" s="137" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D38" s="137" t="inlineStr">
+        <is>
+          <t>Sync Phase 6A to main</t>
+        </is>
+      </c>
+      <c r="E38" s="137" t="inlineStr">
+        <is>
+          <t>Merge dev → main. All compliance fixes confirmed. Autonomous procurement loop working (minus checkout — staging creds). Restaurant OS demo-ready. Phase 6B starts after this.</t>
+        </is>
+      </c>
+      <c r="F38" s="137" t="inlineStr">
+        <is>
+          <t>release: Phase 6A complete — restaurant OS + compliance fixes</t>
+        </is>
+      </c>
+      <c r="G38" s="137" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="H38" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I32" s="80" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J32" s="80" t="inlineStr">
+      <c r="I38" s="136" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J38" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K32" s="80" t="n"/>
-      <c r="L32" s="80" t="n"/>
-      <c r="M32" s="82" t="n">
+      <c r="K38" s="136" t="n"/>
+      <c r="L38" s="136" t="n"/>
+      <c r="M38" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N32" s="81" t="inlineStr">
-        <is>
-          <t>P6-A27</t>
-        </is>
-      </c>
-      <c r="O32" s="81" t="inlineStr">
-        <is>
-          <t>README reflects two-sided platform; all compliance changes documented; screenshots current</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="52.05" customHeight="1" s="90">
-      <c r="A33" s="116" t="inlineStr">
-        <is>
-          <t>P6-A29</t>
-        </is>
-      </c>
-      <c r="B33" s="74" t="inlineStr">
-        <is>
-          <t>dev -&gt; main</t>
-        </is>
-      </c>
-      <c r="C33" s="74" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="D33" s="74" t="inlineStr">
-        <is>
-          <t>Sync Phase 6A to main</t>
-        </is>
-      </c>
-      <c r="E33" s="74" t="inlineStr">
-        <is>
-          <t>Merge dev → main. All compliance fixes confirmed. Autonomous procurement loop working (minus checkout — staging creds). Restaurant OS demo-ready. Phase 6B starts after this.</t>
-        </is>
-      </c>
-      <c r="F33" s="74" t="inlineStr">
-        <is>
-          <t>release: Phase 6A complete — restaurant OS + compliance fixes</t>
-        </is>
-      </c>
-      <c r="G33" s="74" t="inlineStr">
-        <is>
-          <t>README.md</t>
-        </is>
-      </c>
-      <c r="H33" s="71" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="I33" s="73" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J33" s="73" t="inlineStr">
-        <is>
-          <t>Anoushka</t>
-        </is>
-      </c>
-      <c r="K33" s="73" t="n"/>
-      <c r="L33" s="73" t="n"/>
-      <c r="M33" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="74" t="inlineStr">
-        <is>
-          <t>P6-A28</t>
-        </is>
-      </c>
-      <c r="O33" s="74" t="inlineStr">
+      <c r="N38" s="137" t="inlineStr">
+        <is>
+          <t>P6-A33</t>
+        </is>
+      </c>
+      <c r="O38" s="137" t="inlineStr">
         <is>
           <t>Full test suite green; compliance fixes verified; no Zomato references; market intel anonymised; demo flow works</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="7.95" customHeight="1" s="90"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A36:O36"/>
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A31:O31"/>
     <mergeCell ref="A22:O22"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A3:O3"/>
@@ -19688,7 +19990,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>search_products for decorations, cake, drinks, party supplies matching the event brief -- same tool pattern as the Restaurant OS operator-facing get_event_supplies (P6-A23), but consumer-facing and for the guest's own event rather than restaurant procurement. Cart/checkout once creds land.</t>
+          <t>search_products for decorations, cake, drinks, party supplies matching the event brief -- same tool pattern as the Restaurant OS operator-facing get_event_supplies (P6-A28), but consumer-facing and for the guest's own event rather than restaurant procurement. Cart/checkout once creds land.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -20398,7 +20700,7 @@
       </c>
       <c r="N14" s="59" t="inlineStr">
         <is>
-          <t>P6-A22</t>
+          <t>P6-A31</t>
         </is>
       </c>
       <c r="O14" s="59" t="inlineStr">
@@ -22056,7 +22358,7 @@
       </c>
       <c r="E63" s="59" t="inlineStr">
         <is>
-          <t>Audit test coverage for every new service/model added in Phase 6A (Action Queue, workflow triggers, trust-ladder, WhatsApp vendor flow, Vendor/Supplier model, Menu Engineering Matrix) -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (workflow-triggered actions, trust-ladder promotions), since the existing eval sets predate all of this and won't catch regressions in it. (Docs + screenshots refresh is P6-A23, done before the demo video; this is the deeper test/CI/eval hygiene pass that doesn't need to block the video.)</t>
+          <t>Audit test coverage for every new service/model added in Phase 6A (Action Queue, workflow triggers, trust-ladder, WhatsApp vendor flow, Vendor/Supplier model, Menu Engineering Matrix) -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (workflow-triggered actions, trust-ladder promotions), since the existing eval sets predate all of this and won't catch regressions in it. (Docs + screenshots refresh is P6-A33, done before the demo video; this is the deeper test/CI/eval hygiene pass that doesn't need to block the video.)</t>
         </is>
       </c>
       <c r="F63" s="59" t="inlineStr">

</xml_diff>

<commit_message>
chore: add Today Dashboard + Data page redesign to Phase 6A (real-product IA pass)
Adds two new tasks discovered during a product-level review of the page
structure: P6-A26 (merge /operations into /dashboard, live-signals context
strip, give the Action Queue -- Phase 6A's biggest existing feature -- an
actual primary-nav home) and P6-A27 (merge /runs + /data-health into one
Data page, add Action Queue history). Retargets Menu Engineering Matrix
(P6-A28) to the new Data page instead of the now-merged /operations.
Renumbers P6-A26-A34 to P6-A29-A36 to keep IDs sequential; fixes every
stale cross-reference across Dashboard, Phase 6B, and Staging Creds sheets.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -569,7 +569,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -956,6 +956,7 @@
     <xf numFmtId="0" fontId="27" fillId="25" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1356,7 +1357,7 @@
     <row r="5" ht="14.4" customHeight="1" s="90">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Staging creds unlock: Instamart checkout (within P6-A27 procurement loop; also P6-B7 Guest Concierge) + Dineout book_table (P6-B5 Guest Concierge).</t>
+          <t>Staging creds unlock: Instamart checkout (within P6-A30 procurement loop; also P6-B7 Guest Concierge) + Dineout book_table (P6-B5 Guest Concierge).</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -17346,7 +17347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="90" min="1" max="1"/>
@@ -18546,7 +18547,7 @@
     </row>
     <row r="21" ht="7.95" customHeight="1" s="90"/>
     <row r="22" ht="18" customHeight="1" s="90">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="140" t="inlineStr">
         <is>
           <t>RESTAURANT OS — remaining planned tasks (no staging creds needed)</t>
         </is>
@@ -18831,7 +18832,7 @@
       </c>
       <c r="E27" s="137" t="inlineStr">
         <is>
-          <t>Confirmed via audit: all 4 scenarios (friday_rush/weekday_lunch/holiday_spike/low_stock_weekend) are hardcoded end-to-end -- a Pydantic Literal type in PlanningRunRequest, ops_manager_node rejects anything else, and the frontend has the same 4-item array duplicated in dashboard/page.tsx AND TodayIdleState.tsx. demand_forecast doesn't actually branch its algorithm on scenario today -- Prophet runs identically regardless, scenario only affects labeling and target_date. This task: relax PlanningScenarioId off the hardcoded Literal to accept a custom profile payload. New service turns free-form natural language ('we're hosting an event today, expecting large turnover') into an ad-hoc scenario_profile dict (label/service_window/operational_focus, LLM-derived) -- the 4 existing presets remain as one-click shortcuts, NOT replaced (explicit product decision). ops_manager_node's SUPPORTED_SCENARIOS check updated to admit custom profiles alongside the presets. Frontend: dedupe the two duplicated SCENARIO_OPTIONS arrays into one shared source; add a natural-language text input alongside the existing tile picker in PlanShiftModal.tsx -- user's choice of either mode, not a replacement of the tiles.</t>
+          <t>Confirmed via audit: all 4 scenarios (friday_rush/weekday_lunch/holiday_spike/low_stock_weekend) are hardcoded end-to-end -- a Pydantic Literal type in PlanningRunRequest, ops_manager_node rejects anything else, and the frontend has the same 4-item array duplicated in dashboard/page.tsx AND TodayIdleState.tsx. demand_forecast doesn't actually branch its algorithm on scenario today -- Prophet runs identically regardless, scenario only affects labeling and target_date. This task: relax PlanningScenarioId off the hardcoded Literal to accept a custom profile payload. New service turns free-form natural language ('we're hosting an event today, expecting large turnover') into an ad-hoc scenario_profile dict (label/service_window/operational_focus, LLM-derived) -- the 4 existing presets remain as one-click shortcuts, NOT replaced (explicit product decision). ops_manager_node's SUPPORTED_SCENARIOS check updated to admit custom profiles alongside the presets. Frontend: dedupe the two duplicated SCENARIO_OPTIONS arrays into one shared source; add a natural-language text input alongside the existing tile picker in PlanShiftModal.tsx -- user's choice of either mode, not a replacement of the tiles. Scope boundary: this task owns the backend (schema relaxation, natural-language-to-profile service) and the input widget itself; where that widget sits in the page layout, the live-signals context strip, and Action Queue placement belong to the new Today Dashboard redesign task (P6-A26) that follows.</t>
         </is>
       </c>
       <c r="F27" s="137" t="inlineStr">
@@ -18884,27 +18885,27 @@
       </c>
       <c r="C28" s="137" t="inlineStr">
         <is>
-          <t>Eval</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D28" s="137" t="inlineStr">
         <is>
-          <t>Validate action-item specificity after live signals land (conditional)</t>
+          <t>Today Dashboard redesign -- merge /operations in, live-signals context strip, Action Queue front-and-center</t>
         </is>
       </c>
       <c r="E28" s="137" t="inlineStr">
         <is>
-          <t>Not a guaranteed code task -- a validation checkpoint. Research confirmed aggregator.py/critic_service.py already favor structured, itemized output (bulleted restock actions, explicit dish names, numeric thresholds, dimension scores) over narrative paragraphs, so the 'standard, generic response' feedback is more likely an input-richness problem than a prompt-engineering problem. After P6-A24 ships, manually review 3-5 generated plans against known-rich live-signal test dates (a rain-forecast night, a real upcoming holiday, an active trend, a live FSSAI notice) to check whether output is now sufficiently specific/actionable. If yes: close this task, no further work needed. If still generic: scope a real follow-up prompt-engineering task against aggregator/critic with concrete before/after examples.</t>
+          <t>Real-product IA decision: merge /operations (agent cards, forecast chart, critic banner) into /dashboard so triggering a plan and watching it build/complete happens in one continuous view, not a page navigation -- a manager clicking 'plan your shift' shouldn't have to go somewhere else to see what they just asked for. Adds a condensed 'Today's Context' strip (weather/holiday/trend/compliance badges, from the four live signals unified in P6-A24) positioned next to the plan trigger, visible while choosing a scenario or typing a natural-language description (P6-A25) -- not on a separate /market page nobody checks daily. Adds the Action Queue (pending restock alerts, WhatsApp vendor drafts, pricing/promo reviews, trust-ladder approve/reject) prominently on this page -- currently the single biggest existing feature (P6-A7/A8/A9/A12) with no clear primary-nav home at all. Surfaces day-of KPIs (net margin, health score, revenue vs yesterday from GET /business/performance, P6-A6) at the top. /operations route redirects to /dashboard once the merge is verified working.</t>
         </is>
       </c>
       <c r="F28" s="137" t="inlineStr">
         <is>
-          <t>None yet -- validation checkpoint, code only if the review finds a real gap</t>
+          <t>feat: Today Dashboard redesign -- merge /operations, live-signals context strip, Action Queue front-and-center</t>
         </is>
       </c>
       <c r="G28" s="137" t="inlineStr">
         <is>
-          <t>None yet</t>
+          <t>docs/PRODUCT_MODES.md, docs/ARCHITECTURE.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H28" s="138" t="inlineStr">
@@ -18914,7 +18915,7 @@
       </c>
       <c r="I28" s="136" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J28" s="136" t="inlineStr">
@@ -18929,12 +18930,12 @@
       </c>
       <c r="N28" s="137" t="inlineStr">
         <is>
-          <t>P6-A24</t>
+          <t>P6-A24, P6-A25</t>
         </is>
       </c>
       <c r="O28" s="137" t="inlineStr">
         <is>
-          <t>N/A -- manual review checkpoint, not an automated test</t>
+          <t>Triggering a plan from Today shows agent cards/forecast chart/critic banner inline with no navigation; context strip shows all 4 live signals when present and degrades gracefully per-signal when one is missing; Action Queue pending items are visible and directly actionable (approve/reject) from this page; KPI snapshot renders real data from GET /business/performance; /operations redirects correctly</t>
         </is>
       </c>
     </row>
@@ -18946,32 +18947,32 @@
       </c>
       <c r="B29" s="137" t="inlineStr">
         <is>
-          <t>feature/procurement-loop-endtoend</t>
+          <t>feature/live-intelligence-signals</t>
         </is>
       </c>
       <c r="C29" s="137" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D29" s="137" t="inlineStr">
         <is>
-          <t>Autonomous procurement loop — end-to-end wire</t>
+          <t>Data page redesign -- merge /runs + /data-health, add Action Queue history</t>
         </is>
       </c>
       <c r="E29" s="137" t="inlineStr">
         <is>
-          <t>Connect: weather/holiday signal → demand_forecast surge → inventory shortage detection → ProcurementEnricher Instamart prices → ActionQueue APPROVE_REQUIRED action → trust ladder → checkout (staging creds) OR WhatsApp vendor fallback. This is the flagship restaurant OS demo moment. The plan output must clearly show: shortage detected → Instamart has it at Rs.24/kg → approve to order → or WhatsApp vendor if not on Instamart. Wire trust ladder: orders under Rs.500 auto-approved, over Rs.500 needs manual approval in action queue UI.</t>
+          <t>Real-product IA decision: a manager doesn't think of 'run history' as a separate audit concept from 'system data/health' -- merges /runs (plan run history, currently the weakest-looking screen: dense monospace debug trace) and /data-health (sync status, freshness) into one 'Data' page with clearly separated sections, applying the existing design system instead of the current raw trace view. Adds a new section with no home anywhere today: Action Queue history -- the audit trail of every action approved/rejected/executed over time (restocks sent, WhatsApp messages, pricing reviews). Fixes the known unstyled /runs/{id} deep-link 404 while in here.</t>
         </is>
       </c>
       <c r="F29" s="137" t="inlineStr">
         <is>
-          <t>feat: autonomous procurement loop — weather → forecast → shortage → Instamart → action queue</t>
+          <t>feat: Data page redesign -- merge /runs + /data-health, add Action Queue history</t>
         </is>
       </c>
       <c r="G29" s="137" t="inlineStr">
         <is>
-          <t>CLAUDE.md, docs/ARCHITECTURE.md (procurement loop diagram)</t>
+          <t>docs/ARCHITECTURE.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H29" s="138" t="inlineStr">
@@ -18981,7 +18982,7 @@
       </c>
       <c r="I29" s="136" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J29" s="136" t="inlineStr">
@@ -18994,14 +18995,10 @@
       <c r="M29" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N29" s="137" t="inlineStr">
-        <is>
-          <t>P6-A24</t>
-        </is>
-      </c>
+      <c r="N29" s="137" t="n"/>
       <c r="O29" s="137" t="inlineStr">
         <is>
-          <t>Full loop runs end-to-end in demo; trust ladder fires correctly; action queue shows Instamart procurement with price + spinId; WhatsApp fallback triggers when product not found on Instamart</t>
+          <t>/runs and /data-health content both accessible from one page with consistent design-system styling; direct navigation to /runs/{id} deep-link renders the run, not a 404; Action Queue history shows past actions with correct status/timestamps</t>
         </is>
       </c>
     </row>
@@ -19013,32 +19010,32 @@
       </c>
       <c r="B30" s="137" t="inlineStr">
         <is>
-          <t>feature/instamart-event-supplies</t>
+          <t>feature/live-intelligence-signals</t>
         </is>
       </c>
       <c r="C30" s="137" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D30" s="137" t="inlineStr">
         <is>
-          <t>Instamart event supplies in operator chatbot</t>
+          <t>Menu engineering matrix UI</t>
         </is>
       </c>
       <c r="E30" s="137" t="inlineStr">
         <is>
-          <t>Extend operator chatbot with event supplies tool: "we are hosting a birthday event tonight, need supplies." Calls search_products for non-food items: candles, paper plates, cups, napkins, soft drinks, basic decorations, cleaning supplies, batteries. Returns real Instamart prices and availability. Creates ActionQueue procurement action for approval. Key insight: Instamart is not just food ingredients — managers use it for quick supply runs that previously required leaving the restaurant. New chatbot tool: get_event_supplies(event_type, headcount)</t>
+          <t>Visual matrix: dish margin (y-axis) vs order popularity (x-axis). Four quadrants: Stars (high margin + high orders — promote), Plowhorses (low margin + high orders — reprice or remove), Puzzles (high margin + low orders — market better), Dogs (low margin + low orders — remove). Data from BusinessAnalyticsService (already has margin + popularity). Interactive: click a dish to see full margin breakdown. Shown on the new Data page (P6-A27), not /operations -- /operations is merged into Today Dashboard (P6-A26) and this is analytical/historical review, not a daily trigger-time decision, so it belongs with run history, not the plan-trigger flow. Connects to planning: critic uses quadrant data to validate menu recommendations.</t>
         </is>
       </c>
       <c r="F30" s="137" t="inlineStr">
         <is>
-          <t>feat: Instamart event supplies tool in operator chatbot</t>
+          <t>feat: menu engineering matrix — margin vs popularity quadrant chart</t>
         </is>
       </c>
       <c r="G30" s="137" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md (chatbot tools updated)</t>
+          <t>None (frontend only)</t>
         </is>
       </c>
       <c r="H30" s="138" t="inlineStr">
@@ -19048,7 +19045,7 @@
       </c>
       <c r="I30" s="136" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J30" s="136" t="inlineStr">
@@ -19061,70 +19058,81 @@
       <c r="M30" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="137" t="n"/>
+      <c r="N30" s="137" t="inlineStr">
+        <is>
+          <t>P6-A27</t>
+        </is>
+      </c>
       <c r="O30" s="137" t="inlineStr">
         <is>
-          <t>search_products returns real results for non-food queries; ActionQueue action created; trust ladder applied; chatbot responds naturally to event supply requests</t>
+          <t>Matrix renders with correct quadrant assignment; click through shows dish margin detail; Stars/Plowhorses/Puzzles/Dogs correctly classified</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="90">
-      <c r="A31" s="139" t="inlineStr">
+      <c r="A31" s="136" t="inlineStr">
         <is>
           <t>P6-A29</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>feature/menu-engineering-matrix</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Menu engineering matrix UI</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Visual matrix: dish margin (y-axis) vs order popularity (x-axis). Four quadrants: Stars (high margin + high orders — promote), Plowhorses (low margin + high orders — reprice or remove), Puzzles (high margin + low orders — market better), Dogs (low margin + low orders — remove). Data from BusinessAnalyticsService (already has margin + popularity). Interactive: click a dish to see full margin breakdown. Shown on /operations page as a new panel. Connects to planning: critic uses quadrant data to validate menu recommendations.</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>feat: menu engineering matrix — margin vs popularity quadrant chart</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>None (frontend only)</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="B31" s="137" t="inlineStr">
+        <is>
+          <t>feature/live-intelligence-signals</t>
+        </is>
+      </c>
+      <c r="C31" s="137" t="inlineStr">
+        <is>
+          <t>Eval</t>
+        </is>
+      </c>
+      <c r="D31" s="137" t="inlineStr">
+        <is>
+          <t>Validate action-item specificity after live signals land (conditional)</t>
+        </is>
+      </c>
+      <c r="E31" s="137" t="inlineStr">
+        <is>
+          <t>Not a guaranteed code task -- a validation checkpoint. Research confirmed aggregator.py/critic_service.py already favor structured, itemized output (bulleted restock actions, explicit dish names, numeric thresholds, dimension scores) over narrative paragraphs, so the 'standard, generic response' feedback is more likely an input-richness problem than a prompt-engineering problem. After P6-A24 ships, manually review 3-5 generated plans against known-rich live-signal test dates (a rain-forecast night, a real upcoming holiday, an active trend, a live FSSAI notice) to check whether output is now sufficiently specific/actionable. If yes: close this task, no further work needed. If still generic: scope a real follow-up prompt-engineering task against aggregator/critic with concrete before/after examples.</t>
+        </is>
+      </c>
+      <c r="F31" s="137" t="inlineStr">
+        <is>
+          <t>None yet -- validation checkpoint, code only if the review finds a real gap</t>
+        </is>
+      </c>
+      <c r="G31" s="137" t="inlineStr">
+        <is>
+          <t>None yet</t>
+        </is>
+      </c>
+      <c r="H31" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
+      <c r="I31" s="136" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J31" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="M31" t="n">
+      <c r="K31" s="136" t="n"/>
+      <c r="L31" s="136" t="n"/>
+      <c r="M31" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Matrix renders with correct quadrant assignment; click through shows dish margin detail; Stars/Plowhorses/Puzzles/Dogs correctly classified</t>
+      <c r="N31" s="137" t="inlineStr">
+        <is>
+          <t>P6-A24, P6-A26</t>
+        </is>
+      </c>
+      <c r="O31" s="137" t="inlineStr">
+        <is>
+          <t>N/A -- manual review checkpoint, not an automated test</t>
         </is>
       </c>
     </row>
@@ -19136,7 +19144,7 @@
       </c>
       <c r="B32" s="137" t="inlineStr">
         <is>
-          <t>feature/structured-outputs</t>
+          <t>feature/procurement-loop-endtoend</t>
         </is>
       </c>
       <c r="C32" s="137" t="inlineStr">
@@ -19146,22 +19154,22 @@
       </c>
       <c r="D32" s="137" t="inlineStr">
         <is>
-          <t>Structured outputs — tool_choice=required across chatbot</t>
+          <t>Autonomous procurement loop — end-to-end wire</t>
         </is>
       </c>
       <c r="E32" s="137" t="inlineStr">
         <is>
-          <t>Force structured JSON outputs from Groq function calling. Eliminates cases where chatbot returns freeform text instead of calling the right tool. Add response validation layer. Makes chatbot more reliable for demo — no unexpected text responses.</t>
+          <t>Connect: weather/holiday signal → demand_forecast surge → inventory shortage detection → ProcurementEnricher Instamart prices → ActionQueue APPROVE_REQUIRED action → trust ladder → checkout (staging creds) OR WhatsApp vendor fallback. This is the flagship restaurant OS demo moment. The plan output must clearly show: shortage detected → Instamart has it at Rs.24/kg → approve to order → or WhatsApp vendor if not on Instamart. Wire trust ladder: orders under Rs.500 auto-approved, over Rs.500 needs manual approval in action queue UI.</t>
         </is>
       </c>
       <c r="F32" s="137" t="inlineStr">
         <is>
-          <t>feat: structured outputs — force tool_choice=required in chatbot</t>
+          <t>feat: autonomous procurement loop — weather → forecast → shortage → Instamart → action queue</t>
         </is>
       </c>
       <c r="G32" s="137" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CLAUDE.md, docs/ARCHITECTURE.md (procurement loop diagram)</t>
         </is>
       </c>
       <c r="H32" s="138" t="inlineStr">
@@ -19171,7 +19179,7 @@
       </c>
       <c r="I32" s="136" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J32" s="136" t="inlineStr">
@@ -19184,10 +19192,14 @@
       <c r="M32" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N32" s="137" t="n"/>
+      <c r="N32" s="137" t="inlineStr">
+        <is>
+          <t>P6-A24</t>
+        </is>
+      </c>
       <c r="O32" s="137" t="inlineStr">
         <is>
-          <t>Chatbot always calls a tool when one applies; no unexpected freeform responses; existing chatbot tests pass</t>
+          <t>Full loop runs end-to-end in demo; trust ladder fires correctly; action queue shows Instamart procurement with price + spinId; WhatsApp fallback triggers when product not found on Instamart</t>
         </is>
       </c>
     </row>
@@ -19199,32 +19211,32 @@
       </c>
       <c r="B33" s="137" t="inlineStr">
         <is>
-          <t>feature/voice-interface</t>
+          <t>feature/instamart-event-supplies</t>
         </is>
       </c>
       <c r="C33" s="137" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D33" s="137" t="inlineStr">
         <is>
-          <t>Voice interface — Whisper transcription + TTS response</t>
+          <t>Instamart event supplies in operator chatbot</t>
         </is>
       </c>
       <c r="E33" s="137" t="inlineStr">
         <is>
-          <t>Restaurant operator speaks to CortexKitchen instead of typing. Browser MediaRecorder API captures audio. Whisper (via Groq) transcribes to text. Existing chatbot processes the text query. TTS reads back the response. Use case: manager walking the floor asks questions hands-free. "What does the plan say about staffing tonight?" "How many covers are we expecting?" Add mic button to existing /chat page. Works for operator side only initially.</t>
+          <t>Extend operator chatbot with event supplies tool: "we are hosting a birthday event tonight, need supplies." Calls search_products for non-food items: candles, paper plates, cups, napkins, soft drinks, basic decorations, cleaning supplies, batteries. Returns real Instamart prices and availability. Creates ActionQueue procurement action for approval. Key insight: Instamart is not just food ingredients — managers use it for quick supply runs that previously required leaving the restaurant. New chatbot tool: get_event_supplies(event_type, headcount)</t>
         </is>
       </c>
       <c r="F33" s="137" t="inlineStr">
         <is>
-          <t>feat: voice interface — Whisper transcription + TTS on /chat page</t>
+          <t>feat: Instamart event supplies tool in operator chatbot</t>
         </is>
       </c>
       <c r="G33" s="137" t="inlineStr">
         <is>
-          <t>docs/PRODUCT_MODES.md (voice mode section)</t>
+          <t>docs/AGENTS.md (chatbot tools updated)</t>
         </is>
       </c>
       <c r="H33" s="138" t="inlineStr">
@@ -19234,7 +19246,7 @@
       </c>
       <c r="I33" s="136" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J33" s="136" t="inlineStr">
@@ -19250,7 +19262,7 @@
       <c r="N33" s="137" t="n"/>
       <c r="O33" s="137" t="inlineStr">
         <is>
-          <t>Audio recorded and transcribed correctly; chatbot processes transcription; TTS plays response; mic button shows recording state</t>
+          <t>search_products returns real results for non-food queries; ActionQueue action created; trust ladder applied; chatbot responds naturally to event supply requests</t>
         </is>
       </c>
     </row>
@@ -19262,27 +19274,27 @@
       </c>
       <c r="B34" s="137" t="inlineStr">
         <is>
-          <t>feature/eval-pipeline</t>
+          <t>feature/structured-outputs</t>
         </is>
       </c>
       <c r="C34" s="137" t="inlineStr">
         <is>
-          <t>Eval</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D34" s="137" t="inlineStr">
         <is>
-          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
+          <t>Structured outputs — tool_choice=required across chatbot</t>
         </is>
       </c>
       <c r="E34" s="137" t="inlineStr">
         <is>
-          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
+          <t>Force structured JSON outputs from Groq function calling. Eliminates cases where chatbot returns freeform text instead of calling the right tool. Add response validation layer. Makes chatbot more reliable for demo — no unexpected text responses.</t>
         </is>
       </c>
       <c r="F34" s="137" t="inlineStr">
         <is>
-          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
+          <t>feat: structured outputs — force tool_choice=required in chatbot</t>
         </is>
       </c>
       <c r="G34" s="137" t="inlineStr">
@@ -19297,7 +19309,7 @@
       </c>
       <c r="I34" s="136" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J34" s="136" t="inlineStr">
@@ -19310,153 +19322,279 @@
       <c r="M34" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="137" t="inlineStr">
-        <is>
-          <t>P6-A27</t>
-        </is>
-      </c>
+      <c r="N34" s="137" t="n"/>
       <c r="O34" s="137" t="inlineStr">
         <is>
+          <t>Chatbot always calls a tool when one applies; no unexpected freeform responses; existing chatbot tests pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="136" t="inlineStr">
+        <is>
+          <t>P6-A33</t>
+        </is>
+      </c>
+      <c r="B35" s="137" t="inlineStr">
+        <is>
+          <t>feature/voice-interface</t>
+        </is>
+      </c>
+      <c r="C35" s="137" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D35" s="137" t="inlineStr">
+        <is>
+          <t>Voice interface — Whisper transcription + TTS response</t>
+        </is>
+      </c>
+      <c r="E35" s="137" t="inlineStr">
+        <is>
+          <t>Restaurant operator speaks to CortexKitchen instead of typing. Browser MediaRecorder API captures audio. Whisper (via Groq) transcribes to text. Existing chatbot processes the text query. TTS reads back the response. Use case: manager walking the floor asks questions hands-free. "What does the plan say about staffing tonight?" "How many covers are we expecting?" Add mic button to existing /chat page. Works for operator side only initially.</t>
+        </is>
+      </c>
+      <c r="F35" s="137" t="inlineStr">
+        <is>
+          <t>feat: voice interface — Whisper transcription + TTS on /chat page</t>
+        </is>
+      </c>
+      <c r="G35" s="137" t="inlineStr">
+        <is>
+          <t>docs/PRODUCT_MODES.md (voice mode section)</t>
+        </is>
+      </c>
+      <c r="H35" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I35" s="136" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J35" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K35" s="136" t="n"/>
+      <c r="L35" s="136" t="n"/>
+      <c r="M35" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="137" t="n"/>
+      <c r="O35" s="137" t="inlineStr">
+        <is>
+          <t>Audio recorded and transcribed correctly; chatbot processes transcription; TTS plays response; mic button shows recording state</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="136" t="inlineStr">
+        <is>
+          <t>P6-A34</t>
+        </is>
+      </c>
+      <c r="B36" s="137" t="inlineStr">
+        <is>
+          <t>feature/eval-pipeline</t>
+        </is>
+      </c>
+      <c r="C36" s="137" t="inlineStr">
+        <is>
+          <t>Eval</t>
+        </is>
+      </c>
+      <c r="D36" s="137" t="inlineStr">
+        <is>
+          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
+        </is>
+      </c>
+      <c r="E36" s="137" t="inlineStr">
+        <is>
+          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
+        </is>
+      </c>
+      <c r="F36" s="137" t="inlineStr">
+        <is>
+          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
+        </is>
+      </c>
+      <c r="G36" s="137" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H36" s="138" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I36" s="136" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J36" s="136" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K36" s="136" t="n"/>
+      <c r="L36" s="136" t="n"/>
+      <c r="M36" s="136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="137" t="inlineStr">
+        <is>
+          <t>P6-A30</t>
+        </is>
+      </c>
+      <c r="O36" s="137" t="inlineStr">
+        <is>
           <t>CI eval gate passes; golden_runs.json reflects current system; regressions caught in 2+ test scenarios</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="140" t="inlineStr">
         <is>
           <t>DOCS + SYNC — end of Phase 6A</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="136" t="inlineStr">
-        <is>
-          <t>P6-A33</t>
-        </is>
-      </c>
-      <c r="B37" s="137" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="136" t="inlineStr">
+        <is>
+          <t>P6-A35</t>
+        </is>
+      </c>
+      <c r="B39" s="137" t="inlineStr">
         <is>
           <t>feature/documentation</t>
         </is>
       </c>
-      <c r="C37" s="137" t="inlineStr">
+      <c r="C39" s="137" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D37" s="137" t="inlineStr">
+      <c r="D39" s="137" t="inlineStr">
         <is>
           <t>Whole-system documentation + screenshots refresh</t>
         </is>
       </c>
-      <c r="E37" s="137" t="inlineStr">
+      <c r="E39" s="137" t="inlineStr">
         <is>
           <t>Update all docs to reflect: new two-sided product vision, compliance changes (Zomato removed, market intel anonymised), autonomous procurement loop, weather signals, voice interface. New product vision statement in README. Screenshots of the operator portal (dashboard, operations, market, action queue, chat) for portfolio -- Guest Concierge screenshots belong to Phase 6B docs (P6-B9), not here, since Guest Concierge does not exist yet at this point.</t>
         </is>
       </c>
-      <c r="F37" s="137" t="inlineStr">
+      <c r="F39" s="137" t="inlineStr">
         <is>
           <t>docs: whole-system documentation refresh — new product vision</t>
         </is>
       </c>
-      <c r="G37" s="137" t="inlineStr">
+      <c r="G39" s="137" t="inlineStr">
         <is>
           <t>README.md, docs/ARCHITECTURE.md, docs/AGENTS.md, CLAUDE.md</t>
         </is>
       </c>
-      <c r="H37" s="138" t="inlineStr">
+      <c r="H39" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I37" s="136" t="inlineStr">
+      <c r="I39" s="136" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J37" s="136" t="inlineStr">
+      <c r="J39" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K37" s="136" t="n"/>
-      <c r="L37" s="136" t="n"/>
-      <c r="M37" s="136" t="n">
+      <c r="K39" s="136" t="n"/>
+      <c r="L39" s="136" t="n"/>
+      <c r="M39" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N37" s="137" t="inlineStr">
-        <is>
-          <t>P6-A32</t>
-        </is>
-      </c>
-      <c r="O37" s="137" t="inlineStr">
+      <c r="N39" s="137" t="inlineStr">
+        <is>
+          <t>P6-A34</t>
+        </is>
+      </c>
+      <c r="O39" s="137" t="inlineStr">
         <is>
           <t>README reflects two-sided platform; all compliance changes documented; screenshots current</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="136" t="inlineStr">
-        <is>
-          <t>P6-A34</t>
-        </is>
-      </c>
-      <c r="B38" s="137" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="136" t="inlineStr">
+        <is>
+          <t>P6-A36</t>
+        </is>
+      </c>
+      <c r="B40" s="137" t="inlineStr">
         <is>
           <t>dev -&gt; main</t>
         </is>
       </c>
-      <c r="C38" s="137" t="inlineStr">
+      <c r="C40" s="137" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
-      <c r="D38" s="137" t="inlineStr">
+      <c r="D40" s="137" t="inlineStr">
         <is>
           <t>Sync Phase 6A to main</t>
         </is>
       </c>
-      <c r="E38" s="137" t="inlineStr">
+      <c r="E40" s="137" t="inlineStr">
         <is>
           <t>Merge dev → main. All compliance fixes confirmed. Autonomous procurement loop working (minus checkout — staging creds). Restaurant OS demo-ready. Phase 6B starts after this.</t>
         </is>
       </c>
-      <c r="F38" s="137" t="inlineStr">
+      <c r="F40" s="137" t="inlineStr">
         <is>
           <t>release: Phase 6A complete — restaurant OS + compliance fixes</t>
         </is>
       </c>
-      <c r="G38" s="137" t="inlineStr">
+      <c r="G40" s="137" t="inlineStr">
         <is>
           <t>README.md</t>
         </is>
       </c>
-      <c r="H38" s="138" t="inlineStr">
+      <c r="H40" s="138" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="I38" s="136" t="inlineStr">
+      <c r="I40" s="136" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J38" s="136" t="inlineStr">
+      <c r="J40" s="136" t="inlineStr">
         <is>
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K38" s="136" t="n"/>
-      <c r="L38" s="136" t="n"/>
-      <c r="M38" s="136" t="n">
+      <c r="K40" s="136" t="n"/>
+      <c r="L40" s="136" t="n"/>
+      <c r="M40" s="136" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="137" t="inlineStr">
-        <is>
-          <t>P6-A33</t>
-        </is>
-      </c>
-      <c r="O38" s="137" t="inlineStr">
+      <c r="N40" s="137" t="inlineStr">
+        <is>
+          <t>P6-A35</t>
+        </is>
+      </c>
+      <c r="O40" s="137" t="inlineStr">
         <is>
           <t>Full test suite green; compliance fixes verified; no Zomato references; market intel anonymised; demo flow works</t>
         </is>
@@ -19464,7 +19602,7 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A36:O36"/>
+    <mergeCell ref="A38:O38"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A22:O22"/>
     <mergeCell ref="A18:O18"/>
@@ -19990,7 +20128,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>search_products for decorations, cake, drinks, party supplies matching the event brief -- same tool pattern as the Restaurant OS operator-facing get_event_supplies (P6-A28), but consumer-facing and for the guest's own event rather than restaurant procurement. Cart/checkout once creds land.</t>
+          <t>search_products for decorations, cake, drinks, party supplies matching the event brief -- same tool pattern as the Restaurant OS operator-facing get_event_supplies (P6-A31), but consumer-facing and for the guest's own event rather than restaurant procurement. Cart/checkout once creds land.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -20700,7 +20838,7 @@
       </c>
       <c r="N14" s="59" t="inlineStr">
         <is>
-          <t>P6-A31</t>
+          <t>P6-A33</t>
         </is>
       </c>
       <c r="O14" s="59" t="inlineStr">
@@ -22358,7 +22496,7 @@
       </c>
       <c r="E63" s="59" t="inlineStr">
         <is>
-          <t>Audit test coverage for every new service/model added in Phase 6A (Action Queue, workflow triggers, trust-ladder, WhatsApp vendor flow, Vendor/Supplier model, Menu Engineering Matrix) -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (workflow-triggered actions, trust-ladder promotions), since the existing eval sets predate all of this and won't catch regressions in it. (Docs + screenshots refresh is P6-A33, done before the demo video; this is the deeper test/CI/eval hygiene pass that doesn't need to block the video.)</t>
+          <t>Audit test coverage for every new service/model added in Phase 6A (Action Queue, workflow triggers, trust-ladder, WhatsApp vendor flow, Vendor/Supplier model, Menu Engineering Matrix) -- confirm nothing shipped without tests. Re-check the CI pipeline includes all new test files. Re-run/expand RAGAS + DeepEval evals to cover the new agentic behaviors (workflow-triggered actions, trust-ladder promotions), since the existing eval sets predate all of this and won't catch regressions in it. (Docs + screenshots refresh is P6-A35, done before the demo video; this is the deeper test/CI/eval hygiene pass that doesn't need to block the video.)</t>
         </is>
       </c>
       <c r="F63" s="59" t="inlineStr">

</xml_diff>

<commit_message>
feat: P6-A21 -- weather + Indian holiday signals with real forecast adjustment
Adds WeatherService (Open-Meteo, no API key) and a shared calendar_utils
holiday lookup, then applies a real deterministic multiplier to Prophet's
raw forecast (ForecastService._apply_signal_adjustments) instead of only
changing narrative prompt text -- pre-adjustment value, multiplier, and
reasons are all preserved for transparency. Wired into ScenarioRecommender,
GET /market/pulse (independent of swiggy_connected), and a new Weather &
Holidays card on /market. Zero Swiggy MCP involvement.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -18576,7 +18576,7 @@
       </c>
       <c r="E23" s="137" t="inlineStr">
         <is>
-          <t>First of four independently-failing live-intelligence services feeding the planning pipeline (P6-A24 unifies all four). New WeatherService (infrastructure/external/weather_service.py) calls Open-Meteo (free, no API key) for current + 48h forecast at the restaurant's location -- rain/heat forecasts shift the plan toward delivery-heavy staffing and prep, clear days toward walk-in/outdoor capacity. INDIAN_HOLIDAYS_2026 already exists in core/constants.py and already feeds ScenarioRecommender in the background -- this task surfaces it explicitly into demand_forecast's own prompt too ('today is Gandhi Jayanti -- public holiday, expect elevated demand'), not just the scenario suggestion. Never raises -- returns None on any failure so demand_forecast runs fine without it. New OrchestratorState field: weather_signal.</t>
+          <t>DONE on feature/live-intelligence-signals. New WeatherService (infrastructure/external/weather_service.py) -- Open-Meteo, free, keyless -- averages temperature/precipitation across the target date's 18:00-22:00 dinner window, classifies heavy_rain/light_rain/very_hot/clear, returns a conservative demand_multiplier (1.03-1.10) plus descriptive delivery_impact/dinein_impact strings. New app/core/calendar_utils.py extracts the holiday/weekend lookup that used to live only inside ScenarioRecommender._date_context, so it's shared rather than duplicated as a second consumer (demand_forecast) needed it. THE ACTUAL FIX: ForecastService._apply_signal_adjustments() applies a deterministic multiplier (holiday x1.4, weather x1.03-1.10, stacked when both apply) to Prophet's raw predicted_orders/predicted_peak_orders -- previously weather/holiday would only ever have reached the LLM recommendation step as narrative text it may or may not act on; now they move the actual predicted number. Transparent by construction: predicted_orders_pre_adjustment, adjustment_multiplier, and adjustment_reasons are all preserved alongside the adjusted figure, so nothing is a silent change to what Prophet said. demand_forecast_node fetches both signals and passes them into analyse_and_recommend(); writes state['weather_signal']. ScenarioRecommender also wired to use the weather signal alongside its existing holiday context. GET /market/pulse returns weather + upcoming_holiday (a cheap 14-day dict scan against INDIAN_HOLIDAYS_2026, no API call) -- both explicitly independent of swiggy_connected, since neither is Swiggy MCP; the original handler had an early return on Swiggy-unavailable that would have hidden both, fixed during implementation. New 'Weather &amp; Holidays' card on /market (SwiggyLiveMarketPanel.tsx) -- also fixed the same early-return bug on the frontend side so the card renders even when Swiggy isn't connected. Default coordinates (core/constants.py: DEFAULT_RESTAURANT_LAT/LNG, Navi Mumbai, matching SWIGGY_ADDRESS_ID's approximate area) used since RestaurantProfile has no stored lat/lng column. As a side effect, fixed a pre-existing environment issue: reportlab was declared in requirements.txt but never actually installed, breaking test_pdf_export.py's collection (11 tests) -- installed, unrelated to this task's code but blocking a clean full-suite run.</t>
         </is>
       </c>
       <c r="F23" s="137" t="inlineStr">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="H23" s="138" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I23" s="136" t="inlineStr">
@@ -18607,12 +18607,12 @@
       <c r="K23" s="136" t="n"/>
       <c r="L23" s="136" t="n"/>
       <c r="M23" s="136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" s="137" t="n"/>
       <c r="O23" s="137" t="inlineStr">
         <is>
-          <t>Weather API call returns current+forecast conditions for a known lat/lng and gracefully degrades to None on API failure; holiday lookup correctly identifies a known date against INDIAN_HOLIDAYS_2026; both signals appear in demand_forecast's prompt on a known test date</t>
+          <t>VERIFIED: 519 backend tests pass (498 pre-existing + 21 new across test_calendar_utils.py, test_weather_service.py, test_forecast_signal_adjustments.py -- classification thresholds, dinner-window extraction, fail-open on HTTP error/malformed response/out-of-range date, multiplier math including holiday+weather stacking, and the predicted_orders_pre_adjustment/adjustment_multiplier/adjustment_reasons transparency fields); frontend typechecks clean (npx tsc --noEmit, zero errors); zero regressions in existing ScenarioRecommender/ForecastService/demand_forecast tests since all new params are optional with defaults.</t>
         </is>
       </c>
     </row>
@@ -19459,6 +19459,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="140" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: update CLAUDE.md + tracker for P6-A27 -- Langfuse tracing + Kindred replay endpoint done
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -18817,18 +18817,52 @@
           <t>Observability</t>
         </is>
       </c>
-      <c r="D29" s="108" t="n"/>
-      <c r="E29" s="108" t="n"/>
-      <c r="F29" s="108" t="n"/>
-      <c r="G29" s="108" t="n"/>
-      <c r="H29" s="109" t="n"/>
-      <c r="I29" s="107" t="n"/>
-      <c r="J29" s="107" t="n"/>
+      <c r="D29" s="108" t="inlineStr">
+        <is>
+          <t>Observability: Langfuse tracing + Kindred replay debugging endpoint</t>
+        </is>
+      </c>
+      <c r="E29" s="108" t="inlineStr">
+        <is>
+          <t>DONE on feature/kindred. Instruments the planning pipeline with Langfuse (langfuse.langchain.CallbackHandler attached to run_planning_scenario/stream_planning_scenario's RunnableConfig -- one span per LangGraph node per run, zero code change inside the nodes themselves) plus a new BaseLLMProvider._trace_generation() helper called from all 3 concrete providers (Groq/Gemini/Comet) right after record_usage(), so every individual LLM call shows up as its own Langfuse generation (real prompt/completion/token usage), not just which node ran. New settings: LANGFUSE_PUBLIC_KEY/SECRET_KEY/HOST/BASE_URL (SDK checks both host names, so both are supported), KINDRED_AGENT_ID, KINDRED_API_KEY (registered, currently unused -- no documented use case found). New POST /replay (app/api/routes/replay.py), mounted directly on the app in main.py at a bare root path (not under /api/v1) since that's Kindred's Configure Replay URL convention. Kindred replays at the level of one LLM generation, not a whole run -- confirmed from real request logs, which carry back exactly the [system, user] messages array captured for one observation. /replay reuses BaseLLMProvider.complete() directly (the same call path every node already uses) for that one call -- an initial version instead misrouted unrecognised input through ScenarioProfileService.derive_profile() and reran the full 11-node graph per replay (6+ LLM calls), which is both semantically wrong and is what burned a full Groq daily token quota (100k TPD) in 3 live replay clicks before the fix. All 5 Kindred replay metadata fields (kindred_replay_run_id/kindred_original_session_id/kindred_include_prior_context/kindred_turn_trace_id/is_replay) plus their 5 X-Kindred-* header equivalents are threaded onto the Langfuse trace via propagate_attributes(), not just the HTTP response, matching Kindred's own polling-by-trace-metadata model. session_id was originally f'org-{org_id}' (grouping every run from one org into one Langfuse session) -- found live to actively break Kindred's original&lt;-&gt;replay matching (one session had pooled 199 unrelated observations across many runs); changed to scope session_id to the individual run_id instead, which fixed the original/replay trace-tree structure lining up 1:1. ngrok (winget-installed 3.3.1) needed a manual `ngrok update` to 3.39.9 -- the Kindred-linked account requires &gt;=3.20.0. Fail-open throughout: every new code path no-ops when LANGFUSE_SECRET_KEY is unset, exactly like the existing LangSmith integration. KNOWN GAP, Kindred-side not ours: Kindred's own Reproducibility comparison view never renders the original/Reference output for the Agent Output step, even after the session fix gave it a matching trace structure -- directly verified via Langfuse's public API that the original data is fully present and correctly formatted in every case checked, so this is a gap in Kindred's own matching/rendering, not a data or formatting problem on our side. Full-graph replay ("turn 9"/root-span selection in Kindred, or true node re-execution with reconstructed state so a code change downstream could be caught) was scoped and deliberately not built -- would need LangGraph checkpointing that doesn't exist yet, and reopens real LLM cost per replay; explicit product decision to leave for a future task if it becomes a real recurring need.</t>
+        </is>
+      </c>
+      <c r="F29" s="108" t="inlineStr">
+        <is>
+          <t>feat: P6-A27 -- Langfuse tracing + Kindred replay endpoint</t>
+        </is>
+      </c>
+      <c r="G29" s="108" t="inlineStr">
+        <is>
+          <t>CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H29" s="109" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I29" s="107" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J29" s="107" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
       <c r="K29" s="107" t="n"/>
       <c r="L29" s="107" t="n"/>
-      <c r="M29" s="107" t="n"/>
+      <c r="M29" s="107" t="n">
+        <v>1</v>
+      </c>
       <c r="N29" s="108" t="n"/>
-      <c r="O29" s="108" t="n"/>
+      <c r="O29" s="108" t="inlineStr">
+        <is>
+          <t>VERIFIED: 544/544 backend tests pass (no new tests added -- Kindred's own setup prompt explicitly said not to add unrelated tests; existing suite confirms no regressions). Live end-to-end verification (not just unit tests): POST /replay smoke-tested repeatedly against the running local server, confirmed HTTP 200 + correct JSON shape (session_id/run_id/kindred_replay_run_id/output) every time. Cross-checked directly against Langfuse's public API (not just its UI) that resulting traces carry agent_id/session_id/kindred_replay_run_id/is_replay metadata correctly, and that every generation observation (original run's 8 LLM calls and every replay's 1 call) has complete input/output. ngrok tunnel verified reachable end-to-end (GET / through the public URL returned 200). Real Kindred replay runs executed against the live tunnel confirmed the fixed endpoint returns the correct single-step output fast (~1-9s) instead of the original bug's 20-130s full-pipeline reruns.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="52.05" customHeight="1" s="84">
       <c r="A30" s="80" t="inlineStr">

</xml_diff>

<commit_message>
tracker: full Phase 6A replan -- from-scratch IA redesign (Dashboard/Planning split, Action Center, Analytics, Admin) + seed data dynamism fix
Mark P6-A28 (Data page merge) Completed. Insert P6-A29-A33: seed data
redesign (fixes the hardcoded random.seed(42) + always-same-3-shortages +
hardcoded popular-dish bias found in a live agent-prompt hardcoding audit),
Dashboard/Planning split, Action Center as its own primary-nav page,
Analytics (new page, absorbs the previously-standalone Menu Engineering
Matrix task), and Admin (Planning History + Data Health relocated from the
P6-A28 Data page, plus new Observability/AI Infrastructure panels).
Cascade-renumbers A30-A37 to A34-A41, fixing cross-referencing Depends On
cells that pointed at old task numbers.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -17209,7 +17209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="84" min="1" max="1"/>
@@ -18887,12 +18887,12 @@
       </c>
       <c r="E30" s="81" t="inlineStr">
         <is>
-          <t>Real-product IA decision: a manager doesn't think of 'run history' as a separate audit concept from 'system data/health' -- merges /runs (plan run history, currently the weakest-looking screen: dense monospace debug trace) and /data-health (sync status, freshness) into one 'Data' page with clearly separated sections, applying the existing design system instead of the current raw trace view. Adds a new section with no home anywhere today: Action Queue history -- the audit trail of every action approved/rejected/executed over time (restocks sent, WhatsApp messages, pricing reviews). Fixes the known unstyled /runs/{id} deep-link 404 while in here.</t>
+          <t>DONE on feature/page-redesign. Merged /runs (plan run history) and /data-health (sync status, freshness) into one /data page, applying the design-system tokens both pages already used (neither was actually the "dense monospace debug trace" this task's original description assumed -- that description was stale). Extracted both into components/data/RunHistorySection.tsx and DataHealthSection.tsx, plus new components/data/ActionQueueHistory.tsx -- an audit trail of approved/rejected/executed actions with no home anywhere before, built entirely on the existing GET /api/v1/action-queue endpoint (omitting the status filter already returns full history, no backend change needed). Fixed the /runs/{id} 404 for real: there was never a dynamic route for it (run selection was pure React state, never a URL segment) -- added app/runs/[id]/ redirecting to /data?run=&lt;id&gt;, plus /runs and /data-health now redirect to /data for old bookmarks. NavBar's separate Runs/Data entries merged into one. Badge component extended with pending/executed/expired variants. Also removed apps/web/cortexkitchen-ui/AGENTS.md and its CLAUDE.md (an @AGENTS.md-only file) -- AGENTS.md told coding agents to read node_modules/next/dist/docs before writing code, and that folder contains a real injected prompt-injection comment posing as an "AI agent hint" pointing at a non-existent unstable_instant API. npx tsc --noEmit and npx eslint both clean, manually verified in browser. SUPERSEDED IN PART by P6-A30/A31/A33 below: after a from-scratch IA redesign discussion, RunHistorySection relocates to Admin (P6-A33), DataHealthSection relocates to Admin (P6-A33), and ActionQueueHistory relocates to the new Action Center (P6-A31) -- the /data route itself will stop being the destination once those land. Marked Completed because the work genuinely happened, was tested, and is live -- not retroactively erased by being reorganized again, same as how P6-A26 also intentionally gets partially restructured by this same IA pass.</t>
         </is>
       </c>
       <c r="F30" s="81" t="inlineStr">
         <is>
-          <t>feat: Data page redesign -- merge /runs + /data-health, add Action Queue history</t>
+          <t>feat: P6-A28 -- merge /runs + /data-health into /data, add Action Queue history</t>
         </is>
       </c>
       <c r="G30" s="81" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="H30" s="82" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I30" s="80" t="inlineStr">
@@ -18918,12 +18918,12 @@
       <c r="K30" s="80" t="n"/>
       <c r="L30" s="80" t="n"/>
       <c r="M30" s="80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N30" s="81" t="n"/>
       <c r="O30" s="81" t="inlineStr">
         <is>
-          <t>/runs and /data-health content both accessible from one page with consistent design-system styling; direct navigation to /runs/{id} deep-link renders the run, not a 404; Action Queue history shows past actions with correct status/timestamps</t>
+          <t>VERIFIED: npx tsc --noEmit and npx eslint clean; manually clicked through /data (Run History, Data Health, Action Queue History, NavBar) in a running browser and confirmed all render correctly; /runs, /runs/123, /data-health all correctly redirect.</t>
         </is>
       </c>
     </row>
@@ -18940,27 +18940,27 @@
       </c>
       <c r="C31" s="81" t="inlineStr">
         <is>
-          <t>Frontend</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D31" s="81" t="inlineStr">
         <is>
-          <t>Menu engineering matrix UI</t>
+          <t>Seed data redesign -- dynamic reseeding, remove fixed random seed and hardcoded shortages/popular dishes</t>
         </is>
       </c>
       <c r="E31" s="81" t="inlineStr">
         <is>
-          <t>Visual matrix: dish margin (y-axis) vs order popularity (x-axis). Four quadrants: Stars (high margin + high orders — promote), Plowhorses (low margin + high orders — reprice or remove), Puzzles (high margin + low orders — market better), Dogs (low margin + low orders — remove). Data from BusinessAnalyticsService (already has margin + popularity). Interactive: click a dish to see full margin breakdown. Shown on the new Data page (P6-A27), not /operations -- /operations is merged into Today Dashboard (P6-A26) and this is analytical/historical review, not a daily trigger-time decision, so it belongs with run history, not the plan-trigger flow. Connects to planning: critic uses quadrant data to validate menu recommendations.</t>
+          <t>Prompted by a full agent-prompt hardcoding audit (this session): no hardcoding exists in any of the 11 LangGraph node prompts themselves -- every node pulls real DB-derived data into f-string templates, and the two literal-ingredient fixtures found (inventory.py, menu_intelligence.py) are gated behind simulation_mode=True, never set by the frontend, dead code in production. The actual problem is scripts/seed_demo_data.py: random.seed(42) is hardcoded (line 117), so every reseed is byte-for-byte identical except for dates (which ARE already correctly relative to today -- no staleness bug there). Exactly 3 of 18 inventory items (Mozzarella Cheese, Fresh Basil, Garlic) are EVER below threshold, at fixed literal quantities, every single day, forever. A hardcoded popular_pizza set ({Margherita, Pepperoni Feast, Chicken Tikka Pizza}) biases 70% of Friday order generation toward exactly those 3 dishes. Decision-log/RAG memory literally states the same 3 ingredients as retrievable "past context" (line 599), so qdrant_enrichment's retrieval feeds the same names back to the LLM as supposedly-independent corroborating memory, compounding the appearance of scripted output even though the retrieval mechanism itself is genuinely real. Only 3 vendors and 3 VendorPriceQuote rows total, covering just 2 ingredients. Fix: seed by today's date (deterministic within a single day, so a demo session doesn't shift under you mid-demo, but genuinely different data day to day -- replaces the permanently-frozen dataset); randomize which N of 18 inventory items go short each day (weighted so 1-4 are reliably short for demo purposes, but never always the same 3); rotate/randomize the popular-dish set instead of a fixed 3-item constant; generate decision-log/RAG memory content dynamically from whatever was actually seeded that day rather than literal hardcoded text; expand vendor/price-quote coverage beyond 2 ingredients so procurement recommendations aren't artificially narrow either. Foundation for P6-A32 (Analytics) and P6-A33 (Admin/Observability) -- both would otherwise visualize the same frozen 3 ingredients/3 dishes no matter how good the UI is.</t>
         </is>
       </c>
       <c r="F31" s="81" t="inlineStr">
         <is>
-          <t>feat: menu engineering matrix — margin vs popularity quadrant chart</t>
+          <t>feat: seed data redesign -- date-based seeding, randomized shortages/popular dishes, dynamic RAG memory</t>
         </is>
       </c>
       <c r="G31" s="81" t="inlineStr">
         <is>
-          <t>None (frontend only)</t>
+          <t>CLAUDE.md, docs/ARCHITECTURE.md</t>
         </is>
       </c>
       <c r="H31" s="82" t="inlineStr">
@@ -18970,7 +18970,7 @@
       </c>
       <c r="I31" s="80" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J31" s="80" t="inlineStr">
@@ -18983,14 +18983,10 @@
       <c r="M31" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="N31" s="81" t="inlineStr">
-        <is>
-          <t>P6-A27</t>
-        </is>
-      </c>
+      <c r="N31" s="81" t="n"/>
       <c r="O31" s="81" t="inlineStr">
         <is>
-          <t>Matrix renders with correct quadrant assignment; click through shows dish margin detail; Stars/Plowhorses/Puzzles/Dogs correctly classified</t>
+          <t>Running the seed script twice on the same real-world day produces identical data (deterministic within a day); running it on two different days produces different shortage items and different popular dishes; no single ingredient/dish is hardcoded as always-short/always-popular in the script; RAG/decision-log memory content matches whatever was actually seeded that day, not a fixed string; at least 3 vendors offer quotes across at least 6 distinct ingredients.</t>
         </is>
       </c>
     </row>
@@ -19007,27 +19003,27 @@
       </c>
       <c r="C32" s="81" t="inlineStr">
         <is>
-          <t>Eval</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D32" s="81" t="inlineStr">
         <is>
-          <t>Validate action-item specificity after live signals land (conditional)</t>
+          <t>Split /dashboard into Dashboard (overview) and Planning (flagship pipeline experience)</t>
         </is>
       </c>
       <c r="E32" s="81" t="inlineStr">
         <is>
-          <t>Not a guaranteed code task -- a validation checkpoint. Research confirmed aggregator.py/critic_service.py already favor structured, itemized output (bulleted restock actions, explicit dish names, numeric thresholds, dimension scores) over narrative paragraphs, so the 'standard, generic response' feedback is more likely an input-richness problem than a prompt-engineering problem. After P6-A24 ships, manually review 3-5 generated plans against known-rich live-signal test dates (a rain-forecast night, a real upcoming holiday, an active trend, a live FSSAI notice) to check whether output is now sufficiently specific/actionable. If yes: close this task, no further work needed. If still generic: scope a real follow-up prompt-engineering task against aggregator/critic with concrete before/after examples.</t>
+          <t>Real-product IA decision, from a from-scratch v1 redesign discussion: a manager wants a fast overview (health score, KPIs, live intelligence) most of the time, and a smaller number of times wants to actually watch/inspect a plan being generated in depth -- two different jobs currently living on one route (/dashboard) via conditional rendering between TodayIdleState.tsx (idle) and the post-trigger success view. Splits the existing idle state (already has health score, net profit/margin, revenue trend, weather/holiday/market context strip via TodayContextStrip, and the scenario trigger flow) into a leaner /dashboard, and moves the existing success view (ForecastChart, AgentCard x4, CriticBanner, ActionQueuePanel) into a new /planning page that becomes the flagship experience. /planning gains two things that didn't exist before: a per-node observability strip (status/runtime/tokens/model/cost per node -- data already captured in node_traces/llm_usage inside run metadata, just never surfaced in the UI) and an explicit Evidence section listing which data sources fed the plan (Swiggy/weather/RSS/FSSAI/RAG -- already computed as market_intel_output/live_signals_text/rag_context, just never labelled as "evidence" in one place for the user). PDF/Excel export relocates here from Data/Run History (P6-A28) since it's about the current run, not historical browsing.</t>
         </is>
       </c>
       <c r="F32" s="81" t="inlineStr">
         <is>
-          <t>None yet -- validation checkpoint, code only if the review finds a real gap</t>
+          <t>feat: split /dashboard into Dashboard (overview) + Planning (flagship pipeline experience)</t>
         </is>
       </c>
       <c r="G32" s="81" t="inlineStr">
         <is>
-          <t>None yet</t>
+          <t>docs/PRODUCT_MODES.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H32" s="82" t="inlineStr">
@@ -19037,7 +19033,7 @@
       </c>
       <c r="I32" s="80" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J32" s="80" t="inlineStr">
@@ -19052,12 +19048,12 @@
       </c>
       <c r="N32" s="81" t="inlineStr">
         <is>
-          <t>P6-A24, P6-A26</t>
+          <t>P6-A28</t>
         </is>
       </c>
       <c r="O32" s="81" t="inlineStr">
         <is>
-          <t>N/A -- manual review checkpoint, not an automated test</t>
+          <t>/dashboard shows health score/KPIs/live intelligence/trigger only, no pipeline detail; /planning shows the full pipeline run (trigger -&gt; node-by-node progress -&gt; generated plan -&gt; critic verdict -&gt; evidence -&gt; export); per-node cost/token/model visible during and after a run; existing scenario-trigger flow (presets + natural language, P6-A25) works identically from its new home.</t>
         </is>
       </c>
     </row>
@@ -19069,32 +19065,32 @@
       </c>
       <c r="B33" s="81" t="inlineStr">
         <is>
-          <t>feature/procurement-loop-endtoend</t>
+          <t>feature/page-redesign</t>
         </is>
       </c>
       <c r="C33" s="81" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D33" s="81" t="inlineStr">
         <is>
-          <t>Autonomous procurement loop — end-to-end wire</t>
+          <t>Action Center -- pending + historical actions as their own primary-nav page</t>
         </is>
       </c>
       <c r="E33" s="81" t="inlineStr">
         <is>
-          <t>Connect: weather/holiday signal → demand_forecast surge → inventory shortage detection → ProcurementEnricher Instamart prices → ActionQueue APPROVE_REQUIRED action → trust ladder → checkout (staging creds) OR WhatsApp vendor fallback. This is the flagship restaurant OS demo moment. The plan output must clearly show: shortage detected → Instamart has it at Rs.24/kg → approve to order → or WhatsApp vendor if not on Instamart. Wire trust ladder: orders under Rs.500 auto-approved, over Rs.500 needs manual approval in action queue UI.</t>
+          <t>The Action Queue (pending approvals) and Action Queue History (built in P6-A28, currently living inside the Data page) both relocate to a new dedicated /action-center page with its own primary-nav entry -- approving/rejecting real actions (restocks, WhatsApp vendor orders, pricing reviews) is a distinct daily job from either planning or historical data browsing, and deserves its own home rather than being a sub-section of something else. Reuses ActionQueuePanel and components/data/ActionQueueHistory.tsx (P6-A28) as-is, just relocated, plus adds status-filter tabs (pending/approved/executed/rejected/expired) instead of one combined feed. No backend change needed -- GET /api/v1/action-queue already supports an optional status filter.</t>
         </is>
       </c>
       <c r="F33" s="81" t="inlineStr">
         <is>
-          <t>feat: autonomous procurement loop — weather → forecast → shortage → Instamart → action queue</t>
+          <t>feat: Action Center -- pending + historical actions as their own primary-nav page</t>
         </is>
       </c>
       <c r="G33" s="81" t="inlineStr">
         <is>
-          <t>CLAUDE.md, docs/ARCHITECTURE.md (procurement loop diagram)</t>
+          <t>CLAUDE.md</t>
         </is>
       </c>
       <c r="H33" s="82" t="inlineStr">
@@ -19104,7 +19100,7 @@
       </c>
       <c r="I33" s="80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J33" s="80" t="inlineStr">
@@ -19119,12 +19115,12 @@
       </c>
       <c r="N33" s="81" t="inlineStr">
         <is>
-          <t>P6-A24</t>
+          <t>P6-A28</t>
         </is>
       </c>
       <c r="O33" s="81" t="inlineStr">
         <is>
-          <t>Full loop runs end-to-end in demo; trust ladder fires correctly; action queue shows Instamart procurement with price + spinId; WhatsApp fallback triggers when product not found on Instamart</t>
+          <t>/action-center shows pending actions (approve/reject working, unchanged behavior) and full history with status-filter tabs; NavBar has a dedicated Action Center entry; /dashboard and /data no longer show Action Queue content (relocated, not duplicated).</t>
         </is>
       </c>
     </row>
@@ -19136,32 +19132,32 @@
       </c>
       <c r="B34" s="81" t="inlineStr">
         <is>
-          <t>feature/instamart-event-supplies</t>
+          <t>feature/page-redesign</t>
         </is>
       </c>
       <c r="C34" s="81" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D34" s="81" t="inlineStr">
         <is>
-          <t>Instamart event supplies in operator chatbot</t>
+          <t>Analytics -- new historical drill-down page (absorbs Menu Engineering Matrix)</t>
         </is>
       </c>
       <c r="E34" s="81" t="inlineStr">
         <is>
-          <t>Extend operator chatbot with event supplies tool: "we are hosting a birthday event tonight, need supplies." Calls search_products for non-food items: candles, paper plates, cups, napkins, soft drinks, basic decorations, cleaning supplies, batteries. Returns real Instamart prices and availability. Creates ActionQueue procurement action for approval. Key insight: Instamart is not just food ingredients — managers use it for quick supply runs that previously required leaving the restaurant. New chatbot tool: get_event_supplies(event_type, headcount)</t>
+          <t>New page, doesn't exist today in any form. Five sections per the v1 redesign: Business (revenue/orders/AOV/forecast accuracy, from business_analytics_service.py + the existing GET /business/performance endpoint -- already partially surfaced on the old Dashboard idle state, gets a proper historical/trend home here instead), Customers (ratings/complaints/sentiment/repeat, from complaint_intelligence + feedback data), Menu (top sellers/low performers/profitability -- this section IS the previously-separate Menu Engineering Matrix task: dish margin vs. order popularity, four quadrants Stars/Plowhorses/Puzzles/Dogs, from BusinessAnalyticsService's existing margin+popularity data, click-through to full dish margin detail), Operations (occupancy/service time/wait time/table turnover, from reservation + complaint data), Inventory (stock health/waste/supplier performance/food cost, from inventory + vendor data). Absorbs the standalone Menu Engineering Matrix task rather than building it in isolation, since it's genuinely a peer of the other 4 analytics sections, not a run-history concern. Depends on P6-A29 landing first -- otherwise every section visualizes the same permanently-frozen 3 ingredients/3 dishes no matter how good the charts are.</t>
         </is>
       </c>
       <c r="F34" s="81" t="inlineStr">
         <is>
-          <t>feat: Instamart event supplies tool in operator chatbot</t>
+          <t>feat: Analytics page -- business/customers/menu/operations/inventory drill-down, includes menu engineering matrix</t>
         </is>
       </c>
       <c r="G34" s="81" t="inlineStr">
         <is>
-          <t>docs/AGENTS.md (chatbot tools updated)</t>
+          <t>docs/ARCHITECTURE.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H34" s="82" t="inlineStr">
@@ -19171,7 +19167,7 @@
       </c>
       <c r="I34" s="80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J34" s="80" t="inlineStr">
@@ -19184,10 +19180,14 @@
       <c r="M34" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="81" t="n"/>
+      <c r="N34" s="81" t="inlineStr">
+        <is>
+          <t>P6-A29, P6-A27</t>
+        </is>
+      </c>
       <c r="O34" s="81" t="inlineStr">
         <is>
-          <t>search_products returns real results for non-food queries; ActionQueue action created; trust ladder applied; chatbot responds naturally to event supply requests</t>
+          <t>All 5 sections render with real, varying data across different seed days; Menu section's quadrant chart correctly classifies dishes into Stars/Plowhorses/Puzzles/Dogs and supports click-through to margin detail; date-range filter (7/14/30-day) works across sections.</t>
         </is>
       </c>
     </row>
@@ -19199,32 +19199,32 @@
       </c>
       <c r="B35" s="81" t="inlineStr">
         <is>
-          <t>feature/structured-outputs</t>
+          <t>feature/page-redesign</t>
         </is>
       </c>
       <c r="C35" s="81" t="inlineStr">
         <is>
-          <t>Agents</t>
+          <t>Frontend</t>
         </is>
       </c>
       <c r="D35" s="81" t="inlineStr">
         <is>
-          <t>Structured outputs — tool_choice=required across chatbot</t>
+          <t>Admin -- secondary-nav section: Planning History, Data Health, Observability, AI Infrastructure, Audit Trail, Integrations</t>
         </is>
       </c>
       <c r="E35" s="81" t="inlineStr">
         <is>
-          <t>Force structured JSON outputs from Groq function calling. Eliminates cases where chatbot returns freeform text instead of calling the right tool. Add response validation layer. Makes chatbot more reliable for demo — no unexpected text responses.</t>
+          <t>New secondary-nav area (not a primary NavBar tab), for operational/technical concerns rather than daily manager workflows. Planning History and Data Health relocate here verbatim from the Data page built in P6-A28 (components/data/RunHistorySection.tsx, DataHealthSection.tsx -- reused as-is, just moved). Two genuinely new panels: Observability (per-run node_traces/llm_usage already captured in run metadata, plus Langfuse traces from P6-A27, surfaced as a real UI for the first time -- status/latency/errors per node/run) and AI Infrastructure (model/provider routing per node, token usage, cost breakdown -- same underlying llm_usage data sliced differently, plus which comet_tiered model tier served which node when tiered routing is active). Audit Trail is effectively the same data as Action Center's history (P6-A31) but framed as a compliance/audit view rather than an action-management view -- shared component, not a duplicate build. Integrations expands the existing /connectors page's Swiggy-only status view to also show Redis/Postgres/Qdrant/WhatsApp(Twilio)/RSS/Weather connectivity.</t>
         </is>
       </c>
       <c r="F35" s="81" t="inlineStr">
         <is>
-          <t>feat: structured outputs — force tool_choice=required in chatbot</t>
+          <t>feat: Admin section -- Planning History + Data Health relocated, new Observability + AI Infrastructure panels</t>
         </is>
       </c>
       <c r="G35" s="81" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>docs/ARCHITECTURE.md, CLAUDE.md</t>
         </is>
       </c>
       <c r="H35" s="82" t="inlineStr">
@@ -19247,10 +19247,14 @@
       <c r="M35" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="N35" s="81" t="n"/>
+      <c r="N35" s="81" t="inlineStr">
+        <is>
+          <t>P6-A28, P6-A27</t>
+        </is>
+      </c>
       <c r="O35" s="81" t="inlineStr">
         <is>
-          <t>Chatbot always calls a tool when one applies; no unexpected freeform responses; existing chatbot tests pass</t>
+          <t>Admin is reachable but not in the primary nav row (secondary menu); Planning History and Data Health render identically to their P6-A28 versions in the new location; Observability shows real per-node latency/status/errors for at least one real run; AI Infrastructure shows real model/provider/cost breakdown; Integrations shows live status for all 7 listed systems (or a clear "not configured" state where no live health-check exists yet).</t>
         </is>
       </c>
     </row>
@@ -19262,32 +19266,32 @@
       </c>
       <c r="B36" s="81" t="inlineStr">
         <is>
-          <t>feature/voice-interface</t>
+          <t>feature/page-redesign</t>
         </is>
       </c>
       <c r="C36" s="81" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Eval</t>
         </is>
       </c>
       <c r="D36" s="81" t="inlineStr">
         <is>
-          <t>Voice interface — Whisper transcription + TTS response</t>
+          <t>Validate action-item specificity after live signals land (conditional)</t>
         </is>
       </c>
       <c r="E36" s="81" t="inlineStr">
         <is>
-          <t>Restaurant operator speaks to CortexKitchen instead of typing. Browser MediaRecorder API captures audio. Whisper (via Groq) transcribes to text. Existing chatbot processes the text query. TTS reads back the response. Use case: manager walking the floor asks questions hands-free. "What does the plan say about staffing tonight?" "How many covers are we expecting?" Add mic button to existing /chat page. Works for operator side only initially.</t>
+          <t>Not a guaranteed code task -- a validation checkpoint. Research confirmed aggregator.py/critic_service.py already favor structured, itemized output (bulleted restock actions, explicit dish names, numeric thresholds, dimension scores) over narrative paragraphs, so the 'standard, generic response' feedback is more likely an input-richness problem than a prompt-engineering problem. After P6-A24 ships, manually review 3-5 generated plans against known-rich live-signal test dates (a rain-forecast night, a real upcoming holiday, an active trend, a live FSSAI notice) to check whether output is now sufficiently specific/actionable. If yes: close this task, no further work needed. If still generic: scope a real follow-up prompt-engineering task against aggregator/critic with concrete before/after examples.</t>
         </is>
       </c>
       <c r="F36" s="81" t="inlineStr">
         <is>
-          <t>feat: voice interface — Whisper transcription + TTS on /chat page</t>
+          <t>None yet -- validation checkpoint, code only if the review finds a real gap</t>
         </is>
       </c>
       <c r="G36" s="81" t="inlineStr">
         <is>
-          <t>docs/PRODUCT_MODES.md (voice mode section)</t>
+          <t>None yet</t>
         </is>
       </c>
       <c r="H36" s="82" t="inlineStr">
@@ -19297,7 +19301,7 @@
       </c>
       <c r="I36" s="80" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J36" s="80" t="inlineStr">
@@ -19310,10 +19314,14 @@
       <c r="M36" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="81" t="n"/>
+      <c r="N36" s="81" t="inlineStr">
+        <is>
+          <t>P6-A24, P6-A26</t>
+        </is>
+      </c>
       <c r="O36" s="81" t="inlineStr">
         <is>
-          <t>Audio recorded and transcribed correctly; chatbot processes transcription; TTS plays response; mic button shows recording state</t>
+          <t>N/A -- manual review checkpoint, not an automated test</t>
         </is>
       </c>
     </row>
@@ -19325,32 +19333,32 @@
       </c>
       <c r="B37" s="81" t="inlineStr">
         <is>
-          <t>feature/eval-pipeline</t>
+          <t>feature/procurement-loop-endtoend</t>
         </is>
       </c>
       <c r="C37" s="81" t="inlineStr">
         <is>
-          <t>Eval</t>
+          <t>Agents</t>
         </is>
       </c>
       <c r="D37" s="81" t="inlineStr">
         <is>
-          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
+          <t>Autonomous procurement loop — end-to-end wire</t>
         </is>
       </c>
       <c r="E37" s="81" t="inlineStr">
         <is>
-          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
+          <t>Connect: weather/holiday signal → demand_forecast surge → inventory shortage detection → ProcurementEnricher Instamart prices → ActionQueue APPROVE_REQUIRED action → trust ladder → checkout (staging creds) OR WhatsApp vendor fallback. This is the flagship restaurant OS demo moment. The plan output must clearly show: shortage detected → Instamart has it at Rs.24/kg → approve to order → or WhatsApp vendor if not on Instamart. Wire trust ladder: orders under Rs.500 auto-approved, over Rs.500 needs manual approval in action queue UI.</t>
         </is>
       </c>
       <c r="F37" s="81" t="inlineStr">
         <is>
-          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
+          <t>feat: autonomous procurement loop — weather → forecast → shortage → Instamart → action queue</t>
         </is>
       </c>
       <c r="G37" s="81" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CLAUDE.md, docs/ARCHITECTURE.md (procurement loop diagram)</t>
         </is>
       </c>
       <c r="H37" s="82" t="inlineStr">
@@ -19360,7 +19368,7 @@
       </c>
       <c r="I37" s="80" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J37" s="80" t="inlineStr">
@@ -19375,56 +19383,172 @@
       </c>
       <c r="N37" s="81" t="inlineStr">
         <is>
-          <t>P6-A30</t>
+          <t>P6-A24</t>
         </is>
       </c>
       <c r="O37" s="81" t="inlineStr">
         <is>
-          <t>CI eval gate passes; golden_runs.json reflects current system; regressions caught in 2+ test scenarios</t>
+          <t>Full loop runs end-to-end in demo; trust ladder fires correctly; action queue shows Instamart procurement with price + spinId; WhatsApp fallback triggers when product not found on Instamart</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="80" t="inlineStr">
+        <is>
+          <t>P6-A36</t>
+        </is>
+      </c>
+      <c r="B38" s="81" t="inlineStr">
+        <is>
+          <t>feature/instamart-event-supplies</t>
+        </is>
+      </c>
+      <c r="C38" s="81" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D38" s="81" t="inlineStr">
+        <is>
+          <t>Instamart event supplies in operator chatbot</t>
+        </is>
+      </c>
+      <c r="E38" s="81" t="inlineStr">
+        <is>
+          <t>Extend operator chatbot with event supplies tool: "we are hosting a birthday event tonight, need supplies." Calls search_products for non-food items: candles, paper plates, cups, napkins, soft drinks, basic decorations, cleaning supplies, batteries. Returns real Instamart prices and availability. Creates ActionQueue procurement action for approval. Key insight: Instamart is not just food ingredients — managers use it for quick supply runs that previously required leaving the restaurant. New chatbot tool: get_event_supplies(event_type, headcount)</t>
+        </is>
+      </c>
+      <c r="F38" s="81" t="inlineStr">
+        <is>
+          <t>feat: Instamart event supplies tool in operator chatbot</t>
+        </is>
+      </c>
+      <c r="G38" s="81" t="inlineStr">
+        <is>
+          <t>docs/AGENTS.md (chatbot tools updated)</t>
+        </is>
+      </c>
+      <c r="H38" s="82" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I38" s="80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J38" s="80" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K38" s="80" t="n"/>
+      <c r="L38" s="80" t="n"/>
+      <c r="M38" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="81" t="n"/>
+      <c r="O38" s="81" t="inlineStr">
+        <is>
+          <t>search_products returns real results for non-food queries; ActionQueue action created; trust ladder applied; chatbot responds naturally to event supply requests</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="110" t="inlineStr">
-        <is>
-          <t>DOCS + SYNC — end of Phase 6A</t>
+      <c r="A39" s="107" t="inlineStr">
+        <is>
+          <t>P6-A37</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>feature/structured-outputs</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Agents</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Structured outputs -- tool_choice=required across chatbot</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Force structured JSON outputs from Groq function calling. Eliminates cases where chatbot returns freeform text instead of calling the right tool. Add response validation layer. Makes chatbot more reliable for demo -- no unexpected text responses.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>feat: structured outputs -- force tool_choice=required in chatbot</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Chatbot always calls a tool when one applies; no unexpected freeform responses; existing chatbot tests pass</t>
         </is>
       </c>
     </row>
     <row r="40" ht="118.8" customHeight="1" s="84">
-      <c r="A40" s="111" t="inlineStr">
-        <is>
-          <t>P6-A36</t>
+      <c r="A40" s="80" t="inlineStr">
+        <is>
+          <t>P6-A38</t>
         </is>
       </c>
       <c r="B40" s="81" t="inlineStr">
         <is>
-          <t>feature/documentation</t>
+          <t>feature/voice-interface</t>
         </is>
       </c>
       <c r="C40" s="81" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D40" s="81" t="inlineStr">
         <is>
-          <t>Whole-system documentation + screenshots refresh</t>
+          <t>Voice interface — Whisper transcription + TTS response</t>
         </is>
       </c>
       <c r="E40" s="81" t="inlineStr">
         <is>
-          <t>Update all docs to reflect: new two-sided product vision, compliance changes (Zomato removed, market intel anonymised), autonomous procurement loop, weather signals, voice interface. New product vision statement in README. Screenshots of the operator portal (dashboard, operations, market, action queue, chat) for portfolio -- Guest Concierge screenshots belong to Phase 6B docs (P6-B9), not here, since Guest Concierge does not exist yet at this point.</t>
+          <t>Restaurant operator speaks to CortexKitchen instead of typing. Browser MediaRecorder API captures audio. Whisper (via Groq) transcribes to text. Existing chatbot processes the text query. TTS reads back the response. Use case: manager walking the floor asks questions hands-free. "What does the plan say about staffing tonight?" "How many covers are we expecting?" Add mic button to existing /chat page. Works for operator side only initially.</t>
         </is>
       </c>
       <c r="F40" s="81" t="inlineStr">
         <is>
-          <t>docs: whole-system documentation refresh — new product vision</t>
+          <t>feat: voice interface — Whisper transcription + TTS on /chat page</t>
         </is>
       </c>
       <c r="G40" s="81" t="inlineStr">
         <is>
-          <t>README.md, docs/ARCHITECTURE.md, docs/AGENTS.md, CLAUDE.md</t>
+          <t>docs/PRODUCT_MODES.md (voice mode section)</t>
         </is>
       </c>
       <c r="H40" s="82" t="inlineStr">
@@ -19447,51 +19571,47 @@
       <c r="M40" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="N40" s="81" t="inlineStr">
-        <is>
-          <t>P6-A34</t>
-        </is>
-      </c>
+      <c r="N40" s="81" t="n"/>
       <c r="O40" s="81" t="inlineStr">
         <is>
-          <t>README reflects two-sided platform; all compliance changes documented; screenshots current</t>
+          <t>Audio recorded and transcribed correctly; chatbot processes transcription; TTS plays response; mic button shows recording state</t>
         </is>
       </c>
     </row>
     <row r="41" ht="52.8" customHeight="1" s="84">
-      <c r="A41" s="111" t="inlineStr">
-        <is>
-          <t>P6-A37</t>
+      <c r="A41" s="80" t="inlineStr">
+        <is>
+          <t>P6-A39</t>
         </is>
       </c>
       <c r="B41" s="81" t="inlineStr">
         <is>
-          <t>dev -&gt; main</t>
+          <t>feature/eval-pipeline</t>
         </is>
       </c>
       <c r="C41" s="81" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Eval</t>
         </is>
       </c>
       <c r="D41" s="81" t="inlineStr">
         <is>
-          <t>Sync Phase 6A to main</t>
+          <t>Promote RAGAS/DeepEval candidates + regenerate golden runs</t>
         </is>
       </c>
       <c r="E41" s="81" t="inlineStr">
         <is>
-          <t>Merge dev → main. All compliance fixes confirmed. Autonomous procurement loop working (minus checkout — staging creds). Restaurant OS demo-ready. Phase 6B starts after this.</t>
+          <t>Review RAGAS and DeepEval eval candidates. Promote passing ones to the CI gate. Regenerate golden_runs.json against real planning data. Ensures eval pipeline catches regressions after compliance changes and new feature additions.</t>
         </is>
       </c>
       <c r="F41" s="81" t="inlineStr">
         <is>
-          <t>release: Phase 6A complete — restaurant OS + compliance fixes</t>
+          <t>feat: eval pipeline — promote RAGAS/DeepEval + regenerate golden runs</t>
         </is>
       </c>
       <c r="G41" s="81" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H41" s="82" t="inlineStr">
@@ -19501,7 +19621,7 @@
       </c>
       <c r="I41" s="80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J41" s="80" t="inlineStr">
@@ -19516,10 +19636,151 @@
       </c>
       <c r="N41" s="81" t="inlineStr">
         <is>
-          <t>P6-A35</t>
+          <t>P6-A34</t>
         </is>
       </c>
       <c r="O41" s="81" t="inlineStr">
+        <is>
+          <t>CI eval gate passes; golden_runs.json reflects current system; regressions caught in 2+ test scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="110" t="inlineStr">
+        <is>
+          <t>DOCS + SYNC — end of Phase 6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="111" t="inlineStr">
+        <is>
+          <t>P6-A40</t>
+        </is>
+      </c>
+      <c r="B44" s="81" t="inlineStr">
+        <is>
+          <t>feature/documentation</t>
+        </is>
+      </c>
+      <c r="C44" s="81" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D44" s="81" t="inlineStr">
+        <is>
+          <t>Whole-system documentation + screenshots refresh</t>
+        </is>
+      </c>
+      <c r="E44" s="81" t="inlineStr">
+        <is>
+          <t>Update all docs to reflect: new two-sided product vision, compliance changes (Zomato removed, market intel anonymised), autonomous procurement loop, weather signals, voice interface. New product vision statement in README. Screenshots of the operator portal (dashboard, operations, market, action queue, chat) for portfolio -- Guest Concierge screenshots belong to Phase 6B docs (P6-B9), not here, since Guest Concierge does not exist yet at this point.</t>
+        </is>
+      </c>
+      <c r="F44" s="81" t="inlineStr">
+        <is>
+          <t>docs: whole-system documentation refresh — new product vision</t>
+        </is>
+      </c>
+      <c r="G44" s="81" t="inlineStr">
+        <is>
+          <t>README.md, docs/ARCHITECTURE.md, docs/AGENTS.md, CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="H44" s="82" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I44" s="80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J44" s="80" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K44" s="80" t="n"/>
+      <c r="L44" s="80" t="n"/>
+      <c r="M44" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="81" t="inlineStr">
+        <is>
+          <t>P6-A38</t>
+        </is>
+      </c>
+      <c r="O44" s="81" t="inlineStr">
+        <is>
+          <t>README reflects two-sided platform; all compliance changes documented; screenshots current</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="111" t="inlineStr">
+        <is>
+          <t>P6-A41</t>
+        </is>
+      </c>
+      <c r="B45" s="81" t="inlineStr">
+        <is>
+          <t>dev -&gt; main</t>
+        </is>
+      </c>
+      <c r="C45" s="81" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D45" s="81" t="inlineStr">
+        <is>
+          <t>Sync Phase 6A to main</t>
+        </is>
+      </c>
+      <c r="E45" s="81" t="inlineStr">
+        <is>
+          <t>Merge dev → main. All compliance fixes confirmed. Autonomous procurement loop working (minus checkout — staging creds). Restaurant OS demo-ready. Phase 6B starts after this.</t>
+        </is>
+      </c>
+      <c r="F45" s="81" t="inlineStr">
+        <is>
+          <t>release: Phase 6A complete — restaurant OS + compliance fixes</t>
+        </is>
+      </c>
+      <c r="G45" s="81" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="H45" s="82" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="I45" s="80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J45" s="80" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K45" s="80" t="n"/>
+      <c r="L45" s="80" t="n"/>
+      <c r="M45" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="81" t="inlineStr">
+        <is>
+          <t>P6-A39</t>
+        </is>
+      </c>
+      <c r="O45" s="81" t="inlineStr">
         <is>
           <t>Full test suite green; compliance fixes verified; no Zomato references; market intel anonymised; demo flow works</t>
         </is>
@@ -19527,11 +19788,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A43:O43"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A22:O22"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A3:O3"/>
-    <mergeCell ref="A39:O39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tracker: mark P6-A29 (seed data redesign) Completed
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -18965,7 +18965,7 @@
       </c>
       <c r="H31" s="82" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I31" s="80" t="inlineStr">
@@ -18981,12 +18981,12 @@
       <c r="K31" s="80" t="n"/>
       <c r="L31" s="80" t="n"/>
       <c r="M31" s="80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" s="81" t="n"/>
       <c r="O31" s="81" t="inlineStr">
         <is>
-          <t>Running the seed script twice on the same real-world day produces identical data (deterministic within a day); running it on two different days produces different shortage items and different popular dishes; no single ingredient/dish is hardcoded as always-short/always-popular in the script; RAG/decision-log memory content matches whatever was actually seeded that day, not a fixed string; at least 3 vendors offer quotes across at least 6 distinct ingredients.</t>
+          <t>VERIFIED: same-day reseed (run twice) produced identical shortages both times (Burger Buns, Cold Brew Coffee on 2026-07-13); isolated random.seed test confirmed three different dates produce three different draws; direct DB query confirmed decision-log input_summary/action_recommended text matches the actually-seeded low ingredients (not stale hardcoded names) and the comfortable-item note correctly names different ingredients (Mozzarella Cheese, Pizza Dough) that were NOT low this run; 14 vendor price quotes across 12 ingredients confirmed in DB. 544/544 backend tests pass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: post-merge update -- feature/phase6b-guest-concierge closed out
Dashboard sheet: Guest Concierge (P6-A34) marked delivered and no longer
gated on Swiggy consent, Phase 6B row superseded with the corrected
compliance reasoning, Phase 6 progress recalculated to 91%, and the
current-milestone narrative brought up to date.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -1136,12 +1136,15 @@
     <row r="3" ht="14.4" customHeight="1" s="96">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Current: Phase 6A (restaurant OS) -- compliance batch, live-intelligence signals, scenario overhaul, and the Dashboard/Planning/Action Center/Analytics/Data IA redesign are all DONE (P6-A1-A30). Of the UI redesign branch (feature/ui-redesign, P6-A31-A34), P6-A33 (AI Assistant page redesign) is now DONE -- P6-A31 (Action Center tabs), P6-A32 (Analytics 5-section + Menu Matrix), and P6-A34 (Admin panels + connector expansion) are still pending on this same branch. A single debugging session on this branch (2026-07-31) also surfaced and fixed five significant unplanned issues, tracked as P6-A45-A50: two live-intelligence data-integrity bugs (FSSAI site redesign silently broke ComplianceAlertsService; TrendsService was returning empty most days due to a redirect bug + a feed-fairness bug), a manual refresh control for all three live-signal surfaces, and two CRITICAL chat backend bugs -- the chat assistant was 100% broken (every message crashed) due to a DB-session lifecycle bug, and even once fixed, an unbounded Instamart tool result was blowing the Groq free-tier rate limit on ordinary questions. None of this was part of the original plan; all of it is now fixed and verified live against the running app, not just unit tests. Voice interface + chatbot capability expansion (feature/voice-and-chatbot-capabilities, P6-A35-A38), eval/observability/CI (P6-A39-A41), e2e hardening (P6-A42), and docs + sync to main (P6-A43-A44) remain fully ahead and untouched by this session -- Phase 6A is NOT close to done just because of this session's volume of work.</t>
+          <t>Current: Phase 6A (restaurant OS) -- compliance batch, live-intelligence signals, scenario overhaul, and the Dashboard/Planning/Action Center/Analytics/Data IA redesign are all DONE (P6-A1-A30). Of the UI redesign branch (feature/ui-redesign, P6-A31-A34): P6-A32's ComplianceAlertsService/TrendsService fixes + manual refresh control, and P6-A33 (AI Assistant page redesign) are DONE, along with five unplanned bug fixes surfaced during that same debugging session (live-intelligence data-integrity, a 100%-reproducible chat crash, a chat rate-limit failure mode). P6-A31 (Action Center tabs) and P6-A32 (Analytics 5-section + Menu Matrix) remain Planned.
+Last completed branch: feature/phase6b-guest-concierge (P6-A34), merged to dev 2026-08-03. Delivered Guest Concierge -- a no-auth ReAct agent over Swiggy's Food/Instamart/Dineout MCP servers (venue search + booking, food ordering, event-supplies sourcing), as a second, independent platform side with its own /concierge frontend. Same branch also shipped the two-sided homepage redesign, voice input (Whisper transcription) across Dashboard/Planning/chat/Concierge, Market Intelligence page reliability fixes (card-vanishing + a real SSR hydration bug), and a full rewrite of all 22 reference documentation files for accuracy.
+Guest Concierge required no separate Swiggy consent to build -- it is the Proposed Arrangement described in clause 1.1 of the signed Integration Agreement, not a gated feature. The earlier plan to gate it behind written consent under clause 2.1(v) (see row 4, now superseded) was a misreading of the agreement, corrected in docs/DECISIONS.md.
+Next recommended branch: P6-A31 (Action Center tabs) or P6-A32 (Analytics 5-section + Menu Matrix) to close out feature/ui-redesign, then eval/observability/CI automation, e2e hardening, and docs + sync to main.</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Phase 6A: 31 of 44 originally-planned tasks done (P6-A1-A30, A33), plus 6 unplanned fixes (P6-A45-A50) this session. Still pending on feature/ui-redesign: P6-A31, A32, A34. Then, in order: voice + chatbot capabilities branch (A35-A38), eval/observability/CI branch (A39-A41), e2e hardening (A42), docs + sync to main (A43-A44). Then Phase 6B.</t>
+          <t>Phase 6A sheet: 34 of 41 active tasks done. Phase 6 (legacy) sheet: 51 of 55 done, 4 superseded. Guest Concierge (P6-A34) delivered and merged to dev -- no longer gated on Swiggy consent. Still pending: P6-A31 (Action Center tabs), P6-A32 (Analytics 5-section + Menu Matrix), then eval/observability/CI, e2e hardening, and docs + sync to main.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1172,7 +1175,7 @@
     <row r="4" ht="14.4" customHeight="1" s="96">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Phase 6B: guest concierge -- 9 tasks (P6-B1-B9), gated on P6-B1 (Swiggy written consent, clause 2.1v) before any code.</t>
+          <t>Superseded: the original Phase 6B plan (guest concierge as 9 separately-scoped tasks, P6-B1-B9, gated on Swiggy written consent under clause 2.1(v)) never shipped as planned. Guest Concierge was instead delivered inside Phase 6A as P6-A34 (feature/phase6b-guest-concierge, merged to dev 2026-08-03) -- no separate consent was required, since it falls under clause 1.1's Proposed Arrangement. See docs/DECISIONS.md for the corrected compliance reasoning.</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -1208,7 +1211,7 @@
     <row r="5" ht="14.4" customHeight="1" s="96">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Staging creds unlock: the real Instamart checkout() call (bulk-order option surfaced in P6-A38 already works up to approval as a peer option to WhatsApp; the final live checkout is what's still blocked) + Dineout book_table (P6-B5 Guest Concierge). Also P6-B7 Guest Concierge Instamart event supplies.</t>
+          <t>Staging creds unlock: the real Instamart checkout() call (bulk-order option already works up to approval as a peer option to WhatsApp; the final live checkout is what's still blocked) + Dineout book_table and Instamart checkout for Guest Concierge (implemented in ConciergeService as part of P6-A34, blocked on the same staging credentials).</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1244,7 +1247,7 @@
     <row r="6" ht="14.4" customHeight="1" s="96">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Compliance: P6-A19 (remove Zomato stub) + P6-A20 (anonymise market intel) -- DONE, merged to dev.</t>
+          <t>Compliance: P6-A19 (remove Zomato stub) + P6-A20 (anonymise market intel) -- DONE, merged to dev. Guest Concierge (P6-A34) confirmed compliant under clause 1.1 (Proposed Arrangement) -- no separate consent required; see docs/DECISIONS.md.</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1641,11 +1644,11 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>0.7813</v>
+        <v>0.91</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Swiggy-native restaurant OS: connector layer, fourteen-node LangGraph pipeline, Action Queue with approval gates + trust ladder + WhatsApp execution, financial scorecard, MCP server + in-app chatbot tool parity, live-intelligence signals, dynamic scenario composition, Langfuse/Kindred replay, Dashboard/Planning/Action Center/Analytics/Data page split. Next: eval/CI/observability automation, then a unified UI redesign round.</t>
+          <t>Swiggy-native restaurant OS: connector layer, fifteen-node LangGraph pipeline, Action Queue with approval gates + an informational trust-ladder badge + WhatsApp execution, financial scorecard, MCP server + in-app chatbot tool parity, live-intelligence signals, dynamic scenario composition, Langfuse/Kindred replay, Dashboard/Planning/Action Center/Analytics/Data page split, plus Guest Concierge -- a no-auth consumer event-planning agent over Swiggy Food/Instamart/Dineout, delivered as a second, independent platform side (P6-A34). Next: Action Center tabs (P6-A31), Analytics 5-section redesign (P6-A32), eval/CI/observability automation, e2e hardening, then docs + sync to main.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: close out P6-A44 -- dev synced to main
Marks the dev-to-main milestone merge (364 files, +43,141/-6,043) as
Completed, done ahead of the originally planned sequence -- Action
Center tabs, Analytics redesign, and the screenshot recapture remain
outstanding on dev. Retires the stale Phase 6B consent-gating plan;
Guest Concierge already shipped as P6-A34 before this merge.
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker.xlsx
+++ b/CortexKitchen_Progress_Tracker.xlsx
@@ -1139,7 +1139,8 @@
           <t>Current: Phase 6A (restaurant OS) -- compliance batch, live-intelligence signals, scenario overhaul, and the Dashboard/Planning/Action Center/Analytics/Data IA redesign are all DONE (P6-A1-A30). Of the UI redesign branch (feature/ui-redesign, P6-A31-A34): P6-A32's ComplianceAlertsService/TrendsService fixes + manual refresh control, and P6-A33 (AI Assistant page redesign) are DONE, along with five unplanned bug fixes surfaced during that same debugging session (live-intelligence data-integrity, a 100%-reproducible chat crash, a chat rate-limit failure mode). P6-A31 (Action Center tabs) and P6-A32 (Analytics 5-section + Menu Matrix) remain Planned.
 Last completed branch: feature/phase6b-guest-concierge (P6-A34), merged to dev 2026-08-03. Delivered Guest Concierge -- a no-auth ReAct agent over Swiggy's Food/Instamart/Dineout MCP servers (venue search + booking, food ordering, event-supplies sourcing), as a second, independent platform side with its own /concierge frontend. Same branch also shipped the two-sided homepage redesign, voice input (Whisper transcription) across Dashboard/Planning/chat/Concierge, Market Intelligence page reliability fixes (card-vanishing + a real SSR hydration bug), and a full rewrite of all 22 reference documentation files for accuracy.
 Guest Concierge required no separate Swiggy consent to build -- it is the Proposed Arrangement described in clause 1.1 of the signed Integration Agreement, not a gated feature. The earlier plan to gate it behind written consent under clause 2.1(v) (see row 4, now superseded) was a misreading of the agreement, corrected in docs/DECISIONS.md.
-Next recommended branch: P6-A31 (Action Center tabs) or P6-A32 (Analytics 5-section + Menu Matrix) to close out feature/ui-redesign, then eval/observability/CI automation, e2e hardening, and docs + sync to main.</t>
+Next recommended branch: P6-A31 (Action Center tabs) or P6-A32 (Analytics 5-section + Menu Matrix) to close out feature/ui-redesign, then eval/observability/CI automation, e2e hardening, and docs + sync to main.
+Main sync: dev merged to main 2026-08-03 (364 files, +43,141/-6,043 lines) -- everything through Guest Concierge (P6-A34) is now on main. This went ahead of P6-A31/A32 (Action Center tabs, Analytics redesign) and the P6-A43 screenshot recapture, both still outstanding on dev.</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -20015,7 +20016,7 @@
       </c>
       <c r="E56" s="81" t="inlineStr">
         <is>
-          <t>Refresh CLAUDE.md and all docs/ files to match the fully implemented Phase 6A state (UI redesign, voice interface, chatbot capability expansion, eval/CI/observability work, e2e hardening) -- same standard as the prior 2026-07-06 docs rewrite (release-quality, matched to code, no stale content). Replace outdated screenshots across README/docs with current UI.</t>
+          <t>Documentation half of this task is done: all 22 markdown files in the repo audited, 16 rewritten for accuracy against the fully implemented Phase 6A state (Swiggy integration, live signals, IA redesign, Guest Concierge), internal task/decision IDs removed throughout. Screenshot half is NOT done -- the outdated screenshots/ directory was deleted rather than replaced; README now says "Screenshots coming soon" as an honest placeholder until a fresh set is captured against the redesigned UI.</t>
         </is>
       </c>
       <c r="F56" s="93" t="inlineStr">
@@ -20030,7 +20031,7 @@
       </c>
       <c r="H56" s="71" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="I56" s="93" t="inlineStr">
@@ -20046,7 +20047,7 @@
       <c r="K56" s="93" t="n"/>
       <c r="L56" s="93" t="n"/>
       <c r="M56" s="93" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N56" s="93" t="inlineStr">
         <is>
@@ -20082,12 +20083,12 @@
       </c>
       <c r="E57" s="81" t="inlineStr">
         <is>
-          <t>Merge dev -&gt; main once P6-A31-A43 are all done and verified. Marks the close of this Phase 6A milestone. Phase 6B (Guest Concierge) starts only after this merge, and only once P6-B1 (Swiggy written consent) clears -- not before.</t>
+          <t>Merged dev to main via GitHub PR on 2026-08-03, ahead of the original planned sequence: P6-A31 (Action Center tabs) and P6-A32 (Analytics 5-section + Menu Matrix) are still Planned, and P6-A43's screenshot capture is still outstanding. The merge went ahead as a deliberate call to ship the Guest Concierge milestone now rather than wait on the remaining UI polish items. The note that Phase 6B (Guest Concierge) would start only after this merge and only once Swiggy written consent cleared was based on a misreading of the signed agreement -- Guest Concierge shipped as P6-A34, ahead of this merge, requiring no separate consent. 364 files changed, +43,141/-6,043 lines.</t>
         </is>
       </c>
       <c r="F57" s="93" t="inlineStr">
         <is>
-          <t>release: Phase 6A milestone -- dev to main sync</t>
+          <t>release: Swiggy-native platform, Guest Concierge, and full frontend redesign -- dev to main sync</t>
         </is>
       </c>
       <c r="G57" s="93" t="inlineStr">
@@ -20097,7 +20098,7 @@
       </c>
       <c r="H57" s="71" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I57" s="93" t="inlineStr">
@@ -20110,10 +20111,18 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="K57" s="93" t="n"/>
-      <c r="L57" s="93" t="n"/>
+      <c r="K57" s="93" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="L57" s="93" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
       <c r="M57" s="93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N57" s="93" t="inlineStr">
         <is>

</xml_diff>